<commit_message>
docs(tc2-3): chuẩn hóa nội dung văn phong chuyên nghiệp cho cột prompt W07 của Thắng
</commit_message>
<xml_diff>
--- a/docs/evidence/tc2-3-ai-usage/AI Prompt Log - W07 - 2026-10-26_2026-11-01.xlsx
+++ b/docs/evidence/tc2-3-ai-usage/AI Prompt Log - W07 - 2026-10-26_2026-11-01.xlsx
@@ -696,12 +696,12 @@
       </c>
       <c r="D6" s="38" t="inlineStr">
         <is>
-          <t>Cấu hình bảo mật danh tính Git và chuyển thông tin email cá nhân</t>
+          <t>Cấu hình danh tính Git cá nhân và bảo mật thông tin tác giả commit</t>
         </is>
       </c>
       <c r="E6" s="38" t="inlineStr">
         <is>
-          <t>đăng xuất đi, đổi git config lại email đừng lộ @runsystem</t>
+          <t>Đăng xuất thông tin xác thực cũ và cấu hình lại Git config (user.name, user.email) với email cá nhân để đảm bảo không để lộ email tổ chức/doanh nghiệp trong lịch sử commit.</t>
         </is>
       </c>
       <c r="F6" s="38" t="inlineStr">
@@ -726,12 +726,12 @@
       </c>
       <c r="D7" s="41" t="inlineStr">
         <is>
-          <t>Xác thực và đăng nhập tài khoản GitHub cá nhân thanglb2005</t>
+          <t>Xác thực và đăng nhập GitHub CLI với tài khoản cá nhân thanglb2005</t>
         </is>
       </c>
       <c r="E7" s="41" t="inlineStr">
         <is>
-          <t>đăng nhập github đi</t>
+          <t>Kiểm tra và thực hiện đăng nhập tài khoản GitHub cá nhân thanglb2005 qua GitHub CLI (gh auth login) để chuẩn bị thao tác trên repository.</t>
         </is>
       </c>
       <c r="F7" s="41" t="inlineStr">
@@ -761,7 +761,7 @@
       </c>
       <c r="E8" s="41" t="inlineStr">
         <is>
-          <t>vào check repo xem pull hết code chưa nha, sau đó vào jira check 6 task tôi sẽ làm trong week 7</t>
+          <t>Kiểm tra trạng thái repository, đồng bộ nhánh và đối chiếu danh sách 6 task được phân công cho Thắng trong sprint W7 trên bảng Jira backlog (SCRUM-91, SCRUM-92, SCRUM-98, SCRUM-99, SCRUM-100, SCRUM-101).</t>
         </is>
       </c>
       <c r="F8" s="41" t="inlineStr">
@@ -786,12 +786,12 @@
       </c>
       <c r="D9" s="41" t="inlineStr">
         <is>
-          <t>Đồng bộ kéo toàn bộ commit mới nhất từ nhánh remote main</t>
+          <t>Đồng bộ toàn bộ commit mới nhất từ nhánh remote main</t>
         </is>
       </c>
       <c r="E9" s="41" t="inlineStr">
         <is>
-          <t>pull hết code đi</t>
+          <t>Kéo và cập nhật toàn bộ commit mới nhất từ nhánh remote main về local workspace để đảm bảo codebase luôn ở phiên bản mới nhất.</t>
         </is>
       </c>
       <c r="F9" s="41" t="inlineStr">
@@ -816,12 +816,12 @@
       </c>
       <c r="D10" s="41" t="inlineStr">
         <is>
-          <t>Đọc mã nguồn, tạo nhánh feat/SCRUM-* và triển khai tuần tự 6 task W7 kèm PR</t>
+          <t>Triển khai 6 task W7 của Thắng trên các nhánh tính năng feat/SCRUM-* và tạo PR</t>
         </is>
       </c>
       <c r="E10" s="41" t="inlineStr">
         <is>
-          <t>Đọc src liên quan, giờ làm tất cả task của tôi đi, mỗi task tạo 1 nhánh đặt tên cho chuẩn ví dụ feat/SCRUM-92-W7-G2-Tich-hop-va-đua-nhanh-migrate-w7-repo-goc-vao-main , khi làm xong task thì tạo PR nha</t>
+          <t>Nghiên cứu mã nguồn liên quan từ repo gốc và repo nộp bài, thực hiện triển khai toàn bộ các task W7 của Thắng theo từng nhánh tính năng đặt tên chuẩn feat/SCRUM-*, sau khi hoàn thiện mỗi task thì tạo Pull Request tương ứng.</t>
         </is>
       </c>
       <c r="F10" s="41" t="inlineStr">
@@ -846,12 +846,12 @@
       </c>
       <c r="D11" s="41" t="inlineStr">
         <is>
-          <t>Tiếp tục hoàn thiện chuyển các module M02, M08, M11, M14 và kênh tính lượt NetID</t>
+          <t>Hoàn thiện porting các module M02, M08, M11, M14 và kênh tính lượt NetID kèm test</t>
         </is>
       </c>
       <c r="E11" s="41" t="inlineStr">
         <is>
-          <t>continue</t>
+          <t>Tiếp tục hoàn thiện việc port mã nguồn các module M02 (audio QC), M08/M11 (auth, identity, accounts) và M14 (billing, gateways, metering NetID) từ repo gốc sang nhánh tích hợp kèm bộ test đầy đủ.</t>
         </is>
       </c>
       <c r="F11" s="41" t="inlineStr">
@@ -876,12 +876,12 @@
       </c>
       <c r="D12" s="41" t="inlineStr">
         <is>
-          <t>Rà soát kỹ lưỡng mã nguồn, rebase giải quyết conflict, kiểm tra lint, test, provenance và check_forbidden_files</t>
+          <t>Rà soát toàn diện mã nguồn, rebase giải quyết xung đột và chạy kiểm thử an toàn</t>
         </is>
       </c>
       <c r="E12" s="41" t="inlineStr">
         <is>
-          <t>review kĩ lại đi nha</t>
+          <t>Rà soát kỹ lưỡng toàn bộ mã nguồn trên các nhánh PR, rebase giải quyết xung đột với nhánh migrate/w7-repo-goc, kiểm tra chất lượng code qua ruff, pytest, provenance nguồn và bộ công cụ kiểm tra check_forbidden_files, check_md_links.</t>
         </is>
       </c>
       <c r="F12" s="41" t="inlineStr">
@@ -906,12 +906,12 @@
       </c>
       <c r="D13" s="41" t="inlineStr">
         <is>
-          <t>Phê duyệt và merge toàn bộ 6 PR vào nhánh tích hợp và main</t>
+          <t>Phê duyệt và merge toàn bộ 6 PR (#61–#66) vào nhánh tích hợp và main</t>
         </is>
       </c>
       <c r="E13" s="41" t="inlineStr">
         <is>
-          <t>oke duyệt PR và merge hết đi</t>
+          <t>Phê duyệt các PR hợp lệ (#61–#65) và merge tuần tự vào nhánh tích hợp migrate/w7-repo-goc, sau đó đồng bộ nhánh tích hợp vào nhánh feat/SCRUM-92 để merge PR #66 vào main.</t>
         </is>
       </c>
       <c r="F13" s="41" t="inlineStr">
@@ -936,12 +936,12 @@
       </c>
       <c r="D14" s="41" t="inlineStr">
         <is>
-          <t>Kiểm tra và cập nhật trạng thái 6 task W7 sang Done trên Jira board</t>
+          <t>Đối chiếu tiêu chí nghiệm thu và cập nhật trạng thái Done cho 6 task W7 trên Jira</t>
         </is>
       </c>
       <c r="E14" s="41" t="inlineStr">
         <is>
-          <t>bên jira 6task đó để done hết nha</t>
+          <t>Đối chiếu kết quả merge PR với các tiêu chí nghiệm thu của 6 task sprint W7 trên bảng Jira, hướng dẫn và cập nhật trạng thái của tất cả 6 task sang Done.</t>
         </is>
       </c>
       <c r="F14" s="41" t="inlineStr">
@@ -966,12 +966,12 @@
       </c>
       <c r="D15" s="41" t="inlineStr">
         <is>
-          <t>Rà soát toàn diện docs/plan/week-07.md đối chiếu hiện trạng công việc của Thắng</t>
+          <t>Rà soát docs/plan/week-07.md đối chiếu hiện trạng và điều kiện nghiệm thu DoD</t>
         </is>
       </c>
       <c r="E15" s="41" t="inlineStr">
         <is>
-          <t>xem trong docs/plan xem task giao tôi còn cnao chưa làm kh, tôi là thắng</t>
+          <t>Rà soát toàn diện các file kế hoạch trong docs/plan/ (đặc biệt là docs/plan/week-07.md) để đối chiếu mọi nhiệm vụ được giao cho Thắng và xác nhận các điều kiện hoàn thành (DoD).</t>
         </is>
       </c>
       <c r="F15" s="41" t="inlineStr">
@@ -996,12 +996,12 @@
       </c>
       <c r="D16" s="41" t="inlineStr">
         <is>
-          <t>Đóng tag git w7-feature-freeze và khởi tạo, cập nhật AI Prompt Log W07</t>
+          <t>Gắn tag Git w7-feature-freeze và khởi tạo, cập nhật AI Prompt Log W07</t>
         </is>
       </c>
       <c r="E16" s="41" t="inlineStr">
         <is>
-          <t>jira t làm rồi, cái kia bạn làm giùm, với lại bạn làm file AI Promt log w7 chưa, fill đi</t>
+          <t>Tạo và đẩy Git tag w7-feature-freeze lên remote theo yêu cầu DoD W7-G2, đồng thời khởi tạo workbook AI Prompt Log W07 với đầy đủ 4 sheet chuẩn và ghi nhận nhật ký sử dụng AI trong tuần.</t>
         </is>
       </c>
       <c r="F16" s="41" t="inlineStr">

</xml_diff>

<commit_message>
feat(SCRUM-103): migrate M15 pages and E2E
</commit_message>
<xml_diff>
--- a/docs/evidence/tc2-3-ai-usage/AI Prompt Log - W07 - 2026-10-26_2026-11-01.xlsx
+++ b/docs/evidence/tc2-3-ai-usage/AI Prompt Log - W07 - 2026-10-26_2026-11-01.xlsx
@@ -1,14 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet name="Thắng" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Nguyên" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Sang" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Tổng hợp" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thắng" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nguyên" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sang" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tổng hợp" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
+  <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
 </file>
 
@@ -6908,20 +6909,64 @@
       </c>
     </row>
     <row r="6" ht="48" customHeight="1" s="24">
-      <c r="A6" s="32" t="n"/>
-      <c r="B6" s="18" t="n"/>
-      <c r="C6" s="18" t="n"/>
-      <c r="D6" s="33" t="n"/>
-      <c r="E6" s="33" t="n"/>
-      <c r="F6" s="33" t="n"/>
+      <c r="A6" s="32" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>Nguyên</t>
+        </is>
+      </c>
+      <c r="C6" s="18" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="D6" s="33" t="inlineStr">
+        <is>
+          <t>Đọc Jira SCRUM-103; chuyển giao M15 và rà soát kiểm thử E2E</t>
+        </is>
+      </c>
+      <c r="E6" s="33" t="inlineStr">
+        <is>
+          <t>Đóng vai trò như 1 người senior trong lĩnh vực IT và hãy làm task SCRUM-103 trên nhánh SCRUM/103 đã tạo từ đầu và hãy đọc trên jira để có thể làm</t>
+        </is>
+      </c>
+      <c r="F6" s="33" t="inlineStr">
+        <is>
+          <t>../../sdd/modules/m15-product-web/reviews/implementation-transfer-scrum-103-2026-10-28.md</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="48" customHeight="1" s="24">
-      <c r="A7" s="32" t="n"/>
-      <c r="B7" s="18" t="n"/>
-      <c r="C7" s="18" t="n"/>
-      <c r="D7" s="33" t="n"/>
-      <c r="E7" s="33" t="n"/>
-      <c r="F7" s="33" t="n"/>
+      <c r="A7" s="32" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B7" s="18" t="inlineStr">
+        <is>
+          <t>Nguyên</t>
+        </is>
+      </c>
+      <c r="C7" s="18" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="D7" s="33" t="inlineStr">
+        <is>
+          <t>Mở rộng SCRUM-103 sang middleware M16 để gỡ blocker khởi động; kiểm thử hồi quy</t>
+        </is>
+      </c>
+      <c r="E7" s="33" t="inlineStr">
+        <is>
+          <t>Bạn muốn mình mở rộng phạm vi để sửa middleware M16 trên nhánh này mở rộng đi</t>
+        </is>
+      </c>
+      <c r="F7" s="33" t="inlineStr">
+        <is>
+          <t>../../sdd/modules/m16-monolith-runtime/evidence/scrum-103-middleware-integration.md</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="36" customHeight="1" s="24">
       <c r="A8" s="32" t="n"/>
@@ -18791,1182 +18836,1182 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor rgb="FF17324D"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A2:F14"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="12.625" defaultRowHeight="14.25"/>
-  <cols>
-    <col width="24" customWidth="1" style="24" min="1" max="1"/>
-    <col width="15" customWidth="1" style="24" min="2" max="2"/>
-    <col width="4" customWidth="1" style="24" min="3" max="3"/>
-    <col width="24" customWidth="1" style="24" min="4" max="4"/>
-    <col width="15" customWidth="1" style="24" min="5" max="5"/>
-    <col width="8" customWidth="1" style="24" min="6" max="6"/>
-    <col width="8.625" customWidth="1" style="24" min="7" max="26"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="15" customHeight="1" s="24"/>
-    <row r="2" ht="25.5" customHeight="1" s="24">
-      <c r="B2" s="1" t="inlineStr">
-        <is>
-          <t>TỔNG HỢP SỬ DỤNG AI — TUẦN 07</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-    </row>
-    <row r="3" ht="19.5" customHeight="1" s="24">
-      <c r="A3" s="30" t="inlineStr">
-        <is>
-          <t>26/10/2026 – 01/11/2026</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="n"/>
-      <c r="C3" s="2" t="n"/>
-      <c r="D3" s="2" t="n"/>
-      <c r="E3" s="2" t="n"/>
-      <c r="F3" s="2" t="n"/>
-    </row>
-    <row r="4" ht="15" customHeight="1" s="24">
-      <c r="A4" s="2" t="n"/>
-      <c r="B4" s="2" t="n"/>
-      <c r="C4" s="2" t="n"/>
-      <c r="D4" s="2" t="n"/>
-      <c r="E4" s="2" t="n"/>
-      <c r="F4" s="2" t="n"/>
-    </row>
-    <row r="5" ht="33.75" customHeight="1" s="24">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>TỔNG SỐ PROMPT</t>
-        </is>
-      </c>
-      <c r="B5" s="5">
-        <f>SUM(B9:B11)</f>
-        <v>11</v>
-      </c>
-      <c r="C5" s="2" t="n"/>
-      <c r="D5" s="2" t="n"/>
-      <c r="E5" s="2" t="n"/>
-      <c r="F5" s="2" t="n"/>
-    </row>
-    <row r="6" ht="15" customHeight="1" s="24">
-      <c r="A6" s="2" t="n"/>
-      <c r="B6" s="2" t="n"/>
-      <c r="C6" s="2" t="n"/>
-      <c r="D6" s="2" t="n"/>
-      <c r="E6" s="2" t="n"/>
-      <c r="F6" s="2" t="n"/>
-    </row>
-    <row r="7" ht="15" customHeight="1" s="24">
-      <c r="A7" s="2" t="n"/>
-      <c r="B7" s="2" t="n"/>
-      <c r="C7" s="2" t="n"/>
-      <c r="D7" s="2" t="n"/>
-      <c r="E7" s="2" t="n"/>
-      <c r="F7" s="2" t="n"/>
-    </row>
-    <row r="8" ht="27.75" customHeight="1" s="24">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>NGƯỜI TẠO</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>SỐ PROMPT</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="n"/>
-      <c r="D8" s="10" t="inlineStr">
-        <is>
-          <t>TOOL AI</t>
-        </is>
-      </c>
-      <c r="E8" s="10" t="inlineStr">
-        <is>
-          <t>SỐ PROMPT</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="n"/>
-    </row>
-    <row r="9" ht="24.75" customHeight="1" s="24">
-      <c r="A9" s="11" t="inlineStr">
-        <is>
-          <t>Thắng</t>
-        </is>
-      </c>
-      <c r="B9" s="13">
-        <f>COUNTIF(Thắng!$A$6:$A$306,"&lt;&gt;")</f>
-        <v>11</v>
-      </c>
-      <c r="C9" s="2" t="n"/>
-      <c r="D9" s="14" t="inlineStr">
-        <is>
-          <t>Claude</t>
-        </is>
-      </c>
-      <c r="E9" s="16">
-        <f>COUNTIFS(Thắng!$A$6:$A$306,"&lt;&gt;",Thắng!$C$6:$C$306,D9)+COUNTIFS(Sang!$A$6:$A$306,"&lt;&gt;",Sang!$C$6:$C$306,D9)+COUNTIFS(Nguyên!$A$6:$A$306,"&lt;&gt;",Nguyên!$C$6:$C$306,D9)</f>
-        <v>0</v>
-      </c>
-      <c r="F9" s="2" t="n"/>
-    </row>
-    <row r="10" ht="24.75" customHeight="1" s="24">
-      <c r="A10" s="11" t="inlineStr">
-        <is>
-          <t>Sang</t>
-        </is>
-      </c>
-      <c r="B10" s="13">
-        <f>COUNTIF(Sang!$A$6:$A$306,"&lt;&gt;")</f>
-        <v>0</v>
-      </c>
-      <c r="C10" s="2" t="n"/>
-      <c r="D10" s="14" t="inlineStr">
-        <is>
-          <t>Codex</t>
-        </is>
-      </c>
-      <c r="E10" s="16">
-        <f>COUNTIFS(Thắng!$A$6:$A$306,"&lt;&gt;",Thắng!$C$6:$C$306,D10)+COUNTIFS(Sang!$A$6:$A$306,"&lt;&gt;",Sang!$C$6:$C$306,D10)+COUNTIFS(Nguyên!$A$6:$A$306,"&lt;&gt;",Nguyên!$C$6:$C$306,D10)</f>
-        <v>0</v>
-      </c>
-      <c r="F10" s="2" t="n"/>
-    </row>
-    <row r="11" ht="24.75" customHeight="1" s="24">
-      <c r="A11" s="11" t="inlineStr">
-        <is>
-          <t>Nguyên</t>
-        </is>
-      </c>
-      <c r="B11" s="13">
-        <f>COUNTIF(Nguyên!$A$6:$A$306,"&lt;&gt;")</f>
-        <v>0</v>
-      </c>
-      <c r="C11" s="2" t="n"/>
-      <c r="D11" s="14" t="inlineStr">
-        <is>
-          <t>Antigravity</t>
-        </is>
-      </c>
-      <c r="E11" s="16">
-        <f>COUNTIFS(Thắng!$A$6:$A$306,"&lt;&gt;",Thắng!$C$6:$C$306,D11)+COUNTIFS(Sang!$A$6:$A$306,"&lt;&gt;",Sang!$C$6:$C$306,D11)+COUNTIFS(Nguyên!$A$6:$A$306,"&lt;&gt;",Nguyên!$C$6:$C$306,D11)</f>
-        <v>11</v>
-      </c>
-      <c r="F11" s="2" t="n"/>
-    </row>
-    <row r="12" ht="15" customHeight="1" s="24">
-      <c r="A12" s="2" t="n"/>
-      <c r="B12" s="2" t="n"/>
-      <c r="C12" s="2" t="n"/>
-      <c r="D12" s="2" t="n"/>
-      <c r="E12" s="2" t="n"/>
-      <c r="F12" s="2" t="n"/>
-    </row>
-    <row r="13" ht="15" customHeight="1" s="24">
-      <c r="A13" s="2" t="n"/>
-      <c r="B13" s="2" t="n"/>
-      <c r="C13" s="2" t="n"/>
-      <c r="D13" s="2" t="n"/>
-      <c r="E13" s="2" t="n"/>
-      <c r="F13" s="2" t="n"/>
-    </row>
-    <row r="14" ht="15" customHeight="1" s="24">
-      <c r="A14" s="17" t="n"/>
-      <c r="B14" s="2" t="n"/>
-      <c r="C14" s="2" t="n"/>
-      <c r="D14" s="2" t="n"/>
-      <c r="E14" s="2" t="n"/>
-      <c r="F14" s="2" t="n"/>
-    </row>
-    <row r="18" ht="15.75" customHeight="1" s="24"/>
-    <row r="19" ht="15.75" customHeight="1" s="24"/>
-    <row r="20" ht="15.75" customHeight="1" s="24"/>
-    <row r="21" ht="15.75" customHeight="1" s="24"/>
-    <row r="22" ht="15.75" customHeight="1" s="24"/>
-    <row r="23" ht="15.75" customHeight="1" s="24"/>
-    <row r="24" ht="15.75" customHeight="1" s="24"/>
-    <row r="25" ht="15.75" customHeight="1" s="24"/>
-    <row r="26" ht="15.75" customHeight="1" s="24"/>
-    <row r="27" ht="15.75" customHeight="1" s="24"/>
-    <row r="28" ht="15.75" customHeight="1" s="24"/>
-    <row r="29" ht="15.75" customHeight="1" s="24"/>
-    <row r="30" ht="15.75" customHeight="1" s="24"/>
-    <row r="31" ht="15.75" customHeight="1" s="24"/>
-    <row r="32" ht="15.75" customHeight="1" s="24"/>
-    <row r="33" ht="15.75" customHeight="1" s="24"/>
-    <row r="34" ht="15.75" customHeight="1" s="24"/>
-    <row r="35" ht="15.75" customHeight="1" s="24"/>
-    <row r="36" ht="15.75" customHeight="1" s="24"/>
-    <row r="37" ht="15.75" customHeight="1" s="24"/>
-    <row r="38" ht="15.75" customHeight="1" s="24"/>
-    <row r="39" ht="15.75" customHeight="1" s="24"/>
-    <row r="40" ht="15.75" customHeight="1" s="24"/>
-    <row r="41" ht="15.75" customHeight="1" s="24"/>
-    <row r="42" ht="15.75" customHeight="1" s="24"/>
-    <row r="43" ht="15.75" customHeight="1" s="24"/>
-    <row r="44" ht="15.75" customHeight="1" s="24"/>
-    <row r="45" ht="15.75" customHeight="1" s="24"/>
-    <row r="46" ht="15.75" customHeight="1" s="24"/>
-    <row r="47" ht="15.75" customHeight="1" s="24"/>
-    <row r="48" ht="15.75" customHeight="1" s="24"/>
-    <row r="49" ht="15.75" customHeight="1" s="24"/>
-    <row r="50" ht="15.75" customHeight="1" s="24"/>
-    <row r="51" ht="15.75" customHeight="1" s="24"/>
-    <row r="52" ht="15.75" customHeight="1" s="24"/>
-    <row r="53" ht="15.75" customHeight="1" s="24"/>
-    <row r="54" ht="15.75" customHeight="1" s="24"/>
-    <row r="55" ht="15.75" customHeight="1" s="24"/>
-    <row r="56" ht="15.75" customHeight="1" s="24"/>
-    <row r="57" ht="15.75" customHeight="1" s="24"/>
-    <row r="58" ht="15.75" customHeight="1" s="24"/>
-    <row r="59" ht="15.75" customHeight="1" s="24"/>
-    <row r="60" ht="15.75" customHeight="1" s="24"/>
-    <row r="61" ht="15.75" customHeight="1" s="24"/>
-    <row r="62" ht="15.75" customHeight="1" s="24"/>
-    <row r="63" ht="15.75" customHeight="1" s="24"/>
-    <row r="64" ht="15.75" customHeight="1" s="24"/>
-    <row r="65" ht="15.75" customHeight="1" s="24"/>
-    <row r="66" ht="15.75" customHeight="1" s="24"/>
-    <row r="67" ht="15.75" customHeight="1" s="24"/>
-    <row r="68" ht="15.75" customHeight="1" s="24"/>
-    <row r="69" ht="15.75" customHeight="1" s="24"/>
-    <row r="70" ht="15.75" customHeight="1" s="24"/>
-    <row r="71" ht="15.75" customHeight="1" s="24"/>
-    <row r="72" ht="15.75" customHeight="1" s="24"/>
-    <row r="73" ht="15.75" customHeight="1" s="24"/>
-    <row r="74" ht="15.75" customHeight="1" s="24"/>
-    <row r="75" ht="15.75" customHeight="1" s="24"/>
-    <row r="76" ht="15.75" customHeight="1" s="24"/>
-    <row r="77" ht="15.75" customHeight="1" s="24"/>
-    <row r="78" ht="15.75" customHeight="1" s="24"/>
-    <row r="79" ht="15.75" customHeight="1" s="24"/>
-    <row r="80" ht="15.75" customHeight="1" s="24"/>
-    <row r="81" ht="15.75" customHeight="1" s="24"/>
-    <row r="82" ht="15.75" customHeight="1" s="24"/>
-    <row r="83" ht="15.75" customHeight="1" s="24"/>
-    <row r="84" ht="15.75" customHeight="1" s="24"/>
-    <row r="85" ht="15.75" customHeight="1" s="24"/>
-    <row r="86" ht="15.75" customHeight="1" s="24"/>
-    <row r="87" ht="15.75" customHeight="1" s="24"/>
-    <row r="88" ht="15.75" customHeight="1" s="24"/>
-    <row r="89" ht="15.75" customHeight="1" s="24"/>
-    <row r="90" ht="15.75" customHeight="1" s="24"/>
-    <row r="91" ht="15.75" customHeight="1" s="24"/>
-    <row r="92" ht="15.75" customHeight="1" s="24"/>
-    <row r="93" ht="15.75" customHeight="1" s="24"/>
-    <row r="94" ht="15.75" customHeight="1" s="24"/>
-    <row r="95" ht="15.75" customHeight="1" s="24"/>
-    <row r="96" ht="15.75" customHeight="1" s="24"/>
-    <row r="97" ht="15.75" customHeight="1" s="24"/>
-    <row r="98" ht="15.75" customHeight="1" s="24"/>
-    <row r="99" ht="15.75" customHeight="1" s="24"/>
-    <row r="100" ht="15.75" customHeight="1" s="24"/>
-    <row r="101" ht="15.75" customHeight="1" s="24"/>
-    <row r="102" ht="15.75" customHeight="1" s="24"/>
-    <row r="103" ht="15.75" customHeight="1" s="24"/>
-    <row r="104" ht="15.75" customHeight="1" s="24"/>
-    <row r="105" ht="15.75" customHeight="1" s="24"/>
-    <row r="106" ht="15.75" customHeight="1" s="24"/>
-    <row r="107" ht="15.75" customHeight="1" s="24"/>
-    <row r="108" ht="15.75" customHeight="1" s="24"/>
-    <row r="109" ht="15.75" customHeight="1" s="24"/>
-    <row r="110" ht="15.75" customHeight="1" s="24"/>
-    <row r="111" ht="15.75" customHeight="1" s="24"/>
-    <row r="112" ht="15.75" customHeight="1" s="24"/>
-    <row r="113" ht="15.75" customHeight="1" s="24"/>
-    <row r="114" ht="15.75" customHeight="1" s="24"/>
-    <row r="115" ht="15.75" customHeight="1" s="24"/>
-    <row r="116" ht="15.75" customHeight="1" s="24"/>
-    <row r="117" ht="15.75" customHeight="1" s="24"/>
-    <row r="118" ht="15.75" customHeight="1" s="24"/>
-    <row r="119" ht="15.75" customHeight="1" s="24"/>
-    <row r="120" ht="15.75" customHeight="1" s="24"/>
-    <row r="121" ht="15.75" customHeight="1" s="24"/>
-    <row r="122" ht="15.75" customHeight="1" s="24"/>
-    <row r="123" ht="15.75" customHeight="1" s="24"/>
-    <row r="124" ht="15.75" customHeight="1" s="24"/>
-    <row r="125" ht="15.75" customHeight="1" s="24"/>
-    <row r="126" ht="15.75" customHeight="1" s="24"/>
-    <row r="127" ht="15.75" customHeight="1" s="24"/>
-    <row r="128" ht="15.75" customHeight="1" s="24"/>
-    <row r="129" ht="15.75" customHeight="1" s="24"/>
-    <row r="130" ht="15.75" customHeight="1" s="24"/>
-    <row r="131" ht="15.75" customHeight="1" s="24"/>
-    <row r="132" ht="15.75" customHeight="1" s="24"/>
-    <row r="133" ht="15.75" customHeight="1" s="24"/>
-    <row r="134" ht="15.75" customHeight="1" s="24"/>
-    <row r="135" ht="15.75" customHeight="1" s="24"/>
-    <row r="136" ht="15.75" customHeight="1" s="24"/>
-    <row r="137" ht="15.75" customHeight="1" s="24"/>
-    <row r="138" ht="15.75" customHeight="1" s="24"/>
-    <row r="139" ht="15.75" customHeight="1" s="24"/>
-    <row r="140" ht="15.75" customHeight="1" s="24"/>
-    <row r="141" ht="15.75" customHeight="1" s="24"/>
-    <row r="142" ht="15.75" customHeight="1" s="24"/>
-    <row r="143" ht="15.75" customHeight="1" s="24"/>
-    <row r="144" ht="15.75" customHeight="1" s="24"/>
-    <row r="145" ht="15.75" customHeight="1" s="24"/>
-    <row r="146" ht="15.75" customHeight="1" s="24"/>
-    <row r="147" ht="15.75" customHeight="1" s="24"/>
-    <row r="148" ht="15.75" customHeight="1" s="24"/>
-    <row r="149" ht="15.75" customHeight="1" s="24"/>
-    <row r="150" ht="15.75" customHeight="1" s="24"/>
-    <row r="151" ht="15.75" customHeight="1" s="24"/>
-    <row r="152" ht="15.75" customHeight="1" s="24"/>
-    <row r="153" ht="15.75" customHeight="1" s="24"/>
-    <row r="154" ht="15.75" customHeight="1" s="24"/>
-    <row r="155" ht="15.75" customHeight="1" s="24"/>
-    <row r="156" ht="15.75" customHeight="1" s="24"/>
-    <row r="157" ht="15.75" customHeight="1" s="24"/>
-    <row r="158" ht="15.75" customHeight="1" s="24"/>
-    <row r="159" ht="15.75" customHeight="1" s="24"/>
-    <row r="160" ht="15.75" customHeight="1" s="24"/>
-    <row r="161" ht="15.75" customHeight="1" s="24"/>
-    <row r="162" ht="15.75" customHeight="1" s="24"/>
-    <row r="163" ht="15.75" customHeight="1" s="24"/>
-    <row r="164" ht="15.75" customHeight="1" s="24"/>
-    <row r="165" ht="15.75" customHeight="1" s="24"/>
-    <row r="166" ht="15.75" customHeight="1" s="24"/>
-    <row r="167" ht="15.75" customHeight="1" s="24"/>
-    <row r="168" ht="15.75" customHeight="1" s="24"/>
-    <row r="169" ht="15.75" customHeight="1" s="24"/>
-    <row r="170" ht="15.75" customHeight="1" s="24"/>
-    <row r="171" ht="15.75" customHeight="1" s="24"/>
-    <row r="172" ht="15.75" customHeight="1" s="24"/>
-    <row r="173" ht="15.75" customHeight="1" s="24"/>
-    <row r="174" ht="15.75" customHeight="1" s="24"/>
-    <row r="175" ht="15.75" customHeight="1" s="24"/>
-    <row r="176" ht="15.75" customHeight="1" s="24"/>
-    <row r="177" ht="15.75" customHeight="1" s="24"/>
-    <row r="178" ht="15.75" customHeight="1" s="24"/>
-    <row r="179" ht="15.75" customHeight="1" s="24"/>
-    <row r="180" ht="15.75" customHeight="1" s="24"/>
-    <row r="181" ht="15.75" customHeight="1" s="24"/>
-    <row r="182" ht="15.75" customHeight="1" s="24"/>
-    <row r="183" ht="15.75" customHeight="1" s="24"/>
-    <row r="184" ht="15.75" customHeight="1" s="24"/>
-    <row r="185" ht="15.75" customHeight="1" s="24"/>
-    <row r="186" ht="15.75" customHeight="1" s="24"/>
-    <row r="187" ht="15.75" customHeight="1" s="24"/>
-    <row r="188" ht="15.75" customHeight="1" s="24"/>
-    <row r="189" ht="15.75" customHeight="1" s="24"/>
-    <row r="190" ht="15.75" customHeight="1" s="24"/>
-    <row r="191" ht="15.75" customHeight="1" s="24"/>
-    <row r="192" ht="15.75" customHeight="1" s="24"/>
-    <row r="193" ht="15.75" customHeight="1" s="24"/>
-    <row r="194" ht="15.75" customHeight="1" s="24"/>
-    <row r="195" ht="15.75" customHeight="1" s="24"/>
-    <row r="196" ht="15.75" customHeight="1" s="24"/>
-    <row r="197" ht="15.75" customHeight="1" s="24"/>
-    <row r="198" ht="15.75" customHeight="1" s="24"/>
-    <row r="199" ht="15.75" customHeight="1" s="24"/>
-    <row r="200" ht="15.75" customHeight="1" s="24"/>
-    <row r="201" ht="15.75" customHeight="1" s="24"/>
-    <row r="202" ht="15.75" customHeight="1" s="24"/>
-    <row r="203" ht="15.75" customHeight="1" s="24"/>
-    <row r="204" ht="15.75" customHeight="1" s="24"/>
-    <row r="205" ht="15.75" customHeight="1" s="24"/>
-    <row r="206" ht="15.75" customHeight="1" s="24"/>
-    <row r="207" ht="15.75" customHeight="1" s="24"/>
-    <row r="208" ht="15.75" customHeight="1" s="24"/>
-    <row r="209" ht="15.75" customHeight="1" s="24"/>
-    <row r="210" ht="15.75" customHeight="1" s="24"/>
-    <row r="211" ht="15.75" customHeight="1" s="24"/>
-    <row r="212" ht="15.75" customHeight="1" s="24"/>
-    <row r="213" ht="15.75" customHeight="1" s="24"/>
-    <row r="214" ht="15.75" customHeight="1" s="24"/>
-    <row r="215" ht="15.75" customHeight="1" s="24"/>
-    <row r="216" ht="15.75" customHeight="1" s="24"/>
-    <row r="217" ht="15.75" customHeight="1" s="24"/>
-    <row r="218" ht="15.75" customHeight="1" s="24"/>
-    <row r="219" ht="15.75" customHeight="1" s="24"/>
-    <row r="220" ht="15.75" customHeight="1" s="24"/>
-    <row r="221" ht="15.75" customHeight="1" s="24"/>
-    <row r="222" ht="15.75" customHeight="1" s="24"/>
-    <row r="223" ht="15.75" customHeight="1" s="24"/>
-    <row r="224" ht="15.75" customHeight="1" s="24"/>
-    <row r="225" ht="15.75" customHeight="1" s="24"/>
-    <row r="226" ht="15.75" customHeight="1" s="24"/>
-    <row r="227" ht="15.75" customHeight="1" s="24"/>
-    <row r="228" ht="15.75" customHeight="1" s="24"/>
-    <row r="229" ht="15.75" customHeight="1" s="24"/>
-    <row r="230" ht="15.75" customHeight="1" s="24"/>
-    <row r="231" ht="15.75" customHeight="1" s="24"/>
-    <row r="232" ht="15.75" customHeight="1" s="24"/>
-    <row r="233" ht="15.75" customHeight="1" s="24"/>
-    <row r="234" ht="15.75" customHeight="1" s="24"/>
-    <row r="235" ht="15.75" customHeight="1" s="24"/>
-    <row r="236" ht="15.75" customHeight="1" s="24"/>
-    <row r="237" ht="15.75" customHeight="1" s="24"/>
-    <row r="238" ht="15.75" customHeight="1" s="24"/>
-    <row r="239" ht="15.75" customHeight="1" s="24"/>
-    <row r="240" ht="15.75" customHeight="1" s="24"/>
-    <row r="241" ht="15.75" customHeight="1" s="24"/>
-    <row r="242" ht="15.75" customHeight="1" s="24"/>
-    <row r="243" ht="15.75" customHeight="1" s="24"/>
-    <row r="244" ht="15.75" customHeight="1" s="24"/>
-    <row r="245" ht="15.75" customHeight="1" s="24"/>
-    <row r="246" ht="15.75" customHeight="1" s="24"/>
-    <row r="247" ht="15.75" customHeight="1" s="24"/>
-    <row r="248" ht="15.75" customHeight="1" s="24"/>
-    <row r="249" ht="15.75" customHeight="1" s="24"/>
-    <row r="250" ht="15.75" customHeight="1" s="24"/>
-    <row r="251" ht="15.75" customHeight="1" s="24"/>
-    <row r="252" ht="15.75" customHeight="1" s="24"/>
-    <row r="253" ht="15.75" customHeight="1" s="24"/>
-    <row r="254" ht="15.75" customHeight="1" s="24"/>
-    <row r="255" ht="15.75" customHeight="1" s="24"/>
-    <row r="256" ht="15.75" customHeight="1" s="24"/>
-    <row r="257" ht="15.75" customHeight="1" s="24"/>
-    <row r="258" ht="15.75" customHeight="1" s="24"/>
-    <row r="259" ht="15.75" customHeight="1" s="24"/>
-    <row r="260" ht="15.75" customHeight="1" s="24"/>
-    <row r="261" ht="15.75" customHeight="1" s="24"/>
-    <row r="262" ht="15.75" customHeight="1" s="24"/>
-    <row r="263" ht="15.75" customHeight="1" s="24"/>
-    <row r="264" ht="15.75" customHeight="1" s="24"/>
-    <row r="265" ht="15.75" customHeight="1" s="24"/>
-    <row r="266" ht="15.75" customHeight="1" s="24"/>
-    <row r="267" ht="15.75" customHeight="1" s="24"/>
-    <row r="268" ht="15.75" customHeight="1" s="24"/>
-    <row r="269" ht="15.75" customHeight="1" s="24"/>
-    <row r="270" ht="15.75" customHeight="1" s="24"/>
-    <row r="271" ht="15.75" customHeight="1" s="24"/>
-    <row r="272" ht="15.75" customHeight="1" s="24"/>
-    <row r="273" ht="15.75" customHeight="1" s="24"/>
-    <row r="274" ht="15.75" customHeight="1" s="24"/>
-    <row r="275" ht="15.75" customHeight="1" s="24"/>
-    <row r="276" ht="15.75" customHeight="1" s="24"/>
-    <row r="277" ht="15.75" customHeight="1" s="24"/>
-    <row r="278" ht="15.75" customHeight="1" s="24"/>
-    <row r="279" ht="15.75" customHeight="1" s="24"/>
-    <row r="280" ht="15.75" customHeight="1" s="24"/>
-    <row r="281" ht="15.75" customHeight="1" s="24"/>
-    <row r="282" ht="15.75" customHeight="1" s="24"/>
-    <row r="283" ht="15.75" customHeight="1" s="24"/>
-    <row r="284" ht="15.75" customHeight="1" s="24"/>
-    <row r="285" ht="15.75" customHeight="1" s="24"/>
-    <row r="286" ht="15.75" customHeight="1" s="24"/>
-    <row r="287" ht="15.75" customHeight="1" s="24"/>
-    <row r="288" ht="15.75" customHeight="1" s="24"/>
-    <row r="289" ht="15.75" customHeight="1" s="24"/>
-    <row r="290" ht="15.75" customHeight="1" s="24"/>
-    <row r="291" ht="15.75" customHeight="1" s="24"/>
-    <row r="292" ht="15.75" customHeight="1" s="24"/>
-    <row r="293" ht="15.75" customHeight="1" s="24"/>
-    <row r="294" ht="15.75" customHeight="1" s="24"/>
-    <row r="295" ht="15.75" customHeight="1" s="24"/>
-    <row r="296" ht="15.75" customHeight="1" s="24"/>
-    <row r="297" ht="15.75" customHeight="1" s="24"/>
-    <row r="298" ht="15.75" customHeight="1" s="24"/>
-    <row r="299" ht="15.75" customHeight="1" s="24"/>
-    <row r="300" ht="15.75" customHeight="1" s="24"/>
-    <row r="301" ht="15.75" customHeight="1" s="24"/>
-    <row r="302" ht="15.75" customHeight="1" s="24"/>
-    <row r="303" ht="15.75" customHeight="1" s="24"/>
-    <row r="304" ht="15.75" customHeight="1" s="24"/>
-    <row r="305" ht="15.75" customHeight="1" s="24"/>
-    <row r="306" ht="15.75" customHeight="1" s="24"/>
-    <row r="307" ht="15.75" customHeight="1" s="24"/>
-    <row r="308" ht="15.75" customHeight="1" s="24"/>
-    <row r="309" ht="15.75" customHeight="1" s="24"/>
-    <row r="310" ht="15.75" customHeight="1" s="24"/>
-    <row r="311" ht="15.75" customHeight="1" s="24"/>
-    <row r="312" ht="15.75" customHeight="1" s="24"/>
-    <row r="313" ht="15.75" customHeight="1" s="24"/>
-    <row r="314" ht="15.75" customHeight="1" s="24"/>
-    <row r="315" ht="15.75" customHeight="1" s="24"/>
-    <row r="316" ht="15.75" customHeight="1" s="24"/>
-    <row r="317" ht="15.75" customHeight="1" s="24"/>
-    <row r="318" ht="15.75" customHeight="1" s="24"/>
-    <row r="319" ht="15.75" customHeight="1" s="24"/>
-    <row r="320" ht="15.75" customHeight="1" s="24"/>
-    <row r="321" ht="15.75" customHeight="1" s="24"/>
-    <row r="322" ht="15.75" customHeight="1" s="24"/>
-    <row r="323" ht="15.75" customHeight="1" s="24"/>
-    <row r="324" ht="15.75" customHeight="1" s="24"/>
-    <row r="325" ht="15.75" customHeight="1" s="24"/>
-    <row r="326" ht="15.75" customHeight="1" s="24"/>
-    <row r="327" ht="15.75" customHeight="1" s="24"/>
-    <row r="328" ht="15.75" customHeight="1" s="24"/>
-    <row r="329" ht="15.75" customHeight="1" s="24"/>
-    <row r="330" ht="15.75" customHeight="1" s="24"/>
-    <row r="331" ht="15.75" customHeight="1" s="24"/>
-    <row r="332" ht="15.75" customHeight="1" s="24"/>
-    <row r="333" ht="15.75" customHeight="1" s="24"/>
-    <row r="334" ht="15.75" customHeight="1" s="24"/>
-    <row r="335" ht="15.75" customHeight="1" s="24"/>
-    <row r="336" ht="15.75" customHeight="1" s="24"/>
-    <row r="337" ht="15.75" customHeight="1" s="24"/>
-    <row r="338" ht="15.75" customHeight="1" s="24"/>
-    <row r="339" ht="15.75" customHeight="1" s="24"/>
-    <row r="340" ht="15.75" customHeight="1" s="24"/>
-    <row r="341" ht="15.75" customHeight="1" s="24"/>
-    <row r="342" ht="15.75" customHeight="1" s="24"/>
-    <row r="343" ht="15.75" customHeight="1" s="24"/>
-    <row r="344" ht="15.75" customHeight="1" s="24"/>
-    <row r="345" ht="15.75" customHeight="1" s="24"/>
-    <row r="346" ht="15.75" customHeight="1" s="24"/>
-    <row r="347" ht="15.75" customHeight="1" s="24"/>
-    <row r="348" ht="15.75" customHeight="1" s="24"/>
-    <row r="349" ht="15.75" customHeight="1" s="24"/>
-    <row r="350" ht="15.75" customHeight="1" s="24"/>
-    <row r="351" ht="15.75" customHeight="1" s="24"/>
-    <row r="352" ht="15.75" customHeight="1" s="24"/>
-    <row r="353" ht="15.75" customHeight="1" s="24"/>
-    <row r="354" ht="15.75" customHeight="1" s="24"/>
-    <row r="355" ht="15.75" customHeight="1" s="24"/>
-    <row r="356" ht="15.75" customHeight="1" s="24"/>
-    <row r="357" ht="15.75" customHeight="1" s="24"/>
-    <row r="358" ht="15.75" customHeight="1" s="24"/>
-    <row r="359" ht="15.75" customHeight="1" s="24"/>
-    <row r="360" ht="15.75" customHeight="1" s="24"/>
-    <row r="361" ht="15.75" customHeight="1" s="24"/>
-    <row r="362" ht="15.75" customHeight="1" s="24"/>
-    <row r="363" ht="15.75" customHeight="1" s="24"/>
-    <row r="364" ht="15.75" customHeight="1" s="24"/>
-    <row r="365" ht="15.75" customHeight="1" s="24"/>
-    <row r="366" ht="15.75" customHeight="1" s="24"/>
-    <row r="367" ht="15.75" customHeight="1" s="24"/>
-    <row r="368" ht="15.75" customHeight="1" s="24"/>
-    <row r="369" ht="15.75" customHeight="1" s="24"/>
-    <row r="370" ht="15.75" customHeight="1" s="24"/>
-    <row r="371" ht="15.75" customHeight="1" s="24"/>
-    <row r="372" ht="15.75" customHeight="1" s="24"/>
-    <row r="373" ht="15.75" customHeight="1" s="24"/>
-    <row r="374" ht="15.75" customHeight="1" s="24"/>
-    <row r="375" ht="15.75" customHeight="1" s="24"/>
-    <row r="376" ht="15.75" customHeight="1" s="24"/>
-    <row r="377" ht="15.75" customHeight="1" s="24"/>
-    <row r="378" ht="15.75" customHeight="1" s="24"/>
-    <row r="379" ht="15.75" customHeight="1" s="24"/>
-    <row r="380" ht="15.75" customHeight="1" s="24"/>
-    <row r="381" ht="15.75" customHeight="1" s="24"/>
-    <row r="382" ht="15.75" customHeight="1" s="24"/>
-    <row r="383" ht="15.75" customHeight="1" s="24"/>
-    <row r="384" ht="15.75" customHeight="1" s="24"/>
-    <row r="385" ht="15.75" customHeight="1" s="24"/>
-    <row r="386" ht="15.75" customHeight="1" s="24"/>
-    <row r="387" ht="15.75" customHeight="1" s="24"/>
-    <row r="388" ht="15.75" customHeight="1" s="24"/>
-    <row r="389" ht="15.75" customHeight="1" s="24"/>
-    <row r="390" ht="15.75" customHeight="1" s="24"/>
-    <row r="391" ht="15.75" customHeight="1" s="24"/>
-    <row r="392" ht="15.75" customHeight="1" s="24"/>
-    <row r="393" ht="15.75" customHeight="1" s="24"/>
-    <row r="394" ht="15.75" customHeight="1" s="24"/>
-    <row r="395" ht="15.75" customHeight="1" s="24"/>
-    <row r="396" ht="15.75" customHeight="1" s="24"/>
-    <row r="397" ht="15.75" customHeight="1" s="24"/>
-    <row r="398" ht="15.75" customHeight="1" s="24"/>
-    <row r="399" ht="15.75" customHeight="1" s="24"/>
-    <row r="400" ht="15.75" customHeight="1" s="24"/>
-    <row r="401" ht="15.75" customHeight="1" s="24"/>
-    <row r="402" ht="15.75" customHeight="1" s="24"/>
-    <row r="403" ht="15.75" customHeight="1" s="24"/>
-    <row r="404" ht="15.75" customHeight="1" s="24"/>
-    <row r="405" ht="15.75" customHeight="1" s="24"/>
-    <row r="406" ht="15.75" customHeight="1" s="24"/>
-    <row r="407" ht="15.75" customHeight="1" s="24"/>
-    <row r="408" ht="15.75" customHeight="1" s="24"/>
-    <row r="409" ht="15.75" customHeight="1" s="24"/>
-    <row r="410" ht="15.75" customHeight="1" s="24"/>
-    <row r="411" ht="15.75" customHeight="1" s="24"/>
-    <row r="412" ht="15.75" customHeight="1" s="24"/>
-    <row r="413" ht="15.75" customHeight="1" s="24"/>
-    <row r="414" ht="15.75" customHeight="1" s="24"/>
-    <row r="415" ht="15.75" customHeight="1" s="24"/>
-    <row r="416" ht="15.75" customHeight="1" s="24"/>
-    <row r="417" ht="15.75" customHeight="1" s="24"/>
-    <row r="418" ht="15.75" customHeight="1" s="24"/>
-    <row r="419" ht="15.75" customHeight="1" s="24"/>
-    <row r="420" ht="15.75" customHeight="1" s="24"/>
-    <row r="421" ht="15.75" customHeight="1" s="24"/>
-    <row r="422" ht="15.75" customHeight="1" s="24"/>
-    <row r="423" ht="15.75" customHeight="1" s="24"/>
-    <row r="424" ht="15.75" customHeight="1" s="24"/>
-    <row r="425" ht="15.75" customHeight="1" s="24"/>
-    <row r="426" ht="15.75" customHeight="1" s="24"/>
-    <row r="427" ht="15.75" customHeight="1" s="24"/>
-    <row r="428" ht="15.75" customHeight="1" s="24"/>
-    <row r="429" ht="15.75" customHeight="1" s="24"/>
-    <row r="430" ht="15.75" customHeight="1" s="24"/>
-    <row r="431" ht="15.75" customHeight="1" s="24"/>
-    <row r="432" ht="15.75" customHeight="1" s="24"/>
-    <row r="433" ht="15.75" customHeight="1" s="24"/>
-    <row r="434" ht="15.75" customHeight="1" s="24"/>
-    <row r="435" ht="15.75" customHeight="1" s="24"/>
-    <row r="436" ht="15.75" customHeight="1" s="24"/>
-    <row r="437" ht="15.75" customHeight="1" s="24"/>
-    <row r="438" ht="15.75" customHeight="1" s="24"/>
-    <row r="439" ht="15.75" customHeight="1" s="24"/>
-    <row r="440" ht="15.75" customHeight="1" s="24"/>
-    <row r="441" ht="15.75" customHeight="1" s="24"/>
-    <row r="442" ht="15.75" customHeight="1" s="24"/>
-    <row r="443" ht="15.75" customHeight="1" s="24"/>
-    <row r="444" ht="15.75" customHeight="1" s="24"/>
-    <row r="445" ht="15.75" customHeight="1" s="24"/>
-    <row r="446" ht="15.75" customHeight="1" s="24"/>
-    <row r="447" ht="15.75" customHeight="1" s="24"/>
-    <row r="448" ht="15.75" customHeight="1" s="24"/>
-    <row r="449" ht="15.75" customHeight="1" s="24"/>
-    <row r="450" ht="15.75" customHeight="1" s="24"/>
-    <row r="451" ht="15.75" customHeight="1" s="24"/>
-    <row r="452" ht="15.75" customHeight="1" s="24"/>
-    <row r="453" ht="15.75" customHeight="1" s="24"/>
-    <row r="454" ht="15.75" customHeight="1" s="24"/>
-    <row r="455" ht="15.75" customHeight="1" s="24"/>
-    <row r="456" ht="15.75" customHeight="1" s="24"/>
-    <row r="457" ht="15.75" customHeight="1" s="24"/>
-    <row r="458" ht="15.75" customHeight="1" s="24"/>
-    <row r="459" ht="15.75" customHeight="1" s="24"/>
-    <row r="460" ht="15.75" customHeight="1" s="24"/>
-    <row r="461" ht="15.75" customHeight="1" s="24"/>
-    <row r="462" ht="15.75" customHeight="1" s="24"/>
-    <row r="463" ht="15.75" customHeight="1" s="24"/>
-    <row r="464" ht="15.75" customHeight="1" s="24"/>
-    <row r="465" ht="15.75" customHeight="1" s="24"/>
-    <row r="466" ht="15.75" customHeight="1" s="24"/>
-    <row r="467" ht="15.75" customHeight="1" s="24"/>
-    <row r="468" ht="15.75" customHeight="1" s="24"/>
-    <row r="469" ht="15.75" customHeight="1" s="24"/>
-    <row r="470" ht="15.75" customHeight="1" s="24"/>
-    <row r="471" ht="15.75" customHeight="1" s="24"/>
-    <row r="472" ht="15.75" customHeight="1" s="24"/>
-    <row r="473" ht="15.75" customHeight="1" s="24"/>
-    <row r="474" ht="15.75" customHeight="1" s="24"/>
-    <row r="475" ht="15.75" customHeight="1" s="24"/>
-    <row r="476" ht="15.75" customHeight="1" s="24"/>
-    <row r="477" ht="15.75" customHeight="1" s="24"/>
-    <row r="478" ht="15.75" customHeight="1" s="24"/>
-    <row r="479" ht="15.75" customHeight="1" s="24"/>
-    <row r="480" ht="15.75" customHeight="1" s="24"/>
-    <row r="481" ht="15.75" customHeight="1" s="24"/>
-    <row r="482" ht="15.75" customHeight="1" s="24"/>
-    <row r="483" ht="15.75" customHeight="1" s="24"/>
-    <row r="484" ht="15.75" customHeight="1" s="24"/>
-    <row r="485" ht="15.75" customHeight="1" s="24"/>
-    <row r="486" ht="15.75" customHeight="1" s="24"/>
-    <row r="487" ht="15.75" customHeight="1" s="24"/>
-    <row r="488" ht="15.75" customHeight="1" s="24"/>
-    <row r="489" ht="15.75" customHeight="1" s="24"/>
-    <row r="490" ht="15.75" customHeight="1" s="24"/>
-    <row r="491" ht="15.75" customHeight="1" s="24"/>
-    <row r="492" ht="15.75" customHeight="1" s="24"/>
-    <row r="493" ht="15.75" customHeight="1" s="24"/>
-    <row r="494" ht="15.75" customHeight="1" s="24"/>
-    <row r="495" ht="15.75" customHeight="1" s="24"/>
-    <row r="496" ht="15.75" customHeight="1" s="24"/>
-    <row r="497" ht="15.75" customHeight="1" s="24"/>
-    <row r="498" ht="15.75" customHeight="1" s="24"/>
-    <row r="499" ht="15.75" customHeight="1" s="24"/>
-    <row r="500" ht="15.75" customHeight="1" s="24"/>
-    <row r="501" ht="15.75" customHeight="1" s="24"/>
-    <row r="502" ht="15.75" customHeight="1" s="24"/>
-    <row r="503" ht="15.75" customHeight="1" s="24"/>
-    <row r="504" ht="15.75" customHeight="1" s="24"/>
-    <row r="505" ht="15.75" customHeight="1" s="24"/>
-    <row r="506" ht="15.75" customHeight="1" s="24"/>
-    <row r="507" ht="15.75" customHeight="1" s="24"/>
-    <row r="508" ht="15.75" customHeight="1" s="24"/>
-    <row r="509" ht="15.75" customHeight="1" s="24"/>
-    <row r="510" ht="15.75" customHeight="1" s="24"/>
-    <row r="511" ht="15.75" customHeight="1" s="24"/>
-    <row r="512" ht="15.75" customHeight="1" s="24"/>
-    <row r="513" ht="15.75" customHeight="1" s="24"/>
-    <row r="514" ht="15.75" customHeight="1" s="24"/>
-    <row r="515" ht="15.75" customHeight="1" s="24"/>
-    <row r="516" ht="15.75" customHeight="1" s="24"/>
-    <row r="517" ht="15.75" customHeight="1" s="24"/>
-    <row r="518" ht="15.75" customHeight="1" s="24"/>
-    <row r="519" ht="15.75" customHeight="1" s="24"/>
-    <row r="520" ht="15.75" customHeight="1" s="24"/>
-    <row r="521" ht="15.75" customHeight="1" s="24"/>
-    <row r="522" ht="15.75" customHeight="1" s="24"/>
-    <row r="523" ht="15.75" customHeight="1" s="24"/>
-    <row r="524" ht="15.75" customHeight="1" s="24"/>
-    <row r="525" ht="15.75" customHeight="1" s="24"/>
-    <row r="526" ht="15.75" customHeight="1" s="24"/>
-    <row r="527" ht="15.75" customHeight="1" s="24"/>
-    <row r="528" ht="15.75" customHeight="1" s="24"/>
-    <row r="529" ht="15.75" customHeight="1" s="24"/>
-    <row r="530" ht="15.75" customHeight="1" s="24"/>
-    <row r="531" ht="15.75" customHeight="1" s="24"/>
-    <row r="532" ht="15.75" customHeight="1" s="24"/>
-    <row r="533" ht="15.75" customHeight="1" s="24"/>
-    <row r="534" ht="15.75" customHeight="1" s="24"/>
-    <row r="535" ht="15.75" customHeight="1" s="24"/>
-    <row r="536" ht="15.75" customHeight="1" s="24"/>
-    <row r="537" ht="15.75" customHeight="1" s="24"/>
-    <row r="538" ht="15.75" customHeight="1" s="24"/>
-    <row r="539" ht="15.75" customHeight="1" s="24"/>
-    <row r="540" ht="15.75" customHeight="1" s="24"/>
-    <row r="541" ht="15.75" customHeight="1" s="24"/>
-    <row r="542" ht="15.75" customHeight="1" s="24"/>
-    <row r="543" ht="15.75" customHeight="1" s="24"/>
-    <row r="544" ht="15.75" customHeight="1" s="24"/>
-    <row r="545" ht="15.75" customHeight="1" s="24"/>
-    <row r="546" ht="15.75" customHeight="1" s="24"/>
-    <row r="547" ht="15.75" customHeight="1" s="24"/>
-    <row r="548" ht="15.75" customHeight="1" s="24"/>
-    <row r="549" ht="15.75" customHeight="1" s="24"/>
-    <row r="550" ht="15.75" customHeight="1" s="24"/>
-    <row r="551" ht="15.75" customHeight="1" s="24"/>
-    <row r="552" ht="15.75" customHeight="1" s="24"/>
-    <row r="553" ht="15.75" customHeight="1" s="24"/>
-    <row r="554" ht="15.75" customHeight="1" s="24"/>
-    <row r="555" ht="15.75" customHeight="1" s="24"/>
-    <row r="556" ht="15.75" customHeight="1" s="24"/>
-    <row r="557" ht="15.75" customHeight="1" s="24"/>
-    <row r="558" ht="15.75" customHeight="1" s="24"/>
-    <row r="559" ht="15.75" customHeight="1" s="24"/>
-    <row r="560" ht="15.75" customHeight="1" s="24"/>
-    <row r="561" ht="15.75" customHeight="1" s="24"/>
-    <row r="562" ht="15.75" customHeight="1" s="24"/>
-    <row r="563" ht="15.75" customHeight="1" s="24"/>
-    <row r="564" ht="15.75" customHeight="1" s="24"/>
-    <row r="565" ht="15.75" customHeight="1" s="24"/>
-    <row r="566" ht="15.75" customHeight="1" s="24"/>
-    <row r="567" ht="15.75" customHeight="1" s="24"/>
-    <row r="568" ht="15.75" customHeight="1" s="24"/>
-    <row r="569" ht="15.75" customHeight="1" s="24"/>
-    <row r="570" ht="15.75" customHeight="1" s="24"/>
-    <row r="571" ht="15.75" customHeight="1" s="24"/>
-    <row r="572" ht="15.75" customHeight="1" s="24"/>
-    <row r="573" ht="15.75" customHeight="1" s="24"/>
-    <row r="574" ht="15.75" customHeight="1" s="24"/>
-    <row r="575" ht="15.75" customHeight="1" s="24"/>
-    <row r="576" ht="15.75" customHeight="1" s="24"/>
-    <row r="577" ht="15.75" customHeight="1" s="24"/>
-    <row r="578" ht="15.75" customHeight="1" s="24"/>
-    <row r="579" ht="15.75" customHeight="1" s="24"/>
-    <row r="580" ht="15.75" customHeight="1" s="24"/>
-    <row r="581" ht="15.75" customHeight="1" s="24"/>
-    <row r="582" ht="15.75" customHeight="1" s="24"/>
-    <row r="583" ht="15.75" customHeight="1" s="24"/>
-    <row r="584" ht="15.75" customHeight="1" s="24"/>
-    <row r="585" ht="15.75" customHeight="1" s="24"/>
-    <row r="586" ht="15.75" customHeight="1" s="24"/>
-    <row r="587" ht="15.75" customHeight="1" s="24"/>
-    <row r="588" ht="15.75" customHeight="1" s="24"/>
-    <row r="589" ht="15.75" customHeight="1" s="24"/>
-    <row r="590" ht="15.75" customHeight="1" s="24"/>
-    <row r="591" ht="15.75" customHeight="1" s="24"/>
-    <row r="592" ht="15.75" customHeight="1" s="24"/>
-    <row r="593" ht="15.75" customHeight="1" s="24"/>
-    <row r="594" ht="15.75" customHeight="1" s="24"/>
-    <row r="595" ht="15.75" customHeight="1" s="24"/>
-    <row r="596" ht="15.75" customHeight="1" s="24"/>
-    <row r="597" ht="15.75" customHeight="1" s="24"/>
-    <row r="598" ht="15.75" customHeight="1" s="24"/>
-    <row r="599" ht="15.75" customHeight="1" s="24"/>
-    <row r="600" ht="15.75" customHeight="1" s="24"/>
-    <row r="601" ht="15.75" customHeight="1" s="24"/>
-    <row r="602" ht="15.75" customHeight="1" s="24"/>
-    <row r="603" ht="15.75" customHeight="1" s="24"/>
-    <row r="604" ht="15.75" customHeight="1" s="24"/>
-    <row r="605" ht="15.75" customHeight="1" s="24"/>
-    <row r="606" ht="15.75" customHeight="1" s="24"/>
-    <row r="607" ht="15.75" customHeight="1" s="24"/>
-    <row r="608" ht="15.75" customHeight="1" s="24"/>
-    <row r="609" ht="15.75" customHeight="1" s="24"/>
-    <row r="610" ht="15.75" customHeight="1" s="24"/>
-    <row r="611" ht="15.75" customHeight="1" s="24"/>
-    <row r="612" ht="15.75" customHeight="1" s="24"/>
-    <row r="613" ht="15.75" customHeight="1" s="24"/>
-    <row r="614" ht="15.75" customHeight="1" s="24"/>
-    <row r="615" ht="15.75" customHeight="1" s="24"/>
-    <row r="616" ht="15.75" customHeight="1" s="24"/>
-    <row r="617" ht="15.75" customHeight="1" s="24"/>
-    <row r="618" ht="15.75" customHeight="1" s="24"/>
-    <row r="619" ht="15.75" customHeight="1" s="24"/>
-    <row r="620" ht="15.75" customHeight="1" s="24"/>
-    <row r="621" ht="15.75" customHeight="1" s="24"/>
-    <row r="622" ht="15.75" customHeight="1" s="24"/>
-    <row r="623" ht="15.75" customHeight="1" s="24"/>
-    <row r="624" ht="15.75" customHeight="1" s="24"/>
-    <row r="625" ht="15.75" customHeight="1" s="24"/>
-    <row r="626" ht="15.75" customHeight="1" s="24"/>
-    <row r="627" ht="15.75" customHeight="1" s="24"/>
-    <row r="628" ht="15.75" customHeight="1" s="24"/>
-    <row r="629" ht="15.75" customHeight="1" s="24"/>
-    <row r="630" ht="15.75" customHeight="1" s="24"/>
-    <row r="631" ht="15.75" customHeight="1" s="24"/>
-    <row r="632" ht="15.75" customHeight="1" s="24"/>
-    <row r="633" ht="15.75" customHeight="1" s="24"/>
-    <row r="634" ht="15.75" customHeight="1" s="24"/>
-    <row r="635" ht="15.75" customHeight="1" s="24"/>
-    <row r="636" ht="15.75" customHeight="1" s="24"/>
-    <row r="637" ht="15.75" customHeight="1" s="24"/>
-    <row r="638" ht="15.75" customHeight="1" s="24"/>
-    <row r="639" ht="15.75" customHeight="1" s="24"/>
-    <row r="640" ht="15.75" customHeight="1" s="24"/>
-    <row r="641" ht="15.75" customHeight="1" s="24"/>
-    <row r="642" ht="15.75" customHeight="1" s="24"/>
-    <row r="643" ht="15.75" customHeight="1" s="24"/>
-    <row r="644" ht="15.75" customHeight="1" s="24"/>
-    <row r="645" ht="15.75" customHeight="1" s="24"/>
-    <row r="646" ht="15.75" customHeight="1" s="24"/>
-    <row r="647" ht="15.75" customHeight="1" s="24"/>
-    <row r="648" ht="15.75" customHeight="1" s="24"/>
-    <row r="649" ht="15.75" customHeight="1" s="24"/>
-    <row r="650" ht="15.75" customHeight="1" s="24"/>
-    <row r="651" ht="15.75" customHeight="1" s="24"/>
-    <row r="652" ht="15.75" customHeight="1" s="24"/>
-    <row r="653" ht="15.75" customHeight="1" s="24"/>
-    <row r="654" ht="15.75" customHeight="1" s="24"/>
-    <row r="655" ht="15.75" customHeight="1" s="24"/>
-    <row r="656" ht="15.75" customHeight="1" s="24"/>
-    <row r="657" ht="15.75" customHeight="1" s="24"/>
-    <row r="658" ht="15.75" customHeight="1" s="24"/>
-    <row r="659" ht="15.75" customHeight="1" s="24"/>
-    <row r="660" ht="15.75" customHeight="1" s="24"/>
-    <row r="661" ht="15.75" customHeight="1" s="24"/>
-    <row r="662" ht="15.75" customHeight="1" s="24"/>
-    <row r="663" ht="15.75" customHeight="1" s="24"/>
-    <row r="664" ht="15.75" customHeight="1" s="24"/>
-    <row r="665" ht="15.75" customHeight="1" s="24"/>
-    <row r="666" ht="15.75" customHeight="1" s="24"/>
-    <row r="667" ht="15.75" customHeight="1" s="24"/>
-    <row r="668" ht="15.75" customHeight="1" s="24"/>
-    <row r="669" ht="15.75" customHeight="1" s="24"/>
-    <row r="670" ht="15.75" customHeight="1" s="24"/>
-    <row r="671" ht="15.75" customHeight="1" s="24"/>
-    <row r="672" ht="15.75" customHeight="1" s="24"/>
-    <row r="673" ht="15.75" customHeight="1" s="24"/>
-    <row r="674" ht="15.75" customHeight="1" s="24"/>
-    <row r="675" ht="15.75" customHeight="1" s="24"/>
-    <row r="676" ht="15.75" customHeight="1" s="24"/>
-    <row r="677" ht="15.75" customHeight="1" s="24"/>
-    <row r="678" ht="15.75" customHeight="1" s="24"/>
-    <row r="679" ht="15.75" customHeight="1" s="24"/>
-    <row r="680" ht="15.75" customHeight="1" s="24"/>
-    <row r="681" ht="15.75" customHeight="1" s="24"/>
-    <row r="682" ht="15.75" customHeight="1" s="24"/>
-    <row r="683" ht="15.75" customHeight="1" s="24"/>
-    <row r="684" ht="15.75" customHeight="1" s="24"/>
-    <row r="685" ht="15.75" customHeight="1" s="24"/>
-    <row r="686" ht="15.75" customHeight="1" s="24"/>
-    <row r="687" ht="15.75" customHeight="1" s="24"/>
-    <row r="688" ht="15.75" customHeight="1" s="24"/>
-    <row r="689" ht="15.75" customHeight="1" s="24"/>
-    <row r="690" ht="15.75" customHeight="1" s="24"/>
-    <row r="691" ht="15.75" customHeight="1" s="24"/>
-    <row r="692" ht="15.75" customHeight="1" s="24"/>
-    <row r="693" ht="15.75" customHeight="1" s="24"/>
-    <row r="694" ht="15.75" customHeight="1" s="24"/>
-    <row r="695" ht="15.75" customHeight="1" s="24"/>
-    <row r="696" ht="15.75" customHeight="1" s="24"/>
-    <row r="697" ht="15.75" customHeight="1" s="24"/>
-    <row r="698" ht="15.75" customHeight="1" s="24"/>
-    <row r="699" ht="15.75" customHeight="1" s="24"/>
-    <row r="700" ht="15.75" customHeight="1" s="24"/>
-    <row r="701" ht="15.75" customHeight="1" s="24"/>
-    <row r="702" ht="15.75" customHeight="1" s="24"/>
-    <row r="703" ht="15.75" customHeight="1" s="24"/>
-    <row r="704" ht="15.75" customHeight="1" s="24"/>
-    <row r="705" ht="15.75" customHeight="1" s="24"/>
-    <row r="706" ht="15.75" customHeight="1" s="24"/>
-    <row r="707" ht="15.75" customHeight="1" s="24"/>
-    <row r="708" ht="15.75" customHeight="1" s="24"/>
-    <row r="709" ht="15.75" customHeight="1" s="24"/>
-    <row r="710" ht="15.75" customHeight="1" s="24"/>
-    <row r="711" ht="15.75" customHeight="1" s="24"/>
-    <row r="712" ht="15.75" customHeight="1" s="24"/>
-    <row r="713" ht="15.75" customHeight="1" s="24"/>
-    <row r="714" ht="15.75" customHeight="1" s="24"/>
-    <row r="715" ht="15.75" customHeight="1" s="24"/>
-    <row r="716" ht="15.75" customHeight="1" s="24"/>
-    <row r="717" ht="15.75" customHeight="1" s="24"/>
-    <row r="718" ht="15.75" customHeight="1" s="24"/>
-    <row r="719" ht="15.75" customHeight="1" s="24"/>
-    <row r="720" ht="15.75" customHeight="1" s="24"/>
-    <row r="721" ht="15.75" customHeight="1" s="24"/>
-    <row r="722" ht="15.75" customHeight="1" s="24"/>
-    <row r="723" ht="15.75" customHeight="1" s="24"/>
-    <row r="724" ht="15.75" customHeight="1" s="24"/>
-    <row r="725" ht="15.75" customHeight="1" s="24"/>
-    <row r="726" ht="15.75" customHeight="1" s="24"/>
-    <row r="727" ht="15.75" customHeight="1" s="24"/>
-    <row r="728" ht="15.75" customHeight="1" s="24"/>
-    <row r="729" ht="15.75" customHeight="1" s="24"/>
-    <row r="730" ht="15.75" customHeight="1" s="24"/>
-    <row r="731" ht="15.75" customHeight="1" s="24"/>
-    <row r="732" ht="15.75" customHeight="1" s="24"/>
-    <row r="733" ht="15.75" customHeight="1" s="24"/>
-    <row r="734" ht="15.75" customHeight="1" s="24"/>
-    <row r="735" ht="15.75" customHeight="1" s="24"/>
-    <row r="736" ht="15.75" customHeight="1" s="24"/>
-    <row r="737" ht="15.75" customHeight="1" s="24"/>
-    <row r="738" ht="15.75" customHeight="1" s="24"/>
-    <row r="739" ht="15.75" customHeight="1" s="24"/>
-    <row r="740" ht="15.75" customHeight="1" s="24"/>
-    <row r="741" ht="15.75" customHeight="1" s="24"/>
-    <row r="742" ht="15.75" customHeight="1" s="24"/>
-    <row r="743" ht="15.75" customHeight="1" s="24"/>
-    <row r="744" ht="15.75" customHeight="1" s="24"/>
-    <row r="745" ht="15.75" customHeight="1" s="24"/>
-    <row r="746" ht="15.75" customHeight="1" s="24"/>
-    <row r="747" ht="15.75" customHeight="1" s="24"/>
-    <row r="748" ht="15.75" customHeight="1" s="24"/>
-    <row r="749" ht="15.75" customHeight="1" s="24"/>
-    <row r="750" ht="15.75" customHeight="1" s="24"/>
-    <row r="751" ht="15.75" customHeight="1" s="24"/>
-    <row r="752" ht="15.75" customHeight="1" s="24"/>
-    <row r="753" ht="15.75" customHeight="1" s="24"/>
-    <row r="754" ht="15.75" customHeight="1" s="24"/>
-    <row r="755" ht="15.75" customHeight="1" s="24"/>
-    <row r="756" ht="15.75" customHeight="1" s="24"/>
-    <row r="757" ht="15.75" customHeight="1" s="24"/>
-    <row r="758" ht="15.75" customHeight="1" s="24"/>
-    <row r="759" ht="15.75" customHeight="1" s="24"/>
-    <row r="760" ht="15.75" customHeight="1" s="24"/>
-    <row r="761" ht="15.75" customHeight="1" s="24"/>
-    <row r="762" ht="15.75" customHeight="1" s="24"/>
-    <row r="763" ht="15.75" customHeight="1" s="24"/>
-    <row r="764" ht="15.75" customHeight="1" s="24"/>
-    <row r="765" ht="15.75" customHeight="1" s="24"/>
-    <row r="766" ht="15.75" customHeight="1" s="24"/>
-    <row r="767" ht="15.75" customHeight="1" s="24"/>
-    <row r="768" ht="15.75" customHeight="1" s="24"/>
-    <row r="769" ht="15.75" customHeight="1" s="24"/>
-    <row r="770" ht="15.75" customHeight="1" s="24"/>
-    <row r="771" ht="15.75" customHeight="1" s="24"/>
-    <row r="772" ht="15.75" customHeight="1" s="24"/>
-    <row r="773" ht="15.75" customHeight="1" s="24"/>
-    <row r="774" ht="15.75" customHeight="1" s="24"/>
-    <row r="775" ht="15.75" customHeight="1" s="24"/>
-    <row r="776" ht="15.75" customHeight="1" s="24"/>
-    <row r="777" ht="15.75" customHeight="1" s="24"/>
-    <row r="778" ht="15.75" customHeight="1" s="24"/>
-    <row r="779" ht="15.75" customHeight="1" s="24"/>
-    <row r="780" ht="15.75" customHeight="1" s="24"/>
-    <row r="781" ht="15.75" customHeight="1" s="24"/>
-    <row r="782" ht="15.75" customHeight="1" s="24"/>
-    <row r="783" ht="15.75" customHeight="1" s="24"/>
-    <row r="784" ht="15.75" customHeight="1" s="24"/>
-    <row r="785" ht="15.75" customHeight="1" s="24"/>
-    <row r="786" ht="15.75" customHeight="1" s="24"/>
-    <row r="787" ht="15.75" customHeight="1" s="24"/>
-    <row r="788" ht="15.75" customHeight="1" s="24"/>
-    <row r="789" ht="15.75" customHeight="1" s="24"/>
-    <row r="790" ht="15.75" customHeight="1" s="24"/>
-    <row r="791" ht="15.75" customHeight="1" s="24"/>
-    <row r="792" ht="15.75" customHeight="1" s="24"/>
-    <row r="793" ht="15.75" customHeight="1" s="24"/>
-    <row r="794" ht="15.75" customHeight="1" s="24"/>
-    <row r="795" ht="15.75" customHeight="1" s="24"/>
-    <row r="796" ht="15.75" customHeight="1" s="24"/>
-    <row r="797" ht="15.75" customHeight="1" s="24"/>
-    <row r="798" ht="15.75" customHeight="1" s="24"/>
-    <row r="799" ht="15.75" customHeight="1" s="24"/>
-    <row r="800" ht="15.75" customHeight="1" s="24"/>
-    <row r="801" ht="15.75" customHeight="1" s="24"/>
-    <row r="802" ht="15.75" customHeight="1" s="24"/>
-    <row r="803" ht="15.75" customHeight="1" s="24"/>
-    <row r="804" ht="15.75" customHeight="1" s="24"/>
-    <row r="805" ht="15.75" customHeight="1" s="24"/>
-    <row r="806" ht="15.75" customHeight="1" s="24"/>
-    <row r="807" ht="15.75" customHeight="1" s="24"/>
-    <row r="808" ht="15.75" customHeight="1" s="24"/>
-    <row r="809" ht="15.75" customHeight="1" s="24"/>
-    <row r="810" ht="15.75" customHeight="1" s="24"/>
-    <row r="811" ht="15.75" customHeight="1" s="24"/>
-    <row r="812" ht="15.75" customHeight="1" s="24"/>
-    <row r="813" ht="15.75" customHeight="1" s="24"/>
-    <row r="814" ht="15.75" customHeight="1" s="24"/>
-    <row r="815" ht="15.75" customHeight="1" s="24"/>
-    <row r="816" ht="15.75" customHeight="1" s="24"/>
-    <row r="817" ht="15.75" customHeight="1" s="24"/>
-    <row r="818" ht="15.75" customHeight="1" s="24"/>
-    <row r="819" ht="15.75" customHeight="1" s="24"/>
-    <row r="820" ht="15.75" customHeight="1" s="24"/>
-    <row r="821" ht="15.75" customHeight="1" s="24"/>
-    <row r="822" ht="15.75" customHeight="1" s="24"/>
-    <row r="823" ht="15.75" customHeight="1" s="24"/>
-    <row r="824" ht="15.75" customHeight="1" s="24"/>
-    <row r="825" ht="15.75" customHeight="1" s="24"/>
-    <row r="826" ht="15.75" customHeight="1" s="24"/>
-    <row r="827" ht="15.75" customHeight="1" s="24"/>
-    <row r="828" ht="15.75" customHeight="1" s="24"/>
-    <row r="829" ht="15.75" customHeight="1" s="24"/>
-    <row r="830" ht="15.75" customHeight="1" s="24"/>
-    <row r="831" ht="15.75" customHeight="1" s="24"/>
-    <row r="832" ht="15.75" customHeight="1" s="24"/>
-    <row r="833" ht="15.75" customHeight="1" s="24"/>
-    <row r="834" ht="15.75" customHeight="1" s="24"/>
-    <row r="835" ht="15.75" customHeight="1" s="24"/>
-    <row r="836" ht="15.75" customHeight="1" s="24"/>
-    <row r="837" ht="15.75" customHeight="1" s="24"/>
-    <row r="838" ht="15.75" customHeight="1" s="24"/>
-    <row r="839" ht="15.75" customHeight="1" s="24"/>
-    <row r="840" ht="15.75" customHeight="1" s="24"/>
-    <row r="841" ht="15.75" customHeight="1" s="24"/>
-    <row r="842" ht="15.75" customHeight="1" s="24"/>
-    <row r="843" ht="15.75" customHeight="1" s="24"/>
-    <row r="844" ht="15.75" customHeight="1" s="24"/>
-    <row r="845" ht="15.75" customHeight="1" s="24"/>
-    <row r="846" ht="15.75" customHeight="1" s="24"/>
-    <row r="847" ht="15.75" customHeight="1" s="24"/>
-    <row r="848" ht="15.75" customHeight="1" s="24"/>
-    <row r="849" ht="15.75" customHeight="1" s="24"/>
-    <row r="850" ht="15.75" customHeight="1" s="24"/>
-    <row r="851" ht="15.75" customHeight="1" s="24"/>
-    <row r="852" ht="15.75" customHeight="1" s="24"/>
-    <row r="853" ht="15.75" customHeight="1" s="24"/>
-    <row r="854" ht="15.75" customHeight="1" s="24"/>
-    <row r="855" ht="15.75" customHeight="1" s="24"/>
-    <row r="856" ht="15.75" customHeight="1" s="24"/>
-    <row r="857" ht="15.75" customHeight="1" s="24"/>
-    <row r="858" ht="15.75" customHeight="1" s="24"/>
-    <row r="859" ht="15.75" customHeight="1" s="24"/>
-    <row r="860" ht="15.75" customHeight="1" s="24"/>
-    <row r="861" ht="15.75" customHeight="1" s="24"/>
-    <row r="862" ht="15.75" customHeight="1" s="24"/>
-    <row r="863" ht="15.75" customHeight="1" s="24"/>
-    <row r="864" ht="15.75" customHeight="1" s="24"/>
-    <row r="865" ht="15.75" customHeight="1" s="24"/>
-    <row r="866" ht="15.75" customHeight="1" s="24"/>
-    <row r="867" ht="15.75" customHeight="1" s="24"/>
-    <row r="868" ht="15.75" customHeight="1" s="24"/>
-    <row r="869" ht="15.75" customHeight="1" s="24"/>
-    <row r="870" ht="15.75" customHeight="1" s="24"/>
-    <row r="871" ht="15.75" customHeight="1" s="24"/>
-    <row r="872" ht="15.75" customHeight="1" s="24"/>
-    <row r="873" ht="15.75" customHeight="1" s="24"/>
-    <row r="874" ht="15.75" customHeight="1" s="24"/>
-    <row r="875" ht="15.75" customHeight="1" s="24"/>
-    <row r="876" ht="15.75" customHeight="1" s="24"/>
-    <row r="877" ht="15.75" customHeight="1" s="24"/>
-    <row r="878" ht="15.75" customHeight="1" s="24"/>
-    <row r="879" ht="15.75" customHeight="1" s="24"/>
-    <row r="880" ht="15.75" customHeight="1" s="24"/>
-    <row r="881" ht="15.75" customHeight="1" s="24"/>
-    <row r="882" ht="15.75" customHeight="1" s="24"/>
-    <row r="883" ht="15.75" customHeight="1" s="24"/>
-    <row r="884" ht="15.75" customHeight="1" s="24"/>
-    <row r="885" ht="15.75" customHeight="1" s="24"/>
-    <row r="886" ht="15.75" customHeight="1" s="24"/>
-    <row r="887" ht="15.75" customHeight="1" s="24"/>
-    <row r="888" ht="15.75" customHeight="1" s="24"/>
-    <row r="889" ht="15.75" customHeight="1" s="24"/>
-    <row r="890" ht="15.75" customHeight="1" s="24"/>
-    <row r="891" ht="15.75" customHeight="1" s="24"/>
-    <row r="892" ht="15.75" customHeight="1" s="24"/>
-    <row r="893" ht="15.75" customHeight="1" s="24"/>
-    <row r="894" ht="15.75" customHeight="1" s="24"/>
-    <row r="895" ht="15.75" customHeight="1" s="24"/>
-    <row r="896" ht="15.75" customHeight="1" s="24"/>
-    <row r="897" ht="15.75" customHeight="1" s="24"/>
-    <row r="898" ht="15.75" customHeight="1" s="24"/>
-    <row r="899" ht="15.75" customHeight="1" s="24"/>
-    <row r="900" ht="15.75" customHeight="1" s="24"/>
-    <row r="901" ht="15.75" customHeight="1" s="24"/>
-    <row r="902" ht="15.75" customHeight="1" s="24"/>
-    <row r="903" ht="15.75" customHeight="1" s="24"/>
-    <row r="904" ht="15.75" customHeight="1" s="24"/>
-    <row r="905" ht="15.75" customHeight="1" s="24"/>
-    <row r="906" ht="15.75" customHeight="1" s="24"/>
-    <row r="907" ht="15.75" customHeight="1" s="24"/>
-    <row r="908" ht="15.75" customHeight="1" s="24"/>
-    <row r="909" ht="15.75" customHeight="1" s="24"/>
-    <row r="910" ht="15.75" customHeight="1" s="24"/>
-    <row r="911" ht="15.75" customHeight="1" s="24"/>
-    <row r="912" ht="15.75" customHeight="1" s="24"/>
-    <row r="913" ht="15.75" customHeight="1" s="24"/>
-    <row r="914" ht="15.75" customHeight="1" s="24"/>
-    <row r="915" ht="15.75" customHeight="1" s="24"/>
-    <row r="916" ht="15.75" customHeight="1" s="24"/>
-    <row r="917" ht="15.75" customHeight="1" s="24"/>
-    <row r="918" ht="15.75" customHeight="1" s="24"/>
-    <row r="919" ht="15.75" customHeight="1" s="24"/>
-    <row r="920" ht="15.75" customHeight="1" s="24"/>
-    <row r="921" ht="15.75" customHeight="1" s="24"/>
-    <row r="922" ht="15.75" customHeight="1" s="24"/>
-    <row r="923" ht="15.75" customHeight="1" s="24"/>
-    <row r="924" ht="15.75" customHeight="1" s="24"/>
-    <row r="925" ht="15.75" customHeight="1" s="24"/>
-    <row r="926" ht="15.75" customHeight="1" s="24"/>
-    <row r="927" ht="15.75" customHeight="1" s="24"/>
-    <row r="928" ht="15.75" customHeight="1" s="24"/>
-    <row r="929" ht="15.75" customHeight="1" s="24"/>
-    <row r="930" ht="15.75" customHeight="1" s="24"/>
-    <row r="931" ht="15.75" customHeight="1" s="24"/>
-    <row r="932" ht="15.75" customHeight="1" s="24"/>
-    <row r="933" ht="15.75" customHeight="1" s="24"/>
-    <row r="934" ht="15.75" customHeight="1" s="24"/>
-    <row r="935" ht="15.75" customHeight="1" s="24"/>
-    <row r="936" ht="15.75" customHeight="1" s="24"/>
-    <row r="937" ht="15.75" customHeight="1" s="24"/>
-    <row r="938" ht="15.75" customHeight="1" s="24"/>
-    <row r="939" ht="15.75" customHeight="1" s="24"/>
-    <row r="940" ht="15.75" customHeight="1" s="24"/>
-    <row r="941" ht="15.75" customHeight="1" s="24"/>
-    <row r="942" ht="15.75" customHeight="1" s="24"/>
-    <row r="943" ht="15.75" customHeight="1" s="24"/>
-    <row r="944" ht="15.75" customHeight="1" s="24"/>
-    <row r="945" ht="15.75" customHeight="1" s="24"/>
-    <row r="946" ht="15.75" customHeight="1" s="24"/>
-    <row r="947" ht="15.75" customHeight="1" s="24"/>
-    <row r="948" ht="15.75" customHeight="1" s="24"/>
-    <row r="949" ht="15.75" customHeight="1" s="24"/>
-    <row r="950" ht="15.75" customHeight="1" s="24"/>
-    <row r="951" ht="15.75" customHeight="1" s="24"/>
-    <row r="952" ht="15.75" customHeight="1" s="24"/>
-    <row r="953" ht="15.75" customHeight="1" s="24"/>
-    <row r="954" ht="15.75" customHeight="1" s="24"/>
-    <row r="955" ht="15.75" customHeight="1" s="24"/>
-    <row r="956" ht="15.75" customHeight="1" s="24"/>
-    <row r="957" ht="15.75" customHeight="1" s="24"/>
-    <row r="958" ht="15.75" customHeight="1" s="24"/>
-    <row r="959" ht="15.75" customHeight="1" s="24"/>
-    <row r="960" ht="15.75" customHeight="1" s="24"/>
-    <row r="961" ht="15.75" customHeight="1" s="24"/>
-    <row r="962" ht="15.75" customHeight="1" s="24"/>
-    <row r="963" ht="15.75" customHeight="1" s="24"/>
-    <row r="964" ht="15.75" customHeight="1" s="24"/>
-    <row r="965" ht="15.75" customHeight="1" s="24"/>
-    <row r="966" ht="15.75" customHeight="1" s="24"/>
-    <row r="967" ht="15.75" customHeight="1" s="24"/>
-    <row r="968" ht="15.75" customHeight="1" s="24"/>
-    <row r="969" ht="15.75" customHeight="1" s="24"/>
-    <row r="970" ht="15.75" customHeight="1" s="24"/>
-    <row r="971" ht="15.75" customHeight="1" s="24"/>
-    <row r="972" ht="15.75" customHeight="1" s="24"/>
-    <row r="973" ht="15.75" customHeight="1" s="24"/>
-    <row r="974" ht="15.75" customHeight="1" s="24"/>
-    <row r="975" ht="15.75" customHeight="1" s="24"/>
-    <row r="976" ht="15.75" customHeight="1" s="24"/>
-    <row r="977" ht="15.75" customHeight="1" s="24"/>
-    <row r="978" ht="15.75" customHeight="1" s="24"/>
-    <row r="979" ht="15.75" customHeight="1" s="24"/>
-    <row r="980" ht="15.75" customHeight="1" s="24"/>
-    <row r="981" ht="15.75" customHeight="1" s="24"/>
-    <row r="982" ht="15.75" customHeight="1" s="24"/>
-    <row r="983" ht="15.75" customHeight="1" s="24"/>
-    <row r="984" ht="15.75" customHeight="1" s="24"/>
-    <row r="985" ht="15.75" customHeight="1" s="24"/>
-    <row r="986" ht="15.75" customHeight="1" s="24"/>
-    <row r="987" ht="15.75" customHeight="1" s="24"/>
-    <row r="988" ht="15.75" customHeight="1" s="24"/>
-    <row r="989" ht="15.75" customHeight="1" s="24"/>
-    <row r="990" ht="15.75" customHeight="1" s="24"/>
-    <row r="991" ht="15.75" customHeight="1" s="24"/>
-    <row r="992" ht="15.75" customHeight="1" s="24"/>
-    <row r="993" ht="15.75" customHeight="1" s="24"/>
-    <row r="994" ht="15.75" customHeight="1" s="24"/>
-    <row r="995" ht="15.75" customHeight="1" s="24"/>
-    <row r="996" ht="15.75" customHeight="1" s="24"/>
-    <row r="997" ht="15.75" customHeight="1" s="24"/>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
+<ns0:worksheet xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <ns0:sheetPr>
+    <ns0:tabColor rgb="FF17324D"/>
+    <ns0:outlinePr summaryBelow="1" summaryRight="1"/>
+    <ns0:pageSetUpPr/>
+  </ns0:sheetPr>
+  <ns0:dimension ref="A2:F14"/>
+  <ns0:sheetFormatPr baseColWidth="8" defaultColWidth="12.625" defaultRowHeight="14.25"/>
+  <ns0:cols>
+    <ns0:col width="24" customWidth="1" style="24" min="1" max="1"/>
+    <ns0:col width="15" customWidth="1" style="24" min="2" max="2"/>
+    <ns0:col width="4" customWidth="1" style="24" min="3" max="3"/>
+    <ns0:col width="24" customWidth="1" style="24" min="4" max="4"/>
+    <ns0:col width="15" customWidth="1" style="24" min="5" max="5"/>
+    <ns0:col width="8" customWidth="1" style="24" min="6" max="6"/>
+    <ns0:col width="8.625" customWidth="1" style="24" min="7" max="26"/>
+  </ns0:cols>
+  <ns0:sheetData>
+    <ns0:row r="1" ht="15" customHeight="1" s="24"/>
+    <ns0:row r="2" ht="25.5" customHeight="1" s="24">
+      <ns0:c r="B2" s="1" t="inlineStr">
+        <ns0:is>
+          <ns0:t>TỔNG HỢP SỬ DỤNG AI — TUẦN 07</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C2" s="2" t="n"/>
+      <ns0:c r="D2" s="2" t="n"/>
+      <ns0:c r="E2" s="2" t="n"/>
+      <ns0:c r="F2" s="2" t="n"/>
+    </ns0:row>
+    <ns0:row r="3" ht="19.5" customHeight="1" s="24">
+      <ns0:c r="A3" s="30" t="inlineStr">
+        <ns0:is>
+          <ns0:t>26/10/2026 – 01/11/2026</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B3" s="2" t="n"/>
+      <ns0:c r="C3" s="2" t="n"/>
+      <ns0:c r="D3" s="2" t="n"/>
+      <ns0:c r="E3" s="2" t="n"/>
+      <ns0:c r="F3" s="2" t="n"/>
+    </ns0:row>
+    <ns0:row r="4" ht="15" customHeight="1" s="24">
+      <ns0:c r="A4" s="2" t="n"/>
+      <ns0:c r="B4" s="2" t="n"/>
+      <ns0:c r="C4" s="2" t="n"/>
+      <ns0:c r="D4" s="2" t="n"/>
+      <ns0:c r="E4" s="2" t="n"/>
+      <ns0:c r="F4" s="2" t="n"/>
+    </ns0:row>
+    <ns0:row r="5" ht="33.75" customHeight="1" s="24">
+      <ns0:c r="A5" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>TỔNG SỐ PROMPT</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B5" s="5">
+        <ns0:f>SUM(B9:B11)</ns0:f>
+        <ns0:v>13</ns0:v>
+      </ns0:c>
+      <ns0:c r="C5" s="2" t="n"/>
+      <ns0:c r="D5" s="2" t="n"/>
+      <ns0:c r="E5" s="2" t="n"/>
+      <ns0:c r="F5" s="2" t="n"/>
+    </ns0:row>
+    <ns0:row r="6" ht="15" customHeight="1" s="24">
+      <ns0:c r="A6" s="2" t="n"/>
+      <ns0:c r="B6" s="2" t="n"/>
+      <ns0:c r="C6" s="2" t="n"/>
+      <ns0:c r="D6" s="2" t="n"/>
+      <ns0:c r="E6" s="2" t="n"/>
+      <ns0:c r="F6" s="2" t="n"/>
+    </ns0:row>
+    <ns0:row r="7" ht="15" customHeight="1" s="24">
+      <ns0:c r="A7" s="2" t="n"/>
+      <ns0:c r="B7" s="2" t="n"/>
+      <ns0:c r="C7" s="2" t="n"/>
+      <ns0:c r="D7" s="2" t="n"/>
+      <ns0:c r="E7" s="2" t="n"/>
+      <ns0:c r="F7" s="2" t="n"/>
+    </ns0:row>
+    <ns0:row r="8" ht="27.75" customHeight="1" s="24">
+      <ns0:c r="A8" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NGƯỜI TẠO</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B8" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>SỐ PROMPT</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C8" s="2" t="n"/>
+      <ns0:c r="D8" s="10" t="inlineStr">
+        <ns0:is>
+          <ns0:t>TOOL AI</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E8" s="10" t="inlineStr">
+        <ns0:is>
+          <ns0:t>SỐ PROMPT</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F8" s="2" t="n"/>
+    </ns0:row>
+    <ns0:row r="9" ht="24.75" customHeight="1" s="24">
+      <ns0:c r="A9" s="11" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Thắng</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B9" s="13">
+        <ns0:f>COUNTIF(Thắng!$A$6:$A$306,"&lt;&gt;")</ns0:f>
+        <ns0:v>11</ns0:v>
+      </ns0:c>
+      <ns0:c r="C9" s="2" t="n"/>
+      <ns0:c r="D9" s="14" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Claude</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E9" s="16">
+        <ns0:f>COUNTIFS(Thắng!$A$6:$A$306,"&lt;&gt;",Thắng!$C$6:$C$306,D9)+COUNTIFS(Sang!$A$6:$A$306,"&lt;&gt;",Sang!$C$6:$C$306,D9)+COUNTIFS(Nguyên!$A$6:$A$306,"&lt;&gt;",Nguyên!$C$6:$C$306,D9)</ns0:f>
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="F9" s="2" t="n"/>
+    </ns0:row>
+    <ns0:row r="10" ht="24.75" customHeight="1" s="24">
+      <ns0:c r="A10" s="11" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Sang</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B10" s="13">
+        <ns0:f>COUNTIF(Sang!$A$6:$A$306,"&lt;&gt;")</ns0:f>
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="C10" s="2" t="n"/>
+      <ns0:c r="D10" s="14" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Codex</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E10" s="16">
+        <ns0:f>COUNTIFS(Thắng!$A$6:$A$306,"&lt;&gt;",Thắng!$C$6:$C$306,D10)+COUNTIFS(Sang!$A$6:$A$306,"&lt;&gt;",Sang!$C$6:$C$306,D10)+COUNTIFS(Nguyên!$A$6:$A$306,"&lt;&gt;",Nguyên!$C$6:$C$306,D10)</ns0:f>
+        <ns0:v>2</ns0:v>
+      </ns0:c>
+      <ns0:c r="F10" s="2" t="n"/>
+    </ns0:row>
+    <ns0:row r="11" ht="24.75" customHeight="1" s="24">
+      <ns0:c r="A11" s="11" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Nguyên</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B11" s="13">
+        <ns0:f>COUNTIF(Nguyên!$A$6:$A$306,"&lt;&gt;")</ns0:f>
+        <ns0:v>2</ns0:v>
+      </ns0:c>
+      <ns0:c r="C11" s="2" t="n"/>
+      <ns0:c r="D11" s="14" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Antigravity</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E11" s="16">
+        <ns0:f>COUNTIFS(Thắng!$A$6:$A$306,"&lt;&gt;",Thắng!$C$6:$C$306,D11)+COUNTIFS(Sang!$A$6:$A$306,"&lt;&gt;",Sang!$C$6:$C$306,D11)+COUNTIFS(Nguyên!$A$6:$A$306,"&lt;&gt;",Nguyên!$C$6:$C$306,D11)</ns0:f>
+        <ns0:v>11</ns0:v>
+      </ns0:c>
+      <ns0:c r="F11" s="2" t="n"/>
+    </ns0:row>
+    <ns0:row r="12" ht="15" customHeight="1" s="24">
+      <ns0:c r="A12" s="2" t="n"/>
+      <ns0:c r="B12" s="2" t="n"/>
+      <ns0:c r="C12" s="2" t="n"/>
+      <ns0:c r="D12" s="2" t="n"/>
+      <ns0:c r="E12" s="2" t="n"/>
+      <ns0:c r="F12" s="2" t="n"/>
+    </ns0:row>
+    <ns0:row r="13" ht="15" customHeight="1" s="24">
+      <ns0:c r="A13" s="2" t="n"/>
+      <ns0:c r="B13" s="2" t="n"/>
+      <ns0:c r="C13" s="2" t="n"/>
+      <ns0:c r="D13" s="2" t="n"/>
+      <ns0:c r="E13" s="2" t="n"/>
+      <ns0:c r="F13" s="2" t="n"/>
+    </ns0:row>
+    <ns0:row r="14" ht="15" customHeight="1" s="24">
+      <ns0:c r="A14" s="17" t="n"/>
+      <ns0:c r="B14" s="2" t="n"/>
+      <ns0:c r="C14" s="2" t="n"/>
+      <ns0:c r="D14" s="2" t="n"/>
+      <ns0:c r="E14" s="2" t="n"/>
+      <ns0:c r="F14" s="2" t="n"/>
+    </ns0:row>
+    <ns0:row r="18" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="19" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="20" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="21" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="22" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="23" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="24" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="25" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="26" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="27" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="28" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="29" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="30" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="31" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="32" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="33" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="34" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="35" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="36" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="37" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="38" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="39" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="40" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="41" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="42" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="43" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="44" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="45" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="46" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="47" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="48" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="49" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="50" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="51" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="52" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="53" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="54" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="55" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="56" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="57" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="58" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="59" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="60" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="61" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="62" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="63" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="64" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="65" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="66" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="67" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="68" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="69" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="70" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="71" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="72" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="73" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="74" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="75" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="76" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="77" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="78" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="79" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="80" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="81" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="82" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="83" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="84" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="85" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="86" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="87" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="88" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="89" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="90" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="91" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="92" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="93" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="94" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="95" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="96" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="97" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="98" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="99" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="100" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="101" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="102" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="103" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="104" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="105" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="106" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="107" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="108" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="109" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="110" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="111" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="112" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="113" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="114" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="115" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="116" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="117" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="118" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="119" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="120" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="121" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="122" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="123" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="124" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="125" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="126" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="127" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="128" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="129" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="130" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="131" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="132" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="133" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="134" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="135" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="136" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="137" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="138" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="139" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="140" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="141" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="142" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="143" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="144" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="145" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="146" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="147" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="148" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="149" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="150" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="151" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="152" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="153" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="154" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="155" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="156" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="157" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="158" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="159" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="160" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="161" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="162" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="163" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="164" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="165" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="166" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="167" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="168" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="169" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="170" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="171" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="172" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="173" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="174" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="175" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="176" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="177" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="178" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="179" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="180" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="181" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="182" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="183" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="184" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="185" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="186" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="187" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="188" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="189" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="190" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="191" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="192" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="193" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="194" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="195" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="196" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="197" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="198" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="199" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="200" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="201" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="202" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="203" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="204" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="205" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="206" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="207" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="208" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="209" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="210" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="211" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="212" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="213" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="214" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="215" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="216" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="217" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="218" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="219" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="220" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="221" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="222" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="223" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="224" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="225" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="226" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="227" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="228" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="229" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="230" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="231" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="232" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="233" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="234" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="235" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="236" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="237" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="238" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="239" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="240" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="241" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="242" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="243" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="244" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="245" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="246" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="247" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="248" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="249" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="250" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="251" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="252" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="253" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="254" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="255" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="256" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="257" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="258" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="259" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="260" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="261" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="262" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="263" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="264" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="265" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="266" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="267" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="268" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="269" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="270" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="271" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="272" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="273" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="274" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="275" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="276" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="277" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="278" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="279" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="280" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="281" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="282" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="283" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="284" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="285" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="286" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="287" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="288" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="289" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="290" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="291" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="292" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="293" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="294" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="295" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="296" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="297" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="298" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="299" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="300" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="301" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="302" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="303" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="304" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="305" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="306" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="307" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="308" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="309" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="310" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="311" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="312" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="313" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="314" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="315" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="316" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="317" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="318" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="319" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="320" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="321" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="322" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="323" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="324" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="325" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="326" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="327" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="328" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="329" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="330" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="331" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="332" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="333" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="334" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="335" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="336" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="337" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="338" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="339" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="340" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="341" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="342" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="343" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="344" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="345" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="346" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="347" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="348" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="349" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="350" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="351" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="352" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="353" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="354" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="355" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="356" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="357" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="358" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="359" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="360" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="361" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="362" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="363" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="364" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="365" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="366" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="367" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="368" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="369" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="370" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="371" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="372" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="373" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="374" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="375" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="376" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="377" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="378" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="379" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="380" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="381" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="382" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="383" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="384" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="385" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="386" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="387" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="388" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="389" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="390" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="391" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="392" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="393" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="394" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="395" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="396" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="397" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="398" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="399" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="400" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="401" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="402" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="403" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="404" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="405" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="406" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="407" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="408" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="409" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="410" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="411" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="412" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="413" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="414" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="415" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="416" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="417" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="418" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="419" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="420" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="421" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="422" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="423" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="424" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="425" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="426" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="427" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="428" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="429" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="430" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="431" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="432" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="433" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="434" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="435" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="436" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="437" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="438" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="439" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="440" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="441" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="442" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="443" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="444" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="445" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="446" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="447" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="448" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="449" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="450" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="451" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="452" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="453" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="454" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="455" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="456" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="457" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="458" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="459" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="460" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="461" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="462" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="463" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="464" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="465" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="466" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="467" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="468" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="469" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="470" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="471" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="472" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="473" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="474" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="475" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="476" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="477" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="478" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="479" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="480" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="481" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="482" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="483" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="484" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="485" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="486" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="487" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="488" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="489" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="490" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="491" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="492" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="493" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="494" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="495" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="496" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="497" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="498" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="499" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="500" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="501" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="502" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="503" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="504" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="505" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="506" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="507" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="508" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="509" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="510" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="511" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="512" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="513" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="514" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="515" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="516" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="517" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="518" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="519" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="520" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="521" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="522" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="523" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="524" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="525" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="526" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="527" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="528" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="529" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="530" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="531" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="532" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="533" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="534" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="535" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="536" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="537" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="538" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="539" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="540" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="541" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="542" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="543" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="544" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="545" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="546" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="547" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="548" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="549" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="550" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="551" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="552" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="553" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="554" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="555" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="556" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="557" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="558" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="559" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="560" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="561" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="562" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="563" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="564" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="565" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="566" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="567" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="568" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="569" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="570" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="571" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="572" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="573" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="574" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="575" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="576" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="577" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="578" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="579" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="580" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="581" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="582" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="583" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="584" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="585" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="586" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="587" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="588" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="589" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="590" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="591" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="592" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="593" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="594" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="595" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="596" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="597" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="598" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="599" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="600" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="601" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="602" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="603" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="604" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="605" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="606" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="607" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="608" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="609" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="610" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="611" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="612" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="613" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="614" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="615" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="616" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="617" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="618" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="619" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="620" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="621" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="622" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="623" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="624" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="625" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="626" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="627" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="628" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="629" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="630" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="631" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="632" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="633" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="634" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="635" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="636" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="637" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="638" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="639" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="640" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="641" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="642" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="643" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="644" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="645" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="646" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="647" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="648" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="649" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="650" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="651" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="652" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="653" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="654" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="655" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="656" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="657" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="658" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="659" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="660" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="661" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="662" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="663" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="664" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="665" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="666" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="667" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="668" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="669" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="670" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="671" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="672" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="673" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="674" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="675" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="676" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="677" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="678" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="679" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="680" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="681" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="682" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="683" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="684" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="685" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="686" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="687" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="688" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="689" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="690" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="691" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="692" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="693" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="694" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="695" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="696" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="697" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="698" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="699" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="700" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="701" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="702" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="703" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="704" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="705" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="706" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="707" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="708" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="709" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="710" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="711" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="712" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="713" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="714" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="715" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="716" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="717" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="718" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="719" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="720" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="721" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="722" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="723" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="724" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="725" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="726" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="727" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="728" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="729" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="730" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="731" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="732" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="733" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="734" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="735" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="736" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="737" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="738" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="739" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="740" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="741" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="742" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="743" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="744" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="745" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="746" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="747" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="748" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="749" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="750" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="751" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="752" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="753" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="754" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="755" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="756" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="757" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="758" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="759" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="760" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="761" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="762" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="763" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="764" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="765" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="766" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="767" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="768" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="769" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="770" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="771" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="772" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="773" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="774" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="775" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="776" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="777" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="778" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="779" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="780" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="781" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="782" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="783" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="784" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="785" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="786" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="787" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="788" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="789" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="790" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="791" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="792" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="793" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="794" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="795" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="796" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="797" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="798" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="799" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="800" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="801" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="802" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="803" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="804" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="805" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="806" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="807" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="808" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="809" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="810" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="811" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="812" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="813" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="814" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="815" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="816" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="817" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="818" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="819" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="820" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="821" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="822" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="823" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="824" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="825" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="826" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="827" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="828" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="829" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="830" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="831" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="832" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="833" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="834" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="835" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="836" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="837" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="838" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="839" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="840" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="841" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="842" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="843" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="844" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="845" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="846" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="847" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="848" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="849" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="850" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="851" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="852" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="853" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="854" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="855" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="856" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="857" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="858" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="859" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="860" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="861" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="862" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="863" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="864" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="865" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="866" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="867" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="868" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="869" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="870" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="871" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="872" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="873" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="874" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="875" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="876" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="877" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="878" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="879" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="880" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="881" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="882" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="883" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="884" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="885" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="886" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="887" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="888" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="889" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="890" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="891" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="892" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="893" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="894" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="895" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="896" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="897" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="898" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="899" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="900" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="901" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="902" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="903" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="904" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="905" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="906" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="907" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="908" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="909" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="910" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="911" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="912" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="913" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="914" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="915" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="916" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="917" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="918" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="919" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="920" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="921" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="922" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="923" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="924" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="925" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="926" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="927" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="928" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="929" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="930" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="931" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="932" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="933" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="934" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="935" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="936" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="937" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="938" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="939" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="940" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="941" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="942" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="943" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="944" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="945" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="946" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="947" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="948" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="949" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="950" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="951" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="952" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="953" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="954" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="955" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="956" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="957" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="958" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="959" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="960" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="961" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="962" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="963" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="964" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="965" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="966" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="967" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="968" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="969" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="970" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="971" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="972" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="973" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="974" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="975" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="976" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="977" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="978" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="979" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="980" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="981" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="982" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="983" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="984" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="985" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="986" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="987" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="988" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="989" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="990" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="991" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="992" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="993" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="994" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="995" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="996" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="997" ht="15.75" customHeight="1" s="24"/>
+  </ns0:sheetData>
+  <ns0:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</ns0:worksheet>
 </file>
</xml_diff>

<commit_message>
docs(SCRUM-103): record PR and W07 evidence
</commit_message>
<xml_diff>
--- a/docs/evidence/tc2-3-ai-usage/AI Prompt Log - W07 - 2026-10-26_2026-11-01.xlsx
+++ b/docs/evidence/tc2-3-ai-usage/AI Prompt Log - W07 - 2026-10-26_2026-11-01.xlsx
@@ -6968,13 +6968,35 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="36" customHeight="1" s="24">
-      <c r="A8" s="32" t="n"/>
-      <c r="B8" s="18" t="n"/>
-      <c r="C8" s="18" t="n"/>
-      <c r="D8" s="33" t="n"/>
-      <c r="E8" s="33" t="n"/>
-      <c r="F8" s="33" t="n"/>
+    <row r="8" ht="48" customHeight="1" s="24">
+      <c r="A8" s="32" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>Nguyên</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="D8" s="33" t="inlineStr">
+        <is>
+          <t>Tạo PR SCRUM-103 vào main và theo dõi CI trước khi merge</t>
+        </is>
+      </c>
+      <c r="E8" s="33" t="inlineStr">
+        <is>
+          <t>Hãy Tạo PR rồi merge vào main đi</t>
+        </is>
+      </c>
+      <c r="F8" s="33" t="inlineStr">
+        <is>
+          <t>Pull request SCRUM-103: https://github.com/thanglb2005/ai-assessor-cefr/pull/68</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="36" customHeight="1" s="24">
       <c r="A9" s="32" t="n"/>
@@ -18894,7 +18916,7 @@
       </ns0:c>
       <ns0:c r="B5" s="5">
         <ns0:f>SUM(B9:B11)</ns0:f>
-        <ns0:v>13</ns0:v>
+        <ns0:v>14</ns0:v>
       </ns0:c>
       <ns0:c r="C5" s="2" t="n"/>
       <ns0:c r="D5" s="2" t="n"/>
@@ -18981,7 +19003,7 @@
       </ns0:c>
       <ns0:c r="E10" s="16">
         <ns0:f>COUNTIFS(Thắng!$A$6:$A$306,"&lt;&gt;",Thắng!$C$6:$C$306,D10)+COUNTIFS(Sang!$A$6:$A$306,"&lt;&gt;",Sang!$C$6:$C$306,D10)+COUNTIFS(Nguyên!$A$6:$A$306,"&lt;&gt;",Nguyên!$C$6:$C$306,D10)</ns0:f>
-        <ns0:v>2</ns0:v>
+        <ns0:v>3</ns0:v>
       </ns0:c>
       <ns0:c r="F10" s="2" t="n"/>
     </ns0:row>
@@ -18993,7 +19015,7 @@
       </ns0:c>
       <ns0:c r="B11" s="13">
         <ns0:f>COUNTIF(Nguyên!$A$6:$A$306,"&lt;&gt;")</ns0:f>
-        <ns0:v>2</ns0:v>
+        <ns0:v>3</ns0:v>
       </ns0:c>
       <ns0:c r="C11" s="2" t="n"/>
       <ns0:c r="D11" s="14" t="inlineStr">

</xml_diff>

<commit_message>
[SCRUM-103] Chuyển M15: toàn bộ trang và test E2E (#68)
* feat(SCRUM-103): migrate M15 pages and E2E

* docs(SCRUM-103): record PR and W07 evidence
</commit_message>
<xml_diff>
--- a/docs/evidence/tc2-3-ai-usage/AI Prompt Log - W07 - 2026-10-26_2026-11-01.xlsx
+++ b/docs/evidence/tc2-3-ai-usage/AI Prompt Log - W07 - 2026-10-26_2026-11-01.xlsx
@@ -1,14 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet name="Thắng" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Nguyên" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Sang" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Tổng hợp" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thắng" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nguyên" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sang" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tổng hợp" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
+  <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
 </file>
 
@@ -6908,28 +6909,94 @@
       </c>
     </row>
     <row r="6" ht="48" customHeight="1" s="24">
-      <c r="A6" s="32" t="n"/>
-      <c r="B6" s="18" t="n"/>
-      <c r="C6" s="18" t="n"/>
-      <c r="D6" s="33" t="n"/>
-      <c r="E6" s="33" t="n"/>
-      <c r="F6" s="33" t="n"/>
+      <c r="A6" s="32" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>Nguyên</t>
+        </is>
+      </c>
+      <c r="C6" s="18" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="D6" s="33" t="inlineStr">
+        <is>
+          <t>Đọc Jira SCRUM-103; chuyển giao M15 và rà soát kiểm thử E2E</t>
+        </is>
+      </c>
+      <c r="E6" s="33" t="inlineStr">
+        <is>
+          <t>Đóng vai trò như 1 người senior trong lĩnh vực IT và hãy làm task SCRUM-103 trên nhánh SCRUM/103 đã tạo từ đầu và hãy đọc trên jira để có thể làm</t>
+        </is>
+      </c>
+      <c r="F6" s="33" t="inlineStr">
+        <is>
+          <t>../../sdd/modules/m15-product-web/reviews/implementation-transfer-scrum-103-2026-10-28.md</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="48" customHeight="1" s="24">
-      <c r="A7" s="32" t="n"/>
-      <c r="B7" s="18" t="n"/>
-      <c r="C7" s="18" t="n"/>
-      <c r="D7" s="33" t="n"/>
-      <c r="E7" s="33" t="n"/>
-      <c r="F7" s="33" t="n"/>
-    </row>
-    <row r="8" ht="36" customHeight="1" s="24">
-      <c r="A8" s="32" t="n"/>
-      <c r="B8" s="18" t="n"/>
-      <c r="C8" s="18" t="n"/>
-      <c r="D8" s="33" t="n"/>
-      <c r="E8" s="33" t="n"/>
-      <c r="F8" s="33" t="n"/>
+      <c r="A7" s="32" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B7" s="18" t="inlineStr">
+        <is>
+          <t>Nguyên</t>
+        </is>
+      </c>
+      <c r="C7" s="18" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="D7" s="33" t="inlineStr">
+        <is>
+          <t>Mở rộng SCRUM-103 sang middleware M16 để gỡ blocker khởi động; kiểm thử hồi quy</t>
+        </is>
+      </c>
+      <c r="E7" s="33" t="inlineStr">
+        <is>
+          <t>Bạn muốn mình mở rộng phạm vi để sửa middleware M16 trên nhánh này mở rộng đi</t>
+        </is>
+      </c>
+      <c r="F7" s="33" t="inlineStr">
+        <is>
+          <t>../../sdd/modules/m16-monolith-runtime/evidence/scrum-103-middleware-integration.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="48" customHeight="1" s="24">
+      <c r="A8" s="32" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>Nguyên</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="D8" s="33" t="inlineStr">
+        <is>
+          <t>Tạo PR SCRUM-103 vào main và theo dõi CI trước khi merge</t>
+        </is>
+      </c>
+      <c r="E8" s="33" t="inlineStr">
+        <is>
+          <t>Hãy Tạo PR rồi merge vào main đi</t>
+        </is>
+      </c>
+      <c r="F8" s="33" t="inlineStr">
+        <is>
+          <t>Pull request SCRUM-103: https://github.com/thanglb2005/ai-assessor-cefr/pull/68</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="36" customHeight="1" s="24">
       <c r="A9" s="32" t="n"/>
@@ -18791,1182 +18858,1182 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor rgb="FF17324D"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A2:F14"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="12.625" defaultRowHeight="14.25"/>
-  <cols>
-    <col width="24" customWidth="1" style="24" min="1" max="1"/>
-    <col width="15" customWidth="1" style="24" min="2" max="2"/>
-    <col width="4" customWidth="1" style="24" min="3" max="3"/>
-    <col width="24" customWidth="1" style="24" min="4" max="4"/>
-    <col width="15" customWidth="1" style="24" min="5" max="5"/>
-    <col width="8" customWidth="1" style="24" min="6" max="6"/>
-    <col width="8.625" customWidth="1" style="24" min="7" max="26"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="15" customHeight="1" s="24"/>
-    <row r="2" ht="25.5" customHeight="1" s="24">
-      <c r="B2" s="1" t="inlineStr">
-        <is>
-          <t>TỔNG HỢP SỬ DỤNG AI — TUẦN 07</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-    </row>
-    <row r="3" ht="19.5" customHeight="1" s="24">
-      <c r="A3" s="30" t="inlineStr">
-        <is>
-          <t>26/10/2026 – 01/11/2026</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="n"/>
-      <c r="C3" s="2" t="n"/>
-      <c r="D3" s="2" t="n"/>
-      <c r="E3" s="2" t="n"/>
-      <c r="F3" s="2" t="n"/>
-    </row>
-    <row r="4" ht="15" customHeight="1" s="24">
-      <c r="A4" s="2" t="n"/>
-      <c r="B4" s="2" t="n"/>
-      <c r="C4" s="2" t="n"/>
-      <c r="D4" s="2" t="n"/>
-      <c r="E4" s="2" t="n"/>
-      <c r="F4" s="2" t="n"/>
-    </row>
-    <row r="5" ht="33.75" customHeight="1" s="24">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>TỔNG SỐ PROMPT</t>
-        </is>
-      </c>
-      <c r="B5" s="5">
-        <f>SUM(B9:B11)</f>
-        <v>11</v>
-      </c>
-      <c r="C5" s="2" t="n"/>
-      <c r="D5" s="2" t="n"/>
-      <c r="E5" s="2" t="n"/>
-      <c r="F5" s="2" t="n"/>
-    </row>
-    <row r="6" ht="15" customHeight="1" s="24">
-      <c r="A6" s="2" t="n"/>
-      <c r="B6" s="2" t="n"/>
-      <c r="C6" s="2" t="n"/>
-      <c r="D6" s="2" t="n"/>
-      <c r="E6" s="2" t="n"/>
-      <c r="F6" s="2" t="n"/>
-    </row>
-    <row r="7" ht="15" customHeight="1" s="24">
-      <c r="A7" s="2" t="n"/>
-      <c r="B7" s="2" t="n"/>
-      <c r="C7" s="2" t="n"/>
-      <c r="D7" s="2" t="n"/>
-      <c r="E7" s="2" t="n"/>
-      <c r="F7" s="2" t="n"/>
-    </row>
-    <row r="8" ht="27.75" customHeight="1" s="24">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>NGƯỜI TẠO</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>SỐ PROMPT</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="n"/>
-      <c r="D8" s="10" t="inlineStr">
-        <is>
-          <t>TOOL AI</t>
-        </is>
-      </c>
-      <c r="E8" s="10" t="inlineStr">
-        <is>
-          <t>SỐ PROMPT</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="n"/>
-    </row>
-    <row r="9" ht="24.75" customHeight="1" s="24">
-      <c r="A9" s="11" t="inlineStr">
-        <is>
-          <t>Thắng</t>
-        </is>
-      </c>
-      <c r="B9" s="13">
-        <f>COUNTIF(Thắng!$A$6:$A$306,"&lt;&gt;")</f>
-        <v>11</v>
-      </c>
-      <c r="C9" s="2" t="n"/>
-      <c r="D9" s="14" t="inlineStr">
-        <is>
-          <t>Claude</t>
-        </is>
-      </c>
-      <c r="E9" s="16">
-        <f>COUNTIFS(Thắng!$A$6:$A$306,"&lt;&gt;",Thắng!$C$6:$C$306,D9)+COUNTIFS(Sang!$A$6:$A$306,"&lt;&gt;",Sang!$C$6:$C$306,D9)+COUNTIFS(Nguyên!$A$6:$A$306,"&lt;&gt;",Nguyên!$C$6:$C$306,D9)</f>
-        <v>0</v>
-      </c>
-      <c r="F9" s="2" t="n"/>
-    </row>
-    <row r="10" ht="24.75" customHeight="1" s="24">
-      <c r="A10" s="11" t="inlineStr">
-        <is>
-          <t>Sang</t>
-        </is>
-      </c>
-      <c r="B10" s="13">
-        <f>COUNTIF(Sang!$A$6:$A$306,"&lt;&gt;")</f>
-        <v>0</v>
-      </c>
-      <c r="C10" s="2" t="n"/>
-      <c r="D10" s="14" t="inlineStr">
-        <is>
-          <t>Codex</t>
-        </is>
-      </c>
-      <c r="E10" s="16">
-        <f>COUNTIFS(Thắng!$A$6:$A$306,"&lt;&gt;",Thắng!$C$6:$C$306,D10)+COUNTIFS(Sang!$A$6:$A$306,"&lt;&gt;",Sang!$C$6:$C$306,D10)+COUNTIFS(Nguyên!$A$6:$A$306,"&lt;&gt;",Nguyên!$C$6:$C$306,D10)</f>
-        <v>0</v>
-      </c>
-      <c r="F10" s="2" t="n"/>
-    </row>
-    <row r="11" ht="24.75" customHeight="1" s="24">
-      <c r="A11" s="11" t="inlineStr">
-        <is>
-          <t>Nguyên</t>
-        </is>
-      </c>
-      <c r="B11" s="13">
-        <f>COUNTIF(Nguyên!$A$6:$A$306,"&lt;&gt;")</f>
-        <v>0</v>
-      </c>
-      <c r="C11" s="2" t="n"/>
-      <c r="D11" s="14" t="inlineStr">
-        <is>
-          <t>Antigravity</t>
-        </is>
-      </c>
-      <c r="E11" s="16">
-        <f>COUNTIFS(Thắng!$A$6:$A$306,"&lt;&gt;",Thắng!$C$6:$C$306,D11)+COUNTIFS(Sang!$A$6:$A$306,"&lt;&gt;",Sang!$C$6:$C$306,D11)+COUNTIFS(Nguyên!$A$6:$A$306,"&lt;&gt;",Nguyên!$C$6:$C$306,D11)</f>
-        <v>11</v>
-      </c>
-      <c r="F11" s="2" t="n"/>
-    </row>
-    <row r="12" ht="15" customHeight="1" s="24">
-      <c r="A12" s="2" t="n"/>
-      <c r="B12" s="2" t="n"/>
-      <c r="C12" s="2" t="n"/>
-      <c r="D12" s="2" t="n"/>
-      <c r="E12" s="2" t="n"/>
-      <c r="F12" s="2" t="n"/>
-    </row>
-    <row r="13" ht="15" customHeight="1" s="24">
-      <c r="A13" s="2" t="n"/>
-      <c r="B13" s="2" t="n"/>
-      <c r="C13" s="2" t="n"/>
-      <c r="D13" s="2" t="n"/>
-      <c r="E13" s="2" t="n"/>
-      <c r="F13" s="2" t="n"/>
-    </row>
-    <row r="14" ht="15" customHeight="1" s="24">
-      <c r="A14" s="17" t="n"/>
-      <c r="B14" s="2" t="n"/>
-      <c r="C14" s="2" t="n"/>
-      <c r="D14" s="2" t="n"/>
-      <c r="E14" s="2" t="n"/>
-      <c r="F14" s="2" t="n"/>
-    </row>
-    <row r="18" ht="15.75" customHeight="1" s="24"/>
-    <row r="19" ht="15.75" customHeight="1" s="24"/>
-    <row r="20" ht="15.75" customHeight="1" s="24"/>
-    <row r="21" ht="15.75" customHeight="1" s="24"/>
-    <row r="22" ht="15.75" customHeight="1" s="24"/>
-    <row r="23" ht="15.75" customHeight="1" s="24"/>
-    <row r="24" ht="15.75" customHeight="1" s="24"/>
-    <row r="25" ht="15.75" customHeight="1" s="24"/>
-    <row r="26" ht="15.75" customHeight="1" s="24"/>
-    <row r="27" ht="15.75" customHeight="1" s="24"/>
-    <row r="28" ht="15.75" customHeight="1" s="24"/>
-    <row r="29" ht="15.75" customHeight="1" s="24"/>
-    <row r="30" ht="15.75" customHeight="1" s="24"/>
-    <row r="31" ht="15.75" customHeight="1" s="24"/>
-    <row r="32" ht="15.75" customHeight="1" s="24"/>
-    <row r="33" ht="15.75" customHeight="1" s="24"/>
-    <row r="34" ht="15.75" customHeight="1" s="24"/>
-    <row r="35" ht="15.75" customHeight="1" s="24"/>
-    <row r="36" ht="15.75" customHeight="1" s="24"/>
-    <row r="37" ht="15.75" customHeight="1" s="24"/>
-    <row r="38" ht="15.75" customHeight="1" s="24"/>
-    <row r="39" ht="15.75" customHeight="1" s="24"/>
-    <row r="40" ht="15.75" customHeight="1" s="24"/>
-    <row r="41" ht="15.75" customHeight="1" s="24"/>
-    <row r="42" ht="15.75" customHeight="1" s="24"/>
-    <row r="43" ht="15.75" customHeight="1" s="24"/>
-    <row r="44" ht="15.75" customHeight="1" s="24"/>
-    <row r="45" ht="15.75" customHeight="1" s="24"/>
-    <row r="46" ht="15.75" customHeight="1" s="24"/>
-    <row r="47" ht="15.75" customHeight="1" s="24"/>
-    <row r="48" ht="15.75" customHeight="1" s="24"/>
-    <row r="49" ht="15.75" customHeight="1" s="24"/>
-    <row r="50" ht="15.75" customHeight="1" s="24"/>
-    <row r="51" ht="15.75" customHeight="1" s="24"/>
-    <row r="52" ht="15.75" customHeight="1" s="24"/>
-    <row r="53" ht="15.75" customHeight="1" s="24"/>
-    <row r="54" ht="15.75" customHeight="1" s="24"/>
-    <row r="55" ht="15.75" customHeight="1" s="24"/>
-    <row r="56" ht="15.75" customHeight="1" s="24"/>
-    <row r="57" ht="15.75" customHeight="1" s="24"/>
-    <row r="58" ht="15.75" customHeight="1" s="24"/>
-    <row r="59" ht="15.75" customHeight="1" s="24"/>
-    <row r="60" ht="15.75" customHeight="1" s="24"/>
-    <row r="61" ht="15.75" customHeight="1" s="24"/>
-    <row r="62" ht="15.75" customHeight="1" s="24"/>
-    <row r="63" ht="15.75" customHeight="1" s="24"/>
-    <row r="64" ht="15.75" customHeight="1" s="24"/>
-    <row r="65" ht="15.75" customHeight="1" s="24"/>
-    <row r="66" ht="15.75" customHeight="1" s="24"/>
-    <row r="67" ht="15.75" customHeight="1" s="24"/>
-    <row r="68" ht="15.75" customHeight="1" s="24"/>
-    <row r="69" ht="15.75" customHeight="1" s="24"/>
-    <row r="70" ht="15.75" customHeight="1" s="24"/>
-    <row r="71" ht="15.75" customHeight="1" s="24"/>
-    <row r="72" ht="15.75" customHeight="1" s="24"/>
-    <row r="73" ht="15.75" customHeight="1" s="24"/>
-    <row r="74" ht="15.75" customHeight="1" s="24"/>
-    <row r="75" ht="15.75" customHeight="1" s="24"/>
-    <row r="76" ht="15.75" customHeight="1" s="24"/>
-    <row r="77" ht="15.75" customHeight="1" s="24"/>
-    <row r="78" ht="15.75" customHeight="1" s="24"/>
-    <row r="79" ht="15.75" customHeight="1" s="24"/>
-    <row r="80" ht="15.75" customHeight="1" s="24"/>
-    <row r="81" ht="15.75" customHeight="1" s="24"/>
-    <row r="82" ht="15.75" customHeight="1" s="24"/>
-    <row r="83" ht="15.75" customHeight="1" s="24"/>
-    <row r="84" ht="15.75" customHeight="1" s="24"/>
-    <row r="85" ht="15.75" customHeight="1" s="24"/>
-    <row r="86" ht="15.75" customHeight="1" s="24"/>
-    <row r="87" ht="15.75" customHeight="1" s="24"/>
-    <row r="88" ht="15.75" customHeight="1" s="24"/>
-    <row r="89" ht="15.75" customHeight="1" s="24"/>
-    <row r="90" ht="15.75" customHeight="1" s="24"/>
-    <row r="91" ht="15.75" customHeight="1" s="24"/>
-    <row r="92" ht="15.75" customHeight="1" s="24"/>
-    <row r="93" ht="15.75" customHeight="1" s="24"/>
-    <row r="94" ht="15.75" customHeight="1" s="24"/>
-    <row r="95" ht="15.75" customHeight="1" s="24"/>
-    <row r="96" ht="15.75" customHeight="1" s="24"/>
-    <row r="97" ht="15.75" customHeight="1" s="24"/>
-    <row r="98" ht="15.75" customHeight="1" s="24"/>
-    <row r="99" ht="15.75" customHeight="1" s="24"/>
-    <row r="100" ht="15.75" customHeight="1" s="24"/>
-    <row r="101" ht="15.75" customHeight="1" s="24"/>
-    <row r="102" ht="15.75" customHeight="1" s="24"/>
-    <row r="103" ht="15.75" customHeight="1" s="24"/>
-    <row r="104" ht="15.75" customHeight="1" s="24"/>
-    <row r="105" ht="15.75" customHeight="1" s="24"/>
-    <row r="106" ht="15.75" customHeight="1" s="24"/>
-    <row r="107" ht="15.75" customHeight="1" s="24"/>
-    <row r="108" ht="15.75" customHeight="1" s="24"/>
-    <row r="109" ht="15.75" customHeight="1" s="24"/>
-    <row r="110" ht="15.75" customHeight="1" s="24"/>
-    <row r="111" ht="15.75" customHeight="1" s="24"/>
-    <row r="112" ht="15.75" customHeight="1" s="24"/>
-    <row r="113" ht="15.75" customHeight="1" s="24"/>
-    <row r="114" ht="15.75" customHeight="1" s="24"/>
-    <row r="115" ht="15.75" customHeight="1" s="24"/>
-    <row r="116" ht="15.75" customHeight="1" s="24"/>
-    <row r="117" ht="15.75" customHeight="1" s="24"/>
-    <row r="118" ht="15.75" customHeight="1" s="24"/>
-    <row r="119" ht="15.75" customHeight="1" s="24"/>
-    <row r="120" ht="15.75" customHeight="1" s="24"/>
-    <row r="121" ht="15.75" customHeight="1" s="24"/>
-    <row r="122" ht="15.75" customHeight="1" s="24"/>
-    <row r="123" ht="15.75" customHeight="1" s="24"/>
-    <row r="124" ht="15.75" customHeight="1" s="24"/>
-    <row r="125" ht="15.75" customHeight="1" s="24"/>
-    <row r="126" ht="15.75" customHeight="1" s="24"/>
-    <row r="127" ht="15.75" customHeight="1" s="24"/>
-    <row r="128" ht="15.75" customHeight="1" s="24"/>
-    <row r="129" ht="15.75" customHeight="1" s="24"/>
-    <row r="130" ht="15.75" customHeight="1" s="24"/>
-    <row r="131" ht="15.75" customHeight="1" s="24"/>
-    <row r="132" ht="15.75" customHeight="1" s="24"/>
-    <row r="133" ht="15.75" customHeight="1" s="24"/>
-    <row r="134" ht="15.75" customHeight="1" s="24"/>
-    <row r="135" ht="15.75" customHeight="1" s="24"/>
-    <row r="136" ht="15.75" customHeight="1" s="24"/>
-    <row r="137" ht="15.75" customHeight="1" s="24"/>
-    <row r="138" ht="15.75" customHeight="1" s="24"/>
-    <row r="139" ht="15.75" customHeight="1" s="24"/>
-    <row r="140" ht="15.75" customHeight="1" s="24"/>
-    <row r="141" ht="15.75" customHeight="1" s="24"/>
-    <row r="142" ht="15.75" customHeight="1" s="24"/>
-    <row r="143" ht="15.75" customHeight="1" s="24"/>
-    <row r="144" ht="15.75" customHeight="1" s="24"/>
-    <row r="145" ht="15.75" customHeight="1" s="24"/>
-    <row r="146" ht="15.75" customHeight="1" s="24"/>
-    <row r="147" ht="15.75" customHeight="1" s="24"/>
-    <row r="148" ht="15.75" customHeight="1" s="24"/>
-    <row r="149" ht="15.75" customHeight="1" s="24"/>
-    <row r="150" ht="15.75" customHeight="1" s="24"/>
-    <row r="151" ht="15.75" customHeight="1" s="24"/>
-    <row r="152" ht="15.75" customHeight="1" s="24"/>
-    <row r="153" ht="15.75" customHeight="1" s="24"/>
-    <row r="154" ht="15.75" customHeight="1" s="24"/>
-    <row r="155" ht="15.75" customHeight="1" s="24"/>
-    <row r="156" ht="15.75" customHeight="1" s="24"/>
-    <row r="157" ht="15.75" customHeight="1" s="24"/>
-    <row r="158" ht="15.75" customHeight="1" s="24"/>
-    <row r="159" ht="15.75" customHeight="1" s="24"/>
-    <row r="160" ht="15.75" customHeight="1" s="24"/>
-    <row r="161" ht="15.75" customHeight="1" s="24"/>
-    <row r="162" ht="15.75" customHeight="1" s="24"/>
-    <row r="163" ht="15.75" customHeight="1" s="24"/>
-    <row r="164" ht="15.75" customHeight="1" s="24"/>
-    <row r="165" ht="15.75" customHeight="1" s="24"/>
-    <row r="166" ht="15.75" customHeight="1" s="24"/>
-    <row r="167" ht="15.75" customHeight="1" s="24"/>
-    <row r="168" ht="15.75" customHeight="1" s="24"/>
-    <row r="169" ht="15.75" customHeight="1" s="24"/>
-    <row r="170" ht="15.75" customHeight="1" s="24"/>
-    <row r="171" ht="15.75" customHeight="1" s="24"/>
-    <row r="172" ht="15.75" customHeight="1" s="24"/>
-    <row r="173" ht="15.75" customHeight="1" s="24"/>
-    <row r="174" ht="15.75" customHeight="1" s="24"/>
-    <row r="175" ht="15.75" customHeight="1" s="24"/>
-    <row r="176" ht="15.75" customHeight="1" s="24"/>
-    <row r="177" ht="15.75" customHeight="1" s="24"/>
-    <row r="178" ht="15.75" customHeight="1" s="24"/>
-    <row r="179" ht="15.75" customHeight="1" s="24"/>
-    <row r="180" ht="15.75" customHeight="1" s="24"/>
-    <row r="181" ht="15.75" customHeight="1" s="24"/>
-    <row r="182" ht="15.75" customHeight="1" s="24"/>
-    <row r="183" ht="15.75" customHeight="1" s="24"/>
-    <row r="184" ht="15.75" customHeight="1" s="24"/>
-    <row r="185" ht="15.75" customHeight="1" s="24"/>
-    <row r="186" ht="15.75" customHeight="1" s="24"/>
-    <row r="187" ht="15.75" customHeight="1" s="24"/>
-    <row r="188" ht="15.75" customHeight="1" s="24"/>
-    <row r="189" ht="15.75" customHeight="1" s="24"/>
-    <row r="190" ht="15.75" customHeight="1" s="24"/>
-    <row r="191" ht="15.75" customHeight="1" s="24"/>
-    <row r="192" ht="15.75" customHeight="1" s="24"/>
-    <row r="193" ht="15.75" customHeight="1" s="24"/>
-    <row r="194" ht="15.75" customHeight="1" s="24"/>
-    <row r="195" ht="15.75" customHeight="1" s="24"/>
-    <row r="196" ht="15.75" customHeight="1" s="24"/>
-    <row r="197" ht="15.75" customHeight="1" s="24"/>
-    <row r="198" ht="15.75" customHeight="1" s="24"/>
-    <row r="199" ht="15.75" customHeight="1" s="24"/>
-    <row r="200" ht="15.75" customHeight="1" s="24"/>
-    <row r="201" ht="15.75" customHeight="1" s="24"/>
-    <row r="202" ht="15.75" customHeight="1" s="24"/>
-    <row r="203" ht="15.75" customHeight="1" s="24"/>
-    <row r="204" ht="15.75" customHeight="1" s="24"/>
-    <row r="205" ht="15.75" customHeight="1" s="24"/>
-    <row r="206" ht="15.75" customHeight="1" s="24"/>
-    <row r="207" ht="15.75" customHeight="1" s="24"/>
-    <row r="208" ht="15.75" customHeight="1" s="24"/>
-    <row r="209" ht="15.75" customHeight="1" s="24"/>
-    <row r="210" ht="15.75" customHeight="1" s="24"/>
-    <row r="211" ht="15.75" customHeight="1" s="24"/>
-    <row r="212" ht="15.75" customHeight="1" s="24"/>
-    <row r="213" ht="15.75" customHeight="1" s="24"/>
-    <row r="214" ht="15.75" customHeight="1" s="24"/>
-    <row r="215" ht="15.75" customHeight="1" s="24"/>
-    <row r="216" ht="15.75" customHeight="1" s="24"/>
-    <row r="217" ht="15.75" customHeight="1" s="24"/>
-    <row r="218" ht="15.75" customHeight="1" s="24"/>
-    <row r="219" ht="15.75" customHeight="1" s="24"/>
-    <row r="220" ht="15.75" customHeight="1" s="24"/>
-    <row r="221" ht="15.75" customHeight="1" s="24"/>
-    <row r="222" ht="15.75" customHeight="1" s="24"/>
-    <row r="223" ht="15.75" customHeight="1" s="24"/>
-    <row r="224" ht="15.75" customHeight="1" s="24"/>
-    <row r="225" ht="15.75" customHeight="1" s="24"/>
-    <row r="226" ht="15.75" customHeight="1" s="24"/>
-    <row r="227" ht="15.75" customHeight="1" s="24"/>
-    <row r="228" ht="15.75" customHeight="1" s="24"/>
-    <row r="229" ht="15.75" customHeight="1" s="24"/>
-    <row r="230" ht="15.75" customHeight="1" s="24"/>
-    <row r="231" ht="15.75" customHeight="1" s="24"/>
-    <row r="232" ht="15.75" customHeight="1" s="24"/>
-    <row r="233" ht="15.75" customHeight="1" s="24"/>
-    <row r="234" ht="15.75" customHeight="1" s="24"/>
-    <row r="235" ht="15.75" customHeight="1" s="24"/>
-    <row r="236" ht="15.75" customHeight="1" s="24"/>
-    <row r="237" ht="15.75" customHeight="1" s="24"/>
-    <row r="238" ht="15.75" customHeight="1" s="24"/>
-    <row r="239" ht="15.75" customHeight="1" s="24"/>
-    <row r="240" ht="15.75" customHeight="1" s="24"/>
-    <row r="241" ht="15.75" customHeight="1" s="24"/>
-    <row r="242" ht="15.75" customHeight="1" s="24"/>
-    <row r="243" ht="15.75" customHeight="1" s="24"/>
-    <row r="244" ht="15.75" customHeight="1" s="24"/>
-    <row r="245" ht="15.75" customHeight="1" s="24"/>
-    <row r="246" ht="15.75" customHeight="1" s="24"/>
-    <row r="247" ht="15.75" customHeight="1" s="24"/>
-    <row r="248" ht="15.75" customHeight="1" s="24"/>
-    <row r="249" ht="15.75" customHeight="1" s="24"/>
-    <row r="250" ht="15.75" customHeight="1" s="24"/>
-    <row r="251" ht="15.75" customHeight="1" s="24"/>
-    <row r="252" ht="15.75" customHeight="1" s="24"/>
-    <row r="253" ht="15.75" customHeight="1" s="24"/>
-    <row r="254" ht="15.75" customHeight="1" s="24"/>
-    <row r="255" ht="15.75" customHeight="1" s="24"/>
-    <row r="256" ht="15.75" customHeight="1" s="24"/>
-    <row r="257" ht="15.75" customHeight="1" s="24"/>
-    <row r="258" ht="15.75" customHeight="1" s="24"/>
-    <row r="259" ht="15.75" customHeight="1" s="24"/>
-    <row r="260" ht="15.75" customHeight="1" s="24"/>
-    <row r="261" ht="15.75" customHeight="1" s="24"/>
-    <row r="262" ht="15.75" customHeight="1" s="24"/>
-    <row r="263" ht="15.75" customHeight="1" s="24"/>
-    <row r="264" ht="15.75" customHeight="1" s="24"/>
-    <row r="265" ht="15.75" customHeight="1" s="24"/>
-    <row r="266" ht="15.75" customHeight="1" s="24"/>
-    <row r="267" ht="15.75" customHeight="1" s="24"/>
-    <row r="268" ht="15.75" customHeight="1" s="24"/>
-    <row r="269" ht="15.75" customHeight="1" s="24"/>
-    <row r="270" ht="15.75" customHeight="1" s="24"/>
-    <row r="271" ht="15.75" customHeight="1" s="24"/>
-    <row r="272" ht="15.75" customHeight="1" s="24"/>
-    <row r="273" ht="15.75" customHeight="1" s="24"/>
-    <row r="274" ht="15.75" customHeight="1" s="24"/>
-    <row r="275" ht="15.75" customHeight="1" s="24"/>
-    <row r="276" ht="15.75" customHeight="1" s="24"/>
-    <row r="277" ht="15.75" customHeight="1" s="24"/>
-    <row r="278" ht="15.75" customHeight="1" s="24"/>
-    <row r="279" ht="15.75" customHeight="1" s="24"/>
-    <row r="280" ht="15.75" customHeight="1" s="24"/>
-    <row r="281" ht="15.75" customHeight="1" s="24"/>
-    <row r="282" ht="15.75" customHeight="1" s="24"/>
-    <row r="283" ht="15.75" customHeight="1" s="24"/>
-    <row r="284" ht="15.75" customHeight="1" s="24"/>
-    <row r="285" ht="15.75" customHeight="1" s="24"/>
-    <row r="286" ht="15.75" customHeight="1" s="24"/>
-    <row r="287" ht="15.75" customHeight="1" s="24"/>
-    <row r="288" ht="15.75" customHeight="1" s="24"/>
-    <row r="289" ht="15.75" customHeight="1" s="24"/>
-    <row r="290" ht="15.75" customHeight="1" s="24"/>
-    <row r="291" ht="15.75" customHeight="1" s="24"/>
-    <row r="292" ht="15.75" customHeight="1" s="24"/>
-    <row r="293" ht="15.75" customHeight="1" s="24"/>
-    <row r="294" ht="15.75" customHeight="1" s="24"/>
-    <row r="295" ht="15.75" customHeight="1" s="24"/>
-    <row r="296" ht="15.75" customHeight="1" s="24"/>
-    <row r="297" ht="15.75" customHeight="1" s="24"/>
-    <row r="298" ht="15.75" customHeight="1" s="24"/>
-    <row r="299" ht="15.75" customHeight="1" s="24"/>
-    <row r="300" ht="15.75" customHeight="1" s="24"/>
-    <row r="301" ht="15.75" customHeight="1" s="24"/>
-    <row r="302" ht="15.75" customHeight="1" s="24"/>
-    <row r="303" ht="15.75" customHeight="1" s="24"/>
-    <row r="304" ht="15.75" customHeight="1" s="24"/>
-    <row r="305" ht="15.75" customHeight="1" s="24"/>
-    <row r="306" ht="15.75" customHeight="1" s="24"/>
-    <row r="307" ht="15.75" customHeight="1" s="24"/>
-    <row r="308" ht="15.75" customHeight="1" s="24"/>
-    <row r="309" ht="15.75" customHeight="1" s="24"/>
-    <row r="310" ht="15.75" customHeight="1" s="24"/>
-    <row r="311" ht="15.75" customHeight="1" s="24"/>
-    <row r="312" ht="15.75" customHeight="1" s="24"/>
-    <row r="313" ht="15.75" customHeight="1" s="24"/>
-    <row r="314" ht="15.75" customHeight="1" s="24"/>
-    <row r="315" ht="15.75" customHeight="1" s="24"/>
-    <row r="316" ht="15.75" customHeight="1" s="24"/>
-    <row r="317" ht="15.75" customHeight="1" s="24"/>
-    <row r="318" ht="15.75" customHeight="1" s="24"/>
-    <row r="319" ht="15.75" customHeight="1" s="24"/>
-    <row r="320" ht="15.75" customHeight="1" s="24"/>
-    <row r="321" ht="15.75" customHeight="1" s="24"/>
-    <row r="322" ht="15.75" customHeight="1" s="24"/>
-    <row r="323" ht="15.75" customHeight="1" s="24"/>
-    <row r="324" ht="15.75" customHeight="1" s="24"/>
-    <row r="325" ht="15.75" customHeight="1" s="24"/>
-    <row r="326" ht="15.75" customHeight="1" s="24"/>
-    <row r="327" ht="15.75" customHeight="1" s="24"/>
-    <row r="328" ht="15.75" customHeight="1" s="24"/>
-    <row r="329" ht="15.75" customHeight="1" s="24"/>
-    <row r="330" ht="15.75" customHeight="1" s="24"/>
-    <row r="331" ht="15.75" customHeight="1" s="24"/>
-    <row r="332" ht="15.75" customHeight="1" s="24"/>
-    <row r="333" ht="15.75" customHeight="1" s="24"/>
-    <row r="334" ht="15.75" customHeight="1" s="24"/>
-    <row r="335" ht="15.75" customHeight="1" s="24"/>
-    <row r="336" ht="15.75" customHeight="1" s="24"/>
-    <row r="337" ht="15.75" customHeight="1" s="24"/>
-    <row r="338" ht="15.75" customHeight="1" s="24"/>
-    <row r="339" ht="15.75" customHeight="1" s="24"/>
-    <row r="340" ht="15.75" customHeight="1" s="24"/>
-    <row r="341" ht="15.75" customHeight="1" s="24"/>
-    <row r="342" ht="15.75" customHeight="1" s="24"/>
-    <row r="343" ht="15.75" customHeight="1" s="24"/>
-    <row r="344" ht="15.75" customHeight="1" s="24"/>
-    <row r="345" ht="15.75" customHeight="1" s="24"/>
-    <row r="346" ht="15.75" customHeight="1" s="24"/>
-    <row r="347" ht="15.75" customHeight="1" s="24"/>
-    <row r="348" ht="15.75" customHeight="1" s="24"/>
-    <row r="349" ht="15.75" customHeight="1" s="24"/>
-    <row r="350" ht="15.75" customHeight="1" s="24"/>
-    <row r="351" ht="15.75" customHeight="1" s="24"/>
-    <row r="352" ht="15.75" customHeight="1" s="24"/>
-    <row r="353" ht="15.75" customHeight="1" s="24"/>
-    <row r="354" ht="15.75" customHeight="1" s="24"/>
-    <row r="355" ht="15.75" customHeight="1" s="24"/>
-    <row r="356" ht="15.75" customHeight="1" s="24"/>
-    <row r="357" ht="15.75" customHeight="1" s="24"/>
-    <row r="358" ht="15.75" customHeight="1" s="24"/>
-    <row r="359" ht="15.75" customHeight="1" s="24"/>
-    <row r="360" ht="15.75" customHeight="1" s="24"/>
-    <row r="361" ht="15.75" customHeight="1" s="24"/>
-    <row r="362" ht="15.75" customHeight="1" s="24"/>
-    <row r="363" ht="15.75" customHeight="1" s="24"/>
-    <row r="364" ht="15.75" customHeight="1" s="24"/>
-    <row r="365" ht="15.75" customHeight="1" s="24"/>
-    <row r="366" ht="15.75" customHeight="1" s="24"/>
-    <row r="367" ht="15.75" customHeight="1" s="24"/>
-    <row r="368" ht="15.75" customHeight="1" s="24"/>
-    <row r="369" ht="15.75" customHeight="1" s="24"/>
-    <row r="370" ht="15.75" customHeight="1" s="24"/>
-    <row r="371" ht="15.75" customHeight="1" s="24"/>
-    <row r="372" ht="15.75" customHeight="1" s="24"/>
-    <row r="373" ht="15.75" customHeight="1" s="24"/>
-    <row r="374" ht="15.75" customHeight="1" s="24"/>
-    <row r="375" ht="15.75" customHeight="1" s="24"/>
-    <row r="376" ht="15.75" customHeight="1" s="24"/>
-    <row r="377" ht="15.75" customHeight="1" s="24"/>
-    <row r="378" ht="15.75" customHeight="1" s="24"/>
-    <row r="379" ht="15.75" customHeight="1" s="24"/>
-    <row r="380" ht="15.75" customHeight="1" s="24"/>
-    <row r="381" ht="15.75" customHeight="1" s="24"/>
-    <row r="382" ht="15.75" customHeight="1" s="24"/>
-    <row r="383" ht="15.75" customHeight="1" s="24"/>
-    <row r="384" ht="15.75" customHeight="1" s="24"/>
-    <row r="385" ht="15.75" customHeight="1" s="24"/>
-    <row r="386" ht="15.75" customHeight="1" s="24"/>
-    <row r="387" ht="15.75" customHeight="1" s="24"/>
-    <row r="388" ht="15.75" customHeight="1" s="24"/>
-    <row r="389" ht="15.75" customHeight="1" s="24"/>
-    <row r="390" ht="15.75" customHeight="1" s="24"/>
-    <row r="391" ht="15.75" customHeight="1" s="24"/>
-    <row r="392" ht="15.75" customHeight="1" s="24"/>
-    <row r="393" ht="15.75" customHeight="1" s="24"/>
-    <row r="394" ht="15.75" customHeight="1" s="24"/>
-    <row r="395" ht="15.75" customHeight="1" s="24"/>
-    <row r="396" ht="15.75" customHeight="1" s="24"/>
-    <row r="397" ht="15.75" customHeight="1" s="24"/>
-    <row r="398" ht="15.75" customHeight="1" s="24"/>
-    <row r="399" ht="15.75" customHeight="1" s="24"/>
-    <row r="400" ht="15.75" customHeight="1" s="24"/>
-    <row r="401" ht="15.75" customHeight="1" s="24"/>
-    <row r="402" ht="15.75" customHeight="1" s="24"/>
-    <row r="403" ht="15.75" customHeight="1" s="24"/>
-    <row r="404" ht="15.75" customHeight="1" s="24"/>
-    <row r="405" ht="15.75" customHeight="1" s="24"/>
-    <row r="406" ht="15.75" customHeight="1" s="24"/>
-    <row r="407" ht="15.75" customHeight="1" s="24"/>
-    <row r="408" ht="15.75" customHeight="1" s="24"/>
-    <row r="409" ht="15.75" customHeight="1" s="24"/>
-    <row r="410" ht="15.75" customHeight="1" s="24"/>
-    <row r="411" ht="15.75" customHeight="1" s="24"/>
-    <row r="412" ht="15.75" customHeight="1" s="24"/>
-    <row r="413" ht="15.75" customHeight="1" s="24"/>
-    <row r="414" ht="15.75" customHeight="1" s="24"/>
-    <row r="415" ht="15.75" customHeight="1" s="24"/>
-    <row r="416" ht="15.75" customHeight="1" s="24"/>
-    <row r="417" ht="15.75" customHeight="1" s="24"/>
-    <row r="418" ht="15.75" customHeight="1" s="24"/>
-    <row r="419" ht="15.75" customHeight="1" s="24"/>
-    <row r="420" ht="15.75" customHeight="1" s="24"/>
-    <row r="421" ht="15.75" customHeight="1" s="24"/>
-    <row r="422" ht="15.75" customHeight="1" s="24"/>
-    <row r="423" ht="15.75" customHeight="1" s="24"/>
-    <row r="424" ht="15.75" customHeight="1" s="24"/>
-    <row r="425" ht="15.75" customHeight="1" s="24"/>
-    <row r="426" ht="15.75" customHeight="1" s="24"/>
-    <row r="427" ht="15.75" customHeight="1" s="24"/>
-    <row r="428" ht="15.75" customHeight="1" s="24"/>
-    <row r="429" ht="15.75" customHeight="1" s="24"/>
-    <row r="430" ht="15.75" customHeight="1" s="24"/>
-    <row r="431" ht="15.75" customHeight="1" s="24"/>
-    <row r="432" ht="15.75" customHeight="1" s="24"/>
-    <row r="433" ht="15.75" customHeight="1" s="24"/>
-    <row r="434" ht="15.75" customHeight="1" s="24"/>
-    <row r="435" ht="15.75" customHeight="1" s="24"/>
-    <row r="436" ht="15.75" customHeight="1" s="24"/>
-    <row r="437" ht="15.75" customHeight="1" s="24"/>
-    <row r="438" ht="15.75" customHeight="1" s="24"/>
-    <row r="439" ht="15.75" customHeight="1" s="24"/>
-    <row r="440" ht="15.75" customHeight="1" s="24"/>
-    <row r="441" ht="15.75" customHeight="1" s="24"/>
-    <row r="442" ht="15.75" customHeight="1" s="24"/>
-    <row r="443" ht="15.75" customHeight="1" s="24"/>
-    <row r="444" ht="15.75" customHeight="1" s="24"/>
-    <row r="445" ht="15.75" customHeight="1" s="24"/>
-    <row r="446" ht="15.75" customHeight="1" s="24"/>
-    <row r="447" ht="15.75" customHeight="1" s="24"/>
-    <row r="448" ht="15.75" customHeight="1" s="24"/>
-    <row r="449" ht="15.75" customHeight="1" s="24"/>
-    <row r="450" ht="15.75" customHeight="1" s="24"/>
-    <row r="451" ht="15.75" customHeight="1" s="24"/>
-    <row r="452" ht="15.75" customHeight="1" s="24"/>
-    <row r="453" ht="15.75" customHeight="1" s="24"/>
-    <row r="454" ht="15.75" customHeight="1" s="24"/>
-    <row r="455" ht="15.75" customHeight="1" s="24"/>
-    <row r="456" ht="15.75" customHeight="1" s="24"/>
-    <row r="457" ht="15.75" customHeight="1" s="24"/>
-    <row r="458" ht="15.75" customHeight="1" s="24"/>
-    <row r="459" ht="15.75" customHeight="1" s="24"/>
-    <row r="460" ht="15.75" customHeight="1" s="24"/>
-    <row r="461" ht="15.75" customHeight="1" s="24"/>
-    <row r="462" ht="15.75" customHeight="1" s="24"/>
-    <row r="463" ht="15.75" customHeight="1" s="24"/>
-    <row r="464" ht="15.75" customHeight="1" s="24"/>
-    <row r="465" ht="15.75" customHeight="1" s="24"/>
-    <row r="466" ht="15.75" customHeight="1" s="24"/>
-    <row r="467" ht="15.75" customHeight="1" s="24"/>
-    <row r="468" ht="15.75" customHeight="1" s="24"/>
-    <row r="469" ht="15.75" customHeight="1" s="24"/>
-    <row r="470" ht="15.75" customHeight="1" s="24"/>
-    <row r="471" ht="15.75" customHeight="1" s="24"/>
-    <row r="472" ht="15.75" customHeight="1" s="24"/>
-    <row r="473" ht="15.75" customHeight="1" s="24"/>
-    <row r="474" ht="15.75" customHeight="1" s="24"/>
-    <row r="475" ht="15.75" customHeight="1" s="24"/>
-    <row r="476" ht="15.75" customHeight="1" s="24"/>
-    <row r="477" ht="15.75" customHeight="1" s="24"/>
-    <row r="478" ht="15.75" customHeight="1" s="24"/>
-    <row r="479" ht="15.75" customHeight="1" s="24"/>
-    <row r="480" ht="15.75" customHeight="1" s="24"/>
-    <row r="481" ht="15.75" customHeight="1" s="24"/>
-    <row r="482" ht="15.75" customHeight="1" s="24"/>
-    <row r="483" ht="15.75" customHeight="1" s="24"/>
-    <row r="484" ht="15.75" customHeight="1" s="24"/>
-    <row r="485" ht="15.75" customHeight="1" s="24"/>
-    <row r="486" ht="15.75" customHeight="1" s="24"/>
-    <row r="487" ht="15.75" customHeight="1" s="24"/>
-    <row r="488" ht="15.75" customHeight="1" s="24"/>
-    <row r="489" ht="15.75" customHeight="1" s="24"/>
-    <row r="490" ht="15.75" customHeight="1" s="24"/>
-    <row r="491" ht="15.75" customHeight="1" s="24"/>
-    <row r="492" ht="15.75" customHeight="1" s="24"/>
-    <row r="493" ht="15.75" customHeight="1" s="24"/>
-    <row r="494" ht="15.75" customHeight="1" s="24"/>
-    <row r="495" ht="15.75" customHeight="1" s="24"/>
-    <row r="496" ht="15.75" customHeight="1" s="24"/>
-    <row r="497" ht="15.75" customHeight="1" s="24"/>
-    <row r="498" ht="15.75" customHeight="1" s="24"/>
-    <row r="499" ht="15.75" customHeight="1" s="24"/>
-    <row r="500" ht="15.75" customHeight="1" s="24"/>
-    <row r="501" ht="15.75" customHeight="1" s="24"/>
-    <row r="502" ht="15.75" customHeight="1" s="24"/>
-    <row r="503" ht="15.75" customHeight="1" s="24"/>
-    <row r="504" ht="15.75" customHeight="1" s="24"/>
-    <row r="505" ht="15.75" customHeight="1" s="24"/>
-    <row r="506" ht="15.75" customHeight="1" s="24"/>
-    <row r="507" ht="15.75" customHeight="1" s="24"/>
-    <row r="508" ht="15.75" customHeight="1" s="24"/>
-    <row r="509" ht="15.75" customHeight="1" s="24"/>
-    <row r="510" ht="15.75" customHeight="1" s="24"/>
-    <row r="511" ht="15.75" customHeight="1" s="24"/>
-    <row r="512" ht="15.75" customHeight="1" s="24"/>
-    <row r="513" ht="15.75" customHeight="1" s="24"/>
-    <row r="514" ht="15.75" customHeight="1" s="24"/>
-    <row r="515" ht="15.75" customHeight="1" s="24"/>
-    <row r="516" ht="15.75" customHeight="1" s="24"/>
-    <row r="517" ht="15.75" customHeight="1" s="24"/>
-    <row r="518" ht="15.75" customHeight="1" s="24"/>
-    <row r="519" ht="15.75" customHeight="1" s="24"/>
-    <row r="520" ht="15.75" customHeight="1" s="24"/>
-    <row r="521" ht="15.75" customHeight="1" s="24"/>
-    <row r="522" ht="15.75" customHeight="1" s="24"/>
-    <row r="523" ht="15.75" customHeight="1" s="24"/>
-    <row r="524" ht="15.75" customHeight="1" s="24"/>
-    <row r="525" ht="15.75" customHeight="1" s="24"/>
-    <row r="526" ht="15.75" customHeight="1" s="24"/>
-    <row r="527" ht="15.75" customHeight="1" s="24"/>
-    <row r="528" ht="15.75" customHeight="1" s="24"/>
-    <row r="529" ht="15.75" customHeight="1" s="24"/>
-    <row r="530" ht="15.75" customHeight="1" s="24"/>
-    <row r="531" ht="15.75" customHeight="1" s="24"/>
-    <row r="532" ht="15.75" customHeight="1" s="24"/>
-    <row r="533" ht="15.75" customHeight="1" s="24"/>
-    <row r="534" ht="15.75" customHeight="1" s="24"/>
-    <row r="535" ht="15.75" customHeight="1" s="24"/>
-    <row r="536" ht="15.75" customHeight="1" s="24"/>
-    <row r="537" ht="15.75" customHeight="1" s="24"/>
-    <row r="538" ht="15.75" customHeight="1" s="24"/>
-    <row r="539" ht="15.75" customHeight="1" s="24"/>
-    <row r="540" ht="15.75" customHeight="1" s="24"/>
-    <row r="541" ht="15.75" customHeight="1" s="24"/>
-    <row r="542" ht="15.75" customHeight="1" s="24"/>
-    <row r="543" ht="15.75" customHeight="1" s="24"/>
-    <row r="544" ht="15.75" customHeight="1" s="24"/>
-    <row r="545" ht="15.75" customHeight="1" s="24"/>
-    <row r="546" ht="15.75" customHeight="1" s="24"/>
-    <row r="547" ht="15.75" customHeight="1" s="24"/>
-    <row r="548" ht="15.75" customHeight="1" s="24"/>
-    <row r="549" ht="15.75" customHeight="1" s="24"/>
-    <row r="550" ht="15.75" customHeight="1" s="24"/>
-    <row r="551" ht="15.75" customHeight="1" s="24"/>
-    <row r="552" ht="15.75" customHeight="1" s="24"/>
-    <row r="553" ht="15.75" customHeight="1" s="24"/>
-    <row r="554" ht="15.75" customHeight="1" s="24"/>
-    <row r="555" ht="15.75" customHeight="1" s="24"/>
-    <row r="556" ht="15.75" customHeight="1" s="24"/>
-    <row r="557" ht="15.75" customHeight="1" s="24"/>
-    <row r="558" ht="15.75" customHeight="1" s="24"/>
-    <row r="559" ht="15.75" customHeight="1" s="24"/>
-    <row r="560" ht="15.75" customHeight="1" s="24"/>
-    <row r="561" ht="15.75" customHeight="1" s="24"/>
-    <row r="562" ht="15.75" customHeight="1" s="24"/>
-    <row r="563" ht="15.75" customHeight="1" s="24"/>
-    <row r="564" ht="15.75" customHeight="1" s="24"/>
-    <row r="565" ht="15.75" customHeight="1" s="24"/>
-    <row r="566" ht="15.75" customHeight="1" s="24"/>
-    <row r="567" ht="15.75" customHeight="1" s="24"/>
-    <row r="568" ht="15.75" customHeight="1" s="24"/>
-    <row r="569" ht="15.75" customHeight="1" s="24"/>
-    <row r="570" ht="15.75" customHeight="1" s="24"/>
-    <row r="571" ht="15.75" customHeight="1" s="24"/>
-    <row r="572" ht="15.75" customHeight="1" s="24"/>
-    <row r="573" ht="15.75" customHeight="1" s="24"/>
-    <row r="574" ht="15.75" customHeight="1" s="24"/>
-    <row r="575" ht="15.75" customHeight="1" s="24"/>
-    <row r="576" ht="15.75" customHeight="1" s="24"/>
-    <row r="577" ht="15.75" customHeight="1" s="24"/>
-    <row r="578" ht="15.75" customHeight="1" s="24"/>
-    <row r="579" ht="15.75" customHeight="1" s="24"/>
-    <row r="580" ht="15.75" customHeight="1" s="24"/>
-    <row r="581" ht="15.75" customHeight="1" s="24"/>
-    <row r="582" ht="15.75" customHeight="1" s="24"/>
-    <row r="583" ht="15.75" customHeight="1" s="24"/>
-    <row r="584" ht="15.75" customHeight="1" s="24"/>
-    <row r="585" ht="15.75" customHeight="1" s="24"/>
-    <row r="586" ht="15.75" customHeight="1" s="24"/>
-    <row r="587" ht="15.75" customHeight="1" s="24"/>
-    <row r="588" ht="15.75" customHeight="1" s="24"/>
-    <row r="589" ht="15.75" customHeight="1" s="24"/>
-    <row r="590" ht="15.75" customHeight="1" s="24"/>
-    <row r="591" ht="15.75" customHeight="1" s="24"/>
-    <row r="592" ht="15.75" customHeight="1" s="24"/>
-    <row r="593" ht="15.75" customHeight="1" s="24"/>
-    <row r="594" ht="15.75" customHeight="1" s="24"/>
-    <row r="595" ht="15.75" customHeight="1" s="24"/>
-    <row r="596" ht="15.75" customHeight="1" s="24"/>
-    <row r="597" ht="15.75" customHeight="1" s="24"/>
-    <row r="598" ht="15.75" customHeight="1" s="24"/>
-    <row r="599" ht="15.75" customHeight="1" s="24"/>
-    <row r="600" ht="15.75" customHeight="1" s="24"/>
-    <row r="601" ht="15.75" customHeight="1" s="24"/>
-    <row r="602" ht="15.75" customHeight="1" s="24"/>
-    <row r="603" ht="15.75" customHeight="1" s="24"/>
-    <row r="604" ht="15.75" customHeight="1" s="24"/>
-    <row r="605" ht="15.75" customHeight="1" s="24"/>
-    <row r="606" ht="15.75" customHeight="1" s="24"/>
-    <row r="607" ht="15.75" customHeight="1" s="24"/>
-    <row r="608" ht="15.75" customHeight="1" s="24"/>
-    <row r="609" ht="15.75" customHeight="1" s="24"/>
-    <row r="610" ht="15.75" customHeight="1" s="24"/>
-    <row r="611" ht="15.75" customHeight="1" s="24"/>
-    <row r="612" ht="15.75" customHeight="1" s="24"/>
-    <row r="613" ht="15.75" customHeight="1" s="24"/>
-    <row r="614" ht="15.75" customHeight="1" s="24"/>
-    <row r="615" ht="15.75" customHeight="1" s="24"/>
-    <row r="616" ht="15.75" customHeight="1" s="24"/>
-    <row r="617" ht="15.75" customHeight="1" s="24"/>
-    <row r="618" ht="15.75" customHeight="1" s="24"/>
-    <row r="619" ht="15.75" customHeight="1" s="24"/>
-    <row r="620" ht="15.75" customHeight="1" s="24"/>
-    <row r="621" ht="15.75" customHeight="1" s="24"/>
-    <row r="622" ht="15.75" customHeight="1" s="24"/>
-    <row r="623" ht="15.75" customHeight="1" s="24"/>
-    <row r="624" ht="15.75" customHeight="1" s="24"/>
-    <row r="625" ht="15.75" customHeight="1" s="24"/>
-    <row r="626" ht="15.75" customHeight="1" s="24"/>
-    <row r="627" ht="15.75" customHeight="1" s="24"/>
-    <row r="628" ht="15.75" customHeight="1" s="24"/>
-    <row r="629" ht="15.75" customHeight="1" s="24"/>
-    <row r="630" ht="15.75" customHeight="1" s="24"/>
-    <row r="631" ht="15.75" customHeight="1" s="24"/>
-    <row r="632" ht="15.75" customHeight="1" s="24"/>
-    <row r="633" ht="15.75" customHeight="1" s="24"/>
-    <row r="634" ht="15.75" customHeight="1" s="24"/>
-    <row r="635" ht="15.75" customHeight="1" s="24"/>
-    <row r="636" ht="15.75" customHeight="1" s="24"/>
-    <row r="637" ht="15.75" customHeight="1" s="24"/>
-    <row r="638" ht="15.75" customHeight="1" s="24"/>
-    <row r="639" ht="15.75" customHeight="1" s="24"/>
-    <row r="640" ht="15.75" customHeight="1" s="24"/>
-    <row r="641" ht="15.75" customHeight="1" s="24"/>
-    <row r="642" ht="15.75" customHeight="1" s="24"/>
-    <row r="643" ht="15.75" customHeight="1" s="24"/>
-    <row r="644" ht="15.75" customHeight="1" s="24"/>
-    <row r="645" ht="15.75" customHeight="1" s="24"/>
-    <row r="646" ht="15.75" customHeight="1" s="24"/>
-    <row r="647" ht="15.75" customHeight="1" s="24"/>
-    <row r="648" ht="15.75" customHeight="1" s="24"/>
-    <row r="649" ht="15.75" customHeight="1" s="24"/>
-    <row r="650" ht="15.75" customHeight="1" s="24"/>
-    <row r="651" ht="15.75" customHeight="1" s="24"/>
-    <row r="652" ht="15.75" customHeight="1" s="24"/>
-    <row r="653" ht="15.75" customHeight="1" s="24"/>
-    <row r="654" ht="15.75" customHeight="1" s="24"/>
-    <row r="655" ht="15.75" customHeight="1" s="24"/>
-    <row r="656" ht="15.75" customHeight="1" s="24"/>
-    <row r="657" ht="15.75" customHeight="1" s="24"/>
-    <row r="658" ht="15.75" customHeight="1" s="24"/>
-    <row r="659" ht="15.75" customHeight="1" s="24"/>
-    <row r="660" ht="15.75" customHeight="1" s="24"/>
-    <row r="661" ht="15.75" customHeight="1" s="24"/>
-    <row r="662" ht="15.75" customHeight="1" s="24"/>
-    <row r="663" ht="15.75" customHeight="1" s="24"/>
-    <row r="664" ht="15.75" customHeight="1" s="24"/>
-    <row r="665" ht="15.75" customHeight="1" s="24"/>
-    <row r="666" ht="15.75" customHeight="1" s="24"/>
-    <row r="667" ht="15.75" customHeight="1" s="24"/>
-    <row r="668" ht="15.75" customHeight="1" s="24"/>
-    <row r="669" ht="15.75" customHeight="1" s="24"/>
-    <row r="670" ht="15.75" customHeight="1" s="24"/>
-    <row r="671" ht="15.75" customHeight="1" s="24"/>
-    <row r="672" ht="15.75" customHeight="1" s="24"/>
-    <row r="673" ht="15.75" customHeight="1" s="24"/>
-    <row r="674" ht="15.75" customHeight="1" s="24"/>
-    <row r="675" ht="15.75" customHeight="1" s="24"/>
-    <row r="676" ht="15.75" customHeight="1" s="24"/>
-    <row r="677" ht="15.75" customHeight="1" s="24"/>
-    <row r="678" ht="15.75" customHeight="1" s="24"/>
-    <row r="679" ht="15.75" customHeight="1" s="24"/>
-    <row r="680" ht="15.75" customHeight="1" s="24"/>
-    <row r="681" ht="15.75" customHeight="1" s="24"/>
-    <row r="682" ht="15.75" customHeight="1" s="24"/>
-    <row r="683" ht="15.75" customHeight="1" s="24"/>
-    <row r="684" ht="15.75" customHeight="1" s="24"/>
-    <row r="685" ht="15.75" customHeight="1" s="24"/>
-    <row r="686" ht="15.75" customHeight="1" s="24"/>
-    <row r="687" ht="15.75" customHeight="1" s="24"/>
-    <row r="688" ht="15.75" customHeight="1" s="24"/>
-    <row r="689" ht="15.75" customHeight="1" s="24"/>
-    <row r="690" ht="15.75" customHeight="1" s="24"/>
-    <row r="691" ht="15.75" customHeight="1" s="24"/>
-    <row r="692" ht="15.75" customHeight="1" s="24"/>
-    <row r="693" ht="15.75" customHeight="1" s="24"/>
-    <row r="694" ht="15.75" customHeight="1" s="24"/>
-    <row r="695" ht="15.75" customHeight="1" s="24"/>
-    <row r="696" ht="15.75" customHeight="1" s="24"/>
-    <row r="697" ht="15.75" customHeight="1" s="24"/>
-    <row r="698" ht="15.75" customHeight="1" s="24"/>
-    <row r="699" ht="15.75" customHeight="1" s="24"/>
-    <row r="700" ht="15.75" customHeight="1" s="24"/>
-    <row r="701" ht="15.75" customHeight="1" s="24"/>
-    <row r="702" ht="15.75" customHeight="1" s="24"/>
-    <row r="703" ht="15.75" customHeight="1" s="24"/>
-    <row r="704" ht="15.75" customHeight="1" s="24"/>
-    <row r="705" ht="15.75" customHeight="1" s="24"/>
-    <row r="706" ht="15.75" customHeight="1" s="24"/>
-    <row r="707" ht="15.75" customHeight="1" s="24"/>
-    <row r="708" ht="15.75" customHeight="1" s="24"/>
-    <row r="709" ht="15.75" customHeight="1" s="24"/>
-    <row r="710" ht="15.75" customHeight="1" s="24"/>
-    <row r="711" ht="15.75" customHeight="1" s="24"/>
-    <row r="712" ht="15.75" customHeight="1" s="24"/>
-    <row r="713" ht="15.75" customHeight="1" s="24"/>
-    <row r="714" ht="15.75" customHeight="1" s="24"/>
-    <row r="715" ht="15.75" customHeight="1" s="24"/>
-    <row r="716" ht="15.75" customHeight="1" s="24"/>
-    <row r="717" ht="15.75" customHeight="1" s="24"/>
-    <row r="718" ht="15.75" customHeight="1" s="24"/>
-    <row r="719" ht="15.75" customHeight="1" s="24"/>
-    <row r="720" ht="15.75" customHeight="1" s="24"/>
-    <row r="721" ht="15.75" customHeight="1" s="24"/>
-    <row r="722" ht="15.75" customHeight="1" s="24"/>
-    <row r="723" ht="15.75" customHeight="1" s="24"/>
-    <row r="724" ht="15.75" customHeight="1" s="24"/>
-    <row r="725" ht="15.75" customHeight="1" s="24"/>
-    <row r="726" ht="15.75" customHeight="1" s="24"/>
-    <row r="727" ht="15.75" customHeight="1" s="24"/>
-    <row r="728" ht="15.75" customHeight="1" s="24"/>
-    <row r="729" ht="15.75" customHeight="1" s="24"/>
-    <row r="730" ht="15.75" customHeight="1" s="24"/>
-    <row r="731" ht="15.75" customHeight="1" s="24"/>
-    <row r="732" ht="15.75" customHeight="1" s="24"/>
-    <row r="733" ht="15.75" customHeight="1" s="24"/>
-    <row r="734" ht="15.75" customHeight="1" s="24"/>
-    <row r="735" ht="15.75" customHeight="1" s="24"/>
-    <row r="736" ht="15.75" customHeight="1" s="24"/>
-    <row r="737" ht="15.75" customHeight="1" s="24"/>
-    <row r="738" ht="15.75" customHeight="1" s="24"/>
-    <row r="739" ht="15.75" customHeight="1" s="24"/>
-    <row r="740" ht="15.75" customHeight="1" s="24"/>
-    <row r="741" ht="15.75" customHeight="1" s="24"/>
-    <row r="742" ht="15.75" customHeight="1" s="24"/>
-    <row r="743" ht="15.75" customHeight="1" s="24"/>
-    <row r="744" ht="15.75" customHeight="1" s="24"/>
-    <row r="745" ht="15.75" customHeight="1" s="24"/>
-    <row r="746" ht="15.75" customHeight="1" s="24"/>
-    <row r="747" ht="15.75" customHeight="1" s="24"/>
-    <row r="748" ht="15.75" customHeight="1" s="24"/>
-    <row r="749" ht="15.75" customHeight="1" s="24"/>
-    <row r="750" ht="15.75" customHeight="1" s="24"/>
-    <row r="751" ht="15.75" customHeight="1" s="24"/>
-    <row r="752" ht="15.75" customHeight="1" s="24"/>
-    <row r="753" ht="15.75" customHeight="1" s="24"/>
-    <row r="754" ht="15.75" customHeight="1" s="24"/>
-    <row r="755" ht="15.75" customHeight="1" s="24"/>
-    <row r="756" ht="15.75" customHeight="1" s="24"/>
-    <row r="757" ht="15.75" customHeight="1" s="24"/>
-    <row r="758" ht="15.75" customHeight="1" s="24"/>
-    <row r="759" ht="15.75" customHeight="1" s="24"/>
-    <row r="760" ht="15.75" customHeight="1" s="24"/>
-    <row r="761" ht="15.75" customHeight="1" s="24"/>
-    <row r="762" ht="15.75" customHeight="1" s="24"/>
-    <row r="763" ht="15.75" customHeight="1" s="24"/>
-    <row r="764" ht="15.75" customHeight="1" s="24"/>
-    <row r="765" ht="15.75" customHeight="1" s="24"/>
-    <row r="766" ht="15.75" customHeight="1" s="24"/>
-    <row r="767" ht="15.75" customHeight="1" s="24"/>
-    <row r="768" ht="15.75" customHeight="1" s="24"/>
-    <row r="769" ht="15.75" customHeight="1" s="24"/>
-    <row r="770" ht="15.75" customHeight="1" s="24"/>
-    <row r="771" ht="15.75" customHeight="1" s="24"/>
-    <row r="772" ht="15.75" customHeight="1" s="24"/>
-    <row r="773" ht="15.75" customHeight="1" s="24"/>
-    <row r="774" ht="15.75" customHeight="1" s="24"/>
-    <row r="775" ht="15.75" customHeight="1" s="24"/>
-    <row r="776" ht="15.75" customHeight="1" s="24"/>
-    <row r="777" ht="15.75" customHeight="1" s="24"/>
-    <row r="778" ht="15.75" customHeight="1" s="24"/>
-    <row r="779" ht="15.75" customHeight="1" s="24"/>
-    <row r="780" ht="15.75" customHeight="1" s="24"/>
-    <row r="781" ht="15.75" customHeight="1" s="24"/>
-    <row r="782" ht="15.75" customHeight="1" s="24"/>
-    <row r="783" ht="15.75" customHeight="1" s="24"/>
-    <row r="784" ht="15.75" customHeight="1" s="24"/>
-    <row r="785" ht="15.75" customHeight="1" s="24"/>
-    <row r="786" ht="15.75" customHeight="1" s="24"/>
-    <row r="787" ht="15.75" customHeight="1" s="24"/>
-    <row r="788" ht="15.75" customHeight="1" s="24"/>
-    <row r="789" ht="15.75" customHeight="1" s="24"/>
-    <row r="790" ht="15.75" customHeight="1" s="24"/>
-    <row r="791" ht="15.75" customHeight="1" s="24"/>
-    <row r="792" ht="15.75" customHeight="1" s="24"/>
-    <row r="793" ht="15.75" customHeight="1" s="24"/>
-    <row r="794" ht="15.75" customHeight="1" s="24"/>
-    <row r="795" ht="15.75" customHeight="1" s="24"/>
-    <row r="796" ht="15.75" customHeight="1" s="24"/>
-    <row r="797" ht="15.75" customHeight="1" s="24"/>
-    <row r="798" ht="15.75" customHeight="1" s="24"/>
-    <row r="799" ht="15.75" customHeight="1" s="24"/>
-    <row r="800" ht="15.75" customHeight="1" s="24"/>
-    <row r="801" ht="15.75" customHeight="1" s="24"/>
-    <row r="802" ht="15.75" customHeight="1" s="24"/>
-    <row r="803" ht="15.75" customHeight="1" s="24"/>
-    <row r="804" ht="15.75" customHeight="1" s="24"/>
-    <row r="805" ht="15.75" customHeight="1" s="24"/>
-    <row r="806" ht="15.75" customHeight="1" s="24"/>
-    <row r="807" ht="15.75" customHeight="1" s="24"/>
-    <row r="808" ht="15.75" customHeight="1" s="24"/>
-    <row r="809" ht="15.75" customHeight="1" s="24"/>
-    <row r="810" ht="15.75" customHeight="1" s="24"/>
-    <row r="811" ht="15.75" customHeight="1" s="24"/>
-    <row r="812" ht="15.75" customHeight="1" s="24"/>
-    <row r="813" ht="15.75" customHeight="1" s="24"/>
-    <row r="814" ht="15.75" customHeight="1" s="24"/>
-    <row r="815" ht="15.75" customHeight="1" s="24"/>
-    <row r="816" ht="15.75" customHeight="1" s="24"/>
-    <row r="817" ht="15.75" customHeight="1" s="24"/>
-    <row r="818" ht="15.75" customHeight="1" s="24"/>
-    <row r="819" ht="15.75" customHeight="1" s="24"/>
-    <row r="820" ht="15.75" customHeight="1" s="24"/>
-    <row r="821" ht="15.75" customHeight="1" s="24"/>
-    <row r="822" ht="15.75" customHeight="1" s="24"/>
-    <row r="823" ht="15.75" customHeight="1" s="24"/>
-    <row r="824" ht="15.75" customHeight="1" s="24"/>
-    <row r="825" ht="15.75" customHeight="1" s="24"/>
-    <row r="826" ht="15.75" customHeight="1" s="24"/>
-    <row r="827" ht="15.75" customHeight="1" s="24"/>
-    <row r="828" ht="15.75" customHeight="1" s="24"/>
-    <row r="829" ht="15.75" customHeight="1" s="24"/>
-    <row r="830" ht="15.75" customHeight="1" s="24"/>
-    <row r="831" ht="15.75" customHeight="1" s="24"/>
-    <row r="832" ht="15.75" customHeight="1" s="24"/>
-    <row r="833" ht="15.75" customHeight="1" s="24"/>
-    <row r="834" ht="15.75" customHeight="1" s="24"/>
-    <row r="835" ht="15.75" customHeight="1" s="24"/>
-    <row r="836" ht="15.75" customHeight="1" s="24"/>
-    <row r="837" ht="15.75" customHeight="1" s="24"/>
-    <row r="838" ht="15.75" customHeight="1" s="24"/>
-    <row r="839" ht="15.75" customHeight="1" s="24"/>
-    <row r="840" ht="15.75" customHeight="1" s="24"/>
-    <row r="841" ht="15.75" customHeight="1" s="24"/>
-    <row r="842" ht="15.75" customHeight="1" s="24"/>
-    <row r="843" ht="15.75" customHeight="1" s="24"/>
-    <row r="844" ht="15.75" customHeight="1" s="24"/>
-    <row r="845" ht="15.75" customHeight="1" s="24"/>
-    <row r="846" ht="15.75" customHeight="1" s="24"/>
-    <row r="847" ht="15.75" customHeight="1" s="24"/>
-    <row r="848" ht="15.75" customHeight="1" s="24"/>
-    <row r="849" ht="15.75" customHeight="1" s="24"/>
-    <row r="850" ht="15.75" customHeight="1" s="24"/>
-    <row r="851" ht="15.75" customHeight="1" s="24"/>
-    <row r="852" ht="15.75" customHeight="1" s="24"/>
-    <row r="853" ht="15.75" customHeight="1" s="24"/>
-    <row r="854" ht="15.75" customHeight="1" s="24"/>
-    <row r="855" ht="15.75" customHeight="1" s="24"/>
-    <row r="856" ht="15.75" customHeight="1" s="24"/>
-    <row r="857" ht="15.75" customHeight="1" s="24"/>
-    <row r="858" ht="15.75" customHeight="1" s="24"/>
-    <row r="859" ht="15.75" customHeight="1" s="24"/>
-    <row r="860" ht="15.75" customHeight="1" s="24"/>
-    <row r="861" ht="15.75" customHeight="1" s="24"/>
-    <row r="862" ht="15.75" customHeight="1" s="24"/>
-    <row r="863" ht="15.75" customHeight="1" s="24"/>
-    <row r="864" ht="15.75" customHeight="1" s="24"/>
-    <row r="865" ht="15.75" customHeight="1" s="24"/>
-    <row r="866" ht="15.75" customHeight="1" s="24"/>
-    <row r="867" ht="15.75" customHeight="1" s="24"/>
-    <row r="868" ht="15.75" customHeight="1" s="24"/>
-    <row r="869" ht="15.75" customHeight="1" s="24"/>
-    <row r="870" ht="15.75" customHeight="1" s="24"/>
-    <row r="871" ht="15.75" customHeight="1" s="24"/>
-    <row r="872" ht="15.75" customHeight="1" s="24"/>
-    <row r="873" ht="15.75" customHeight="1" s="24"/>
-    <row r="874" ht="15.75" customHeight="1" s="24"/>
-    <row r="875" ht="15.75" customHeight="1" s="24"/>
-    <row r="876" ht="15.75" customHeight="1" s="24"/>
-    <row r="877" ht="15.75" customHeight="1" s="24"/>
-    <row r="878" ht="15.75" customHeight="1" s="24"/>
-    <row r="879" ht="15.75" customHeight="1" s="24"/>
-    <row r="880" ht="15.75" customHeight="1" s="24"/>
-    <row r="881" ht="15.75" customHeight="1" s="24"/>
-    <row r="882" ht="15.75" customHeight="1" s="24"/>
-    <row r="883" ht="15.75" customHeight="1" s="24"/>
-    <row r="884" ht="15.75" customHeight="1" s="24"/>
-    <row r="885" ht="15.75" customHeight="1" s="24"/>
-    <row r="886" ht="15.75" customHeight="1" s="24"/>
-    <row r="887" ht="15.75" customHeight="1" s="24"/>
-    <row r="888" ht="15.75" customHeight="1" s="24"/>
-    <row r="889" ht="15.75" customHeight="1" s="24"/>
-    <row r="890" ht="15.75" customHeight="1" s="24"/>
-    <row r="891" ht="15.75" customHeight="1" s="24"/>
-    <row r="892" ht="15.75" customHeight="1" s="24"/>
-    <row r="893" ht="15.75" customHeight="1" s="24"/>
-    <row r="894" ht="15.75" customHeight="1" s="24"/>
-    <row r="895" ht="15.75" customHeight="1" s="24"/>
-    <row r="896" ht="15.75" customHeight="1" s="24"/>
-    <row r="897" ht="15.75" customHeight="1" s="24"/>
-    <row r="898" ht="15.75" customHeight="1" s="24"/>
-    <row r="899" ht="15.75" customHeight="1" s="24"/>
-    <row r="900" ht="15.75" customHeight="1" s="24"/>
-    <row r="901" ht="15.75" customHeight="1" s="24"/>
-    <row r="902" ht="15.75" customHeight="1" s="24"/>
-    <row r="903" ht="15.75" customHeight="1" s="24"/>
-    <row r="904" ht="15.75" customHeight="1" s="24"/>
-    <row r="905" ht="15.75" customHeight="1" s="24"/>
-    <row r="906" ht="15.75" customHeight="1" s="24"/>
-    <row r="907" ht="15.75" customHeight="1" s="24"/>
-    <row r="908" ht="15.75" customHeight="1" s="24"/>
-    <row r="909" ht="15.75" customHeight="1" s="24"/>
-    <row r="910" ht="15.75" customHeight="1" s="24"/>
-    <row r="911" ht="15.75" customHeight="1" s="24"/>
-    <row r="912" ht="15.75" customHeight="1" s="24"/>
-    <row r="913" ht="15.75" customHeight="1" s="24"/>
-    <row r="914" ht="15.75" customHeight="1" s="24"/>
-    <row r="915" ht="15.75" customHeight="1" s="24"/>
-    <row r="916" ht="15.75" customHeight="1" s="24"/>
-    <row r="917" ht="15.75" customHeight="1" s="24"/>
-    <row r="918" ht="15.75" customHeight="1" s="24"/>
-    <row r="919" ht="15.75" customHeight="1" s="24"/>
-    <row r="920" ht="15.75" customHeight="1" s="24"/>
-    <row r="921" ht="15.75" customHeight="1" s="24"/>
-    <row r="922" ht="15.75" customHeight="1" s="24"/>
-    <row r="923" ht="15.75" customHeight="1" s="24"/>
-    <row r="924" ht="15.75" customHeight="1" s="24"/>
-    <row r="925" ht="15.75" customHeight="1" s="24"/>
-    <row r="926" ht="15.75" customHeight="1" s="24"/>
-    <row r="927" ht="15.75" customHeight="1" s="24"/>
-    <row r="928" ht="15.75" customHeight="1" s="24"/>
-    <row r="929" ht="15.75" customHeight="1" s="24"/>
-    <row r="930" ht="15.75" customHeight="1" s="24"/>
-    <row r="931" ht="15.75" customHeight="1" s="24"/>
-    <row r="932" ht="15.75" customHeight="1" s="24"/>
-    <row r="933" ht="15.75" customHeight="1" s="24"/>
-    <row r="934" ht="15.75" customHeight="1" s="24"/>
-    <row r="935" ht="15.75" customHeight="1" s="24"/>
-    <row r="936" ht="15.75" customHeight="1" s="24"/>
-    <row r="937" ht="15.75" customHeight="1" s="24"/>
-    <row r="938" ht="15.75" customHeight="1" s="24"/>
-    <row r="939" ht="15.75" customHeight="1" s="24"/>
-    <row r="940" ht="15.75" customHeight="1" s="24"/>
-    <row r="941" ht="15.75" customHeight="1" s="24"/>
-    <row r="942" ht="15.75" customHeight="1" s="24"/>
-    <row r="943" ht="15.75" customHeight="1" s="24"/>
-    <row r="944" ht="15.75" customHeight="1" s="24"/>
-    <row r="945" ht="15.75" customHeight="1" s="24"/>
-    <row r="946" ht="15.75" customHeight="1" s="24"/>
-    <row r="947" ht="15.75" customHeight="1" s="24"/>
-    <row r="948" ht="15.75" customHeight="1" s="24"/>
-    <row r="949" ht="15.75" customHeight="1" s="24"/>
-    <row r="950" ht="15.75" customHeight="1" s="24"/>
-    <row r="951" ht="15.75" customHeight="1" s="24"/>
-    <row r="952" ht="15.75" customHeight="1" s="24"/>
-    <row r="953" ht="15.75" customHeight="1" s="24"/>
-    <row r="954" ht="15.75" customHeight="1" s="24"/>
-    <row r="955" ht="15.75" customHeight="1" s="24"/>
-    <row r="956" ht="15.75" customHeight="1" s="24"/>
-    <row r="957" ht="15.75" customHeight="1" s="24"/>
-    <row r="958" ht="15.75" customHeight="1" s="24"/>
-    <row r="959" ht="15.75" customHeight="1" s="24"/>
-    <row r="960" ht="15.75" customHeight="1" s="24"/>
-    <row r="961" ht="15.75" customHeight="1" s="24"/>
-    <row r="962" ht="15.75" customHeight="1" s="24"/>
-    <row r="963" ht="15.75" customHeight="1" s="24"/>
-    <row r="964" ht="15.75" customHeight="1" s="24"/>
-    <row r="965" ht="15.75" customHeight="1" s="24"/>
-    <row r="966" ht="15.75" customHeight="1" s="24"/>
-    <row r="967" ht="15.75" customHeight="1" s="24"/>
-    <row r="968" ht="15.75" customHeight="1" s="24"/>
-    <row r="969" ht="15.75" customHeight="1" s="24"/>
-    <row r="970" ht="15.75" customHeight="1" s="24"/>
-    <row r="971" ht="15.75" customHeight="1" s="24"/>
-    <row r="972" ht="15.75" customHeight="1" s="24"/>
-    <row r="973" ht="15.75" customHeight="1" s="24"/>
-    <row r="974" ht="15.75" customHeight="1" s="24"/>
-    <row r="975" ht="15.75" customHeight="1" s="24"/>
-    <row r="976" ht="15.75" customHeight="1" s="24"/>
-    <row r="977" ht="15.75" customHeight="1" s="24"/>
-    <row r="978" ht="15.75" customHeight="1" s="24"/>
-    <row r="979" ht="15.75" customHeight="1" s="24"/>
-    <row r="980" ht="15.75" customHeight="1" s="24"/>
-    <row r="981" ht="15.75" customHeight="1" s="24"/>
-    <row r="982" ht="15.75" customHeight="1" s="24"/>
-    <row r="983" ht="15.75" customHeight="1" s="24"/>
-    <row r="984" ht="15.75" customHeight="1" s="24"/>
-    <row r="985" ht="15.75" customHeight="1" s="24"/>
-    <row r="986" ht="15.75" customHeight="1" s="24"/>
-    <row r="987" ht="15.75" customHeight="1" s="24"/>
-    <row r="988" ht="15.75" customHeight="1" s="24"/>
-    <row r="989" ht="15.75" customHeight="1" s="24"/>
-    <row r="990" ht="15.75" customHeight="1" s="24"/>
-    <row r="991" ht="15.75" customHeight="1" s="24"/>
-    <row r="992" ht="15.75" customHeight="1" s="24"/>
-    <row r="993" ht="15.75" customHeight="1" s="24"/>
-    <row r="994" ht="15.75" customHeight="1" s="24"/>
-    <row r="995" ht="15.75" customHeight="1" s="24"/>
-    <row r="996" ht="15.75" customHeight="1" s="24"/>
-    <row r="997" ht="15.75" customHeight="1" s="24"/>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
+<ns0:worksheet xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <ns0:sheetPr>
+    <ns0:tabColor rgb="FF17324D"/>
+    <ns0:outlinePr summaryBelow="1" summaryRight="1"/>
+    <ns0:pageSetUpPr/>
+  </ns0:sheetPr>
+  <ns0:dimension ref="A2:F14"/>
+  <ns0:sheetFormatPr baseColWidth="8" defaultColWidth="12.625" defaultRowHeight="14.25"/>
+  <ns0:cols>
+    <ns0:col width="24" customWidth="1" style="24" min="1" max="1"/>
+    <ns0:col width="15" customWidth="1" style="24" min="2" max="2"/>
+    <ns0:col width="4" customWidth="1" style="24" min="3" max="3"/>
+    <ns0:col width="24" customWidth="1" style="24" min="4" max="4"/>
+    <ns0:col width="15" customWidth="1" style="24" min="5" max="5"/>
+    <ns0:col width="8" customWidth="1" style="24" min="6" max="6"/>
+    <ns0:col width="8.625" customWidth="1" style="24" min="7" max="26"/>
+  </ns0:cols>
+  <ns0:sheetData>
+    <ns0:row r="1" ht="15" customHeight="1" s="24"/>
+    <ns0:row r="2" ht="25.5" customHeight="1" s="24">
+      <ns0:c r="B2" s="1" t="inlineStr">
+        <ns0:is>
+          <ns0:t>TỔNG HỢP SỬ DỤNG AI — TUẦN 07</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C2" s="2" t="n"/>
+      <ns0:c r="D2" s="2" t="n"/>
+      <ns0:c r="E2" s="2" t="n"/>
+      <ns0:c r="F2" s="2" t="n"/>
+    </ns0:row>
+    <ns0:row r="3" ht="19.5" customHeight="1" s="24">
+      <ns0:c r="A3" s="30" t="inlineStr">
+        <ns0:is>
+          <ns0:t>26/10/2026 – 01/11/2026</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B3" s="2" t="n"/>
+      <ns0:c r="C3" s="2" t="n"/>
+      <ns0:c r="D3" s="2" t="n"/>
+      <ns0:c r="E3" s="2" t="n"/>
+      <ns0:c r="F3" s="2" t="n"/>
+    </ns0:row>
+    <ns0:row r="4" ht="15" customHeight="1" s="24">
+      <ns0:c r="A4" s="2" t="n"/>
+      <ns0:c r="B4" s="2" t="n"/>
+      <ns0:c r="C4" s="2" t="n"/>
+      <ns0:c r="D4" s="2" t="n"/>
+      <ns0:c r="E4" s="2" t="n"/>
+      <ns0:c r="F4" s="2" t="n"/>
+    </ns0:row>
+    <ns0:row r="5" ht="33.75" customHeight="1" s="24">
+      <ns0:c r="A5" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>TỔNG SỐ PROMPT</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B5" s="5">
+        <ns0:f>SUM(B9:B11)</ns0:f>
+        <ns0:v>14</ns0:v>
+      </ns0:c>
+      <ns0:c r="C5" s="2" t="n"/>
+      <ns0:c r="D5" s="2" t="n"/>
+      <ns0:c r="E5" s="2" t="n"/>
+      <ns0:c r="F5" s="2" t="n"/>
+    </ns0:row>
+    <ns0:row r="6" ht="15" customHeight="1" s="24">
+      <ns0:c r="A6" s="2" t="n"/>
+      <ns0:c r="B6" s="2" t="n"/>
+      <ns0:c r="C6" s="2" t="n"/>
+      <ns0:c r="D6" s="2" t="n"/>
+      <ns0:c r="E6" s="2" t="n"/>
+      <ns0:c r="F6" s="2" t="n"/>
+    </ns0:row>
+    <ns0:row r="7" ht="15" customHeight="1" s="24">
+      <ns0:c r="A7" s="2" t="n"/>
+      <ns0:c r="B7" s="2" t="n"/>
+      <ns0:c r="C7" s="2" t="n"/>
+      <ns0:c r="D7" s="2" t="n"/>
+      <ns0:c r="E7" s="2" t="n"/>
+      <ns0:c r="F7" s="2" t="n"/>
+    </ns0:row>
+    <ns0:row r="8" ht="27.75" customHeight="1" s="24">
+      <ns0:c r="A8" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NGƯỜI TẠO</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B8" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>SỐ PROMPT</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C8" s="2" t="n"/>
+      <ns0:c r="D8" s="10" t="inlineStr">
+        <ns0:is>
+          <ns0:t>TOOL AI</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E8" s="10" t="inlineStr">
+        <ns0:is>
+          <ns0:t>SỐ PROMPT</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F8" s="2" t="n"/>
+    </ns0:row>
+    <ns0:row r="9" ht="24.75" customHeight="1" s="24">
+      <ns0:c r="A9" s="11" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Thắng</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B9" s="13">
+        <ns0:f>COUNTIF(Thắng!$A$6:$A$306,"&lt;&gt;")</ns0:f>
+        <ns0:v>11</ns0:v>
+      </ns0:c>
+      <ns0:c r="C9" s="2" t="n"/>
+      <ns0:c r="D9" s="14" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Claude</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E9" s="16">
+        <ns0:f>COUNTIFS(Thắng!$A$6:$A$306,"&lt;&gt;",Thắng!$C$6:$C$306,D9)+COUNTIFS(Sang!$A$6:$A$306,"&lt;&gt;",Sang!$C$6:$C$306,D9)+COUNTIFS(Nguyên!$A$6:$A$306,"&lt;&gt;",Nguyên!$C$6:$C$306,D9)</ns0:f>
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="F9" s="2" t="n"/>
+    </ns0:row>
+    <ns0:row r="10" ht="24.75" customHeight="1" s="24">
+      <ns0:c r="A10" s="11" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Sang</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B10" s="13">
+        <ns0:f>COUNTIF(Sang!$A$6:$A$306,"&lt;&gt;")</ns0:f>
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="C10" s="2" t="n"/>
+      <ns0:c r="D10" s="14" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Codex</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E10" s="16">
+        <ns0:f>COUNTIFS(Thắng!$A$6:$A$306,"&lt;&gt;",Thắng!$C$6:$C$306,D10)+COUNTIFS(Sang!$A$6:$A$306,"&lt;&gt;",Sang!$C$6:$C$306,D10)+COUNTIFS(Nguyên!$A$6:$A$306,"&lt;&gt;",Nguyên!$C$6:$C$306,D10)</ns0:f>
+        <ns0:v>3</ns0:v>
+      </ns0:c>
+      <ns0:c r="F10" s="2" t="n"/>
+    </ns0:row>
+    <ns0:row r="11" ht="24.75" customHeight="1" s="24">
+      <ns0:c r="A11" s="11" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Nguyên</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B11" s="13">
+        <ns0:f>COUNTIF(Nguyên!$A$6:$A$306,"&lt;&gt;")</ns0:f>
+        <ns0:v>3</ns0:v>
+      </ns0:c>
+      <ns0:c r="C11" s="2" t="n"/>
+      <ns0:c r="D11" s="14" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Antigravity</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E11" s="16">
+        <ns0:f>COUNTIFS(Thắng!$A$6:$A$306,"&lt;&gt;",Thắng!$C$6:$C$306,D11)+COUNTIFS(Sang!$A$6:$A$306,"&lt;&gt;",Sang!$C$6:$C$306,D11)+COUNTIFS(Nguyên!$A$6:$A$306,"&lt;&gt;",Nguyên!$C$6:$C$306,D11)</ns0:f>
+        <ns0:v>11</ns0:v>
+      </ns0:c>
+      <ns0:c r="F11" s="2" t="n"/>
+    </ns0:row>
+    <ns0:row r="12" ht="15" customHeight="1" s="24">
+      <ns0:c r="A12" s="2" t="n"/>
+      <ns0:c r="B12" s="2" t="n"/>
+      <ns0:c r="C12" s="2" t="n"/>
+      <ns0:c r="D12" s="2" t="n"/>
+      <ns0:c r="E12" s="2" t="n"/>
+      <ns0:c r="F12" s="2" t="n"/>
+    </ns0:row>
+    <ns0:row r="13" ht="15" customHeight="1" s="24">
+      <ns0:c r="A13" s="2" t="n"/>
+      <ns0:c r="B13" s="2" t="n"/>
+      <ns0:c r="C13" s="2" t="n"/>
+      <ns0:c r="D13" s="2" t="n"/>
+      <ns0:c r="E13" s="2" t="n"/>
+      <ns0:c r="F13" s="2" t="n"/>
+    </ns0:row>
+    <ns0:row r="14" ht="15" customHeight="1" s="24">
+      <ns0:c r="A14" s="17" t="n"/>
+      <ns0:c r="B14" s="2" t="n"/>
+      <ns0:c r="C14" s="2" t="n"/>
+      <ns0:c r="D14" s="2" t="n"/>
+      <ns0:c r="E14" s="2" t="n"/>
+      <ns0:c r="F14" s="2" t="n"/>
+    </ns0:row>
+    <ns0:row r="18" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="19" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="20" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="21" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="22" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="23" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="24" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="25" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="26" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="27" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="28" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="29" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="30" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="31" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="32" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="33" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="34" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="35" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="36" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="37" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="38" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="39" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="40" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="41" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="42" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="43" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="44" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="45" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="46" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="47" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="48" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="49" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="50" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="51" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="52" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="53" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="54" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="55" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="56" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="57" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="58" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="59" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="60" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="61" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="62" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="63" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="64" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="65" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="66" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="67" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="68" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="69" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="70" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="71" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="72" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="73" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="74" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="75" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="76" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="77" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="78" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="79" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="80" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="81" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="82" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="83" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="84" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="85" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="86" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="87" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="88" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="89" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="90" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="91" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="92" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="93" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="94" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="95" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="96" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="97" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="98" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="99" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="100" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="101" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="102" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="103" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="104" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="105" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="106" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="107" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="108" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="109" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="110" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="111" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="112" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="113" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="114" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="115" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="116" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="117" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="118" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="119" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="120" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="121" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="122" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="123" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="124" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="125" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="126" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="127" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="128" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="129" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="130" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="131" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="132" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="133" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="134" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="135" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="136" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="137" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="138" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="139" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="140" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="141" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="142" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="143" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="144" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="145" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="146" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="147" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="148" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="149" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="150" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="151" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="152" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="153" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="154" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="155" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="156" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="157" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="158" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="159" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="160" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="161" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="162" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="163" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="164" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="165" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="166" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="167" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="168" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="169" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="170" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="171" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="172" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="173" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="174" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="175" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="176" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="177" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="178" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="179" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="180" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="181" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="182" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="183" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="184" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="185" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="186" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="187" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="188" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="189" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="190" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="191" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="192" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="193" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="194" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="195" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="196" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="197" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="198" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="199" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="200" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="201" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="202" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="203" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="204" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="205" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="206" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="207" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="208" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="209" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="210" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="211" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="212" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="213" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="214" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="215" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="216" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="217" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="218" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="219" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="220" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="221" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="222" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="223" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="224" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="225" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="226" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="227" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="228" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="229" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="230" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="231" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="232" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="233" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="234" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="235" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="236" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="237" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="238" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="239" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="240" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="241" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="242" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="243" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="244" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="245" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="246" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="247" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="248" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="249" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="250" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="251" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="252" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="253" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="254" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="255" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="256" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="257" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="258" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="259" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="260" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="261" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="262" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="263" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="264" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="265" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="266" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="267" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="268" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="269" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="270" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="271" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="272" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="273" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="274" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="275" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="276" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="277" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="278" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="279" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="280" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="281" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="282" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="283" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="284" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="285" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="286" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="287" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="288" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="289" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="290" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="291" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="292" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="293" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="294" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="295" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="296" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="297" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="298" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="299" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="300" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="301" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="302" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="303" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="304" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="305" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="306" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="307" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="308" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="309" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="310" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="311" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="312" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="313" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="314" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="315" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="316" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="317" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="318" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="319" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="320" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="321" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="322" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="323" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="324" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="325" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="326" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="327" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="328" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="329" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="330" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="331" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="332" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="333" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="334" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="335" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="336" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="337" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="338" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="339" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="340" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="341" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="342" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="343" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="344" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="345" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="346" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="347" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="348" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="349" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="350" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="351" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="352" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="353" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="354" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="355" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="356" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="357" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="358" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="359" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="360" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="361" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="362" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="363" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="364" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="365" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="366" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="367" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="368" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="369" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="370" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="371" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="372" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="373" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="374" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="375" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="376" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="377" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="378" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="379" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="380" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="381" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="382" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="383" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="384" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="385" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="386" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="387" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="388" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="389" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="390" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="391" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="392" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="393" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="394" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="395" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="396" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="397" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="398" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="399" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="400" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="401" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="402" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="403" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="404" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="405" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="406" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="407" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="408" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="409" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="410" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="411" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="412" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="413" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="414" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="415" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="416" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="417" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="418" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="419" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="420" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="421" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="422" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="423" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="424" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="425" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="426" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="427" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="428" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="429" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="430" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="431" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="432" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="433" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="434" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="435" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="436" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="437" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="438" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="439" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="440" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="441" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="442" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="443" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="444" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="445" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="446" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="447" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="448" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="449" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="450" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="451" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="452" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="453" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="454" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="455" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="456" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="457" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="458" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="459" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="460" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="461" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="462" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="463" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="464" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="465" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="466" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="467" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="468" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="469" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="470" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="471" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="472" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="473" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="474" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="475" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="476" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="477" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="478" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="479" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="480" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="481" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="482" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="483" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="484" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="485" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="486" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="487" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="488" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="489" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="490" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="491" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="492" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="493" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="494" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="495" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="496" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="497" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="498" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="499" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="500" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="501" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="502" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="503" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="504" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="505" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="506" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="507" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="508" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="509" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="510" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="511" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="512" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="513" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="514" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="515" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="516" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="517" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="518" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="519" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="520" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="521" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="522" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="523" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="524" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="525" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="526" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="527" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="528" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="529" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="530" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="531" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="532" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="533" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="534" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="535" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="536" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="537" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="538" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="539" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="540" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="541" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="542" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="543" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="544" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="545" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="546" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="547" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="548" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="549" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="550" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="551" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="552" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="553" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="554" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="555" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="556" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="557" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="558" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="559" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="560" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="561" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="562" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="563" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="564" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="565" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="566" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="567" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="568" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="569" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="570" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="571" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="572" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="573" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="574" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="575" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="576" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="577" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="578" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="579" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="580" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="581" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="582" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="583" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="584" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="585" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="586" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="587" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="588" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="589" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="590" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="591" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="592" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="593" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="594" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="595" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="596" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="597" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="598" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="599" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="600" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="601" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="602" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="603" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="604" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="605" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="606" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="607" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="608" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="609" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="610" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="611" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="612" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="613" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="614" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="615" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="616" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="617" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="618" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="619" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="620" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="621" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="622" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="623" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="624" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="625" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="626" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="627" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="628" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="629" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="630" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="631" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="632" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="633" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="634" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="635" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="636" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="637" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="638" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="639" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="640" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="641" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="642" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="643" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="644" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="645" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="646" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="647" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="648" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="649" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="650" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="651" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="652" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="653" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="654" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="655" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="656" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="657" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="658" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="659" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="660" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="661" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="662" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="663" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="664" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="665" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="666" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="667" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="668" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="669" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="670" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="671" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="672" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="673" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="674" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="675" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="676" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="677" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="678" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="679" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="680" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="681" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="682" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="683" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="684" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="685" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="686" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="687" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="688" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="689" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="690" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="691" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="692" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="693" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="694" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="695" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="696" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="697" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="698" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="699" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="700" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="701" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="702" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="703" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="704" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="705" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="706" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="707" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="708" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="709" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="710" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="711" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="712" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="713" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="714" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="715" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="716" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="717" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="718" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="719" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="720" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="721" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="722" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="723" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="724" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="725" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="726" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="727" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="728" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="729" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="730" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="731" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="732" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="733" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="734" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="735" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="736" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="737" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="738" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="739" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="740" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="741" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="742" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="743" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="744" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="745" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="746" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="747" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="748" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="749" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="750" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="751" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="752" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="753" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="754" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="755" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="756" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="757" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="758" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="759" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="760" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="761" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="762" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="763" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="764" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="765" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="766" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="767" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="768" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="769" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="770" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="771" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="772" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="773" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="774" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="775" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="776" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="777" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="778" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="779" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="780" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="781" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="782" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="783" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="784" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="785" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="786" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="787" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="788" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="789" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="790" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="791" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="792" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="793" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="794" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="795" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="796" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="797" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="798" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="799" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="800" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="801" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="802" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="803" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="804" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="805" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="806" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="807" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="808" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="809" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="810" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="811" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="812" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="813" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="814" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="815" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="816" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="817" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="818" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="819" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="820" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="821" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="822" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="823" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="824" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="825" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="826" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="827" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="828" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="829" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="830" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="831" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="832" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="833" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="834" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="835" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="836" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="837" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="838" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="839" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="840" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="841" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="842" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="843" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="844" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="845" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="846" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="847" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="848" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="849" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="850" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="851" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="852" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="853" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="854" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="855" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="856" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="857" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="858" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="859" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="860" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="861" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="862" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="863" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="864" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="865" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="866" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="867" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="868" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="869" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="870" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="871" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="872" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="873" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="874" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="875" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="876" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="877" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="878" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="879" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="880" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="881" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="882" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="883" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="884" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="885" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="886" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="887" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="888" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="889" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="890" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="891" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="892" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="893" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="894" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="895" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="896" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="897" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="898" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="899" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="900" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="901" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="902" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="903" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="904" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="905" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="906" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="907" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="908" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="909" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="910" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="911" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="912" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="913" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="914" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="915" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="916" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="917" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="918" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="919" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="920" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="921" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="922" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="923" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="924" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="925" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="926" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="927" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="928" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="929" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="930" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="931" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="932" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="933" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="934" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="935" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="936" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="937" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="938" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="939" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="940" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="941" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="942" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="943" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="944" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="945" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="946" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="947" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="948" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="949" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="950" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="951" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="952" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="953" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="954" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="955" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="956" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="957" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="958" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="959" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="960" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="961" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="962" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="963" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="964" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="965" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="966" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="967" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="968" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="969" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="970" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="971" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="972" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="973" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="974" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="975" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="976" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="977" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="978" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="979" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="980" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="981" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="982" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="983" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="984" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="985" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="986" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="987" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="988" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="989" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="990" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="991" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="992" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="993" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="994" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="995" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="996" ht="15.75" customHeight="1" s="24"/>
+    <ns0:row r="997" ht="15.75" customHeight="1" s="24"/>
+  </ns0:sheetData>
+  <ns0:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</ns0:worksheet>
 </file>
</xml_diff>

<commit_message>
docs(W7): báo cáo tuần 7 của Sang và AI Prompt Log tuần 7 (sheet Sang)
Báo cáo đối chiếu W7-S01..S05 với kế hoạch W7, phần làm lại sau W7 đã vào
main (#78: D058, D059, D060, sơ đồ lớp thực thể), kết quả kiểm thử, vướng mắc
và kế hoạch tuần 8. AI log W07 sheet Sang 10 dòng ngày 28–29/10, mỗi dòng có
PR hoặc tệp làm minh chứng; README cập nhật số liệu W07 (24 bản ghi).
</commit_message>
<xml_diff>
--- a/docs/evidence/tc2-3-ai-usage/AI Prompt Log - W07 - 2026-10-26_2026-11-01.xlsx
+++ b/docs/evidence/tc2-3-ai-usage/AI Prompt Log - W07 - 2026-10-26_2026-11-01.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thắng" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nguyên" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sang" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tổng hợp" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Thắng" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Nguyên" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Sang" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Tổng hợp" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
@@ -12960,84 +12960,304 @@
       </c>
     </row>
     <row r="6" ht="36" customHeight="1" s="24">
-      <c r="A6" s="20" t="n"/>
-      <c r="B6" s="18" t="n"/>
-      <c r="C6" s="18" t="n"/>
-      <c r="D6" s="33" t="n"/>
-      <c r="E6" s="33" t="n"/>
-      <c r="F6" s="33" t="n"/>
+      <c r="A6" s="36" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B6" s="37" t="inlineStr">
+        <is>
+          <t>Sang</t>
+        </is>
+      </c>
+      <c r="C6" s="37" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="D6" s="38" t="inlineStr">
+        <is>
+          <t>Rà soát kế hoạch W7 sau khi chuyển sang MongoDB; làm main xanh trở lại và gỡ số đo S&amp;I còn sót</t>
+        </is>
+      </c>
+      <c r="E6" s="38" t="inlineStr">
+        <is>
+          <t>Đối chiếu kế hoạch W7 với những gì nhóm đã chuyển sang repo nộp bài (kiến trúc nay dùng MongoDB, không còn PostgreSQL), chỉ ra các mục sai lệch, rồi thực hiện ngay hai bước: đưa nhánh main về trạng thái CI xanh với code khớp bản nguồn đã chuyển, và gỡ các số đo suy ra từ Speak &amp; Improve còn sót trong tài liệu, kèm chuyển các tài liệu vận hành cần thiết từ repo gốc.</t>
+        </is>
+      </c>
+      <c r="F6" s="38" t="inlineStr">
+        <is>
+          <t>https://github.com/thanglb2005/ai-assessor-cefr/pull/71; https://github.com/thanglb2005/ai-assessor-cefr/pull/72; https://github.com/thanglb2005/ai-assessor-cefr/pull/73</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="36" customHeight="1" s="24">
-      <c r="A7" s="20" t="n"/>
-      <c r="B7" s="18" t="n"/>
-      <c r="C7" s="18" t="n"/>
-      <c r="D7" s="33" t="n"/>
-      <c r="E7" s="33" t="n"/>
-      <c r="F7" s="33" t="n"/>
+      <c r="A7" s="36" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B7" s="37" t="inlineStr">
+        <is>
+          <t>Sang</t>
+        </is>
+      </c>
+      <c r="C7" s="37" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="D7" s="38" t="inlineStr">
+        <is>
+          <t>D058: bỏ đồng thuận nghiên cứu, thay bằng đồng ý điều khoản sử dụng</t>
+        </is>
+      </c>
+      <c r="E7" s="38" t="inlineStr">
+        <is>
+          <t>Giai đoạn thu giọng người Việt để huấn luyện mô hình đã kết thúc; loại bỏ tính năng ký đồng thuận nghiên cứu khỏi toàn hệ thống và thay bằng một lần đồng ý điều khoản sử dụng, có migration chuyển dữ liệu cũ.</t>
+        </is>
+      </c>
+      <c r="F7" s="38" t="inlineStr">
+        <is>
+          <t>https://github.com/thanglb2005/ai-assessor-cefr/pull/75 (gộp vào main qua #78)</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="36" customHeight="1" s="24">
-      <c r="A8" s="20" t="n"/>
-      <c r="B8" s="18" t="n"/>
-      <c r="C8" s="18" t="n"/>
-      <c r="D8" s="33" t="n"/>
-      <c r="E8" s="33" t="n"/>
-      <c r="F8" s="33" t="n"/>
+      <c r="A8" s="36" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B8" s="37" t="inlineStr">
+        <is>
+          <t>Sang</t>
+        </is>
+      </c>
+      <c r="C8" s="37" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="D8" s="38" t="inlineStr">
+        <is>
+          <t>Rút gọn sơ đồ lớp, bỏ thuộc tính thừa trong sơ đồ và code, cập nhật bản draw.io</t>
+        </is>
+      </c>
+      <c r="E8" s="38" t="inlineStr">
+        <is>
+          <t>Rà lại class diagram trên draw.io: chỉ giữ lớp và thuộc tính phục vụ nghiệp vụ, bỏ thuộc tính không ai đọc ở cả sơ đồ lẫn code, giảm số bảng xuống mức hợp lý theo chuẩn OOP (khoảng 20, được phép chênh lệch nếu có lý do), rồi cập nhật lại trang "So do lop" trên Drive.</t>
+        </is>
+      </c>
+      <c r="F8" s="38" t="inlineStr">
+        <is>
+          <t>https://github.com/thanglb2005/ai-assessor-cefr/pull/69; https://github.com/thanglb2005/ai-assessor-cefr/pull/70; https://github.com/thanglb2005/ai-assessor-cefr/pull/74</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="36" customHeight="1" s="24">
-      <c r="A9" s="20" t="n"/>
-      <c r="B9" s="18" t="n"/>
-      <c r="C9" s="18" t="n"/>
-      <c r="D9" s="33" t="n"/>
-      <c r="E9" s="33" t="n"/>
-      <c r="F9" s="33" t="n"/>
+      <c r="A9" s="36" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B9" s="37" t="inlineStr">
+        <is>
+          <t>Sang</t>
+        </is>
+      </c>
+      <c r="C9" s="37" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="D9" s="38" t="inlineStr">
+        <is>
+          <t>D059: hỗ trợ đủ sáu band CEFR từ A1 đến C2</t>
+        </is>
+      </c>
+      <c r="E9" s="38" t="inlineStr">
+        <is>
+          <t>Mở rộng thang band từ A2–B2 lên đủ A1–C2 ở mọi nơi: ánh xạ điểm sang band, ngân hàng luyện tập, lộ trình mẫu, chấm mù, giao diện và test; ghi rõ ba ngưỡng ngoài chưa được hiệu chuẩn.</t>
+        </is>
+      </c>
+      <c r="F9" s="38" t="inlineStr">
+        <is>
+          <t>https://github.com/thanglb2005/ai-assessor-cefr/pull/76 (gộp vào main qua #78); src/aicefr/scoring/band_map.py</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="36" customHeight="1" s="24">
-      <c r="A10" s="20" t="n"/>
-      <c r="B10" s="18" t="n"/>
-      <c r="C10" s="18" t="n"/>
-      <c r="D10" s="33" t="n"/>
-      <c r="E10" s="33" t="n"/>
-      <c r="F10" s="33" t="n"/>
+      <c r="A10" s="36" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B10" s="37" t="inlineStr">
+        <is>
+          <t>Sang</t>
+        </is>
+      </c>
+      <c r="C10" s="37" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="D10" s="38" t="inlineStr">
+        <is>
+          <t>Kiểm tra độ phủ nghiệp vụ của sơ đồ lớp, thiết kế lại chỉ gồm thực thể và chạy toàn bộ test ở local</t>
+        </is>
+      </c>
+      <c r="E10" s="38" t="inlineStr">
+        <is>
+          <t>Đánh giá bộ khoảng 20 collection đã đề xuất có phủ hết nghiệp vụ của bài toán hay chưa (số lượng được linh hoạt); thiết kế lại class diagram chỉ chứa thực thể, không lớp trừu tượng; sau đó chạy toàn bộ test đơn vị và E2E ở local.</t>
+        </is>
+      </c>
+      <c r="F10" s="38" t="inlineStr">
+        <is>
+          <t>https://github.com/thanglb2005/ai-assessor-cefr/pull/70; docs/sdd/thiet-ke-gon-so-do-lop-va-collection.md</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="36" customHeight="1" s="24">
-      <c r="A11" s="20" t="n"/>
-      <c r="B11" s="18" t="n"/>
-      <c r="C11" s="18" t="n"/>
-      <c r="D11" s="33" t="n"/>
-      <c r="E11" s="33" t="n"/>
-      <c r="F11" s="33" t="n"/>
+      <c r="A11" s="36" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B11" s="37" t="inlineStr">
+        <is>
+          <t>Sang</t>
+        </is>
+      </c>
+      <c r="C11" s="37" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="D11" s="38" t="inlineStr">
+        <is>
+          <t>Bổ sung enum vào sơ đồ lớp, rút còn enum điều khiển nghiệp vụ, chia khung theo phần nghiệp vụ</t>
+        </is>
+      </c>
+      <c r="E11" s="38" t="inlineStr">
+        <is>
+          <t>Thêm các kiểu liệt kê vào class diagram và xác nhận sơ đồ phủ đủ nghiệp vụ; sau đó lược bớt enum không cần thiết, gộp collection hợp lý, vẽ sơ đồ chia khung theo phần nghiệp vụ để các đường không chồng chéo và nối mỗi enum với thực thể dùng nó.</t>
+        </is>
+      </c>
+      <c r="F11" s="38" t="inlineStr">
+        <is>
+          <t>https://github.com/thanglb2005/ai-assessor-cefr/pull/77; tools/zone_layout.py; docs/sdd/diagrams/02_class.drawio</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="36" customHeight="1" s="24">
-      <c r="A12" s="20" t="n"/>
-      <c r="B12" s="18" t="n"/>
-      <c r="C12" s="18" t="n"/>
-      <c r="D12" s="33" t="n"/>
-      <c r="E12" s="33" t="n"/>
-      <c r="F12" s="33" t="n"/>
+      <c r="A12" s="36" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B12" s="37" t="inlineStr">
+        <is>
+          <t>Sang</t>
+        </is>
+      </c>
+      <c r="C12" s="37" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="D12" s="38" t="inlineStr">
+        <is>
+          <t>D060: quan hệ thể hiện qua thuộc tính, gộp collection theo aggregate root và rã sơ đồ xuống code</t>
+        </is>
+      </c>
+      <c r="E12" s="38" t="inlineStr">
+        <is>
+          <t>Sửa class diagram theo quy tắc của nhóm: mỗi quan hệ phải có thuộc tính ở lớp giữ quan hệ, bội số chỉ ghi trên đường giữa hai thực thể, thuộc tính trỏ tới enum mang kiểu enum; tiếp tục gộp collection nếu hợp lý, rồi chuyển code theo đúng sơ đồ (lớp miền, migration dữ liệu, test đối chiếu sơ đồ với code).</t>
+        </is>
+      </c>
+      <c r="F12" s="38" t="inlineStr">
+        <is>
+          <t>https://github.com/thanglb2005/ai-assessor-cefr/pull/77; src/aicefr/storage/migrations.py; tests/test_d060_collections.py; tests/test_diagrams.py</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="36" customHeight="1" s="24">
-      <c r="A13" s="20" t="n"/>
-      <c r="B13" s="18" t="n"/>
-      <c r="C13" s="18" t="n"/>
-      <c r="D13" s="33" t="n"/>
-      <c r="E13" s="33" t="n"/>
-      <c r="F13" s="33" t="n"/>
+      <c r="A13" s="36" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B13" s="37" t="inlineStr">
+        <is>
+          <t>Sang</t>
+        </is>
+      </c>
+      <c r="C13" s="37" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="D13" s="38" t="inlineStr">
+        <is>
+          <t>Đưa toàn bộ phần làm lại sau W7 lên main của repo nộp bài</t>
+        </is>
+      </c>
+      <c r="E13" s="38" t="inlineStr">
+        <is>
+          <t>Hoàn thiện bố cục sơ đồ, merge D060, rồi gộp toàn bộ phần làm lại sau W7 vào main của repo nhóm thành một commit; repo gốc của Sang không dùng nữa. Xử lý các check CI đỏ (link tài liệu hỏng, giới hạn thời gian job kiểm thử).</t>
+        </is>
+      </c>
+      <c r="F13" s="38" t="inlineStr">
+        <is>
+          <t>https://github.com/thanglb2005/ai-assessor-cefr/pull/78 (squash 130ffea); .github/workflows/ci.yml</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="36" customHeight="1" s="24">
-      <c r="A14" s="20" t="n"/>
-      <c r="B14" s="18" t="n"/>
-      <c r="C14" s="18" t="n"/>
-      <c r="D14" s="33" t="n"/>
-      <c r="E14" s="33" t="n"/>
-      <c r="F14" s="33" t="n"/>
+      <c r="A14" s="36" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B14" s="37" t="inlineStr">
+        <is>
+          <t>Sang</t>
+        </is>
+      </c>
+      <c r="C14" s="37" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="D14" s="38" t="inlineStr">
+        <is>
+          <t>Merge PR gỡ số đo S&amp;I và đóng các PR đã được gộp</t>
+        </is>
+      </c>
+      <c r="E14" s="38" t="inlineStr">
+        <is>
+          <t>Cập nhật nhánh gỡ số đo S&amp;I theo main mới, sửa link tới tài liệu nội bộ, merge vào main, rồi đóng các PR đã nằm trong lần gộp kèm ghi chú lý do.</t>
+        </is>
+      </c>
+      <c r="F14" s="38" t="inlineStr">
+        <is>
+          <t>https://github.com/thanglb2005/ai-assessor-cefr/pull/73 (squash 856bd5f)</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="36" customHeight="1" s="24">
-      <c r="A15" s="20" t="n"/>
-      <c r="B15" s="18" t="n"/>
-      <c r="C15" s="18" t="n"/>
-      <c r="D15" s="33" t="n"/>
-      <c r="E15" s="33" t="n"/>
-      <c r="F15" s="33" t="n"/>
+      <c r="A15" s="36" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B15" s="37" t="inlineStr">
+        <is>
+          <t>Sang</t>
+        </is>
+      </c>
+      <c r="C15" s="37" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="D15" s="38" t="inlineStr">
+        <is>
+          <t>Soạn báo cáo tuần 7 và ghi AI Prompt Log tuần 7</t>
+        </is>
+      </c>
+      <c r="E15" s="38" t="inlineStr">
+        <is>
+          <t>Cập nhật báo cáo tiến độ tuần 7 của Sang và nhật ký sử dụng AI của tuần, đối chiếu từng mục với PR và commit thật.</t>
+        </is>
+      </c>
+      <c r="F15" s="38" t="inlineStr">
+        <is>
+          <t>docs/reports/week-07/bao-cao-tuan-07-sang.md; docs/evidence/tc2-3-ai-usage/README.md</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="36" customHeight="1" s="24">
       <c r="A16" s="20" t="n"/>
@@ -18858,1182 +19078,1182 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<ns0:worksheet xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <ns0:sheetPr>
-    <ns0:tabColor rgb="FF17324D"/>
-    <ns0:outlinePr summaryBelow="1" summaryRight="1"/>
-    <ns0:pageSetUpPr/>
-  </ns0:sheetPr>
-  <ns0:dimension ref="A2:F14"/>
-  <ns0:sheetFormatPr baseColWidth="8" defaultColWidth="12.625" defaultRowHeight="14.25"/>
-  <ns0:cols>
-    <ns0:col width="24" customWidth="1" style="24" min="1" max="1"/>
-    <ns0:col width="15" customWidth="1" style="24" min="2" max="2"/>
-    <ns0:col width="4" customWidth="1" style="24" min="3" max="3"/>
-    <ns0:col width="24" customWidth="1" style="24" min="4" max="4"/>
-    <ns0:col width="15" customWidth="1" style="24" min="5" max="5"/>
-    <ns0:col width="8" customWidth="1" style="24" min="6" max="6"/>
-    <ns0:col width="8.625" customWidth="1" style="24" min="7" max="26"/>
-  </ns0:cols>
-  <ns0:sheetData>
-    <ns0:row r="1" ht="15" customHeight="1" s="24"/>
-    <ns0:row r="2" ht="25.5" customHeight="1" s="24">
-      <ns0:c r="B2" s="1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>TỔNG HỢP SỬ DỤNG AI — TUẦN 07</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C2" s="2" t="n"/>
-      <ns0:c r="D2" s="2" t="n"/>
-      <ns0:c r="E2" s="2" t="n"/>
-      <ns0:c r="F2" s="2" t="n"/>
-    </ns0:row>
-    <ns0:row r="3" ht="19.5" customHeight="1" s="24">
-      <ns0:c r="A3" s="30" t="inlineStr">
-        <ns0:is>
-          <ns0:t>26/10/2026 – 01/11/2026</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B3" s="2" t="n"/>
-      <ns0:c r="C3" s="2" t="n"/>
-      <ns0:c r="D3" s="2" t="n"/>
-      <ns0:c r="E3" s="2" t="n"/>
-      <ns0:c r="F3" s="2" t="n"/>
-    </ns0:row>
-    <ns0:row r="4" ht="15" customHeight="1" s="24">
-      <ns0:c r="A4" s="2" t="n"/>
-      <ns0:c r="B4" s="2" t="n"/>
-      <ns0:c r="C4" s="2" t="n"/>
-      <ns0:c r="D4" s="2" t="n"/>
-      <ns0:c r="E4" s="2" t="n"/>
-      <ns0:c r="F4" s="2" t="n"/>
-    </ns0:row>
-    <ns0:row r="5" ht="33.75" customHeight="1" s="24">
-      <ns0:c r="A5" s="4" t="inlineStr">
-        <ns0:is>
-          <ns0:t>TỔNG SỐ PROMPT</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B5" s="5">
-        <ns0:f>SUM(B9:B11)</ns0:f>
-        <ns0:v>14</ns0:v>
-      </ns0:c>
-      <ns0:c r="C5" s="2" t="n"/>
-      <ns0:c r="D5" s="2" t="n"/>
-      <ns0:c r="E5" s="2" t="n"/>
-      <ns0:c r="F5" s="2" t="n"/>
-    </ns0:row>
-    <ns0:row r="6" ht="15" customHeight="1" s="24">
-      <ns0:c r="A6" s="2" t="n"/>
-      <ns0:c r="B6" s="2" t="n"/>
-      <ns0:c r="C6" s="2" t="n"/>
-      <ns0:c r="D6" s="2" t="n"/>
-      <ns0:c r="E6" s="2" t="n"/>
-      <ns0:c r="F6" s="2" t="n"/>
-    </ns0:row>
-    <ns0:row r="7" ht="15" customHeight="1" s="24">
-      <ns0:c r="A7" s="2" t="n"/>
-      <ns0:c r="B7" s="2" t="n"/>
-      <ns0:c r="C7" s="2" t="n"/>
-      <ns0:c r="D7" s="2" t="n"/>
-      <ns0:c r="E7" s="2" t="n"/>
-      <ns0:c r="F7" s="2" t="n"/>
-    </ns0:row>
-    <ns0:row r="8" ht="27.75" customHeight="1" s="24">
-      <ns0:c r="A8" s="4" t="inlineStr">
-        <ns0:is>
-          <ns0:t>NGƯỜI TẠO</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B8" s="4" t="inlineStr">
-        <ns0:is>
-          <ns0:t>SỐ PROMPT</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C8" s="2" t="n"/>
-      <ns0:c r="D8" s="10" t="inlineStr">
-        <ns0:is>
-          <ns0:t>TOOL AI</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="E8" s="10" t="inlineStr">
-        <ns0:is>
-          <ns0:t>SỐ PROMPT</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="F8" s="2" t="n"/>
-    </ns0:row>
-    <ns0:row r="9" ht="24.75" customHeight="1" s="24">
-      <ns0:c r="A9" s="11" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Thắng</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B9" s="13">
-        <ns0:f>COUNTIF(Thắng!$A$6:$A$306,"&lt;&gt;")</ns0:f>
-        <ns0:v>11</ns0:v>
-      </ns0:c>
-      <ns0:c r="C9" s="2" t="n"/>
-      <ns0:c r="D9" s="14" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Claude</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="E9" s="16">
-        <ns0:f>COUNTIFS(Thắng!$A$6:$A$306,"&lt;&gt;",Thắng!$C$6:$C$306,D9)+COUNTIFS(Sang!$A$6:$A$306,"&lt;&gt;",Sang!$C$6:$C$306,D9)+COUNTIFS(Nguyên!$A$6:$A$306,"&lt;&gt;",Nguyên!$C$6:$C$306,D9)</ns0:f>
-        <ns0:v>0</ns0:v>
-      </ns0:c>
-      <ns0:c r="F9" s="2" t="n"/>
-    </ns0:row>
-    <ns0:row r="10" ht="24.75" customHeight="1" s="24">
-      <ns0:c r="A10" s="11" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Sang</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B10" s="13">
-        <ns0:f>COUNTIF(Sang!$A$6:$A$306,"&lt;&gt;")</ns0:f>
-        <ns0:v>0</ns0:v>
-      </ns0:c>
-      <ns0:c r="C10" s="2" t="n"/>
-      <ns0:c r="D10" s="14" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Codex</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="E10" s="16">
-        <ns0:f>COUNTIFS(Thắng!$A$6:$A$306,"&lt;&gt;",Thắng!$C$6:$C$306,D10)+COUNTIFS(Sang!$A$6:$A$306,"&lt;&gt;",Sang!$C$6:$C$306,D10)+COUNTIFS(Nguyên!$A$6:$A$306,"&lt;&gt;",Nguyên!$C$6:$C$306,D10)</ns0:f>
-        <ns0:v>3</ns0:v>
-      </ns0:c>
-      <ns0:c r="F10" s="2" t="n"/>
-    </ns0:row>
-    <ns0:row r="11" ht="24.75" customHeight="1" s="24">
-      <ns0:c r="A11" s="11" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Nguyên</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B11" s="13">
-        <ns0:f>COUNTIF(Nguyên!$A$6:$A$306,"&lt;&gt;")</ns0:f>
-        <ns0:v>3</ns0:v>
-      </ns0:c>
-      <ns0:c r="C11" s="2" t="n"/>
-      <ns0:c r="D11" s="14" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Antigravity</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="E11" s="16">
-        <ns0:f>COUNTIFS(Thắng!$A$6:$A$306,"&lt;&gt;",Thắng!$C$6:$C$306,D11)+COUNTIFS(Sang!$A$6:$A$306,"&lt;&gt;",Sang!$C$6:$C$306,D11)+COUNTIFS(Nguyên!$A$6:$A$306,"&lt;&gt;",Nguyên!$C$6:$C$306,D11)</ns0:f>
-        <ns0:v>11</ns0:v>
-      </ns0:c>
-      <ns0:c r="F11" s="2" t="n"/>
-    </ns0:row>
-    <ns0:row r="12" ht="15" customHeight="1" s="24">
-      <ns0:c r="A12" s="2" t="n"/>
-      <ns0:c r="B12" s="2" t="n"/>
-      <ns0:c r="C12" s="2" t="n"/>
-      <ns0:c r="D12" s="2" t="n"/>
-      <ns0:c r="E12" s="2" t="n"/>
-      <ns0:c r="F12" s="2" t="n"/>
-    </ns0:row>
-    <ns0:row r="13" ht="15" customHeight="1" s="24">
-      <ns0:c r="A13" s="2" t="n"/>
-      <ns0:c r="B13" s="2" t="n"/>
-      <ns0:c r="C13" s="2" t="n"/>
-      <ns0:c r="D13" s="2" t="n"/>
-      <ns0:c r="E13" s="2" t="n"/>
-      <ns0:c r="F13" s="2" t="n"/>
-    </ns0:row>
-    <ns0:row r="14" ht="15" customHeight="1" s="24">
-      <ns0:c r="A14" s="17" t="n"/>
-      <ns0:c r="B14" s="2" t="n"/>
-      <ns0:c r="C14" s="2" t="n"/>
-      <ns0:c r="D14" s="2" t="n"/>
-      <ns0:c r="E14" s="2" t="n"/>
-      <ns0:c r="F14" s="2" t="n"/>
-    </ns0:row>
-    <ns0:row r="18" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="19" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="20" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="21" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="22" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="23" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="24" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="25" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="26" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="27" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="28" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="29" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="30" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="31" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="32" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="33" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="34" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="35" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="36" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="37" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="38" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="39" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="40" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="41" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="42" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="43" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="44" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="45" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="46" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="47" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="48" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="49" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="50" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="51" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="52" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="53" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="54" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="55" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="56" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="57" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="58" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="59" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="60" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="61" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="62" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="63" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="64" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="65" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="66" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="67" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="68" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="69" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="70" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="71" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="72" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="73" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="74" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="75" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="76" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="77" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="78" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="79" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="80" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="81" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="82" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="83" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="84" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="85" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="86" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="87" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="88" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="89" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="90" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="91" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="92" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="93" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="94" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="95" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="96" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="97" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="98" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="99" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="100" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="101" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="102" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="103" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="104" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="105" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="106" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="107" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="108" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="109" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="110" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="111" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="112" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="113" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="114" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="115" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="116" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="117" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="118" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="119" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="120" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="121" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="122" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="123" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="124" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="125" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="126" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="127" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="128" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="129" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="130" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="131" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="132" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="133" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="134" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="135" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="136" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="137" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="138" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="139" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="140" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="141" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="142" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="143" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="144" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="145" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="146" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="147" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="148" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="149" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="150" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="151" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="152" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="153" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="154" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="155" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="156" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="157" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="158" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="159" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="160" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="161" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="162" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="163" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="164" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="165" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="166" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="167" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="168" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="169" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="170" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="171" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="172" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="173" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="174" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="175" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="176" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="177" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="178" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="179" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="180" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="181" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="182" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="183" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="184" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="185" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="186" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="187" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="188" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="189" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="190" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="191" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="192" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="193" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="194" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="195" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="196" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="197" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="198" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="199" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="200" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="201" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="202" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="203" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="204" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="205" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="206" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="207" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="208" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="209" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="210" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="211" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="212" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="213" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="214" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="215" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="216" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="217" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="218" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="219" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="220" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="221" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="222" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="223" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="224" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="225" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="226" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="227" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="228" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="229" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="230" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="231" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="232" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="233" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="234" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="235" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="236" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="237" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="238" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="239" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="240" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="241" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="242" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="243" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="244" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="245" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="246" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="247" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="248" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="249" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="250" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="251" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="252" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="253" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="254" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="255" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="256" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="257" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="258" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="259" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="260" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="261" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="262" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="263" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="264" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="265" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="266" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="267" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="268" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="269" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="270" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="271" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="272" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="273" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="274" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="275" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="276" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="277" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="278" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="279" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="280" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="281" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="282" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="283" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="284" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="285" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="286" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="287" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="288" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="289" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="290" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="291" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="292" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="293" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="294" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="295" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="296" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="297" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="298" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="299" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="300" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="301" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="302" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="303" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="304" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="305" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="306" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="307" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="308" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="309" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="310" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="311" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="312" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="313" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="314" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="315" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="316" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="317" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="318" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="319" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="320" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="321" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="322" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="323" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="324" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="325" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="326" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="327" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="328" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="329" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="330" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="331" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="332" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="333" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="334" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="335" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="336" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="337" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="338" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="339" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="340" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="341" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="342" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="343" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="344" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="345" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="346" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="347" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="348" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="349" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="350" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="351" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="352" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="353" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="354" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="355" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="356" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="357" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="358" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="359" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="360" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="361" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="362" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="363" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="364" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="365" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="366" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="367" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="368" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="369" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="370" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="371" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="372" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="373" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="374" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="375" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="376" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="377" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="378" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="379" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="380" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="381" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="382" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="383" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="384" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="385" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="386" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="387" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="388" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="389" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="390" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="391" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="392" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="393" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="394" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="395" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="396" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="397" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="398" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="399" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="400" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="401" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="402" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="403" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="404" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="405" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="406" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="407" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="408" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="409" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="410" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="411" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="412" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="413" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="414" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="415" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="416" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="417" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="418" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="419" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="420" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="421" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="422" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="423" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="424" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="425" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="426" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="427" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="428" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="429" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="430" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="431" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="432" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="433" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="434" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="435" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="436" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="437" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="438" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="439" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="440" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="441" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="442" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="443" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="444" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="445" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="446" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="447" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="448" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="449" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="450" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="451" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="452" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="453" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="454" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="455" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="456" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="457" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="458" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="459" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="460" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="461" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="462" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="463" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="464" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="465" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="466" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="467" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="468" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="469" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="470" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="471" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="472" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="473" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="474" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="475" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="476" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="477" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="478" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="479" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="480" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="481" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="482" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="483" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="484" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="485" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="486" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="487" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="488" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="489" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="490" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="491" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="492" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="493" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="494" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="495" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="496" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="497" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="498" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="499" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="500" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="501" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="502" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="503" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="504" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="505" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="506" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="507" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="508" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="509" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="510" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="511" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="512" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="513" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="514" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="515" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="516" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="517" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="518" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="519" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="520" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="521" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="522" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="523" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="524" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="525" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="526" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="527" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="528" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="529" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="530" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="531" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="532" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="533" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="534" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="535" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="536" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="537" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="538" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="539" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="540" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="541" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="542" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="543" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="544" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="545" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="546" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="547" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="548" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="549" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="550" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="551" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="552" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="553" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="554" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="555" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="556" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="557" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="558" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="559" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="560" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="561" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="562" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="563" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="564" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="565" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="566" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="567" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="568" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="569" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="570" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="571" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="572" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="573" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="574" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="575" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="576" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="577" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="578" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="579" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="580" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="581" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="582" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="583" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="584" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="585" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="586" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="587" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="588" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="589" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="590" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="591" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="592" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="593" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="594" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="595" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="596" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="597" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="598" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="599" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="600" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="601" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="602" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="603" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="604" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="605" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="606" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="607" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="608" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="609" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="610" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="611" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="612" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="613" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="614" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="615" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="616" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="617" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="618" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="619" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="620" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="621" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="622" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="623" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="624" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="625" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="626" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="627" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="628" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="629" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="630" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="631" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="632" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="633" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="634" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="635" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="636" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="637" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="638" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="639" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="640" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="641" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="642" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="643" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="644" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="645" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="646" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="647" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="648" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="649" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="650" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="651" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="652" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="653" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="654" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="655" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="656" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="657" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="658" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="659" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="660" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="661" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="662" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="663" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="664" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="665" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="666" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="667" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="668" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="669" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="670" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="671" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="672" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="673" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="674" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="675" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="676" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="677" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="678" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="679" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="680" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="681" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="682" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="683" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="684" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="685" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="686" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="687" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="688" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="689" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="690" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="691" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="692" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="693" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="694" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="695" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="696" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="697" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="698" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="699" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="700" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="701" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="702" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="703" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="704" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="705" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="706" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="707" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="708" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="709" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="710" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="711" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="712" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="713" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="714" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="715" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="716" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="717" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="718" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="719" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="720" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="721" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="722" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="723" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="724" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="725" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="726" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="727" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="728" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="729" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="730" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="731" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="732" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="733" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="734" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="735" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="736" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="737" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="738" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="739" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="740" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="741" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="742" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="743" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="744" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="745" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="746" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="747" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="748" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="749" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="750" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="751" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="752" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="753" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="754" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="755" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="756" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="757" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="758" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="759" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="760" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="761" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="762" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="763" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="764" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="765" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="766" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="767" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="768" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="769" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="770" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="771" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="772" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="773" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="774" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="775" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="776" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="777" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="778" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="779" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="780" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="781" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="782" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="783" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="784" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="785" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="786" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="787" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="788" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="789" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="790" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="791" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="792" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="793" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="794" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="795" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="796" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="797" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="798" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="799" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="800" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="801" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="802" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="803" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="804" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="805" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="806" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="807" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="808" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="809" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="810" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="811" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="812" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="813" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="814" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="815" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="816" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="817" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="818" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="819" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="820" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="821" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="822" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="823" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="824" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="825" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="826" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="827" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="828" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="829" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="830" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="831" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="832" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="833" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="834" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="835" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="836" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="837" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="838" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="839" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="840" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="841" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="842" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="843" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="844" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="845" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="846" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="847" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="848" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="849" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="850" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="851" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="852" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="853" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="854" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="855" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="856" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="857" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="858" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="859" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="860" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="861" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="862" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="863" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="864" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="865" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="866" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="867" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="868" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="869" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="870" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="871" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="872" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="873" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="874" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="875" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="876" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="877" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="878" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="879" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="880" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="881" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="882" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="883" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="884" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="885" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="886" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="887" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="888" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="889" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="890" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="891" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="892" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="893" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="894" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="895" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="896" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="897" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="898" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="899" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="900" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="901" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="902" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="903" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="904" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="905" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="906" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="907" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="908" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="909" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="910" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="911" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="912" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="913" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="914" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="915" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="916" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="917" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="918" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="919" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="920" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="921" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="922" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="923" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="924" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="925" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="926" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="927" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="928" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="929" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="930" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="931" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="932" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="933" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="934" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="935" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="936" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="937" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="938" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="939" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="940" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="941" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="942" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="943" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="944" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="945" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="946" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="947" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="948" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="949" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="950" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="951" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="952" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="953" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="954" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="955" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="956" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="957" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="958" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="959" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="960" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="961" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="962" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="963" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="964" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="965" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="966" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="967" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="968" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="969" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="970" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="971" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="972" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="973" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="974" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="975" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="976" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="977" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="978" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="979" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="980" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="981" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="982" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="983" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="984" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="985" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="986" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="987" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="988" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="989" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="990" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="991" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="992" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="993" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="994" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="995" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="996" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="997" ht="15.75" customHeight="1" s="24"/>
-  </ns0:sheetData>
-  <ns0:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</ns0:worksheet>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="FF17324D"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A2:F14"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.625" defaultRowHeight="14.25"/>
+  <cols>
+    <col width="24" customWidth="1" style="24" min="1" max="1"/>
+    <col width="15" customWidth="1" style="24" min="2" max="2"/>
+    <col width="4" customWidth="1" style="24" min="3" max="3"/>
+    <col width="24" customWidth="1" style="24" min="4" max="4"/>
+    <col width="15" customWidth="1" style="24" min="5" max="5"/>
+    <col width="8" customWidth="1" style="24" min="6" max="6"/>
+    <col width="8.625" customWidth="1" style="24" min="7" max="26"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="15" customHeight="1" s="24"/>
+    <row r="2" ht="25.5" customHeight="1" s="24">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>TỔNG HỢP SỬ DỤNG AI — TUẦN 07</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+    </row>
+    <row r="3" ht="19.5" customHeight="1" s="24">
+      <c r="A3" s="30" t="inlineStr">
+        <is>
+          <t>26/10/2026 – 01/11/2026</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n"/>
+      <c r="C3" s="2" t="n"/>
+      <c r="D3" s="2" t="n"/>
+      <c r="E3" s="2" t="n"/>
+      <c r="F3" s="2" t="n"/>
+    </row>
+    <row r="4" ht="15" customHeight="1" s="24">
+      <c r="A4" s="2" t="n"/>
+      <c r="B4" s="2" t="n"/>
+      <c r="C4" s="2" t="n"/>
+      <c r="D4" s="2" t="n"/>
+      <c r="E4" s="2" t="n"/>
+      <c r="F4" s="2" t="n"/>
+    </row>
+    <row r="5" ht="33.75" customHeight="1" s="24">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>TỔNG SỐ PROMPT</t>
+        </is>
+      </c>
+      <c r="B5" s="5">
+        <f>SUM(B9:B11)</f>
+        <v/>
+      </c>
+      <c r="C5" s="2" t="n"/>
+      <c r="D5" s="2" t="n"/>
+      <c r="E5" s="2" t="n"/>
+      <c r="F5" s="2" t="n"/>
+    </row>
+    <row r="6" ht="15" customHeight="1" s="24">
+      <c r="A6" s="2" t="n"/>
+      <c r="B6" s="2" t="n"/>
+      <c r="C6" s="2" t="n"/>
+      <c r="D6" s="2" t="n"/>
+      <c r="E6" s="2" t="n"/>
+      <c r="F6" s="2" t="n"/>
+    </row>
+    <row r="7" ht="15" customHeight="1" s="24">
+      <c r="A7" s="2" t="n"/>
+      <c r="B7" s="2" t="n"/>
+      <c r="C7" s="2" t="n"/>
+      <c r="D7" s="2" t="n"/>
+      <c r="E7" s="2" t="n"/>
+      <c r="F7" s="2" t="n"/>
+    </row>
+    <row r="8" ht="27.75" customHeight="1" s="24">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>NGƯỜI TẠO</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>SỐ PROMPT</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="n"/>
+      <c r="D8" s="10" t="inlineStr">
+        <is>
+          <t>TOOL AI</t>
+        </is>
+      </c>
+      <c r="E8" s="10" t="inlineStr">
+        <is>
+          <t>SỐ PROMPT</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="n"/>
+    </row>
+    <row r="9" ht="24.75" customHeight="1" s="24">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>Thắng</t>
+        </is>
+      </c>
+      <c r="B9" s="13">
+        <f>COUNTIF(Thắng!$A$6:$A$306,"&lt;&gt;")</f>
+        <v/>
+      </c>
+      <c r="C9" s="2" t="n"/>
+      <c r="D9" s="14" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="E9" s="16">
+        <f>COUNTIFS(Thắng!$A$6:$A$306,"&lt;&gt;",Thắng!$C$6:$C$306,D9)+COUNTIFS(Sang!$A$6:$A$306,"&lt;&gt;",Sang!$C$6:$C$306,D9)+COUNTIFS(Nguyên!$A$6:$A$306,"&lt;&gt;",Nguyên!$C$6:$C$306,D9)</f>
+        <v/>
+      </c>
+      <c r="F9" s="2" t="n"/>
+    </row>
+    <row r="10" ht="24.75" customHeight="1" s="24">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>Sang</t>
+        </is>
+      </c>
+      <c r="B10" s="13">
+        <f>COUNTIF(Sang!$A$6:$A$306,"&lt;&gt;")</f>
+        <v/>
+      </c>
+      <c r="C10" s="2" t="n"/>
+      <c r="D10" s="14" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="E10" s="16">
+        <f>COUNTIFS(Thắng!$A$6:$A$306,"&lt;&gt;",Thắng!$C$6:$C$306,D10)+COUNTIFS(Sang!$A$6:$A$306,"&lt;&gt;",Sang!$C$6:$C$306,D10)+COUNTIFS(Nguyên!$A$6:$A$306,"&lt;&gt;",Nguyên!$C$6:$C$306,D10)</f>
+        <v/>
+      </c>
+      <c r="F10" s="2" t="n"/>
+    </row>
+    <row r="11" ht="24.75" customHeight="1" s="24">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>Nguyên</t>
+        </is>
+      </c>
+      <c r="B11" s="13">
+        <f>COUNTIF(Nguyên!$A$6:$A$306,"&lt;&gt;")</f>
+        <v/>
+      </c>
+      <c r="C11" s="2" t="n"/>
+      <c r="D11" s="14" t="inlineStr">
+        <is>
+          <t>Antigravity</t>
+        </is>
+      </c>
+      <c r="E11" s="16">
+        <f>COUNTIFS(Thắng!$A$6:$A$306,"&lt;&gt;",Thắng!$C$6:$C$306,D11)+COUNTIFS(Sang!$A$6:$A$306,"&lt;&gt;",Sang!$C$6:$C$306,D11)+COUNTIFS(Nguyên!$A$6:$A$306,"&lt;&gt;",Nguyên!$C$6:$C$306,D11)</f>
+        <v/>
+      </c>
+      <c r="F11" s="2" t="n"/>
+    </row>
+    <row r="12" ht="15" customHeight="1" s="24">
+      <c r="A12" s="2" t="n"/>
+      <c r="B12" s="2" t="n"/>
+      <c r="C12" s="2" t="n"/>
+      <c r="D12" s="2" t="n"/>
+      <c r="E12" s="2" t="n"/>
+      <c r="F12" s="2" t="n"/>
+    </row>
+    <row r="13" ht="15" customHeight="1" s="24">
+      <c r="A13" s="2" t="n"/>
+      <c r="B13" s="2" t="n"/>
+      <c r="C13" s="2" t="n"/>
+      <c r="D13" s="2" t="n"/>
+      <c r="E13" s="2" t="n"/>
+      <c r="F13" s="2" t="n"/>
+    </row>
+    <row r="14" ht="15" customHeight="1" s="24">
+      <c r="A14" s="17" t="n"/>
+      <c r="B14" s="2" t="n"/>
+      <c r="C14" s="2" t="n"/>
+      <c r="D14" s="2" t="n"/>
+      <c r="E14" s="2" t="n"/>
+      <c r="F14" s="2" t="n"/>
+    </row>
+    <row r="18" ht="15.75" customHeight="1" s="24"/>
+    <row r="19" ht="15.75" customHeight="1" s="24"/>
+    <row r="20" ht="15.75" customHeight="1" s="24"/>
+    <row r="21" ht="15.75" customHeight="1" s="24"/>
+    <row r="22" ht="15.75" customHeight="1" s="24"/>
+    <row r="23" ht="15.75" customHeight="1" s="24"/>
+    <row r="24" ht="15.75" customHeight="1" s="24"/>
+    <row r="25" ht="15.75" customHeight="1" s="24"/>
+    <row r="26" ht="15.75" customHeight="1" s="24"/>
+    <row r="27" ht="15.75" customHeight="1" s="24"/>
+    <row r="28" ht="15.75" customHeight="1" s="24"/>
+    <row r="29" ht="15.75" customHeight="1" s="24"/>
+    <row r="30" ht="15.75" customHeight="1" s="24"/>
+    <row r="31" ht="15.75" customHeight="1" s="24"/>
+    <row r="32" ht="15.75" customHeight="1" s="24"/>
+    <row r="33" ht="15.75" customHeight="1" s="24"/>
+    <row r="34" ht="15.75" customHeight="1" s="24"/>
+    <row r="35" ht="15.75" customHeight="1" s="24"/>
+    <row r="36" ht="15.75" customHeight="1" s="24"/>
+    <row r="37" ht="15.75" customHeight="1" s="24"/>
+    <row r="38" ht="15.75" customHeight="1" s="24"/>
+    <row r="39" ht="15.75" customHeight="1" s="24"/>
+    <row r="40" ht="15.75" customHeight="1" s="24"/>
+    <row r="41" ht="15.75" customHeight="1" s="24"/>
+    <row r="42" ht="15.75" customHeight="1" s="24"/>
+    <row r="43" ht="15.75" customHeight="1" s="24"/>
+    <row r="44" ht="15.75" customHeight="1" s="24"/>
+    <row r="45" ht="15.75" customHeight="1" s="24"/>
+    <row r="46" ht="15.75" customHeight="1" s="24"/>
+    <row r="47" ht="15.75" customHeight="1" s="24"/>
+    <row r="48" ht="15.75" customHeight="1" s="24"/>
+    <row r="49" ht="15.75" customHeight="1" s="24"/>
+    <row r="50" ht="15.75" customHeight="1" s="24"/>
+    <row r="51" ht="15.75" customHeight="1" s="24"/>
+    <row r="52" ht="15.75" customHeight="1" s="24"/>
+    <row r="53" ht="15.75" customHeight="1" s="24"/>
+    <row r="54" ht="15.75" customHeight="1" s="24"/>
+    <row r="55" ht="15.75" customHeight="1" s="24"/>
+    <row r="56" ht="15.75" customHeight="1" s="24"/>
+    <row r="57" ht="15.75" customHeight="1" s="24"/>
+    <row r="58" ht="15.75" customHeight="1" s="24"/>
+    <row r="59" ht="15.75" customHeight="1" s="24"/>
+    <row r="60" ht="15.75" customHeight="1" s="24"/>
+    <row r="61" ht="15.75" customHeight="1" s="24"/>
+    <row r="62" ht="15.75" customHeight="1" s="24"/>
+    <row r="63" ht="15.75" customHeight="1" s="24"/>
+    <row r="64" ht="15.75" customHeight="1" s="24"/>
+    <row r="65" ht="15.75" customHeight="1" s="24"/>
+    <row r="66" ht="15.75" customHeight="1" s="24"/>
+    <row r="67" ht="15.75" customHeight="1" s="24"/>
+    <row r="68" ht="15.75" customHeight="1" s="24"/>
+    <row r="69" ht="15.75" customHeight="1" s="24"/>
+    <row r="70" ht="15.75" customHeight="1" s="24"/>
+    <row r="71" ht="15.75" customHeight="1" s="24"/>
+    <row r="72" ht="15.75" customHeight="1" s="24"/>
+    <row r="73" ht="15.75" customHeight="1" s="24"/>
+    <row r="74" ht="15.75" customHeight="1" s="24"/>
+    <row r="75" ht="15.75" customHeight="1" s="24"/>
+    <row r="76" ht="15.75" customHeight="1" s="24"/>
+    <row r="77" ht="15.75" customHeight="1" s="24"/>
+    <row r="78" ht="15.75" customHeight="1" s="24"/>
+    <row r="79" ht="15.75" customHeight="1" s="24"/>
+    <row r="80" ht="15.75" customHeight="1" s="24"/>
+    <row r="81" ht="15.75" customHeight="1" s="24"/>
+    <row r="82" ht="15.75" customHeight="1" s="24"/>
+    <row r="83" ht="15.75" customHeight="1" s="24"/>
+    <row r="84" ht="15.75" customHeight="1" s="24"/>
+    <row r="85" ht="15.75" customHeight="1" s="24"/>
+    <row r="86" ht="15.75" customHeight="1" s="24"/>
+    <row r="87" ht="15.75" customHeight="1" s="24"/>
+    <row r="88" ht="15.75" customHeight="1" s="24"/>
+    <row r="89" ht="15.75" customHeight="1" s="24"/>
+    <row r="90" ht="15.75" customHeight="1" s="24"/>
+    <row r="91" ht="15.75" customHeight="1" s="24"/>
+    <row r="92" ht="15.75" customHeight="1" s="24"/>
+    <row r="93" ht="15.75" customHeight="1" s="24"/>
+    <row r="94" ht="15.75" customHeight="1" s="24"/>
+    <row r="95" ht="15.75" customHeight="1" s="24"/>
+    <row r="96" ht="15.75" customHeight="1" s="24"/>
+    <row r="97" ht="15.75" customHeight="1" s="24"/>
+    <row r="98" ht="15.75" customHeight="1" s="24"/>
+    <row r="99" ht="15.75" customHeight="1" s="24"/>
+    <row r="100" ht="15.75" customHeight="1" s="24"/>
+    <row r="101" ht="15.75" customHeight="1" s="24"/>
+    <row r="102" ht="15.75" customHeight="1" s="24"/>
+    <row r="103" ht="15.75" customHeight="1" s="24"/>
+    <row r="104" ht="15.75" customHeight="1" s="24"/>
+    <row r="105" ht="15.75" customHeight="1" s="24"/>
+    <row r="106" ht="15.75" customHeight="1" s="24"/>
+    <row r="107" ht="15.75" customHeight="1" s="24"/>
+    <row r="108" ht="15.75" customHeight="1" s="24"/>
+    <row r="109" ht="15.75" customHeight="1" s="24"/>
+    <row r="110" ht="15.75" customHeight="1" s="24"/>
+    <row r="111" ht="15.75" customHeight="1" s="24"/>
+    <row r="112" ht="15.75" customHeight="1" s="24"/>
+    <row r="113" ht="15.75" customHeight="1" s="24"/>
+    <row r="114" ht="15.75" customHeight="1" s="24"/>
+    <row r="115" ht="15.75" customHeight="1" s="24"/>
+    <row r="116" ht="15.75" customHeight="1" s="24"/>
+    <row r="117" ht="15.75" customHeight="1" s="24"/>
+    <row r="118" ht="15.75" customHeight="1" s="24"/>
+    <row r="119" ht="15.75" customHeight="1" s="24"/>
+    <row r="120" ht="15.75" customHeight="1" s="24"/>
+    <row r="121" ht="15.75" customHeight="1" s="24"/>
+    <row r="122" ht="15.75" customHeight="1" s="24"/>
+    <row r="123" ht="15.75" customHeight="1" s="24"/>
+    <row r="124" ht="15.75" customHeight="1" s="24"/>
+    <row r="125" ht="15.75" customHeight="1" s="24"/>
+    <row r="126" ht="15.75" customHeight="1" s="24"/>
+    <row r="127" ht="15.75" customHeight="1" s="24"/>
+    <row r="128" ht="15.75" customHeight="1" s="24"/>
+    <row r="129" ht="15.75" customHeight="1" s="24"/>
+    <row r="130" ht="15.75" customHeight="1" s="24"/>
+    <row r="131" ht="15.75" customHeight="1" s="24"/>
+    <row r="132" ht="15.75" customHeight="1" s="24"/>
+    <row r="133" ht="15.75" customHeight="1" s="24"/>
+    <row r="134" ht="15.75" customHeight="1" s="24"/>
+    <row r="135" ht="15.75" customHeight="1" s="24"/>
+    <row r="136" ht="15.75" customHeight="1" s="24"/>
+    <row r="137" ht="15.75" customHeight="1" s="24"/>
+    <row r="138" ht="15.75" customHeight="1" s="24"/>
+    <row r="139" ht="15.75" customHeight="1" s="24"/>
+    <row r="140" ht="15.75" customHeight="1" s="24"/>
+    <row r="141" ht="15.75" customHeight="1" s="24"/>
+    <row r="142" ht="15.75" customHeight="1" s="24"/>
+    <row r="143" ht="15.75" customHeight="1" s="24"/>
+    <row r="144" ht="15.75" customHeight="1" s="24"/>
+    <row r="145" ht="15.75" customHeight="1" s="24"/>
+    <row r="146" ht="15.75" customHeight="1" s="24"/>
+    <row r="147" ht="15.75" customHeight="1" s="24"/>
+    <row r="148" ht="15.75" customHeight="1" s="24"/>
+    <row r="149" ht="15.75" customHeight="1" s="24"/>
+    <row r="150" ht="15.75" customHeight="1" s="24"/>
+    <row r="151" ht="15.75" customHeight="1" s="24"/>
+    <row r="152" ht="15.75" customHeight="1" s="24"/>
+    <row r="153" ht="15.75" customHeight="1" s="24"/>
+    <row r="154" ht="15.75" customHeight="1" s="24"/>
+    <row r="155" ht="15.75" customHeight="1" s="24"/>
+    <row r="156" ht="15.75" customHeight="1" s="24"/>
+    <row r="157" ht="15.75" customHeight="1" s="24"/>
+    <row r="158" ht="15.75" customHeight="1" s="24"/>
+    <row r="159" ht="15.75" customHeight="1" s="24"/>
+    <row r="160" ht="15.75" customHeight="1" s="24"/>
+    <row r="161" ht="15.75" customHeight="1" s="24"/>
+    <row r="162" ht="15.75" customHeight="1" s="24"/>
+    <row r="163" ht="15.75" customHeight="1" s="24"/>
+    <row r="164" ht="15.75" customHeight="1" s="24"/>
+    <row r="165" ht="15.75" customHeight="1" s="24"/>
+    <row r="166" ht="15.75" customHeight="1" s="24"/>
+    <row r="167" ht="15.75" customHeight="1" s="24"/>
+    <row r="168" ht="15.75" customHeight="1" s="24"/>
+    <row r="169" ht="15.75" customHeight="1" s="24"/>
+    <row r="170" ht="15.75" customHeight="1" s="24"/>
+    <row r="171" ht="15.75" customHeight="1" s="24"/>
+    <row r="172" ht="15.75" customHeight="1" s="24"/>
+    <row r="173" ht="15.75" customHeight="1" s="24"/>
+    <row r="174" ht="15.75" customHeight="1" s="24"/>
+    <row r="175" ht="15.75" customHeight="1" s="24"/>
+    <row r="176" ht="15.75" customHeight="1" s="24"/>
+    <row r="177" ht="15.75" customHeight="1" s="24"/>
+    <row r="178" ht="15.75" customHeight="1" s="24"/>
+    <row r="179" ht="15.75" customHeight="1" s="24"/>
+    <row r="180" ht="15.75" customHeight="1" s="24"/>
+    <row r="181" ht="15.75" customHeight="1" s="24"/>
+    <row r="182" ht="15.75" customHeight="1" s="24"/>
+    <row r="183" ht="15.75" customHeight="1" s="24"/>
+    <row r="184" ht="15.75" customHeight="1" s="24"/>
+    <row r="185" ht="15.75" customHeight="1" s="24"/>
+    <row r="186" ht="15.75" customHeight="1" s="24"/>
+    <row r="187" ht="15.75" customHeight="1" s="24"/>
+    <row r="188" ht="15.75" customHeight="1" s="24"/>
+    <row r="189" ht="15.75" customHeight="1" s="24"/>
+    <row r="190" ht="15.75" customHeight="1" s="24"/>
+    <row r="191" ht="15.75" customHeight="1" s="24"/>
+    <row r="192" ht="15.75" customHeight="1" s="24"/>
+    <row r="193" ht="15.75" customHeight="1" s="24"/>
+    <row r="194" ht="15.75" customHeight="1" s="24"/>
+    <row r="195" ht="15.75" customHeight="1" s="24"/>
+    <row r="196" ht="15.75" customHeight="1" s="24"/>
+    <row r="197" ht="15.75" customHeight="1" s="24"/>
+    <row r="198" ht="15.75" customHeight="1" s="24"/>
+    <row r="199" ht="15.75" customHeight="1" s="24"/>
+    <row r="200" ht="15.75" customHeight="1" s="24"/>
+    <row r="201" ht="15.75" customHeight="1" s="24"/>
+    <row r="202" ht="15.75" customHeight="1" s="24"/>
+    <row r="203" ht="15.75" customHeight="1" s="24"/>
+    <row r="204" ht="15.75" customHeight="1" s="24"/>
+    <row r="205" ht="15.75" customHeight="1" s="24"/>
+    <row r="206" ht="15.75" customHeight="1" s="24"/>
+    <row r="207" ht="15.75" customHeight="1" s="24"/>
+    <row r="208" ht="15.75" customHeight="1" s="24"/>
+    <row r="209" ht="15.75" customHeight="1" s="24"/>
+    <row r="210" ht="15.75" customHeight="1" s="24"/>
+    <row r="211" ht="15.75" customHeight="1" s="24"/>
+    <row r="212" ht="15.75" customHeight="1" s="24"/>
+    <row r="213" ht="15.75" customHeight="1" s="24"/>
+    <row r="214" ht="15.75" customHeight="1" s="24"/>
+    <row r="215" ht="15.75" customHeight="1" s="24"/>
+    <row r="216" ht="15.75" customHeight="1" s="24"/>
+    <row r="217" ht="15.75" customHeight="1" s="24"/>
+    <row r="218" ht="15.75" customHeight="1" s="24"/>
+    <row r="219" ht="15.75" customHeight="1" s="24"/>
+    <row r="220" ht="15.75" customHeight="1" s="24"/>
+    <row r="221" ht="15.75" customHeight="1" s="24"/>
+    <row r="222" ht="15.75" customHeight="1" s="24"/>
+    <row r="223" ht="15.75" customHeight="1" s="24"/>
+    <row r="224" ht="15.75" customHeight="1" s="24"/>
+    <row r="225" ht="15.75" customHeight="1" s="24"/>
+    <row r="226" ht="15.75" customHeight="1" s="24"/>
+    <row r="227" ht="15.75" customHeight="1" s="24"/>
+    <row r="228" ht="15.75" customHeight="1" s="24"/>
+    <row r="229" ht="15.75" customHeight="1" s="24"/>
+    <row r="230" ht="15.75" customHeight="1" s="24"/>
+    <row r="231" ht="15.75" customHeight="1" s="24"/>
+    <row r="232" ht="15.75" customHeight="1" s="24"/>
+    <row r="233" ht="15.75" customHeight="1" s="24"/>
+    <row r="234" ht="15.75" customHeight="1" s="24"/>
+    <row r="235" ht="15.75" customHeight="1" s="24"/>
+    <row r="236" ht="15.75" customHeight="1" s="24"/>
+    <row r="237" ht="15.75" customHeight="1" s="24"/>
+    <row r="238" ht="15.75" customHeight="1" s="24"/>
+    <row r="239" ht="15.75" customHeight="1" s="24"/>
+    <row r="240" ht="15.75" customHeight="1" s="24"/>
+    <row r="241" ht="15.75" customHeight="1" s="24"/>
+    <row r="242" ht="15.75" customHeight="1" s="24"/>
+    <row r="243" ht="15.75" customHeight="1" s="24"/>
+    <row r="244" ht="15.75" customHeight="1" s="24"/>
+    <row r="245" ht="15.75" customHeight="1" s="24"/>
+    <row r="246" ht="15.75" customHeight="1" s="24"/>
+    <row r="247" ht="15.75" customHeight="1" s="24"/>
+    <row r="248" ht="15.75" customHeight="1" s="24"/>
+    <row r="249" ht="15.75" customHeight="1" s="24"/>
+    <row r="250" ht="15.75" customHeight="1" s="24"/>
+    <row r="251" ht="15.75" customHeight="1" s="24"/>
+    <row r="252" ht="15.75" customHeight="1" s="24"/>
+    <row r="253" ht="15.75" customHeight="1" s="24"/>
+    <row r="254" ht="15.75" customHeight="1" s="24"/>
+    <row r="255" ht="15.75" customHeight="1" s="24"/>
+    <row r="256" ht="15.75" customHeight="1" s="24"/>
+    <row r="257" ht="15.75" customHeight="1" s="24"/>
+    <row r="258" ht="15.75" customHeight="1" s="24"/>
+    <row r="259" ht="15.75" customHeight="1" s="24"/>
+    <row r="260" ht="15.75" customHeight="1" s="24"/>
+    <row r="261" ht="15.75" customHeight="1" s="24"/>
+    <row r="262" ht="15.75" customHeight="1" s="24"/>
+    <row r="263" ht="15.75" customHeight="1" s="24"/>
+    <row r="264" ht="15.75" customHeight="1" s="24"/>
+    <row r="265" ht="15.75" customHeight="1" s="24"/>
+    <row r="266" ht="15.75" customHeight="1" s="24"/>
+    <row r="267" ht="15.75" customHeight="1" s="24"/>
+    <row r="268" ht="15.75" customHeight="1" s="24"/>
+    <row r="269" ht="15.75" customHeight="1" s="24"/>
+    <row r="270" ht="15.75" customHeight="1" s="24"/>
+    <row r="271" ht="15.75" customHeight="1" s="24"/>
+    <row r="272" ht="15.75" customHeight="1" s="24"/>
+    <row r="273" ht="15.75" customHeight="1" s="24"/>
+    <row r="274" ht="15.75" customHeight="1" s="24"/>
+    <row r="275" ht="15.75" customHeight="1" s="24"/>
+    <row r="276" ht="15.75" customHeight="1" s="24"/>
+    <row r="277" ht="15.75" customHeight="1" s="24"/>
+    <row r="278" ht="15.75" customHeight="1" s="24"/>
+    <row r="279" ht="15.75" customHeight="1" s="24"/>
+    <row r="280" ht="15.75" customHeight="1" s="24"/>
+    <row r="281" ht="15.75" customHeight="1" s="24"/>
+    <row r="282" ht="15.75" customHeight="1" s="24"/>
+    <row r="283" ht="15.75" customHeight="1" s="24"/>
+    <row r="284" ht="15.75" customHeight="1" s="24"/>
+    <row r="285" ht="15.75" customHeight="1" s="24"/>
+    <row r="286" ht="15.75" customHeight="1" s="24"/>
+    <row r="287" ht="15.75" customHeight="1" s="24"/>
+    <row r="288" ht="15.75" customHeight="1" s="24"/>
+    <row r="289" ht="15.75" customHeight="1" s="24"/>
+    <row r="290" ht="15.75" customHeight="1" s="24"/>
+    <row r="291" ht="15.75" customHeight="1" s="24"/>
+    <row r="292" ht="15.75" customHeight="1" s="24"/>
+    <row r="293" ht="15.75" customHeight="1" s="24"/>
+    <row r="294" ht="15.75" customHeight="1" s="24"/>
+    <row r="295" ht="15.75" customHeight="1" s="24"/>
+    <row r="296" ht="15.75" customHeight="1" s="24"/>
+    <row r="297" ht="15.75" customHeight="1" s="24"/>
+    <row r="298" ht="15.75" customHeight="1" s="24"/>
+    <row r="299" ht="15.75" customHeight="1" s="24"/>
+    <row r="300" ht="15.75" customHeight="1" s="24"/>
+    <row r="301" ht="15.75" customHeight="1" s="24"/>
+    <row r="302" ht="15.75" customHeight="1" s="24"/>
+    <row r="303" ht="15.75" customHeight="1" s="24"/>
+    <row r="304" ht="15.75" customHeight="1" s="24"/>
+    <row r="305" ht="15.75" customHeight="1" s="24"/>
+    <row r="306" ht="15.75" customHeight="1" s="24"/>
+    <row r="307" ht="15.75" customHeight="1" s="24"/>
+    <row r="308" ht="15.75" customHeight="1" s="24"/>
+    <row r="309" ht="15.75" customHeight="1" s="24"/>
+    <row r="310" ht="15.75" customHeight="1" s="24"/>
+    <row r="311" ht="15.75" customHeight="1" s="24"/>
+    <row r="312" ht="15.75" customHeight="1" s="24"/>
+    <row r="313" ht="15.75" customHeight="1" s="24"/>
+    <row r="314" ht="15.75" customHeight="1" s="24"/>
+    <row r="315" ht="15.75" customHeight="1" s="24"/>
+    <row r="316" ht="15.75" customHeight="1" s="24"/>
+    <row r="317" ht="15.75" customHeight="1" s="24"/>
+    <row r="318" ht="15.75" customHeight="1" s="24"/>
+    <row r="319" ht="15.75" customHeight="1" s="24"/>
+    <row r="320" ht="15.75" customHeight="1" s="24"/>
+    <row r="321" ht="15.75" customHeight="1" s="24"/>
+    <row r="322" ht="15.75" customHeight="1" s="24"/>
+    <row r="323" ht="15.75" customHeight="1" s="24"/>
+    <row r="324" ht="15.75" customHeight="1" s="24"/>
+    <row r="325" ht="15.75" customHeight="1" s="24"/>
+    <row r="326" ht="15.75" customHeight="1" s="24"/>
+    <row r="327" ht="15.75" customHeight="1" s="24"/>
+    <row r="328" ht="15.75" customHeight="1" s="24"/>
+    <row r="329" ht="15.75" customHeight="1" s="24"/>
+    <row r="330" ht="15.75" customHeight="1" s="24"/>
+    <row r="331" ht="15.75" customHeight="1" s="24"/>
+    <row r="332" ht="15.75" customHeight="1" s="24"/>
+    <row r="333" ht="15.75" customHeight="1" s="24"/>
+    <row r="334" ht="15.75" customHeight="1" s="24"/>
+    <row r="335" ht="15.75" customHeight="1" s="24"/>
+    <row r="336" ht="15.75" customHeight="1" s="24"/>
+    <row r="337" ht="15.75" customHeight="1" s="24"/>
+    <row r="338" ht="15.75" customHeight="1" s="24"/>
+    <row r="339" ht="15.75" customHeight="1" s="24"/>
+    <row r="340" ht="15.75" customHeight="1" s="24"/>
+    <row r="341" ht="15.75" customHeight="1" s="24"/>
+    <row r="342" ht="15.75" customHeight="1" s="24"/>
+    <row r="343" ht="15.75" customHeight="1" s="24"/>
+    <row r="344" ht="15.75" customHeight="1" s="24"/>
+    <row r="345" ht="15.75" customHeight="1" s="24"/>
+    <row r="346" ht="15.75" customHeight="1" s="24"/>
+    <row r="347" ht="15.75" customHeight="1" s="24"/>
+    <row r="348" ht="15.75" customHeight="1" s="24"/>
+    <row r="349" ht="15.75" customHeight="1" s="24"/>
+    <row r="350" ht="15.75" customHeight="1" s="24"/>
+    <row r="351" ht="15.75" customHeight="1" s="24"/>
+    <row r="352" ht="15.75" customHeight="1" s="24"/>
+    <row r="353" ht="15.75" customHeight="1" s="24"/>
+    <row r="354" ht="15.75" customHeight="1" s="24"/>
+    <row r="355" ht="15.75" customHeight="1" s="24"/>
+    <row r="356" ht="15.75" customHeight="1" s="24"/>
+    <row r="357" ht="15.75" customHeight="1" s="24"/>
+    <row r="358" ht="15.75" customHeight="1" s="24"/>
+    <row r="359" ht="15.75" customHeight="1" s="24"/>
+    <row r="360" ht="15.75" customHeight="1" s="24"/>
+    <row r="361" ht="15.75" customHeight="1" s="24"/>
+    <row r="362" ht="15.75" customHeight="1" s="24"/>
+    <row r="363" ht="15.75" customHeight="1" s="24"/>
+    <row r="364" ht="15.75" customHeight="1" s="24"/>
+    <row r="365" ht="15.75" customHeight="1" s="24"/>
+    <row r="366" ht="15.75" customHeight="1" s="24"/>
+    <row r="367" ht="15.75" customHeight="1" s="24"/>
+    <row r="368" ht="15.75" customHeight="1" s="24"/>
+    <row r="369" ht="15.75" customHeight="1" s="24"/>
+    <row r="370" ht="15.75" customHeight="1" s="24"/>
+    <row r="371" ht="15.75" customHeight="1" s="24"/>
+    <row r="372" ht="15.75" customHeight="1" s="24"/>
+    <row r="373" ht="15.75" customHeight="1" s="24"/>
+    <row r="374" ht="15.75" customHeight="1" s="24"/>
+    <row r="375" ht="15.75" customHeight="1" s="24"/>
+    <row r="376" ht="15.75" customHeight="1" s="24"/>
+    <row r="377" ht="15.75" customHeight="1" s="24"/>
+    <row r="378" ht="15.75" customHeight="1" s="24"/>
+    <row r="379" ht="15.75" customHeight="1" s="24"/>
+    <row r="380" ht="15.75" customHeight="1" s="24"/>
+    <row r="381" ht="15.75" customHeight="1" s="24"/>
+    <row r="382" ht="15.75" customHeight="1" s="24"/>
+    <row r="383" ht="15.75" customHeight="1" s="24"/>
+    <row r="384" ht="15.75" customHeight="1" s="24"/>
+    <row r="385" ht="15.75" customHeight="1" s="24"/>
+    <row r="386" ht="15.75" customHeight="1" s="24"/>
+    <row r="387" ht="15.75" customHeight="1" s="24"/>
+    <row r="388" ht="15.75" customHeight="1" s="24"/>
+    <row r="389" ht="15.75" customHeight="1" s="24"/>
+    <row r="390" ht="15.75" customHeight="1" s="24"/>
+    <row r="391" ht="15.75" customHeight="1" s="24"/>
+    <row r="392" ht="15.75" customHeight="1" s="24"/>
+    <row r="393" ht="15.75" customHeight="1" s="24"/>
+    <row r="394" ht="15.75" customHeight="1" s="24"/>
+    <row r="395" ht="15.75" customHeight="1" s="24"/>
+    <row r="396" ht="15.75" customHeight="1" s="24"/>
+    <row r="397" ht="15.75" customHeight="1" s="24"/>
+    <row r="398" ht="15.75" customHeight="1" s="24"/>
+    <row r="399" ht="15.75" customHeight="1" s="24"/>
+    <row r="400" ht="15.75" customHeight="1" s="24"/>
+    <row r="401" ht="15.75" customHeight="1" s="24"/>
+    <row r="402" ht="15.75" customHeight="1" s="24"/>
+    <row r="403" ht="15.75" customHeight="1" s="24"/>
+    <row r="404" ht="15.75" customHeight="1" s="24"/>
+    <row r="405" ht="15.75" customHeight="1" s="24"/>
+    <row r="406" ht="15.75" customHeight="1" s="24"/>
+    <row r="407" ht="15.75" customHeight="1" s="24"/>
+    <row r="408" ht="15.75" customHeight="1" s="24"/>
+    <row r="409" ht="15.75" customHeight="1" s="24"/>
+    <row r="410" ht="15.75" customHeight="1" s="24"/>
+    <row r="411" ht="15.75" customHeight="1" s="24"/>
+    <row r="412" ht="15.75" customHeight="1" s="24"/>
+    <row r="413" ht="15.75" customHeight="1" s="24"/>
+    <row r="414" ht="15.75" customHeight="1" s="24"/>
+    <row r="415" ht="15.75" customHeight="1" s="24"/>
+    <row r="416" ht="15.75" customHeight="1" s="24"/>
+    <row r="417" ht="15.75" customHeight="1" s="24"/>
+    <row r="418" ht="15.75" customHeight="1" s="24"/>
+    <row r="419" ht="15.75" customHeight="1" s="24"/>
+    <row r="420" ht="15.75" customHeight="1" s="24"/>
+    <row r="421" ht="15.75" customHeight="1" s="24"/>
+    <row r="422" ht="15.75" customHeight="1" s="24"/>
+    <row r="423" ht="15.75" customHeight="1" s="24"/>
+    <row r="424" ht="15.75" customHeight="1" s="24"/>
+    <row r="425" ht="15.75" customHeight="1" s="24"/>
+    <row r="426" ht="15.75" customHeight="1" s="24"/>
+    <row r="427" ht="15.75" customHeight="1" s="24"/>
+    <row r="428" ht="15.75" customHeight="1" s="24"/>
+    <row r="429" ht="15.75" customHeight="1" s="24"/>
+    <row r="430" ht="15.75" customHeight="1" s="24"/>
+    <row r="431" ht="15.75" customHeight="1" s="24"/>
+    <row r="432" ht="15.75" customHeight="1" s="24"/>
+    <row r="433" ht="15.75" customHeight="1" s="24"/>
+    <row r="434" ht="15.75" customHeight="1" s="24"/>
+    <row r="435" ht="15.75" customHeight="1" s="24"/>
+    <row r="436" ht="15.75" customHeight="1" s="24"/>
+    <row r="437" ht="15.75" customHeight="1" s="24"/>
+    <row r="438" ht="15.75" customHeight="1" s="24"/>
+    <row r="439" ht="15.75" customHeight="1" s="24"/>
+    <row r="440" ht="15.75" customHeight="1" s="24"/>
+    <row r="441" ht="15.75" customHeight="1" s="24"/>
+    <row r="442" ht="15.75" customHeight="1" s="24"/>
+    <row r="443" ht="15.75" customHeight="1" s="24"/>
+    <row r="444" ht="15.75" customHeight="1" s="24"/>
+    <row r="445" ht="15.75" customHeight="1" s="24"/>
+    <row r="446" ht="15.75" customHeight="1" s="24"/>
+    <row r="447" ht="15.75" customHeight="1" s="24"/>
+    <row r="448" ht="15.75" customHeight="1" s="24"/>
+    <row r="449" ht="15.75" customHeight="1" s="24"/>
+    <row r="450" ht="15.75" customHeight="1" s="24"/>
+    <row r="451" ht="15.75" customHeight="1" s="24"/>
+    <row r="452" ht="15.75" customHeight="1" s="24"/>
+    <row r="453" ht="15.75" customHeight="1" s="24"/>
+    <row r="454" ht="15.75" customHeight="1" s="24"/>
+    <row r="455" ht="15.75" customHeight="1" s="24"/>
+    <row r="456" ht="15.75" customHeight="1" s="24"/>
+    <row r="457" ht="15.75" customHeight="1" s="24"/>
+    <row r="458" ht="15.75" customHeight="1" s="24"/>
+    <row r="459" ht="15.75" customHeight="1" s="24"/>
+    <row r="460" ht="15.75" customHeight="1" s="24"/>
+    <row r="461" ht="15.75" customHeight="1" s="24"/>
+    <row r="462" ht="15.75" customHeight="1" s="24"/>
+    <row r="463" ht="15.75" customHeight="1" s="24"/>
+    <row r="464" ht="15.75" customHeight="1" s="24"/>
+    <row r="465" ht="15.75" customHeight="1" s="24"/>
+    <row r="466" ht="15.75" customHeight="1" s="24"/>
+    <row r="467" ht="15.75" customHeight="1" s="24"/>
+    <row r="468" ht="15.75" customHeight="1" s="24"/>
+    <row r="469" ht="15.75" customHeight="1" s="24"/>
+    <row r="470" ht="15.75" customHeight="1" s="24"/>
+    <row r="471" ht="15.75" customHeight="1" s="24"/>
+    <row r="472" ht="15.75" customHeight="1" s="24"/>
+    <row r="473" ht="15.75" customHeight="1" s="24"/>
+    <row r="474" ht="15.75" customHeight="1" s="24"/>
+    <row r="475" ht="15.75" customHeight="1" s="24"/>
+    <row r="476" ht="15.75" customHeight="1" s="24"/>
+    <row r="477" ht="15.75" customHeight="1" s="24"/>
+    <row r="478" ht="15.75" customHeight="1" s="24"/>
+    <row r="479" ht="15.75" customHeight="1" s="24"/>
+    <row r="480" ht="15.75" customHeight="1" s="24"/>
+    <row r="481" ht="15.75" customHeight="1" s="24"/>
+    <row r="482" ht="15.75" customHeight="1" s="24"/>
+    <row r="483" ht="15.75" customHeight="1" s="24"/>
+    <row r="484" ht="15.75" customHeight="1" s="24"/>
+    <row r="485" ht="15.75" customHeight="1" s="24"/>
+    <row r="486" ht="15.75" customHeight="1" s="24"/>
+    <row r="487" ht="15.75" customHeight="1" s="24"/>
+    <row r="488" ht="15.75" customHeight="1" s="24"/>
+    <row r="489" ht="15.75" customHeight="1" s="24"/>
+    <row r="490" ht="15.75" customHeight="1" s="24"/>
+    <row r="491" ht="15.75" customHeight="1" s="24"/>
+    <row r="492" ht="15.75" customHeight="1" s="24"/>
+    <row r="493" ht="15.75" customHeight="1" s="24"/>
+    <row r="494" ht="15.75" customHeight="1" s="24"/>
+    <row r="495" ht="15.75" customHeight="1" s="24"/>
+    <row r="496" ht="15.75" customHeight="1" s="24"/>
+    <row r="497" ht="15.75" customHeight="1" s="24"/>
+    <row r="498" ht="15.75" customHeight="1" s="24"/>
+    <row r="499" ht="15.75" customHeight="1" s="24"/>
+    <row r="500" ht="15.75" customHeight="1" s="24"/>
+    <row r="501" ht="15.75" customHeight="1" s="24"/>
+    <row r="502" ht="15.75" customHeight="1" s="24"/>
+    <row r="503" ht="15.75" customHeight="1" s="24"/>
+    <row r="504" ht="15.75" customHeight="1" s="24"/>
+    <row r="505" ht="15.75" customHeight="1" s="24"/>
+    <row r="506" ht="15.75" customHeight="1" s="24"/>
+    <row r="507" ht="15.75" customHeight="1" s="24"/>
+    <row r="508" ht="15.75" customHeight="1" s="24"/>
+    <row r="509" ht="15.75" customHeight="1" s="24"/>
+    <row r="510" ht="15.75" customHeight="1" s="24"/>
+    <row r="511" ht="15.75" customHeight="1" s="24"/>
+    <row r="512" ht="15.75" customHeight="1" s="24"/>
+    <row r="513" ht="15.75" customHeight="1" s="24"/>
+    <row r="514" ht="15.75" customHeight="1" s="24"/>
+    <row r="515" ht="15.75" customHeight="1" s="24"/>
+    <row r="516" ht="15.75" customHeight="1" s="24"/>
+    <row r="517" ht="15.75" customHeight="1" s="24"/>
+    <row r="518" ht="15.75" customHeight="1" s="24"/>
+    <row r="519" ht="15.75" customHeight="1" s="24"/>
+    <row r="520" ht="15.75" customHeight="1" s="24"/>
+    <row r="521" ht="15.75" customHeight="1" s="24"/>
+    <row r="522" ht="15.75" customHeight="1" s="24"/>
+    <row r="523" ht="15.75" customHeight="1" s="24"/>
+    <row r="524" ht="15.75" customHeight="1" s="24"/>
+    <row r="525" ht="15.75" customHeight="1" s="24"/>
+    <row r="526" ht="15.75" customHeight="1" s="24"/>
+    <row r="527" ht="15.75" customHeight="1" s="24"/>
+    <row r="528" ht="15.75" customHeight="1" s="24"/>
+    <row r="529" ht="15.75" customHeight="1" s="24"/>
+    <row r="530" ht="15.75" customHeight="1" s="24"/>
+    <row r="531" ht="15.75" customHeight="1" s="24"/>
+    <row r="532" ht="15.75" customHeight="1" s="24"/>
+    <row r="533" ht="15.75" customHeight="1" s="24"/>
+    <row r="534" ht="15.75" customHeight="1" s="24"/>
+    <row r="535" ht="15.75" customHeight="1" s="24"/>
+    <row r="536" ht="15.75" customHeight="1" s="24"/>
+    <row r="537" ht="15.75" customHeight="1" s="24"/>
+    <row r="538" ht="15.75" customHeight="1" s="24"/>
+    <row r="539" ht="15.75" customHeight="1" s="24"/>
+    <row r="540" ht="15.75" customHeight="1" s="24"/>
+    <row r="541" ht="15.75" customHeight="1" s="24"/>
+    <row r="542" ht="15.75" customHeight="1" s="24"/>
+    <row r="543" ht="15.75" customHeight="1" s="24"/>
+    <row r="544" ht="15.75" customHeight="1" s="24"/>
+    <row r="545" ht="15.75" customHeight="1" s="24"/>
+    <row r="546" ht="15.75" customHeight="1" s="24"/>
+    <row r="547" ht="15.75" customHeight="1" s="24"/>
+    <row r="548" ht="15.75" customHeight="1" s="24"/>
+    <row r="549" ht="15.75" customHeight="1" s="24"/>
+    <row r="550" ht="15.75" customHeight="1" s="24"/>
+    <row r="551" ht="15.75" customHeight="1" s="24"/>
+    <row r="552" ht="15.75" customHeight="1" s="24"/>
+    <row r="553" ht="15.75" customHeight="1" s="24"/>
+    <row r="554" ht="15.75" customHeight="1" s="24"/>
+    <row r="555" ht="15.75" customHeight="1" s="24"/>
+    <row r="556" ht="15.75" customHeight="1" s="24"/>
+    <row r="557" ht="15.75" customHeight="1" s="24"/>
+    <row r="558" ht="15.75" customHeight="1" s="24"/>
+    <row r="559" ht="15.75" customHeight="1" s="24"/>
+    <row r="560" ht="15.75" customHeight="1" s="24"/>
+    <row r="561" ht="15.75" customHeight="1" s="24"/>
+    <row r="562" ht="15.75" customHeight="1" s="24"/>
+    <row r="563" ht="15.75" customHeight="1" s="24"/>
+    <row r="564" ht="15.75" customHeight="1" s="24"/>
+    <row r="565" ht="15.75" customHeight="1" s="24"/>
+    <row r="566" ht="15.75" customHeight="1" s="24"/>
+    <row r="567" ht="15.75" customHeight="1" s="24"/>
+    <row r="568" ht="15.75" customHeight="1" s="24"/>
+    <row r="569" ht="15.75" customHeight="1" s="24"/>
+    <row r="570" ht="15.75" customHeight="1" s="24"/>
+    <row r="571" ht="15.75" customHeight="1" s="24"/>
+    <row r="572" ht="15.75" customHeight="1" s="24"/>
+    <row r="573" ht="15.75" customHeight="1" s="24"/>
+    <row r="574" ht="15.75" customHeight="1" s="24"/>
+    <row r="575" ht="15.75" customHeight="1" s="24"/>
+    <row r="576" ht="15.75" customHeight="1" s="24"/>
+    <row r="577" ht="15.75" customHeight="1" s="24"/>
+    <row r="578" ht="15.75" customHeight="1" s="24"/>
+    <row r="579" ht="15.75" customHeight="1" s="24"/>
+    <row r="580" ht="15.75" customHeight="1" s="24"/>
+    <row r="581" ht="15.75" customHeight="1" s="24"/>
+    <row r="582" ht="15.75" customHeight="1" s="24"/>
+    <row r="583" ht="15.75" customHeight="1" s="24"/>
+    <row r="584" ht="15.75" customHeight="1" s="24"/>
+    <row r="585" ht="15.75" customHeight="1" s="24"/>
+    <row r="586" ht="15.75" customHeight="1" s="24"/>
+    <row r="587" ht="15.75" customHeight="1" s="24"/>
+    <row r="588" ht="15.75" customHeight="1" s="24"/>
+    <row r="589" ht="15.75" customHeight="1" s="24"/>
+    <row r="590" ht="15.75" customHeight="1" s="24"/>
+    <row r="591" ht="15.75" customHeight="1" s="24"/>
+    <row r="592" ht="15.75" customHeight="1" s="24"/>
+    <row r="593" ht="15.75" customHeight="1" s="24"/>
+    <row r="594" ht="15.75" customHeight="1" s="24"/>
+    <row r="595" ht="15.75" customHeight="1" s="24"/>
+    <row r="596" ht="15.75" customHeight="1" s="24"/>
+    <row r="597" ht="15.75" customHeight="1" s="24"/>
+    <row r="598" ht="15.75" customHeight="1" s="24"/>
+    <row r="599" ht="15.75" customHeight="1" s="24"/>
+    <row r="600" ht="15.75" customHeight="1" s="24"/>
+    <row r="601" ht="15.75" customHeight="1" s="24"/>
+    <row r="602" ht="15.75" customHeight="1" s="24"/>
+    <row r="603" ht="15.75" customHeight="1" s="24"/>
+    <row r="604" ht="15.75" customHeight="1" s="24"/>
+    <row r="605" ht="15.75" customHeight="1" s="24"/>
+    <row r="606" ht="15.75" customHeight="1" s="24"/>
+    <row r="607" ht="15.75" customHeight="1" s="24"/>
+    <row r="608" ht="15.75" customHeight="1" s="24"/>
+    <row r="609" ht="15.75" customHeight="1" s="24"/>
+    <row r="610" ht="15.75" customHeight="1" s="24"/>
+    <row r="611" ht="15.75" customHeight="1" s="24"/>
+    <row r="612" ht="15.75" customHeight="1" s="24"/>
+    <row r="613" ht="15.75" customHeight="1" s="24"/>
+    <row r="614" ht="15.75" customHeight="1" s="24"/>
+    <row r="615" ht="15.75" customHeight="1" s="24"/>
+    <row r="616" ht="15.75" customHeight="1" s="24"/>
+    <row r="617" ht="15.75" customHeight="1" s="24"/>
+    <row r="618" ht="15.75" customHeight="1" s="24"/>
+    <row r="619" ht="15.75" customHeight="1" s="24"/>
+    <row r="620" ht="15.75" customHeight="1" s="24"/>
+    <row r="621" ht="15.75" customHeight="1" s="24"/>
+    <row r="622" ht="15.75" customHeight="1" s="24"/>
+    <row r="623" ht="15.75" customHeight="1" s="24"/>
+    <row r="624" ht="15.75" customHeight="1" s="24"/>
+    <row r="625" ht="15.75" customHeight="1" s="24"/>
+    <row r="626" ht="15.75" customHeight="1" s="24"/>
+    <row r="627" ht="15.75" customHeight="1" s="24"/>
+    <row r="628" ht="15.75" customHeight="1" s="24"/>
+    <row r="629" ht="15.75" customHeight="1" s="24"/>
+    <row r="630" ht="15.75" customHeight="1" s="24"/>
+    <row r="631" ht="15.75" customHeight="1" s="24"/>
+    <row r="632" ht="15.75" customHeight="1" s="24"/>
+    <row r="633" ht="15.75" customHeight="1" s="24"/>
+    <row r="634" ht="15.75" customHeight="1" s="24"/>
+    <row r="635" ht="15.75" customHeight="1" s="24"/>
+    <row r="636" ht="15.75" customHeight="1" s="24"/>
+    <row r="637" ht="15.75" customHeight="1" s="24"/>
+    <row r="638" ht="15.75" customHeight="1" s="24"/>
+    <row r="639" ht="15.75" customHeight="1" s="24"/>
+    <row r="640" ht="15.75" customHeight="1" s="24"/>
+    <row r="641" ht="15.75" customHeight="1" s="24"/>
+    <row r="642" ht="15.75" customHeight="1" s="24"/>
+    <row r="643" ht="15.75" customHeight="1" s="24"/>
+    <row r="644" ht="15.75" customHeight="1" s="24"/>
+    <row r="645" ht="15.75" customHeight="1" s="24"/>
+    <row r="646" ht="15.75" customHeight="1" s="24"/>
+    <row r="647" ht="15.75" customHeight="1" s="24"/>
+    <row r="648" ht="15.75" customHeight="1" s="24"/>
+    <row r="649" ht="15.75" customHeight="1" s="24"/>
+    <row r="650" ht="15.75" customHeight="1" s="24"/>
+    <row r="651" ht="15.75" customHeight="1" s="24"/>
+    <row r="652" ht="15.75" customHeight="1" s="24"/>
+    <row r="653" ht="15.75" customHeight="1" s="24"/>
+    <row r="654" ht="15.75" customHeight="1" s="24"/>
+    <row r="655" ht="15.75" customHeight="1" s="24"/>
+    <row r="656" ht="15.75" customHeight="1" s="24"/>
+    <row r="657" ht="15.75" customHeight="1" s="24"/>
+    <row r="658" ht="15.75" customHeight="1" s="24"/>
+    <row r="659" ht="15.75" customHeight="1" s="24"/>
+    <row r="660" ht="15.75" customHeight="1" s="24"/>
+    <row r="661" ht="15.75" customHeight="1" s="24"/>
+    <row r="662" ht="15.75" customHeight="1" s="24"/>
+    <row r="663" ht="15.75" customHeight="1" s="24"/>
+    <row r="664" ht="15.75" customHeight="1" s="24"/>
+    <row r="665" ht="15.75" customHeight="1" s="24"/>
+    <row r="666" ht="15.75" customHeight="1" s="24"/>
+    <row r="667" ht="15.75" customHeight="1" s="24"/>
+    <row r="668" ht="15.75" customHeight="1" s="24"/>
+    <row r="669" ht="15.75" customHeight="1" s="24"/>
+    <row r="670" ht="15.75" customHeight="1" s="24"/>
+    <row r="671" ht="15.75" customHeight="1" s="24"/>
+    <row r="672" ht="15.75" customHeight="1" s="24"/>
+    <row r="673" ht="15.75" customHeight="1" s="24"/>
+    <row r="674" ht="15.75" customHeight="1" s="24"/>
+    <row r="675" ht="15.75" customHeight="1" s="24"/>
+    <row r="676" ht="15.75" customHeight="1" s="24"/>
+    <row r="677" ht="15.75" customHeight="1" s="24"/>
+    <row r="678" ht="15.75" customHeight="1" s="24"/>
+    <row r="679" ht="15.75" customHeight="1" s="24"/>
+    <row r="680" ht="15.75" customHeight="1" s="24"/>
+    <row r="681" ht="15.75" customHeight="1" s="24"/>
+    <row r="682" ht="15.75" customHeight="1" s="24"/>
+    <row r="683" ht="15.75" customHeight="1" s="24"/>
+    <row r="684" ht="15.75" customHeight="1" s="24"/>
+    <row r="685" ht="15.75" customHeight="1" s="24"/>
+    <row r="686" ht="15.75" customHeight="1" s="24"/>
+    <row r="687" ht="15.75" customHeight="1" s="24"/>
+    <row r="688" ht="15.75" customHeight="1" s="24"/>
+    <row r="689" ht="15.75" customHeight="1" s="24"/>
+    <row r="690" ht="15.75" customHeight="1" s="24"/>
+    <row r="691" ht="15.75" customHeight="1" s="24"/>
+    <row r="692" ht="15.75" customHeight="1" s="24"/>
+    <row r="693" ht="15.75" customHeight="1" s="24"/>
+    <row r="694" ht="15.75" customHeight="1" s="24"/>
+    <row r="695" ht="15.75" customHeight="1" s="24"/>
+    <row r="696" ht="15.75" customHeight="1" s="24"/>
+    <row r="697" ht="15.75" customHeight="1" s="24"/>
+    <row r="698" ht="15.75" customHeight="1" s="24"/>
+    <row r="699" ht="15.75" customHeight="1" s="24"/>
+    <row r="700" ht="15.75" customHeight="1" s="24"/>
+    <row r="701" ht="15.75" customHeight="1" s="24"/>
+    <row r="702" ht="15.75" customHeight="1" s="24"/>
+    <row r="703" ht="15.75" customHeight="1" s="24"/>
+    <row r="704" ht="15.75" customHeight="1" s="24"/>
+    <row r="705" ht="15.75" customHeight="1" s="24"/>
+    <row r="706" ht="15.75" customHeight="1" s="24"/>
+    <row r="707" ht="15.75" customHeight="1" s="24"/>
+    <row r="708" ht="15.75" customHeight="1" s="24"/>
+    <row r="709" ht="15.75" customHeight="1" s="24"/>
+    <row r="710" ht="15.75" customHeight="1" s="24"/>
+    <row r="711" ht="15.75" customHeight="1" s="24"/>
+    <row r="712" ht="15.75" customHeight="1" s="24"/>
+    <row r="713" ht="15.75" customHeight="1" s="24"/>
+    <row r="714" ht="15.75" customHeight="1" s="24"/>
+    <row r="715" ht="15.75" customHeight="1" s="24"/>
+    <row r="716" ht="15.75" customHeight="1" s="24"/>
+    <row r="717" ht="15.75" customHeight="1" s="24"/>
+    <row r="718" ht="15.75" customHeight="1" s="24"/>
+    <row r="719" ht="15.75" customHeight="1" s="24"/>
+    <row r="720" ht="15.75" customHeight="1" s="24"/>
+    <row r="721" ht="15.75" customHeight="1" s="24"/>
+    <row r="722" ht="15.75" customHeight="1" s="24"/>
+    <row r="723" ht="15.75" customHeight="1" s="24"/>
+    <row r="724" ht="15.75" customHeight="1" s="24"/>
+    <row r="725" ht="15.75" customHeight="1" s="24"/>
+    <row r="726" ht="15.75" customHeight="1" s="24"/>
+    <row r="727" ht="15.75" customHeight="1" s="24"/>
+    <row r="728" ht="15.75" customHeight="1" s="24"/>
+    <row r="729" ht="15.75" customHeight="1" s="24"/>
+    <row r="730" ht="15.75" customHeight="1" s="24"/>
+    <row r="731" ht="15.75" customHeight="1" s="24"/>
+    <row r="732" ht="15.75" customHeight="1" s="24"/>
+    <row r="733" ht="15.75" customHeight="1" s="24"/>
+    <row r="734" ht="15.75" customHeight="1" s="24"/>
+    <row r="735" ht="15.75" customHeight="1" s="24"/>
+    <row r="736" ht="15.75" customHeight="1" s="24"/>
+    <row r="737" ht="15.75" customHeight="1" s="24"/>
+    <row r="738" ht="15.75" customHeight="1" s="24"/>
+    <row r="739" ht="15.75" customHeight="1" s="24"/>
+    <row r="740" ht="15.75" customHeight="1" s="24"/>
+    <row r="741" ht="15.75" customHeight="1" s="24"/>
+    <row r="742" ht="15.75" customHeight="1" s="24"/>
+    <row r="743" ht="15.75" customHeight="1" s="24"/>
+    <row r="744" ht="15.75" customHeight="1" s="24"/>
+    <row r="745" ht="15.75" customHeight="1" s="24"/>
+    <row r="746" ht="15.75" customHeight="1" s="24"/>
+    <row r="747" ht="15.75" customHeight="1" s="24"/>
+    <row r="748" ht="15.75" customHeight="1" s="24"/>
+    <row r="749" ht="15.75" customHeight="1" s="24"/>
+    <row r="750" ht="15.75" customHeight="1" s="24"/>
+    <row r="751" ht="15.75" customHeight="1" s="24"/>
+    <row r="752" ht="15.75" customHeight="1" s="24"/>
+    <row r="753" ht="15.75" customHeight="1" s="24"/>
+    <row r="754" ht="15.75" customHeight="1" s="24"/>
+    <row r="755" ht="15.75" customHeight="1" s="24"/>
+    <row r="756" ht="15.75" customHeight="1" s="24"/>
+    <row r="757" ht="15.75" customHeight="1" s="24"/>
+    <row r="758" ht="15.75" customHeight="1" s="24"/>
+    <row r="759" ht="15.75" customHeight="1" s="24"/>
+    <row r="760" ht="15.75" customHeight="1" s="24"/>
+    <row r="761" ht="15.75" customHeight="1" s="24"/>
+    <row r="762" ht="15.75" customHeight="1" s="24"/>
+    <row r="763" ht="15.75" customHeight="1" s="24"/>
+    <row r="764" ht="15.75" customHeight="1" s="24"/>
+    <row r="765" ht="15.75" customHeight="1" s="24"/>
+    <row r="766" ht="15.75" customHeight="1" s="24"/>
+    <row r="767" ht="15.75" customHeight="1" s="24"/>
+    <row r="768" ht="15.75" customHeight="1" s="24"/>
+    <row r="769" ht="15.75" customHeight="1" s="24"/>
+    <row r="770" ht="15.75" customHeight="1" s="24"/>
+    <row r="771" ht="15.75" customHeight="1" s="24"/>
+    <row r="772" ht="15.75" customHeight="1" s="24"/>
+    <row r="773" ht="15.75" customHeight="1" s="24"/>
+    <row r="774" ht="15.75" customHeight="1" s="24"/>
+    <row r="775" ht="15.75" customHeight="1" s="24"/>
+    <row r="776" ht="15.75" customHeight="1" s="24"/>
+    <row r="777" ht="15.75" customHeight="1" s="24"/>
+    <row r="778" ht="15.75" customHeight="1" s="24"/>
+    <row r="779" ht="15.75" customHeight="1" s="24"/>
+    <row r="780" ht="15.75" customHeight="1" s="24"/>
+    <row r="781" ht="15.75" customHeight="1" s="24"/>
+    <row r="782" ht="15.75" customHeight="1" s="24"/>
+    <row r="783" ht="15.75" customHeight="1" s="24"/>
+    <row r="784" ht="15.75" customHeight="1" s="24"/>
+    <row r="785" ht="15.75" customHeight="1" s="24"/>
+    <row r="786" ht="15.75" customHeight="1" s="24"/>
+    <row r="787" ht="15.75" customHeight="1" s="24"/>
+    <row r="788" ht="15.75" customHeight="1" s="24"/>
+    <row r="789" ht="15.75" customHeight="1" s="24"/>
+    <row r="790" ht="15.75" customHeight="1" s="24"/>
+    <row r="791" ht="15.75" customHeight="1" s="24"/>
+    <row r="792" ht="15.75" customHeight="1" s="24"/>
+    <row r="793" ht="15.75" customHeight="1" s="24"/>
+    <row r="794" ht="15.75" customHeight="1" s="24"/>
+    <row r="795" ht="15.75" customHeight="1" s="24"/>
+    <row r="796" ht="15.75" customHeight="1" s="24"/>
+    <row r="797" ht="15.75" customHeight="1" s="24"/>
+    <row r="798" ht="15.75" customHeight="1" s="24"/>
+    <row r="799" ht="15.75" customHeight="1" s="24"/>
+    <row r="800" ht="15.75" customHeight="1" s="24"/>
+    <row r="801" ht="15.75" customHeight="1" s="24"/>
+    <row r="802" ht="15.75" customHeight="1" s="24"/>
+    <row r="803" ht="15.75" customHeight="1" s="24"/>
+    <row r="804" ht="15.75" customHeight="1" s="24"/>
+    <row r="805" ht="15.75" customHeight="1" s="24"/>
+    <row r="806" ht="15.75" customHeight="1" s="24"/>
+    <row r="807" ht="15.75" customHeight="1" s="24"/>
+    <row r="808" ht="15.75" customHeight="1" s="24"/>
+    <row r="809" ht="15.75" customHeight="1" s="24"/>
+    <row r="810" ht="15.75" customHeight="1" s="24"/>
+    <row r="811" ht="15.75" customHeight="1" s="24"/>
+    <row r="812" ht="15.75" customHeight="1" s="24"/>
+    <row r="813" ht="15.75" customHeight="1" s="24"/>
+    <row r="814" ht="15.75" customHeight="1" s="24"/>
+    <row r="815" ht="15.75" customHeight="1" s="24"/>
+    <row r="816" ht="15.75" customHeight="1" s="24"/>
+    <row r="817" ht="15.75" customHeight="1" s="24"/>
+    <row r="818" ht="15.75" customHeight="1" s="24"/>
+    <row r="819" ht="15.75" customHeight="1" s="24"/>
+    <row r="820" ht="15.75" customHeight="1" s="24"/>
+    <row r="821" ht="15.75" customHeight="1" s="24"/>
+    <row r="822" ht="15.75" customHeight="1" s="24"/>
+    <row r="823" ht="15.75" customHeight="1" s="24"/>
+    <row r="824" ht="15.75" customHeight="1" s="24"/>
+    <row r="825" ht="15.75" customHeight="1" s="24"/>
+    <row r="826" ht="15.75" customHeight="1" s="24"/>
+    <row r="827" ht="15.75" customHeight="1" s="24"/>
+    <row r="828" ht="15.75" customHeight="1" s="24"/>
+    <row r="829" ht="15.75" customHeight="1" s="24"/>
+    <row r="830" ht="15.75" customHeight="1" s="24"/>
+    <row r="831" ht="15.75" customHeight="1" s="24"/>
+    <row r="832" ht="15.75" customHeight="1" s="24"/>
+    <row r="833" ht="15.75" customHeight="1" s="24"/>
+    <row r="834" ht="15.75" customHeight="1" s="24"/>
+    <row r="835" ht="15.75" customHeight="1" s="24"/>
+    <row r="836" ht="15.75" customHeight="1" s="24"/>
+    <row r="837" ht="15.75" customHeight="1" s="24"/>
+    <row r="838" ht="15.75" customHeight="1" s="24"/>
+    <row r="839" ht="15.75" customHeight="1" s="24"/>
+    <row r="840" ht="15.75" customHeight="1" s="24"/>
+    <row r="841" ht="15.75" customHeight="1" s="24"/>
+    <row r="842" ht="15.75" customHeight="1" s="24"/>
+    <row r="843" ht="15.75" customHeight="1" s="24"/>
+    <row r="844" ht="15.75" customHeight="1" s="24"/>
+    <row r="845" ht="15.75" customHeight="1" s="24"/>
+    <row r="846" ht="15.75" customHeight="1" s="24"/>
+    <row r="847" ht="15.75" customHeight="1" s="24"/>
+    <row r="848" ht="15.75" customHeight="1" s="24"/>
+    <row r="849" ht="15.75" customHeight="1" s="24"/>
+    <row r="850" ht="15.75" customHeight="1" s="24"/>
+    <row r="851" ht="15.75" customHeight="1" s="24"/>
+    <row r="852" ht="15.75" customHeight="1" s="24"/>
+    <row r="853" ht="15.75" customHeight="1" s="24"/>
+    <row r="854" ht="15.75" customHeight="1" s="24"/>
+    <row r="855" ht="15.75" customHeight="1" s="24"/>
+    <row r="856" ht="15.75" customHeight="1" s="24"/>
+    <row r="857" ht="15.75" customHeight="1" s="24"/>
+    <row r="858" ht="15.75" customHeight="1" s="24"/>
+    <row r="859" ht="15.75" customHeight="1" s="24"/>
+    <row r="860" ht="15.75" customHeight="1" s="24"/>
+    <row r="861" ht="15.75" customHeight="1" s="24"/>
+    <row r="862" ht="15.75" customHeight="1" s="24"/>
+    <row r="863" ht="15.75" customHeight="1" s="24"/>
+    <row r="864" ht="15.75" customHeight="1" s="24"/>
+    <row r="865" ht="15.75" customHeight="1" s="24"/>
+    <row r="866" ht="15.75" customHeight="1" s="24"/>
+    <row r="867" ht="15.75" customHeight="1" s="24"/>
+    <row r="868" ht="15.75" customHeight="1" s="24"/>
+    <row r="869" ht="15.75" customHeight="1" s="24"/>
+    <row r="870" ht="15.75" customHeight="1" s="24"/>
+    <row r="871" ht="15.75" customHeight="1" s="24"/>
+    <row r="872" ht="15.75" customHeight="1" s="24"/>
+    <row r="873" ht="15.75" customHeight="1" s="24"/>
+    <row r="874" ht="15.75" customHeight="1" s="24"/>
+    <row r="875" ht="15.75" customHeight="1" s="24"/>
+    <row r="876" ht="15.75" customHeight="1" s="24"/>
+    <row r="877" ht="15.75" customHeight="1" s="24"/>
+    <row r="878" ht="15.75" customHeight="1" s="24"/>
+    <row r="879" ht="15.75" customHeight="1" s="24"/>
+    <row r="880" ht="15.75" customHeight="1" s="24"/>
+    <row r="881" ht="15.75" customHeight="1" s="24"/>
+    <row r="882" ht="15.75" customHeight="1" s="24"/>
+    <row r="883" ht="15.75" customHeight="1" s="24"/>
+    <row r="884" ht="15.75" customHeight="1" s="24"/>
+    <row r="885" ht="15.75" customHeight="1" s="24"/>
+    <row r="886" ht="15.75" customHeight="1" s="24"/>
+    <row r="887" ht="15.75" customHeight="1" s="24"/>
+    <row r="888" ht="15.75" customHeight="1" s="24"/>
+    <row r="889" ht="15.75" customHeight="1" s="24"/>
+    <row r="890" ht="15.75" customHeight="1" s="24"/>
+    <row r="891" ht="15.75" customHeight="1" s="24"/>
+    <row r="892" ht="15.75" customHeight="1" s="24"/>
+    <row r="893" ht="15.75" customHeight="1" s="24"/>
+    <row r="894" ht="15.75" customHeight="1" s="24"/>
+    <row r="895" ht="15.75" customHeight="1" s="24"/>
+    <row r="896" ht="15.75" customHeight="1" s="24"/>
+    <row r="897" ht="15.75" customHeight="1" s="24"/>
+    <row r="898" ht="15.75" customHeight="1" s="24"/>
+    <row r="899" ht="15.75" customHeight="1" s="24"/>
+    <row r="900" ht="15.75" customHeight="1" s="24"/>
+    <row r="901" ht="15.75" customHeight="1" s="24"/>
+    <row r="902" ht="15.75" customHeight="1" s="24"/>
+    <row r="903" ht="15.75" customHeight="1" s="24"/>
+    <row r="904" ht="15.75" customHeight="1" s="24"/>
+    <row r="905" ht="15.75" customHeight="1" s="24"/>
+    <row r="906" ht="15.75" customHeight="1" s="24"/>
+    <row r="907" ht="15.75" customHeight="1" s="24"/>
+    <row r="908" ht="15.75" customHeight="1" s="24"/>
+    <row r="909" ht="15.75" customHeight="1" s="24"/>
+    <row r="910" ht="15.75" customHeight="1" s="24"/>
+    <row r="911" ht="15.75" customHeight="1" s="24"/>
+    <row r="912" ht="15.75" customHeight="1" s="24"/>
+    <row r="913" ht="15.75" customHeight="1" s="24"/>
+    <row r="914" ht="15.75" customHeight="1" s="24"/>
+    <row r="915" ht="15.75" customHeight="1" s="24"/>
+    <row r="916" ht="15.75" customHeight="1" s="24"/>
+    <row r="917" ht="15.75" customHeight="1" s="24"/>
+    <row r="918" ht="15.75" customHeight="1" s="24"/>
+    <row r="919" ht="15.75" customHeight="1" s="24"/>
+    <row r="920" ht="15.75" customHeight="1" s="24"/>
+    <row r="921" ht="15.75" customHeight="1" s="24"/>
+    <row r="922" ht="15.75" customHeight="1" s="24"/>
+    <row r="923" ht="15.75" customHeight="1" s="24"/>
+    <row r="924" ht="15.75" customHeight="1" s="24"/>
+    <row r="925" ht="15.75" customHeight="1" s="24"/>
+    <row r="926" ht="15.75" customHeight="1" s="24"/>
+    <row r="927" ht="15.75" customHeight="1" s="24"/>
+    <row r="928" ht="15.75" customHeight="1" s="24"/>
+    <row r="929" ht="15.75" customHeight="1" s="24"/>
+    <row r="930" ht="15.75" customHeight="1" s="24"/>
+    <row r="931" ht="15.75" customHeight="1" s="24"/>
+    <row r="932" ht="15.75" customHeight="1" s="24"/>
+    <row r="933" ht="15.75" customHeight="1" s="24"/>
+    <row r="934" ht="15.75" customHeight="1" s="24"/>
+    <row r="935" ht="15.75" customHeight="1" s="24"/>
+    <row r="936" ht="15.75" customHeight="1" s="24"/>
+    <row r="937" ht="15.75" customHeight="1" s="24"/>
+    <row r="938" ht="15.75" customHeight="1" s="24"/>
+    <row r="939" ht="15.75" customHeight="1" s="24"/>
+    <row r="940" ht="15.75" customHeight="1" s="24"/>
+    <row r="941" ht="15.75" customHeight="1" s="24"/>
+    <row r="942" ht="15.75" customHeight="1" s="24"/>
+    <row r="943" ht="15.75" customHeight="1" s="24"/>
+    <row r="944" ht="15.75" customHeight="1" s="24"/>
+    <row r="945" ht="15.75" customHeight="1" s="24"/>
+    <row r="946" ht="15.75" customHeight="1" s="24"/>
+    <row r="947" ht="15.75" customHeight="1" s="24"/>
+    <row r="948" ht="15.75" customHeight="1" s="24"/>
+    <row r="949" ht="15.75" customHeight="1" s="24"/>
+    <row r="950" ht="15.75" customHeight="1" s="24"/>
+    <row r="951" ht="15.75" customHeight="1" s="24"/>
+    <row r="952" ht="15.75" customHeight="1" s="24"/>
+    <row r="953" ht="15.75" customHeight="1" s="24"/>
+    <row r="954" ht="15.75" customHeight="1" s="24"/>
+    <row r="955" ht="15.75" customHeight="1" s="24"/>
+    <row r="956" ht="15.75" customHeight="1" s="24"/>
+    <row r="957" ht="15.75" customHeight="1" s="24"/>
+    <row r="958" ht="15.75" customHeight="1" s="24"/>
+    <row r="959" ht="15.75" customHeight="1" s="24"/>
+    <row r="960" ht="15.75" customHeight="1" s="24"/>
+    <row r="961" ht="15.75" customHeight="1" s="24"/>
+    <row r="962" ht="15.75" customHeight="1" s="24"/>
+    <row r="963" ht="15.75" customHeight="1" s="24"/>
+    <row r="964" ht="15.75" customHeight="1" s="24"/>
+    <row r="965" ht="15.75" customHeight="1" s="24"/>
+    <row r="966" ht="15.75" customHeight="1" s="24"/>
+    <row r="967" ht="15.75" customHeight="1" s="24"/>
+    <row r="968" ht="15.75" customHeight="1" s="24"/>
+    <row r="969" ht="15.75" customHeight="1" s="24"/>
+    <row r="970" ht="15.75" customHeight="1" s="24"/>
+    <row r="971" ht="15.75" customHeight="1" s="24"/>
+    <row r="972" ht="15.75" customHeight="1" s="24"/>
+    <row r="973" ht="15.75" customHeight="1" s="24"/>
+    <row r="974" ht="15.75" customHeight="1" s="24"/>
+    <row r="975" ht="15.75" customHeight="1" s="24"/>
+    <row r="976" ht="15.75" customHeight="1" s="24"/>
+    <row r="977" ht="15.75" customHeight="1" s="24"/>
+    <row r="978" ht="15.75" customHeight="1" s="24"/>
+    <row r="979" ht="15.75" customHeight="1" s="24"/>
+    <row r="980" ht="15.75" customHeight="1" s="24"/>
+    <row r="981" ht="15.75" customHeight="1" s="24"/>
+    <row r="982" ht="15.75" customHeight="1" s="24"/>
+    <row r="983" ht="15.75" customHeight="1" s="24"/>
+    <row r="984" ht="15.75" customHeight="1" s="24"/>
+    <row r="985" ht="15.75" customHeight="1" s="24"/>
+    <row r="986" ht="15.75" customHeight="1" s="24"/>
+    <row r="987" ht="15.75" customHeight="1" s="24"/>
+    <row r="988" ht="15.75" customHeight="1" s="24"/>
+    <row r="989" ht="15.75" customHeight="1" s="24"/>
+    <row r="990" ht="15.75" customHeight="1" s="24"/>
+    <row r="991" ht="15.75" customHeight="1" s="24"/>
+    <row r="992" ht="15.75" customHeight="1" s="24"/>
+    <row r="993" ht="15.75" customHeight="1" s="24"/>
+    <row r="994" ht="15.75" customHeight="1" s="24"/>
+    <row r="995" ht="15.75" customHeight="1" s="24"/>
+    <row r="996" ht="15.75" customHeight="1" s="24"/>
+    <row r="997" ht="15.75" customHeight="1" s="24"/>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
docs(W7): báo cáo tuần 7 của Sang và AI Prompt Log tuần 7 (sheet Sang) (#79)
Báo cáo đối chiếu W7-S01..S05 với kế hoạch W7, phần làm lại sau W7 đã vào
main (#78: D058, D059, D060, sơ đồ lớp thực thể), kết quả kiểm thử, vướng mắc
và kế hoạch tuần 8. AI log W07 sheet Sang 10 dòng ngày 28–29/10, mỗi dòng có
PR hoặc tệp làm minh chứng; README cập nhật số liệu W07 (24 bản ghi).
</commit_message>
<xml_diff>
--- a/docs/evidence/tc2-3-ai-usage/AI Prompt Log - W07 - 2026-10-26_2026-11-01.xlsx
+++ b/docs/evidence/tc2-3-ai-usage/AI Prompt Log - W07 - 2026-10-26_2026-11-01.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thắng" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nguyên" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sang" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tổng hợp" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Thắng" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Nguyên" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Sang" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Tổng hợp" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
@@ -12960,84 +12960,304 @@
       </c>
     </row>
     <row r="6" ht="36" customHeight="1" s="24">
-      <c r="A6" s="20" t="n"/>
-      <c r="B6" s="18" t="n"/>
-      <c r="C6" s="18" t="n"/>
-      <c r="D6" s="33" t="n"/>
-      <c r="E6" s="33" t="n"/>
-      <c r="F6" s="33" t="n"/>
+      <c r="A6" s="36" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B6" s="37" t="inlineStr">
+        <is>
+          <t>Sang</t>
+        </is>
+      </c>
+      <c r="C6" s="37" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="D6" s="38" t="inlineStr">
+        <is>
+          <t>Rà soát kế hoạch W7 sau khi chuyển sang MongoDB; làm main xanh trở lại và gỡ số đo S&amp;I còn sót</t>
+        </is>
+      </c>
+      <c r="E6" s="38" t="inlineStr">
+        <is>
+          <t>Đối chiếu kế hoạch W7 với những gì nhóm đã chuyển sang repo nộp bài (kiến trúc nay dùng MongoDB, không còn PostgreSQL), chỉ ra các mục sai lệch, rồi thực hiện ngay hai bước: đưa nhánh main về trạng thái CI xanh với code khớp bản nguồn đã chuyển, và gỡ các số đo suy ra từ Speak &amp; Improve còn sót trong tài liệu, kèm chuyển các tài liệu vận hành cần thiết từ repo gốc.</t>
+        </is>
+      </c>
+      <c r="F6" s="38" t="inlineStr">
+        <is>
+          <t>https://github.com/thanglb2005/ai-assessor-cefr/pull/71; https://github.com/thanglb2005/ai-assessor-cefr/pull/72; https://github.com/thanglb2005/ai-assessor-cefr/pull/73</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="36" customHeight="1" s="24">
-      <c r="A7" s="20" t="n"/>
-      <c r="B7" s="18" t="n"/>
-      <c r="C7" s="18" t="n"/>
-      <c r="D7" s="33" t="n"/>
-      <c r="E7" s="33" t="n"/>
-      <c r="F7" s="33" t="n"/>
+      <c r="A7" s="36" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B7" s="37" t="inlineStr">
+        <is>
+          <t>Sang</t>
+        </is>
+      </c>
+      <c r="C7" s="37" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="D7" s="38" t="inlineStr">
+        <is>
+          <t>D058: bỏ đồng thuận nghiên cứu, thay bằng đồng ý điều khoản sử dụng</t>
+        </is>
+      </c>
+      <c r="E7" s="38" t="inlineStr">
+        <is>
+          <t>Giai đoạn thu giọng người Việt để huấn luyện mô hình đã kết thúc; loại bỏ tính năng ký đồng thuận nghiên cứu khỏi toàn hệ thống và thay bằng một lần đồng ý điều khoản sử dụng, có migration chuyển dữ liệu cũ.</t>
+        </is>
+      </c>
+      <c r="F7" s="38" t="inlineStr">
+        <is>
+          <t>https://github.com/thanglb2005/ai-assessor-cefr/pull/75 (gộp vào main qua #78)</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="36" customHeight="1" s="24">
-      <c r="A8" s="20" t="n"/>
-      <c r="B8" s="18" t="n"/>
-      <c r="C8" s="18" t="n"/>
-      <c r="D8" s="33" t="n"/>
-      <c r="E8" s="33" t="n"/>
-      <c r="F8" s="33" t="n"/>
+      <c r="A8" s="36" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B8" s="37" t="inlineStr">
+        <is>
+          <t>Sang</t>
+        </is>
+      </c>
+      <c r="C8" s="37" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="D8" s="38" t="inlineStr">
+        <is>
+          <t>Rút gọn sơ đồ lớp, bỏ thuộc tính thừa trong sơ đồ và code, cập nhật bản draw.io</t>
+        </is>
+      </c>
+      <c r="E8" s="38" t="inlineStr">
+        <is>
+          <t>Rà lại class diagram trên draw.io: chỉ giữ lớp và thuộc tính phục vụ nghiệp vụ, bỏ thuộc tính không ai đọc ở cả sơ đồ lẫn code, giảm số bảng xuống mức hợp lý theo chuẩn OOP (khoảng 20, được phép chênh lệch nếu có lý do), rồi cập nhật lại trang "So do lop" trên Drive.</t>
+        </is>
+      </c>
+      <c r="F8" s="38" t="inlineStr">
+        <is>
+          <t>https://github.com/thanglb2005/ai-assessor-cefr/pull/69; https://github.com/thanglb2005/ai-assessor-cefr/pull/70; https://github.com/thanglb2005/ai-assessor-cefr/pull/74</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="36" customHeight="1" s="24">
-      <c r="A9" s="20" t="n"/>
-      <c r="B9" s="18" t="n"/>
-      <c r="C9" s="18" t="n"/>
-      <c r="D9" s="33" t="n"/>
-      <c r="E9" s="33" t="n"/>
-      <c r="F9" s="33" t="n"/>
+      <c r="A9" s="36" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B9" s="37" t="inlineStr">
+        <is>
+          <t>Sang</t>
+        </is>
+      </c>
+      <c r="C9" s="37" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="D9" s="38" t="inlineStr">
+        <is>
+          <t>D059: hỗ trợ đủ sáu band CEFR từ A1 đến C2</t>
+        </is>
+      </c>
+      <c r="E9" s="38" t="inlineStr">
+        <is>
+          <t>Mở rộng thang band từ A2–B2 lên đủ A1–C2 ở mọi nơi: ánh xạ điểm sang band, ngân hàng luyện tập, lộ trình mẫu, chấm mù, giao diện và test; ghi rõ ba ngưỡng ngoài chưa được hiệu chuẩn.</t>
+        </is>
+      </c>
+      <c r="F9" s="38" t="inlineStr">
+        <is>
+          <t>https://github.com/thanglb2005/ai-assessor-cefr/pull/76 (gộp vào main qua #78); src/aicefr/scoring/band_map.py</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="36" customHeight="1" s="24">
-      <c r="A10" s="20" t="n"/>
-      <c r="B10" s="18" t="n"/>
-      <c r="C10" s="18" t="n"/>
-      <c r="D10" s="33" t="n"/>
-      <c r="E10" s="33" t="n"/>
-      <c r="F10" s="33" t="n"/>
+      <c r="A10" s="36" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B10" s="37" t="inlineStr">
+        <is>
+          <t>Sang</t>
+        </is>
+      </c>
+      <c r="C10" s="37" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="D10" s="38" t="inlineStr">
+        <is>
+          <t>Kiểm tra độ phủ nghiệp vụ của sơ đồ lớp, thiết kế lại chỉ gồm thực thể và chạy toàn bộ test ở local</t>
+        </is>
+      </c>
+      <c r="E10" s="38" t="inlineStr">
+        <is>
+          <t>Đánh giá bộ khoảng 20 collection đã đề xuất có phủ hết nghiệp vụ của bài toán hay chưa (số lượng được linh hoạt); thiết kế lại class diagram chỉ chứa thực thể, không lớp trừu tượng; sau đó chạy toàn bộ test đơn vị và E2E ở local.</t>
+        </is>
+      </c>
+      <c r="F10" s="38" t="inlineStr">
+        <is>
+          <t>https://github.com/thanglb2005/ai-assessor-cefr/pull/70; docs/sdd/thiet-ke-gon-so-do-lop-va-collection.md</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="36" customHeight="1" s="24">
-      <c r="A11" s="20" t="n"/>
-      <c r="B11" s="18" t="n"/>
-      <c r="C11" s="18" t="n"/>
-      <c r="D11" s="33" t="n"/>
-      <c r="E11" s="33" t="n"/>
-      <c r="F11" s="33" t="n"/>
+      <c r="A11" s="36" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B11" s="37" t="inlineStr">
+        <is>
+          <t>Sang</t>
+        </is>
+      </c>
+      <c r="C11" s="37" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="D11" s="38" t="inlineStr">
+        <is>
+          <t>Bổ sung enum vào sơ đồ lớp, rút còn enum điều khiển nghiệp vụ, chia khung theo phần nghiệp vụ</t>
+        </is>
+      </c>
+      <c r="E11" s="38" t="inlineStr">
+        <is>
+          <t>Thêm các kiểu liệt kê vào class diagram và xác nhận sơ đồ phủ đủ nghiệp vụ; sau đó lược bớt enum không cần thiết, gộp collection hợp lý, vẽ sơ đồ chia khung theo phần nghiệp vụ để các đường không chồng chéo và nối mỗi enum với thực thể dùng nó.</t>
+        </is>
+      </c>
+      <c r="F11" s="38" t="inlineStr">
+        <is>
+          <t>https://github.com/thanglb2005/ai-assessor-cefr/pull/77; tools/zone_layout.py; docs/sdd/diagrams/02_class.drawio</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="36" customHeight="1" s="24">
-      <c r="A12" s="20" t="n"/>
-      <c r="B12" s="18" t="n"/>
-      <c r="C12" s="18" t="n"/>
-      <c r="D12" s="33" t="n"/>
-      <c r="E12" s="33" t="n"/>
-      <c r="F12" s="33" t="n"/>
+      <c r="A12" s="36" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B12" s="37" t="inlineStr">
+        <is>
+          <t>Sang</t>
+        </is>
+      </c>
+      <c r="C12" s="37" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="D12" s="38" t="inlineStr">
+        <is>
+          <t>D060: quan hệ thể hiện qua thuộc tính, gộp collection theo aggregate root và rã sơ đồ xuống code</t>
+        </is>
+      </c>
+      <c r="E12" s="38" t="inlineStr">
+        <is>
+          <t>Sửa class diagram theo quy tắc của nhóm: mỗi quan hệ phải có thuộc tính ở lớp giữ quan hệ, bội số chỉ ghi trên đường giữa hai thực thể, thuộc tính trỏ tới enum mang kiểu enum; tiếp tục gộp collection nếu hợp lý, rồi chuyển code theo đúng sơ đồ (lớp miền, migration dữ liệu, test đối chiếu sơ đồ với code).</t>
+        </is>
+      </c>
+      <c r="F12" s="38" t="inlineStr">
+        <is>
+          <t>https://github.com/thanglb2005/ai-assessor-cefr/pull/77; src/aicefr/storage/migrations.py; tests/test_d060_collections.py; tests/test_diagrams.py</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="36" customHeight="1" s="24">
-      <c r="A13" s="20" t="n"/>
-      <c r="B13" s="18" t="n"/>
-      <c r="C13" s="18" t="n"/>
-      <c r="D13" s="33" t="n"/>
-      <c r="E13" s="33" t="n"/>
-      <c r="F13" s="33" t="n"/>
+      <c r="A13" s="36" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B13" s="37" t="inlineStr">
+        <is>
+          <t>Sang</t>
+        </is>
+      </c>
+      <c r="C13" s="37" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="D13" s="38" t="inlineStr">
+        <is>
+          <t>Đưa toàn bộ phần làm lại sau W7 lên main của repo nộp bài</t>
+        </is>
+      </c>
+      <c r="E13" s="38" t="inlineStr">
+        <is>
+          <t>Hoàn thiện bố cục sơ đồ, merge D060, rồi gộp toàn bộ phần làm lại sau W7 vào main của repo nhóm thành một commit; repo gốc của Sang không dùng nữa. Xử lý các check CI đỏ (link tài liệu hỏng, giới hạn thời gian job kiểm thử).</t>
+        </is>
+      </c>
+      <c r="F13" s="38" t="inlineStr">
+        <is>
+          <t>https://github.com/thanglb2005/ai-assessor-cefr/pull/78 (squash 130ffea); .github/workflows/ci.yml</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="36" customHeight="1" s="24">
-      <c r="A14" s="20" t="n"/>
-      <c r="B14" s="18" t="n"/>
-      <c r="C14" s="18" t="n"/>
-      <c r="D14" s="33" t="n"/>
-      <c r="E14" s="33" t="n"/>
-      <c r="F14" s="33" t="n"/>
+      <c r="A14" s="36" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B14" s="37" t="inlineStr">
+        <is>
+          <t>Sang</t>
+        </is>
+      </c>
+      <c r="C14" s="37" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="D14" s="38" t="inlineStr">
+        <is>
+          <t>Merge PR gỡ số đo S&amp;I và đóng các PR đã được gộp</t>
+        </is>
+      </c>
+      <c r="E14" s="38" t="inlineStr">
+        <is>
+          <t>Cập nhật nhánh gỡ số đo S&amp;I theo main mới, sửa link tới tài liệu nội bộ, merge vào main, rồi đóng các PR đã nằm trong lần gộp kèm ghi chú lý do.</t>
+        </is>
+      </c>
+      <c r="F14" s="38" t="inlineStr">
+        <is>
+          <t>https://github.com/thanglb2005/ai-assessor-cefr/pull/73 (squash 856bd5f)</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="36" customHeight="1" s="24">
-      <c r="A15" s="20" t="n"/>
-      <c r="B15" s="18" t="n"/>
-      <c r="C15" s="18" t="n"/>
-      <c r="D15" s="33" t="n"/>
-      <c r="E15" s="33" t="n"/>
-      <c r="F15" s="33" t="n"/>
+      <c r="A15" s="36" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B15" s="37" t="inlineStr">
+        <is>
+          <t>Sang</t>
+        </is>
+      </c>
+      <c r="C15" s="37" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="D15" s="38" t="inlineStr">
+        <is>
+          <t>Soạn báo cáo tuần 7 và ghi AI Prompt Log tuần 7</t>
+        </is>
+      </c>
+      <c r="E15" s="38" t="inlineStr">
+        <is>
+          <t>Cập nhật báo cáo tiến độ tuần 7 của Sang và nhật ký sử dụng AI của tuần, đối chiếu từng mục với PR và commit thật.</t>
+        </is>
+      </c>
+      <c r="F15" s="38" t="inlineStr">
+        <is>
+          <t>docs/reports/week-07/bao-cao-tuan-07-sang.md; docs/evidence/tc2-3-ai-usage/README.md</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="36" customHeight="1" s="24">
       <c r="A16" s="20" t="n"/>
@@ -18858,1182 +19078,1182 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<ns0:worksheet xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <ns0:sheetPr>
-    <ns0:tabColor rgb="FF17324D"/>
-    <ns0:outlinePr summaryBelow="1" summaryRight="1"/>
-    <ns0:pageSetUpPr/>
-  </ns0:sheetPr>
-  <ns0:dimension ref="A2:F14"/>
-  <ns0:sheetFormatPr baseColWidth="8" defaultColWidth="12.625" defaultRowHeight="14.25"/>
-  <ns0:cols>
-    <ns0:col width="24" customWidth="1" style="24" min="1" max="1"/>
-    <ns0:col width="15" customWidth="1" style="24" min="2" max="2"/>
-    <ns0:col width="4" customWidth="1" style="24" min="3" max="3"/>
-    <ns0:col width="24" customWidth="1" style="24" min="4" max="4"/>
-    <ns0:col width="15" customWidth="1" style="24" min="5" max="5"/>
-    <ns0:col width="8" customWidth="1" style="24" min="6" max="6"/>
-    <ns0:col width="8.625" customWidth="1" style="24" min="7" max="26"/>
-  </ns0:cols>
-  <ns0:sheetData>
-    <ns0:row r="1" ht="15" customHeight="1" s="24"/>
-    <ns0:row r="2" ht="25.5" customHeight="1" s="24">
-      <ns0:c r="B2" s="1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>TỔNG HỢP SỬ DỤNG AI — TUẦN 07</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C2" s="2" t="n"/>
-      <ns0:c r="D2" s="2" t="n"/>
-      <ns0:c r="E2" s="2" t="n"/>
-      <ns0:c r="F2" s="2" t="n"/>
-    </ns0:row>
-    <ns0:row r="3" ht="19.5" customHeight="1" s="24">
-      <ns0:c r="A3" s="30" t="inlineStr">
-        <ns0:is>
-          <ns0:t>26/10/2026 – 01/11/2026</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B3" s="2" t="n"/>
-      <ns0:c r="C3" s="2" t="n"/>
-      <ns0:c r="D3" s="2" t="n"/>
-      <ns0:c r="E3" s="2" t="n"/>
-      <ns0:c r="F3" s="2" t="n"/>
-    </ns0:row>
-    <ns0:row r="4" ht="15" customHeight="1" s="24">
-      <ns0:c r="A4" s="2" t="n"/>
-      <ns0:c r="B4" s="2" t="n"/>
-      <ns0:c r="C4" s="2" t="n"/>
-      <ns0:c r="D4" s="2" t="n"/>
-      <ns0:c r="E4" s="2" t="n"/>
-      <ns0:c r="F4" s="2" t="n"/>
-    </ns0:row>
-    <ns0:row r="5" ht="33.75" customHeight="1" s="24">
-      <ns0:c r="A5" s="4" t="inlineStr">
-        <ns0:is>
-          <ns0:t>TỔNG SỐ PROMPT</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B5" s="5">
-        <ns0:f>SUM(B9:B11)</ns0:f>
-        <ns0:v>14</ns0:v>
-      </ns0:c>
-      <ns0:c r="C5" s="2" t="n"/>
-      <ns0:c r="D5" s="2" t="n"/>
-      <ns0:c r="E5" s="2" t="n"/>
-      <ns0:c r="F5" s="2" t="n"/>
-    </ns0:row>
-    <ns0:row r="6" ht="15" customHeight="1" s="24">
-      <ns0:c r="A6" s="2" t="n"/>
-      <ns0:c r="B6" s="2" t="n"/>
-      <ns0:c r="C6" s="2" t="n"/>
-      <ns0:c r="D6" s="2" t="n"/>
-      <ns0:c r="E6" s="2" t="n"/>
-      <ns0:c r="F6" s="2" t="n"/>
-    </ns0:row>
-    <ns0:row r="7" ht="15" customHeight="1" s="24">
-      <ns0:c r="A7" s="2" t="n"/>
-      <ns0:c r="B7" s="2" t="n"/>
-      <ns0:c r="C7" s="2" t="n"/>
-      <ns0:c r="D7" s="2" t="n"/>
-      <ns0:c r="E7" s="2" t="n"/>
-      <ns0:c r="F7" s="2" t="n"/>
-    </ns0:row>
-    <ns0:row r="8" ht="27.75" customHeight="1" s="24">
-      <ns0:c r="A8" s="4" t="inlineStr">
-        <ns0:is>
-          <ns0:t>NGƯỜI TẠO</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B8" s="4" t="inlineStr">
-        <ns0:is>
-          <ns0:t>SỐ PROMPT</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C8" s="2" t="n"/>
-      <ns0:c r="D8" s="10" t="inlineStr">
-        <ns0:is>
-          <ns0:t>TOOL AI</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="E8" s="10" t="inlineStr">
-        <ns0:is>
-          <ns0:t>SỐ PROMPT</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="F8" s="2" t="n"/>
-    </ns0:row>
-    <ns0:row r="9" ht="24.75" customHeight="1" s="24">
-      <ns0:c r="A9" s="11" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Thắng</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B9" s="13">
-        <ns0:f>COUNTIF(Thắng!$A$6:$A$306,"&lt;&gt;")</ns0:f>
-        <ns0:v>11</ns0:v>
-      </ns0:c>
-      <ns0:c r="C9" s="2" t="n"/>
-      <ns0:c r="D9" s="14" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Claude</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="E9" s="16">
-        <ns0:f>COUNTIFS(Thắng!$A$6:$A$306,"&lt;&gt;",Thắng!$C$6:$C$306,D9)+COUNTIFS(Sang!$A$6:$A$306,"&lt;&gt;",Sang!$C$6:$C$306,D9)+COUNTIFS(Nguyên!$A$6:$A$306,"&lt;&gt;",Nguyên!$C$6:$C$306,D9)</ns0:f>
-        <ns0:v>0</ns0:v>
-      </ns0:c>
-      <ns0:c r="F9" s="2" t="n"/>
-    </ns0:row>
-    <ns0:row r="10" ht="24.75" customHeight="1" s="24">
-      <ns0:c r="A10" s="11" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Sang</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B10" s="13">
-        <ns0:f>COUNTIF(Sang!$A$6:$A$306,"&lt;&gt;")</ns0:f>
-        <ns0:v>0</ns0:v>
-      </ns0:c>
-      <ns0:c r="C10" s="2" t="n"/>
-      <ns0:c r="D10" s="14" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Codex</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="E10" s="16">
-        <ns0:f>COUNTIFS(Thắng!$A$6:$A$306,"&lt;&gt;",Thắng!$C$6:$C$306,D10)+COUNTIFS(Sang!$A$6:$A$306,"&lt;&gt;",Sang!$C$6:$C$306,D10)+COUNTIFS(Nguyên!$A$6:$A$306,"&lt;&gt;",Nguyên!$C$6:$C$306,D10)</ns0:f>
-        <ns0:v>3</ns0:v>
-      </ns0:c>
-      <ns0:c r="F10" s="2" t="n"/>
-    </ns0:row>
-    <ns0:row r="11" ht="24.75" customHeight="1" s="24">
-      <ns0:c r="A11" s="11" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Nguyên</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B11" s="13">
-        <ns0:f>COUNTIF(Nguyên!$A$6:$A$306,"&lt;&gt;")</ns0:f>
-        <ns0:v>3</ns0:v>
-      </ns0:c>
-      <ns0:c r="C11" s="2" t="n"/>
-      <ns0:c r="D11" s="14" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Antigravity</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="E11" s="16">
-        <ns0:f>COUNTIFS(Thắng!$A$6:$A$306,"&lt;&gt;",Thắng!$C$6:$C$306,D11)+COUNTIFS(Sang!$A$6:$A$306,"&lt;&gt;",Sang!$C$6:$C$306,D11)+COUNTIFS(Nguyên!$A$6:$A$306,"&lt;&gt;",Nguyên!$C$6:$C$306,D11)</ns0:f>
-        <ns0:v>11</ns0:v>
-      </ns0:c>
-      <ns0:c r="F11" s="2" t="n"/>
-    </ns0:row>
-    <ns0:row r="12" ht="15" customHeight="1" s="24">
-      <ns0:c r="A12" s="2" t="n"/>
-      <ns0:c r="B12" s="2" t="n"/>
-      <ns0:c r="C12" s="2" t="n"/>
-      <ns0:c r="D12" s="2" t="n"/>
-      <ns0:c r="E12" s="2" t="n"/>
-      <ns0:c r="F12" s="2" t="n"/>
-    </ns0:row>
-    <ns0:row r="13" ht="15" customHeight="1" s="24">
-      <ns0:c r="A13" s="2" t="n"/>
-      <ns0:c r="B13" s="2" t="n"/>
-      <ns0:c r="C13" s="2" t="n"/>
-      <ns0:c r="D13" s="2" t="n"/>
-      <ns0:c r="E13" s="2" t="n"/>
-      <ns0:c r="F13" s="2" t="n"/>
-    </ns0:row>
-    <ns0:row r="14" ht="15" customHeight="1" s="24">
-      <ns0:c r="A14" s="17" t="n"/>
-      <ns0:c r="B14" s="2" t="n"/>
-      <ns0:c r="C14" s="2" t="n"/>
-      <ns0:c r="D14" s="2" t="n"/>
-      <ns0:c r="E14" s="2" t="n"/>
-      <ns0:c r="F14" s="2" t="n"/>
-    </ns0:row>
-    <ns0:row r="18" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="19" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="20" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="21" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="22" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="23" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="24" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="25" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="26" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="27" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="28" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="29" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="30" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="31" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="32" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="33" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="34" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="35" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="36" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="37" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="38" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="39" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="40" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="41" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="42" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="43" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="44" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="45" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="46" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="47" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="48" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="49" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="50" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="51" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="52" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="53" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="54" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="55" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="56" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="57" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="58" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="59" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="60" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="61" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="62" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="63" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="64" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="65" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="66" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="67" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="68" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="69" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="70" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="71" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="72" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="73" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="74" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="75" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="76" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="77" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="78" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="79" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="80" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="81" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="82" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="83" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="84" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="85" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="86" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="87" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="88" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="89" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="90" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="91" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="92" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="93" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="94" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="95" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="96" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="97" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="98" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="99" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="100" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="101" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="102" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="103" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="104" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="105" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="106" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="107" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="108" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="109" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="110" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="111" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="112" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="113" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="114" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="115" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="116" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="117" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="118" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="119" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="120" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="121" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="122" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="123" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="124" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="125" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="126" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="127" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="128" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="129" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="130" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="131" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="132" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="133" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="134" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="135" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="136" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="137" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="138" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="139" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="140" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="141" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="142" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="143" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="144" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="145" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="146" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="147" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="148" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="149" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="150" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="151" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="152" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="153" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="154" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="155" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="156" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="157" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="158" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="159" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="160" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="161" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="162" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="163" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="164" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="165" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="166" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="167" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="168" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="169" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="170" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="171" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="172" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="173" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="174" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="175" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="176" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="177" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="178" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="179" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="180" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="181" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="182" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="183" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="184" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="185" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="186" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="187" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="188" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="189" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="190" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="191" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="192" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="193" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="194" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="195" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="196" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="197" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="198" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="199" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="200" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="201" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="202" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="203" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="204" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="205" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="206" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="207" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="208" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="209" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="210" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="211" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="212" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="213" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="214" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="215" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="216" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="217" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="218" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="219" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="220" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="221" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="222" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="223" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="224" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="225" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="226" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="227" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="228" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="229" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="230" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="231" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="232" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="233" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="234" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="235" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="236" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="237" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="238" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="239" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="240" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="241" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="242" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="243" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="244" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="245" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="246" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="247" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="248" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="249" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="250" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="251" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="252" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="253" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="254" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="255" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="256" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="257" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="258" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="259" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="260" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="261" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="262" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="263" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="264" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="265" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="266" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="267" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="268" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="269" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="270" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="271" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="272" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="273" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="274" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="275" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="276" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="277" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="278" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="279" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="280" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="281" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="282" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="283" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="284" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="285" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="286" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="287" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="288" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="289" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="290" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="291" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="292" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="293" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="294" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="295" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="296" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="297" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="298" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="299" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="300" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="301" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="302" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="303" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="304" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="305" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="306" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="307" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="308" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="309" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="310" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="311" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="312" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="313" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="314" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="315" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="316" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="317" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="318" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="319" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="320" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="321" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="322" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="323" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="324" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="325" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="326" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="327" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="328" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="329" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="330" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="331" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="332" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="333" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="334" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="335" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="336" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="337" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="338" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="339" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="340" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="341" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="342" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="343" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="344" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="345" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="346" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="347" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="348" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="349" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="350" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="351" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="352" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="353" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="354" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="355" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="356" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="357" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="358" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="359" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="360" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="361" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="362" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="363" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="364" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="365" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="366" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="367" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="368" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="369" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="370" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="371" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="372" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="373" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="374" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="375" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="376" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="377" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="378" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="379" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="380" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="381" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="382" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="383" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="384" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="385" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="386" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="387" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="388" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="389" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="390" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="391" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="392" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="393" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="394" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="395" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="396" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="397" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="398" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="399" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="400" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="401" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="402" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="403" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="404" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="405" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="406" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="407" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="408" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="409" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="410" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="411" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="412" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="413" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="414" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="415" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="416" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="417" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="418" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="419" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="420" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="421" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="422" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="423" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="424" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="425" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="426" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="427" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="428" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="429" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="430" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="431" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="432" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="433" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="434" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="435" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="436" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="437" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="438" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="439" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="440" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="441" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="442" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="443" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="444" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="445" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="446" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="447" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="448" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="449" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="450" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="451" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="452" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="453" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="454" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="455" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="456" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="457" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="458" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="459" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="460" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="461" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="462" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="463" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="464" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="465" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="466" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="467" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="468" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="469" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="470" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="471" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="472" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="473" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="474" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="475" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="476" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="477" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="478" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="479" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="480" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="481" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="482" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="483" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="484" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="485" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="486" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="487" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="488" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="489" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="490" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="491" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="492" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="493" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="494" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="495" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="496" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="497" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="498" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="499" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="500" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="501" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="502" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="503" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="504" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="505" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="506" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="507" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="508" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="509" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="510" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="511" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="512" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="513" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="514" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="515" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="516" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="517" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="518" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="519" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="520" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="521" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="522" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="523" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="524" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="525" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="526" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="527" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="528" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="529" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="530" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="531" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="532" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="533" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="534" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="535" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="536" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="537" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="538" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="539" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="540" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="541" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="542" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="543" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="544" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="545" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="546" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="547" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="548" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="549" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="550" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="551" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="552" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="553" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="554" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="555" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="556" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="557" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="558" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="559" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="560" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="561" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="562" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="563" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="564" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="565" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="566" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="567" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="568" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="569" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="570" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="571" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="572" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="573" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="574" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="575" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="576" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="577" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="578" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="579" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="580" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="581" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="582" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="583" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="584" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="585" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="586" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="587" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="588" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="589" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="590" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="591" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="592" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="593" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="594" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="595" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="596" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="597" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="598" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="599" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="600" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="601" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="602" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="603" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="604" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="605" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="606" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="607" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="608" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="609" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="610" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="611" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="612" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="613" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="614" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="615" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="616" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="617" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="618" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="619" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="620" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="621" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="622" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="623" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="624" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="625" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="626" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="627" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="628" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="629" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="630" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="631" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="632" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="633" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="634" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="635" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="636" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="637" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="638" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="639" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="640" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="641" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="642" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="643" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="644" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="645" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="646" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="647" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="648" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="649" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="650" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="651" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="652" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="653" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="654" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="655" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="656" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="657" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="658" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="659" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="660" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="661" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="662" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="663" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="664" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="665" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="666" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="667" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="668" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="669" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="670" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="671" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="672" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="673" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="674" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="675" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="676" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="677" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="678" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="679" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="680" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="681" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="682" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="683" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="684" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="685" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="686" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="687" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="688" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="689" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="690" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="691" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="692" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="693" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="694" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="695" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="696" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="697" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="698" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="699" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="700" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="701" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="702" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="703" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="704" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="705" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="706" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="707" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="708" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="709" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="710" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="711" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="712" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="713" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="714" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="715" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="716" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="717" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="718" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="719" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="720" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="721" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="722" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="723" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="724" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="725" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="726" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="727" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="728" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="729" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="730" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="731" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="732" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="733" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="734" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="735" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="736" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="737" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="738" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="739" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="740" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="741" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="742" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="743" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="744" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="745" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="746" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="747" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="748" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="749" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="750" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="751" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="752" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="753" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="754" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="755" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="756" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="757" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="758" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="759" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="760" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="761" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="762" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="763" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="764" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="765" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="766" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="767" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="768" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="769" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="770" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="771" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="772" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="773" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="774" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="775" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="776" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="777" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="778" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="779" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="780" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="781" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="782" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="783" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="784" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="785" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="786" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="787" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="788" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="789" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="790" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="791" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="792" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="793" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="794" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="795" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="796" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="797" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="798" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="799" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="800" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="801" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="802" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="803" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="804" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="805" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="806" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="807" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="808" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="809" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="810" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="811" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="812" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="813" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="814" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="815" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="816" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="817" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="818" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="819" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="820" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="821" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="822" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="823" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="824" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="825" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="826" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="827" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="828" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="829" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="830" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="831" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="832" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="833" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="834" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="835" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="836" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="837" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="838" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="839" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="840" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="841" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="842" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="843" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="844" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="845" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="846" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="847" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="848" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="849" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="850" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="851" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="852" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="853" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="854" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="855" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="856" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="857" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="858" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="859" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="860" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="861" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="862" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="863" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="864" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="865" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="866" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="867" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="868" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="869" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="870" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="871" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="872" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="873" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="874" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="875" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="876" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="877" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="878" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="879" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="880" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="881" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="882" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="883" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="884" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="885" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="886" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="887" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="888" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="889" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="890" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="891" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="892" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="893" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="894" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="895" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="896" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="897" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="898" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="899" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="900" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="901" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="902" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="903" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="904" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="905" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="906" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="907" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="908" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="909" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="910" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="911" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="912" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="913" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="914" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="915" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="916" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="917" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="918" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="919" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="920" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="921" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="922" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="923" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="924" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="925" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="926" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="927" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="928" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="929" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="930" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="931" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="932" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="933" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="934" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="935" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="936" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="937" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="938" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="939" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="940" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="941" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="942" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="943" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="944" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="945" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="946" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="947" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="948" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="949" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="950" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="951" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="952" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="953" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="954" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="955" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="956" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="957" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="958" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="959" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="960" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="961" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="962" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="963" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="964" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="965" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="966" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="967" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="968" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="969" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="970" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="971" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="972" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="973" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="974" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="975" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="976" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="977" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="978" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="979" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="980" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="981" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="982" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="983" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="984" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="985" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="986" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="987" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="988" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="989" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="990" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="991" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="992" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="993" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="994" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="995" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="996" ht="15.75" customHeight="1" s="24"/>
-    <ns0:row r="997" ht="15.75" customHeight="1" s="24"/>
-  </ns0:sheetData>
-  <ns0:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</ns0:worksheet>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="FF17324D"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A2:F14"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.625" defaultRowHeight="14.25"/>
+  <cols>
+    <col width="24" customWidth="1" style="24" min="1" max="1"/>
+    <col width="15" customWidth="1" style="24" min="2" max="2"/>
+    <col width="4" customWidth="1" style="24" min="3" max="3"/>
+    <col width="24" customWidth="1" style="24" min="4" max="4"/>
+    <col width="15" customWidth="1" style="24" min="5" max="5"/>
+    <col width="8" customWidth="1" style="24" min="6" max="6"/>
+    <col width="8.625" customWidth="1" style="24" min="7" max="26"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="15" customHeight="1" s="24"/>
+    <row r="2" ht="25.5" customHeight="1" s="24">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>TỔNG HỢP SỬ DỤNG AI — TUẦN 07</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+    </row>
+    <row r="3" ht="19.5" customHeight="1" s="24">
+      <c r="A3" s="30" t="inlineStr">
+        <is>
+          <t>26/10/2026 – 01/11/2026</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n"/>
+      <c r="C3" s="2" t="n"/>
+      <c r="D3" s="2" t="n"/>
+      <c r="E3" s="2" t="n"/>
+      <c r="F3" s="2" t="n"/>
+    </row>
+    <row r="4" ht="15" customHeight="1" s="24">
+      <c r="A4" s="2" t="n"/>
+      <c r="B4" s="2" t="n"/>
+      <c r="C4" s="2" t="n"/>
+      <c r="D4" s="2" t="n"/>
+      <c r="E4" s="2" t="n"/>
+      <c r="F4" s="2" t="n"/>
+    </row>
+    <row r="5" ht="33.75" customHeight="1" s="24">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>TỔNG SỐ PROMPT</t>
+        </is>
+      </c>
+      <c r="B5" s="5">
+        <f>SUM(B9:B11)</f>
+        <v/>
+      </c>
+      <c r="C5" s="2" t="n"/>
+      <c r="D5" s="2" t="n"/>
+      <c r="E5" s="2" t="n"/>
+      <c r="F5" s="2" t="n"/>
+    </row>
+    <row r="6" ht="15" customHeight="1" s="24">
+      <c r="A6" s="2" t="n"/>
+      <c r="B6" s="2" t="n"/>
+      <c r="C6" s="2" t="n"/>
+      <c r="D6" s="2" t="n"/>
+      <c r="E6" s="2" t="n"/>
+      <c r="F6" s="2" t="n"/>
+    </row>
+    <row r="7" ht="15" customHeight="1" s="24">
+      <c r="A7" s="2" t="n"/>
+      <c r="B7" s="2" t="n"/>
+      <c r="C7" s="2" t="n"/>
+      <c r="D7" s="2" t="n"/>
+      <c r="E7" s="2" t="n"/>
+      <c r="F7" s="2" t="n"/>
+    </row>
+    <row r="8" ht="27.75" customHeight="1" s="24">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>NGƯỜI TẠO</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>SỐ PROMPT</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="n"/>
+      <c r="D8" s="10" t="inlineStr">
+        <is>
+          <t>TOOL AI</t>
+        </is>
+      </c>
+      <c r="E8" s="10" t="inlineStr">
+        <is>
+          <t>SỐ PROMPT</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="n"/>
+    </row>
+    <row r="9" ht="24.75" customHeight="1" s="24">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>Thắng</t>
+        </is>
+      </c>
+      <c r="B9" s="13">
+        <f>COUNTIF(Thắng!$A$6:$A$306,"&lt;&gt;")</f>
+        <v/>
+      </c>
+      <c r="C9" s="2" t="n"/>
+      <c r="D9" s="14" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="E9" s="16">
+        <f>COUNTIFS(Thắng!$A$6:$A$306,"&lt;&gt;",Thắng!$C$6:$C$306,D9)+COUNTIFS(Sang!$A$6:$A$306,"&lt;&gt;",Sang!$C$6:$C$306,D9)+COUNTIFS(Nguyên!$A$6:$A$306,"&lt;&gt;",Nguyên!$C$6:$C$306,D9)</f>
+        <v/>
+      </c>
+      <c r="F9" s="2" t="n"/>
+    </row>
+    <row r="10" ht="24.75" customHeight="1" s="24">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>Sang</t>
+        </is>
+      </c>
+      <c r="B10" s="13">
+        <f>COUNTIF(Sang!$A$6:$A$306,"&lt;&gt;")</f>
+        <v/>
+      </c>
+      <c r="C10" s="2" t="n"/>
+      <c r="D10" s="14" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="E10" s="16">
+        <f>COUNTIFS(Thắng!$A$6:$A$306,"&lt;&gt;",Thắng!$C$6:$C$306,D10)+COUNTIFS(Sang!$A$6:$A$306,"&lt;&gt;",Sang!$C$6:$C$306,D10)+COUNTIFS(Nguyên!$A$6:$A$306,"&lt;&gt;",Nguyên!$C$6:$C$306,D10)</f>
+        <v/>
+      </c>
+      <c r="F10" s="2" t="n"/>
+    </row>
+    <row r="11" ht="24.75" customHeight="1" s="24">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>Nguyên</t>
+        </is>
+      </c>
+      <c r="B11" s="13">
+        <f>COUNTIF(Nguyên!$A$6:$A$306,"&lt;&gt;")</f>
+        <v/>
+      </c>
+      <c r="C11" s="2" t="n"/>
+      <c r="D11" s="14" t="inlineStr">
+        <is>
+          <t>Antigravity</t>
+        </is>
+      </c>
+      <c r="E11" s="16">
+        <f>COUNTIFS(Thắng!$A$6:$A$306,"&lt;&gt;",Thắng!$C$6:$C$306,D11)+COUNTIFS(Sang!$A$6:$A$306,"&lt;&gt;",Sang!$C$6:$C$306,D11)+COUNTIFS(Nguyên!$A$6:$A$306,"&lt;&gt;",Nguyên!$C$6:$C$306,D11)</f>
+        <v/>
+      </c>
+      <c r="F11" s="2" t="n"/>
+    </row>
+    <row r="12" ht="15" customHeight="1" s="24">
+      <c r="A12" s="2" t="n"/>
+      <c r="B12" s="2" t="n"/>
+      <c r="C12" s="2" t="n"/>
+      <c r="D12" s="2" t="n"/>
+      <c r="E12" s="2" t="n"/>
+      <c r="F12" s="2" t="n"/>
+    </row>
+    <row r="13" ht="15" customHeight="1" s="24">
+      <c r="A13" s="2" t="n"/>
+      <c r="B13" s="2" t="n"/>
+      <c r="C13" s="2" t="n"/>
+      <c r="D13" s="2" t="n"/>
+      <c r="E13" s="2" t="n"/>
+      <c r="F13" s="2" t="n"/>
+    </row>
+    <row r="14" ht="15" customHeight="1" s="24">
+      <c r="A14" s="17" t="n"/>
+      <c r="B14" s="2" t="n"/>
+      <c r="C14" s="2" t="n"/>
+      <c r="D14" s="2" t="n"/>
+      <c r="E14" s="2" t="n"/>
+      <c r="F14" s="2" t="n"/>
+    </row>
+    <row r="18" ht="15.75" customHeight="1" s="24"/>
+    <row r="19" ht="15.75" customHeight="1" s="24"/>
+    <row r="20" ht="15.75" customHeight="1" s="24"/>
+    <row r="21" ht="15.75" customHeight="1" s="24"/>
+    <row r="22" ht="15.75" customHeight="1" s="24"/>
+    <row r="23" ht="15.75" customHeight="1" s="24"/>
+    <row r="24" ht="15.75" customHeight="1" s="24"/>
+    <row r="25" ht="15.75" customHeight="1" s="24"/>
+    <row r="26" ht="15.75" customHeight="1" s="24"/>
+    <row r="27" ht="15.75" customHeight="1" s="24"/>
+    <row r="28" ht="15.75" customHeight="1" s="24"/>
+    <row r="29" ht="15.75" customHeight="1" s="24"/>
+    <row r="30" ht="15.75" customHeight="1" s="24"/>
+    <row r="31" ht="15.75" customHeight="1" s="24"/>
+    <row r="32" ht="15.75" customHeight="1" s="24"/>
+    <row r="33" ht="15.75" customHeight="1" s="24"/>
+    <row r="34" ht="15.75" customHeight="1" s="24"/>
+    <row r="35" ht="15.75" customHeight="1" s="24"/>
+    <row r="36" ht="15.75" customHeight="1" s="24"/>
+    <row r="37" ht="15.75" customHeight="1" s="24"/>
+    <row r="38" ht="15.75" customHeight="1" s="24"/>
+    <row r="39" ht="15.75" customHeight="1" s="24"/>
+    <row r="40" ht="15.75" customHeight="1" s="24"/>
+    <row r="41" ht="15.75" customHeight="1" s="24"/>
+    <row r="42" ht="15.75" customHeight="1" s="24"/>
+    <row r="43" ht="15.75" customHeight="1" s="24"/>
+    <row r="44" ht="15.75" customHeight="1" s="24"/>
+    <row r="45" ht="15.75" customHeight="1" s="24"/>
+    <row r="46" ht="15.75" customHeight="1" s="24"/>
+    <row r="47" ht="15.75" customHeight="1" s="24"/>
+    <row r="48" ht="15.75" customHeight="1" s="24"/>
+    <row r="49" ht="15.75" customHeight="1" s="24"/>
+    <row r="50" ht="15.75" customHeight="1" s="24"/>
+    <row r="51" ht="15.75" customHeight="1" s="24"/>
+    <row r="52" ht="15.75" customHeight="1" s="24"/>
+    <row r="53" ht="15.75" customHeight="1" s="24"/>
+    <row r="54" ht="15.75" customHeight="1" s="24"/>
+    <row r="55" ht="15.75" customHeight="1" s="24"/>
+    <row r="56" ht="15.75" customHeight="1" s="24"/>
+    <row r="57" ht="15.75" customHeight="1" s="24"/>
+    <row r="58" ht="15.75" customHeight="1" s="24"/>
+    <row r="59" ht="15.75" customHeight="1" s="24"/>
+    <row r="60" ht="15.75" customHeight="1" s="24"/>
+    <row r="61" ht="15.75" customHeight="1" s="24"/>
+    <row r="62" ht="15.75" customHeight="1" s="24"/>
+    <row r="63" ht="15.75" customHeight="1" s="24"/>
+    <row r="64" ht="15.75" customHeight="1" s="24"/>
+    <row r="65" ht="15.75" customHeight="1" s="24"/>
+    <row r="66" ht="15.75" customHeight="1" s="24"/>
+    <row r="67" ht="15.75" customHeight="1" s="24"/>
+    <row r="68" ht="15.75" customHeight="1" s="24"/>
+    <row r="69" ht="15.75" customHeight="1" s="24"/>
+    <row r="70" ht="15.75" customHeight="1" s="24"/>
+    <row r="71" ht="15.75" customHeight="1" s="24"/>
+    <row r="72" ht="15.75" customHeight="1" s="24"/>
+    <row r="73" ht="15.75" customHeight="1" s="24"/>
+    <row r="74" ht="15.75" customHeight="1" s="24"/>
+    <row r="75" ht="15.75" customHeight="1" s="24"/>
+    <row r="76" ht="15.75" customHeight="1" s="24"/>
+    <row r="77" ht="15.75" customHeight="1" s="24"/>
+    <row r="78" ht="15.75" customHeight="1" s="24"/>
+    <row r="79" ht="15.75" customHeight="1" s="24"/>
+    <row r="80" ht="15.75" customHeight="1" s="24"/>
+    <row r="81" ht="15.75" customHeight="1" s="24"/>
+    <row r="82" ht="15.75" customHeight="1" s="24"/>
+    <row r="83" ht="15.75" customHeight="1" s="24"/>
+    <row r="84" ht="15.75" customHeight="1" s="24"/>
+    <row r="85" ht="15.75" customHeight="1" s="24"/>
+    <row r="86" ht="15.75" customHeight="1" s="24"/>
+    <row r="87" ht="15.75" customHeight="1" s="24"/>
+    <row r="88" ht="15.75" customHeight="1" s="24"/>
+    <row r="89" ht="15.75" customHeight="1" s="24"/>
+    <row r="90" ht="15.75" customHeight="1" s="24"/>
+    <row r="91" ht="15.75" customHeight="1" s="24"/>
+    <row r="92" ht="15.75" customHeight="1" s="24"/>
+    <row r="93" ht="15.75" customHeight="1" s="24"/>
+    <row r="94" ht="15.75" customHeight="1" s="24"/>
+    <row r="95" ht="15.75" customHeight="1" s="24"/>
+    <row r="96" ht="15.75" customHeight="1" s="24"/>
+    <row r="97" ht="15.75" customHeight="1" s="24"/>
+    <row r="98" ht="15.75" customHeight="1" s="24"/>
+    <row r="99" ht="15.75" customHeight="1" s="24"/>
+    <row r="100" ht="15.75" customHeight="1" s="24"/>
+    <row r="101" ht="15.75" customHeight="1" s="24"/>
+    <row r="102" ht="15.75" customHeight="1" s="24"/>
+    <row r="103" ht="15.75" customHeight="1" s="24"/>
+    <row r="104" ht="15.75" customHeight="1" s="24"/>
+    <row r="105" ht="15.75" customHeight="1" s="24"/>
+    <row r="106" ht="15.75" customHeight="1" s="24"/>
+    <row r="107" ht="15.75" customHeight="1" s="24"/>
+    <row r="108" ht="15.75" customHeight="1" s="24"/>
+    <row r="109" ht="15.75" customHeight="1" s="24"/>
+    <row r="110" ht="15.75" customHeight="1" s="24"/>
+    <row r="111" ht="15.75" customHeight="1" s="24"/>
+    <row r="112" ht="15.75" customHeight="1" s="24"/>
+    <row r="113" ht="15.75" customHeight="1" s="24"/>
+    <row r="114" ht="15.75" customHeight="1" s="24"/>
+    <row r="115" ht="15.75" customHeight="1" s="24"/>
+    <row r="116" ht="15.75" customHeight="1" s="24"/>
+    <row r="117" ht="15.75" customHeight="1" s="24"/>
+    <row r="118" ht="15.75" customHeight="1" s="24"/>
+    <row r="119" ht="15.75" customHeight="1" s="24"/>
+    <row r="120" ht="15.75" customHeight="1" s="24"/>
+    <row r="121" ht="15.75" customHeight="1" s="24"/>
+    <row r="122" ht="15.75" customHeight="1" s="24"/>
+    <row r="123" ht="15.75" customHeight="1" s="24"/>
+    <row r="124" ht="15.75" customHeight="1" s="24"/>
+    <row r="125" ht="15.75" customHeight="1" s="24"/>
+    <row r="126" ht="15.75" customHeight="1" s="24"/>
+    <row r="127" ht="15.75" customHeight="1" s="24"/>
+    <row r="128" ht="15.75" customHeight="1" s="24"/>
+    <row r="129" ht="15.75" customHeight="1" s="24"/>
+    <row r="130" ht="15.75" customHeight="1" s="24"/>
+    <row r="131" ht="15.75" customHeight="1" s="24"/>
+    <row r="132" ht="15.75" customHeight="1" s="24"/>
+    <row r="133" ht="15.75" customHeight="1" s="24"/>
+    <row r="134" ht="15.75" customHeight="1" s="24"/>
+    <row r="135" ht="15.75" customHeight="1" s="24"/>
+    <row r="136" ht="15.75" customHeight="1" s="24"/>
+    <row r="137" ht="15.75" customHeight="1" s="24"/>
+    <row r="138" ht="15.75" customHeight="1" s="24"/>
+    <row r="139" ht="15.75" customHeight="1" s="24"/>
+    <row r="140" ht="15.75" customHeight="1" s="24"/>
+    <row r="141" ht="15.75" customHeight="1" s="24"/>
+    <row r="142" ht="15.75" customHeight="1" s="24"/>
+    <row r="143" ht="15.75" customHeight="1" s="24"/>
+    <row r="144" ht="15.75" customHeight="1" s="24"/>
+    <row r="145" ht="15.75" customHeight="1" s="24"/>
+    <row r="146" ht="15.75" customHeight="1" s="24"/>
+    <row r="147" ht="15.75" customHeight="1" s="24"/>
+    <row r="148" ht="15.75" customHeight="1" s="24"/>
+    <row r="149" ht="15.75" customHeight="1" s="24"/>
+    <row r="150" ht="15.75" customHeight="1" s="24"/>
+    <row r="151" ht="15.75" customHeight="1" s="24"/>
+    <row r="152" ht="15.75" customHeight="1" s="24"/>
+    <row r="153" ht="15.75" customHeight="1" s="24"/>
+    <row r="154" ht="15.75" customHeight="1" s="24"/>
+    <row r="155" ht="15.75" customHeight="1" s="24"/>
+    <row r="156" ht="15.75" customHeight="1" s="24"/>
+    <row r="157" ht="15.75" customHeight="1" s="24"/>
+    <row r="158" ht="15.75" customHeight="1" s="24"/>
+    <row r="159" ht="15.75" customHeight="1" s="24"/>
+    <row r="160" ht="15.75" customHeight="1" s="24"/>
+    <row r="161" ht="15.75" customHeight="1" s="24"/>
+    <row r="162" ht="15.75" customHeight="1" s="24"/>
+    <row r="163" ht="15.75" customHeight="1" s="24"/>
+    <row r="164" ht="15.75" customHeight="1" s="24"/>
+    <row r="165" ht="15.75" customHeight="1" s="24"/>
+    <row r="166" ht="15.75" customHeight="1" s="24"/>
+    <row r="167" ht="15.75" customHeight="1" s="24"/>
+    <row r="168" ht="15.75" customHeight="1" s="24"/>
+    <row r="169" ht="15.75" customHeight="1" s="24"/>
+    <row r="170" ht="15.75" customHeight="1" s="24"/>
+    <row r="171" ht="15.75" customHeight="1" s="24"/>
+    <row r="172" ht="15.75" customHeight="1" s="24"/>
+    <row r="173" ht="15.75" customHeight="1" s="24"/>
+    <row r="174" ht="15.75" customHeight="1" s="24"/>
+    <row r="175" ht="15.75" customHeight="1" s="24"/>
+    <row r="176" ht="15.75" customHeight="1" s="24"/>
+    <row r="177" ht="15.75" customHeight="1" s="24"/>
+    <row r="178" ht="15.75" customHeight="1" s="24"/>
+    <row r="179" ht="15.75" customHeight="1" s="24"/>
+    <row r="180" ht="15.75" customHeight="1" s="24"/>
+    <row r="181" ht="15.75" customHeight="1" s="24"/>
+    <row r="182" ht="15.75" customHeight="1" s="24"/>
+    <row r="183" ht="15.75" customHeight="1" s="24"/>
+    <row r="184" ht="15.75" customHeight="1" s="24"/>
+    <row r="185" ht="15.75" customHeight="1" s="24"/>
+    <row r="186" ht="15.75" customHeight="1" s="24"/>
+    <row r="187" ht="15.75" customHeight="1" s="24"/>
+    <row r="188" ht="15.75" customHeight="1" s="24"/>
+    <row r="189" ht="15.75" customHeight="1" s="24"/>
+    <row r="190" ht="15.75" customHeight="1" s="24"/>
+    <row r="191" ht="15.75" customHeight="1" s="24"/>
+    <row r="192" ht="15.75" customHeight="1" s="24"/>
+    <row r="193" ht="15.75" customHeight="1" s="24"/>
+    <row r="194" ht="15.75" customHeight="1" s="24"/>
+    <row r="195" ht="15.75" customHeight="1" s="24"/>
+    <row r="196" ht="15.75" customHeight="1" s="24"/>
+    <row r="197" ht="15.75" customHeight="1" s="24"/>
+    <row r="198" ht="15.75" customHeight="1" s="24"/>
+    <row r="199" ht="15.75" customHeight="1" s="24"/>
+    <row r="200" ht="15.75" customHeight="1" s="24"/>
+    <row r="201" ht="15.75" customHeight="1" s="24"/>
+    <row r="202" ht="15.75" customHeight="1" s="24"/>
+    <row r="203" ht="15.75" customHeight="1" s="24"/>
+    <row r="204" ht="15.75" customHeight="1" s="24"/>
+    <row r="205" ht="15.75" customHeight="1" s="24"/>
+    <row r="206" ht="15.75" customHeight="1" s="24"/>
+    <row r="207" ht="15.75" customHeight="1" s="24"/>
+    <row r="208" ht="15.75" customHeight="1" s="24"/>
+    <row r="209" ht="15.75" customHeight="1" s="24"/>
+    <row r="210" ht="15.75" customHeight="1" s="24"/>
+    <row r="211" ht="15.75" customHeight="1" s="24"/>
+    <row r="212" ht="15.75" customHeight="1" s="24"/>
+    <row r="213" ht="15.75" customHeight="1" s="24"/>
+    <row r="214" ht="15.75" customHeight="1" s="24"/>
+    <row r="215" ht="15.75" customHeight="1" s="24"/>
+    <row r="216" ht="15.75" customHeight="1" s="24"/>
+    <row r="217" ht="15.75" customHeight="1" s="24"/>
+    <row r="218" ht="15.75" customHeight="1" s="24"/>
+    <row r="219" ht="15.75" customHeight="1" s="24"/>
+    <row r="220" ht="15.75" customHeight="1" s="24"/>
+    <row r="221" ht="15.75" customHeight="1" s="24"/>
+    <row r="222" ht="15.75" customHeight="1" s="24"/>
+    <row r="223" ht="15.75" customHeight="1" s="24"/>
+    <row r="224" ht="15.75" customHeight="1" s="24"/>
+    <row r="225" ht="15.75" customHeight="1" s="24"/>
+    <row r="226" ht="15.75" customHeight="1" s="24"/>
+    <row r="227" ht="15.75" customHeight="1" s="24"/>
+    <row r="228" ht="15.75" customHeight="1" s="24"/>
+    <row r="229" ht="15.75" customHeight="1" s="24"/>
+    <row r="230" ht="15.75" customHeight="1" s="24"/>
+    <row r="231" ht="15.75" customHeight="1" s="24"/>
+    <row r="232" ht="15.75" customHeight="1" s="24"/>
+    <row r="233" ht="15.75" customHeight="1" s="24"/>
+    <row r="234" ht="15.75" customHeight="1" s="24"/>
+    <row r="235" ht="15.75" customHeight="1" s="24"/>
+    <row r="236" ht="15.75" customHeight="1" s="24"/>
+    <row r="237" ht="15.75" customHeight="1" s="24"/>
+    <row r="238" ht="15.75" customHeight="1" s="24"/>
+    <row r="239" ht="15.75" customHeight="1" s="24"/>
+    <row r="240" ht="15.75" customHeight="1" s="24"/>
+    <row r="241" ht="15.75" customHeight="1" s="24"/>
+    <row r="242" ht="15.75" customHeight="1" s="24"/>
+    <row r="243" ht="15.75" customHeight="1" s="24"/>
+    <row r="244" ht="15.75" customHeight="1" s="24"/>
+    <row r="245" ht="15.75" customHeight="1" s="24"/>
+    <row r="246" ht="15.75" customHeight="1" s="24"/>
+    <row r="247" ht="15.75" customHeight="1" s="24"/>
+    <row r="248" ht="15.75" customHeight="1" s="24"/>
+    <row r="249" ht="15.75" customHeight="1" s="24"/>
+    <row r="250" ht="15.75" customHeight="1" s="24"/>
+    <row r="251" ht="15.75" customHeight="1" s="24"/>
+    <row r="252" ht="15.75" customHeight="1" s="24"/>
+    <row r="253" ht="15.75" customHeight="1" s="24"/>
+    <row r="254" ht="15.75" customHeight="1" s="24"/>
+    <row r="255" ht="15.75" customHeight="1" s="24"/>
+    <row r="256" ht="15.75" customHeight="1" s="24"/>
+    <row r="257" ht="15.75" customHeight="1" s="24"/>
+    <row r="258" ht="15.75" customHeight="1" s="24"/>
+    <row r="259" ht="15.75" customHeight="1" s="24"/>
+    <row r="260" ht="15.75" customHeight="1" s="24"/>
+    <row r="261" ht="15.75" customHeight="1" s="24"/>
+    <row r="262" ht="15.75" customHeight="1" s="24"/>
+    <row r="263" ht="15.75" customHeight="1" s="24"/>
+    <row r="264" ht="15.75" customHeight="1" s="24"/>
+    <row r="265" ht="15.75" customHeight="1" s="24"/>
+    <row r="266" ht="15.75" customHeight="1" s="24"/>
+    <row r="267" ht="15.75" customHeight="1" s="24"/>
+    <row r="268" ht="15.75" customHeight="1" s="24"/>
+    <row r="269" ht="15.75" customHeight="1" s="24"/>
+    <row r="270" ht="15.75" customHeight="1" s="24"/>
+    <row r="271" ht="15.75" customHeight="1" s="24"/>
+    <row r="272" ht="15.75" customHeight="1" s="24"/>
+    <row r="273" ht="15.75" customHeight="1" s="24"/>
+    <row r="274" ht="15.75" customHeight="1" s="24"/>
+    <row r="275" ht="15.75" customHeight="1" s="24"/>
+    <row r="276" ht="15.75" customHeight="1" s="24"/>
+    <row r="277" ht="15.75" customHeight="1" s="24"/>
+    <row r="278" ht="15.75" customHeight="1" s="24"/>
+    <row r="279" ht="15.75" customHeight="1" s="24"/>
+    <row r="280" ht="15.75" customHeight="1" s="24"/>
+    <row r="281" ht="15.75" customHeight="1" s="24"/>
+    <row r="282" ht="15.75" customHeight="1" s="24"/>
+    <row r="283" ht="15.75" customHeight="1" s="24"/>
+    <row r="284" ht="15.75" customHeight="1" s="24"/>
+    <row r="285" ht="15.75" customHeight="1" s="24"/>
+    <row r="286" ht="15.75" customHeight="1" s="24"/>
+    <row r="287" ht="15.75" customHeight="1" s="24"/>
+    <row r="288" ht="15.75" customHeight="1" s="24"/>
+    <row r="289" ht="15.75" customHeight="1" s="24"/>
+    <row r="290" ht="15.75" customHeight="1" s="24"/>
+    <row r="291" ht="15.75" customHeight="1" s="24"/>
+    <row r="292" ht="15.75" customHeight="1" s="24"/>
+    <row r="293" ht="15.75" customHeight="1" s="24"/>
+    <row r="294" ht="15.75" customHeight="1" s="24"/>
+    <row r="295" ht="15.75" customHeight="1" s="24"/>
+    <row r="296" ht="15.75" customHeight="1" s="24"/>
+    <row r="297" ht="15.75" customHeight="1" s="24"/>
+    <row r="298" ht="15.75" customHeight="1" s="24"/>
+    <row r="299" ht="15.75" customHeight="1" s="24"/>
+    <row r="300" ht="15.75" customHeight="1" s="24"/>
+    <row r="301" ht="15.75" customHeight="1" s="24"/>
+    <row r="302" ht="15.75" customHeight="1" s="24"/>
+    <row r="303" ht="15.75" customHeight="1" s="24"/>
+    <row r="304" ht="15.75" customHeight="1" s="24"/>
+    <row r="305" ht="15.75" customHeight="1" s="24"/>
+    <row r="306" ht="15.75" customHeight="1" s="24"/>
+    <row r="307" ht="15.75" customHeight="1" s="24"/>
+    <row r="308" ht="15.75" customHeight="1" s="24"/>
+    <row r="309" ht="15.75" customHeight="1" s="24"/>
+    <row r="310" ht="15.75" customHeight="1" s="24"/>
+    <row r="311" ht="15.75" customHeight="1" s="24"/>
+    <row r="312" ht="15.75" customHeight="1" s="24"/>
+    <row r="313" ht="15.75" customHeight="1" s="24"/>
+    <row r="314" ht="15.75" customHeight="1" s="24"/>
+    <row r="315" ht="15.75" customHeight="1" s="24"/>
+    <row r="316" ht="15.75" customHeight="1" s="24"/>
+    <row r="317" ht="15.75" customHeight="1" s="24"/>
+    <row r="318" ht="15.75" customHeight="1" s="24"/>
+    <row r="319" ht="15.75" customHeight="1" s="24"/>
+    <row r="320" ht="15.75" customHeight="1" s="24"/>
+    <row r="321" ht="15.75" customHeight="1" s="24"/>
+    <row r="322" ht="15.75" customHeight="1" s="24"/>
+    <row r="323" ht="15.75" customHeight="1" s="24"/>
+    <row r="324" ht="15.75" customHeight="1" s="24"/>
+    <row r="325" ht="15.75" customHeight="1" s="24"/>
+    <row r="326" ht="15.75" customHeight="1" s="24"/>
+    <row r="327" ht="15.75" customHeight="1" s="24"/>
+    <row r="328" ht="15.75" customHeight="1" s="24"/>
+    <row r="329" ht="15.75" customHeight="1" s="24"/>
+    <row r="330" ht="15.75" customHeight="1" s="24"/>
+    <row r="331" ht="15.75" customHeight="1" s="24"/>
+    <row r="332" ht="15.75" customHeight="1" s="24"/>
+    <row r="333" ht="15.75" customHeight="1" s="24"/>
+    <row r="334" ht="15.75" customHeight="1" s="24"/>
+    <row r="335" ht="15.75" customHeight="1" s="24"/>
+    <row r="336" ht="15.75" customHeight="1" s="24"/>
+    <row r="337" ht="15.75" customHeight="1" s="24"/>
+    <row r="338" ht="15.75" customHeight="1" s="24"/>
+    <row r="339" ht="15.75" customHeight="1" s="24"/>
+    <row r="340" ht="15.75" customHeight="1" s="24"/>
+    <row r="341" ht="15.75" customHeight="1" s="24"/>
+    <row r="342" ht="15.75" customHeight="1" s="24"/>
+    <row r="343" ht="15.75" customHeight="1" s="24"/>
+    <row r="344" ht="15.75" customHeight="1" s="24"/>
+    <row r="345" ht="15.75" customHeight="1" s="24"/>
+    <row r="346" ht="15.75" customHeight="1" s="24"/>
+    <row r="347" ht="15.75" customHeight="1" s="24"/>
+    <row r="348" ht="15.75" customHeight="1" s="24"/>
+    <row r="349" ht="15.75" customHeight="1" s="24"/>
+    <row r="350" ht="15.75" customHeight="1" s="24"/>
+    <row r="351" ht="15.75" customHeight="1" s="24"/>
+    <row r="352" ht="15.75" customHeight="1" s="24"/>
+    <row r="353" ht="15.75" customHeight="1" s="24"/>
+    <row r="354" ht="15.75" customHeight="1" s="24"/>
+    <row r="355" ht="15.75" customHeight="1" s="24"/>
+    <row r="356" ht="15.75" customHeight="1" s="24"/>
+    <row r="357" ht="15.75" customHeight="1" s="24"/>
+    <row r="358" ht="15.75" customHeight="1" s="24"/>
+    <row r="359" ht="15.75" customHeight="1" s="24"/>
+    <row r="360" ht="15.75" customHeight="1" s="24"/>
+    <row r="361" ht="15.75" customHeight="1" s="24"/>
+    <row r="362" ht="15.75" customHeight="1" s="24"/>
+    <row r="363" ht="15.75" customHeight="1" s="24"/>
+    <row r="364" ht="15.75" customHeight="1" s="24"/>
+    <row r="365" ht="15.75" customHeight="1" s="24"/>
+    <row r="366" ht="15.75" customHeight="1" s="24"/>
+    <row r="367" ht="15.75" customHeight="1" s="24"/>
+    <row r="368" ht="15.75" customHeight="1" s="24"/>
+    <row r="369" ht="15.75" customHeight="1" s="24"/>
+    <row r="370" ht="15.75" customHeight="1" s="24"/>
+    <row r="371" ht="15.75" customHeight="1" s="24"/>
+    <row r="372" ht="15.75" customHeight="1" s="24"/>
+    <row r="373" ht="15.75" customHeight="1" s="24"/>
+    <row r="374" ht="15.75" customHeight="1" s="24"/>
+    <row r="375" ht="15.75" customHeight="1" s="24"/>
+    <row r="376" ht="15.75" customHeight="1" s="24"/>
+    <row r="377" ht="15.75" customHeight="1" s="24"/>
+    <row r="378" ht="15.75" customHeight="1" s="24"/>
+    <row r="379" ht="15.75" customHeight="1" s="24"/>
+    <row r="380" ht="15.75" customHeight="1" s="24"/>
+    <row r="381" ht="15.75" customHeight="1" s="24"/>
+    <row r="382" ht="15.75" customHeight="1" s="24"/>
+    <row r="383" ht="15.75" customHeight="1" s="24"/>
+    <row r="384" ht="15.75" customHeight="1" s="24"/>
+    <row r="385" ht="15.75" customHeight="1" s="24"/>
+    <row r="386" ht="15.75" customHeight="1" s="24"/>
+    <row r="387" ht="15.75" customHeight="1" s="24"/>
+    <row r="388" ht="15.75" customHeight="1" s="24"/>
+    <row r="389" ht="15.75" customHeight="1" s="24"/>
+    <row r="390" ht="15.75" customHeight="1" s="24"/>
+    <row r="391" ht="15.75" customHeight="1" s="24"/>
+    <row r="392" ht="15.75" customHeight="1" s="24"/>
+    <row r="393" ht="15.75" customHeight="1" s="24"/>
+    <row r="394" ht="15.75" customHeight="1" s="24"/>
+    <row r="395" ht="15.75" customHeight="1" s="24"/>
+    <row r="396" ht="15.75" customHeight="1" s="24"/>
+    <row r="397" ht="15.75" customHeight="1" s="24"/>
+    <row r="398" ht="15.75" customHeight="1" s="24"/>
+    <row r="399" ht="15.75" customHeight="1" s="24"/>
+    <row r="400" ht="15.75" customHeight="1" s="24"/>
+    <row r="401" ht="15.75" customHeight="1" s="24"/>
+    <row r="402" ht="15.75" customHeight="1" s="24"/>
+    <row r="403" ht="15.75" customHeight="1" s="24"/>
+    <row r="404" ht="15.75" customHeight="1" s="24"/>
+    <row r="405" ht="15.75" customHeight="1" s="24"/>
+    <row r="406" ht="15.75" customHeight="1" s="24"/>
+    <row r="407" ht="15.75" customHeight="1" s="24"/>
+    <row r="408" ht="15.75" customHeight="1" s="24"/>
+    <row r="409" ht="15.75" customHeight="1" s="24"/>
+    <row r="410" ht="15.75" customHeight="1" s="24"/>
+    <row r="411" ht="15.75" customHeight="1" s="24"/>
+    <row r="412" ht="15.75" customHeight="1" s="24"/>
+    <row r="413" ht="15.75" customHeight="1" s="24"/>
+    <row r="414" ht="15.75" customHeight="1" s="24"/>
+    <row r="415" ht="15.75" customHeight="1" s="24"/>
+    <row r="416" ht="15.75" customHeight="1" s="24"/>
+    <row r="417" ht="15.75" customHeight="1" s="24"/>
+    <row r="418" ht="15.75" customHeight="1" s="24"/>
+    <row r="419" ht="15.75" customHeight="1" s="24"/>
+    <row r="420" ht="15.75" customHeight="1" s="24"/>
+    <row r="421" ht="15.75" customHeight="1" s="24"/>
+    <row r="422" ht="15.75" customHeight="1" s="24"/>
+    <row r="423" ht="15.75" customHeight="1" s="24"/>
+    <row r="424" ht="15.75" customHeight="1" s="24"/>
+    <row r="425" ht="15.75" customHeight="1" s="24"/>
+    <row r="426" ht="15.75" customHeight="1" s="24"/>
+    <row r="427" ht="15.75" customHeight="1" s="24"/>
+    <row r="428" ht="15.75" customHeight="1" s="24"/>
+    <row r="429" ht="15.75" customHeight="1" s="24"/>
+    <row r="430" ht="15.75" customHeight="1" s="24"/>
+    <row r="431" ht="15.75" customHeight="1" s="24"/>
+    <row r="432" ht="15.75" customHeight="1" s="24"/>
+    <row r="433" ht="15.75" customHeight="1" s="24"/>
+    <row r="434" ht="15.75" customHeight="1" s="24"/>
+    <row r="435" ht="15.75" customHeight="1" s="24"/>
+    <row r="436" ht="15.75" customHeight="1" s="24"/>
+    <row r="437" ht="15.75" customHeight="1" s="24"/>
+    <row r="438" ht="15.75" customHeight="1" s="24"/>
+    <row r="439" ht="15.75" customHeight="1" s="24"/>
+    <row r="440" ht="15.75" customHeight="1" s="24"/>
+    <row r="441" ht="15.75" customHeight="1" s="24"/>
+    <row r="442" ht="15.75" customHeight="1" s="24"/>
+    <row r="443" ht="15.75" customHeight="1" s="24"/>
+    <row r="444" ht="15.75" customHeight="1" s="24"/>
+    <row r="445" ht="15.75" customHeight="1" s="24"/>
+    <row r="446" ht="15.75" customHeight="1" s="24"/>
+    <row r="447" ht="15.75" customHeight="1" s="24"/>
+    <row r="448" ht="15.75" customHeight="1" s="24"/>
+    <row r="449" ht="15.75" customHeight="1" s="24"/>
+    <row r="450" ht="15.75" customHeight="1" s="24"/>
+    <row r="451" ht="15.75" customHeight="1" s="24"/>
+    <row r="452" ht="15.75" customHeight="1" s="24"/>
+    <row r="453" ht="15.75" customHeight="1" s="24"/>
+    <row r="454" ht="15.75" customHeight="1" s="24"/>
+    <row r="455" ht="15.75" customHeight="1" s="24"/>
+    <row r="456" ht="15.75" customHeight="1" s="24"/>
+    <row r="457" ht="15.75" customHeight="1" s="24"/>
+    <row r="458" ht="15.75" customHeight="1" s="24"/>
+    <row r="459" ht="15.75" customHeight="1" s="24"/>
+    <row r="460" ht="15.75" customHeight="1" s="24"/>
+    <row r="461" ht="15.75" customHeight="1" s="24"/>
+    <row r="462" ht="15.75" customHeight="1" s="24"/>
+    <row r="463" ht="15.75" customHeight="1" s="24"/>
+    <row r="464" ht="15.75" customHeight="1" s="24"/>
+    <row r="465" ht="15.75" customHeight="1" s="24"/>
+    <row r="466" ht="15.75" customHeight="1" s="24"/>
+    <row r="467" ht="15.75" customHeight="1" s="24"/>
+    <row r="468" ht="15.75" customHeight="1" s="24"/>
+    <row r="469" ht="15.75" customHeight="1" s="24"/>
+    <row r="470" ht="15.75" customHeight="1" s="24"/>
+    <row r="471" ht="15.75" customHeight="1" s="24"/>
+    <row r="472" ht="15.75" customHeight="1" s="24"/>
+    <row r="473" ht="15.75" customHeight="1" s="24"/>
+    <row r="474" ht="15.75" customHeight="1" s="24"/>
+    <row r="475" ht="15.75" customHeight="1" s="24"/>
+    <row r="476" ht="15.75" customHeight="1" s="24"/>
+    <row r="477" ht="15.75" customHeight="1" s="24"/>
+    <row r="478" ht="15.75" customHeight="1" s="24"/>
+    <row r="479" ht="15.75" customHeight="1" s="24"/>
+    <row r="480" ht="15.75" customHeight="1" s="24"/>
+    <row r="481" ht="15.75" customHeight="1" s="24"/>
+    <row r="482" ht="15.75" customHeight="1" s="24"/>
+    <row r="483" ht="15.75" customHeight="1" s="24"/>
+    <row r="484" ht="15.75" customHeight="1" s="24"/>
+    <row r="485" ht="15.75" customHeight="1" s="24"/>
+    <row r="486" ht="15.75" customHeight="1" s="24"/>
+    <row r="487" ht="15.75" customHeight="1" s="24"/>
+    <row r="488" ht="15.75" customHeight="1" s="24"/>
+    <row r="489" ht="15.75" customHeight="1" s="24"/>
+    <row r="490" ht="15.75" customHeight="1" s="24"/>
+    <row r="491" ht="15.75" customHeight="1" s="24"/>
+    <row r="492" ht="15.75" customHeight="1" s="24"/>
+    <row r="493" ht="15.75" customHeight="1" s="24"/>
+    <row r="494" ht="15.75" customHeight="1" s="24"/>
+    <row r="495" ht="15.75" customHeight="1" s="24"/>
+    <row r="496" ht="15.75" customHeight="1" s="24"/>
+    <row r="497" ht="15.75" customHeight="1" s="24"/>
+    <row r="498" ht="15.75" customHeight="1" s="24"/>
+    <row r="499" ht="15.75" customHeight="1" s="24"/>
+    <row r="500" ht="15.75" customHeight="1" s="24"/>
+    <row r="501" ht="15.75" customHeight="1" s="24"/>
+    <row r="502" ht="15.75" customHeight="1" s="24"/>
+    <row r="503" ht="15.75" customHeight="1" s="24"/>
+    <row r="504" ht="15.75" customHeight="1" s="24"/>
+    <row r="505" ht="15.75" customHeight="1" s="24"/>
+    <row r="506" ht="15.75" customHeight="1" s="24"/>
+    <row r="507" ht="15.75" customHeight="1" s="24"/>
+    <row r="508" ht="15.75" customHeight="1" s="24"/>
+    <row r="509" ht="15.75" customHeight="1" s="24"/>
+    <row r="510" ht="15.75" customHeight="1" s="24"/>
+    <row r="511" ht="15.75" customHeight="1" s="24"/>
+    <row r="512" ht="15.75" customHeight="1" s="24"/>
+    <row r="513" ht="15.75" customHeight="1" s="24"/>
+    <row r="514" ht="15.75" customHeight="1" s="24"/>
+    <row r="515" ht="15.75" customHeight="1" s="24"/>
+    <row r="516" ht="15.75" customHeight="1" s="24"/>
+    <row r="517" ht="15.75" customHeight="1" s="24"/>
+    <row r="518" ht="15.75" customHeight="1" s="24"/>
+    <row r="519" ht="15.75" customHeight="1" s="24"/>
+    <row r="520" ht="15.75" customHeight="1" s="24"/>
+    <row r="521" ht="15.75" customHeight="1" s="24"/>
+    <row r="522" ht="15.75" customHeight="1" s="24"/>
+    <row r="523" ht="15.75" customHeight="1" s="24"/>
+    <row r="524" ht="15.75" customHeight="1" s="24"/>
+    <row r="525" ht="15.75" customHeight="1" s="24"/>
+    <row r="526" ht="15.75" customHeight="1" s="24"/>
+    <row r="527" ht="15.75" customHeight="1" s="24"/>
+    <row r="528" ht="15.75" customHeight="1" s="24"/>
+    <row r="529" ht="15.75" customHeight="1" s="24"/>
+    <row r="530" ht="15.75" customHeight="1" s="24"/>
+    <row r="531" ht="15.75" customHeight="1" s="24"/>
+    <row r="532" ht="15.75" customHeight="1" s="24"/>
+    <row r="533" ht="15.75" customHeight="1" s="24"/>
+    <row r="534" ht="15.75" customHeight="1" s="24"/>
+    <row r="535" ht="15.75" customHeight="1" s="24"/>
+    <row r="536" ht="15.75" customHeight="1" s="24"/>
+    <row r="537" ht="15.75" customHeight="1" s="24"/>
+    <row r="538" ht="15.75" customHeight="1" s="24"/>
+    <row r="539" ht="15.75" customHeight="1" s="24"/>
+    <row r="540" ht="15.75" customHeight="1" s="24"/>
+    <row r="541" ht="15.75" customHeight="1" s="24"/>
+    <row r="542" ht="15.75" customHeight="1" s="24"/>
+    <row r="543" ht="15.75" customHeight="1" s="24"/>
+    <row r="544" ht="15.75" customHeight="1" s="24"/>
+    <row r="545" ht="15.75" customHeight="1" s="24"/>
+    <row r="546" ht="15.75" customHeight="1" s="24"/>
+    <row r="547" ht="15.75" customHeight="1" s="24"/>
+    <row r="548" ht="15.75" customHeight="1" s="24"/>
+    <row r="549" ht="15.75" customHeight="1" s="24"/>
+    <row r="550" ht="15.75" customHeight="1" s="24"/>
+    <row r="551" ht="15.75" customHeight="1" s="24"/>
+    <row r="552" ht="15.75" customHeight="1" s="24"/>
+    <row r="553" ht="15.75" customHeight="1" s="24"/>
+    <row r="554" ht="15.75" customHeight="1" s="24"/>
+    <row r="555" ht="15.75" customHeight="1" s="24"/>
+    <row r="556" ht="15.75" customHeight="1" s="24"/>
+    <row r="557" ht="15.75" customHeight="1" s="24"/>
+    <row r="558" ht="15.75" customHeight="1" s="24"/>
+    <row r="559" ht="15.75" customHeight="1" s="24"/>
+    <row r="560" ht="15.75" customHeight="1" s="24"/>
+    <row r="561" ht="15.75" customHeight="1" s="24"/>
+    <row r="562" ht="15.75" customHeight="1" s="24"/>
+    <row r="563" ht="15.75" customHeight="1" s="24"/>
+    <row r="564" ht="15.75" customHeight="1" s="24"/>
+    <row r="565" ht="15.75" customHeight="1" s="24"/>
+    <row r="566" ht="15.75" customHeight="1" s="24"/>
+    <row r="567" ht="15.75" customHeight="1" s="24"/>
+    <row r="568" ht="15.75" customHeight="1" s="24"/>
+    <row r="569" ht="15.75" customHeight="1" s="24"/>
+    <row r="570" ht="15.75" customHeight="1" s="24"/>
+    <row r="571" ht="15.75" customHeight="1" s="24"/>
+    <row r="572" ht="15.75" customHeight="1" s="24"/>
+    <row r="573" ht="15.75" customHeight="1" s="24"/>
+    <row r="574" ht="15.75" customHeight="1" s="24"/>
+    <row r="575" ht="15.75" customHeight="1" s="24"/>
+    <row r="576" ht="15.75" customHeight="1" s="24"/>
+    <row r="577" ht="15.75" customHeight="1" s="24"/>
+    <row r="578" ht="15.75" customHeight="1" s="24"/>
+    <row r="579" ht="15.75" customHeight="1" s="24"/>
+    <row r="580" ht="15.75" customHeight="1" s="24"/>
+    <row r="581" ht="15.75" customHeight="1" s="24"/>
+    <row r="582" ht="15.75" customHeight="1" s="24"/>
+    <row r="583" ht="15.75" customHeight="1" s="24"/>
+    <row r="584" ht="15.75" customHeight="1" s="24"/>
+    <row r="585" ht="15.75" customHeight="1" s="24"/>
+    <row r="586" ht="15.75" customHeight="1" s="24"/>
+    <row r="587" ht="15.75" customHeight="1" s="24"/>
+    <row r="588" ht="15.75" customHeight="1" s="24"/>
+    <row r="589" ht="15.75" customHeight="1" s="24"/>
+    <row r="590" ht="15.75" customHeight="1" s="24"/>
+    <row r="591" ht="15.75" customHeight="1" s="24"/>
+    <row r="592" ht="15.75" customHeight="1" s="24"/>
+    <row r="593" ht="15.75" customHeight="1" s="24"/>
+    <row r="594" ht="15.75" customHeight="1" s="24"/>
+    <row r="595" ht="15.75" customHeight="1" s="24"/>
+    <row r="596" ht="15.75" customHeight="1" s="24"/>
+    <row r="597" ht="15.75" customHeight="1" s="24"/>
+    <row r="598" ht="15.75" customHeight="1" s="24"/>
+    <row r="599" ht="15.75" customHeight="1" s="24"/>
+    <row r="600" ht="15.75" customHeight="1" s="24"/>
+    <row r="601" ht="15.75" customHeight="1" s="24"/>
+    <row r="602" ht="15.75" customHeight="1" s="24"/>
+    <row r="603" ht="15.75" customHeight="1" s="24"/>
+    <row r="604" ht="15.75" customHeight="1" s="24"/>
+    <row r="605" ht="15.75" customHeight="1" s="24"/>
+    <row r="606" ht="15.75" customHeight="1" s="24"/>
+    <row r="607" ht="15.75" customHeight="1" s="24"/>
+    <row r="608" ht="15.75" customHeight="1" s="24"/>
+    <row r="609" ht="15.75" customHeight="1" s="24"/>
+    <row r="610" ht="15.75" customHeight="1" s="24"/>
+    <row r="611" ht="15.75" customHeight="1" s="24"/>
+    <row r="612" ht="15.75" customHeight="1" s="24"/>
+    <row r="613" ht="15.75" customHeight="1" s="24"/>
+    <row r="614" ht="15.75" customHeight="1" s="24"/>
+    <row r="615" ht="15.75" customHeight="1" s="24"/>
+    <row r="616" ht="15.75" customHeight="1" s="24"/>
+    <row r="617" ht="15.75" customHeight="1" s="24"/>
+    <row r="618" ht="15.75" customHeight="1" s="24"/>
+    <row r="619" ht="15.75" customHeight="1" s="24"/>
+    <row r="620" ht="15.75" customHeight="1" s="24"/>
+    <row r="621" ht="15.75" customHeight="1" s="24"/>
+    <row r="622" ht="15.75" customHeight="1" s="24"/>
+    <row r="623" ht="15.75" customHeight="1" s="24"/>
+    <row r="624" ht="15.75" customHeight="1" s="24"/>
+    <row r="625" ht="15.75" customHeight="1" s="24"/>
+    <row r="626" ht="15.75" customHeight="1" s="24"/>
+    <row r="627" ht="15.75" customHeight="1" s="24"/>
+    <row r="628" ht="15.75" customHeight="1" s="24"/>
+    <row r="629" ht="15.75" customHeight="1" s="24"/>
+    <row r="630" ht="15.75" customHeight="1" s="24"/>
+    <row r="631" ht="15.75" customHeight="1" s="24"/>
+    <row r="632" ht="15.75" customHeight="1" s="24"/>
+    <row r="633" ht="15.75" customHeight="1" s="24"/>
+    <row r="634" ht="15.75" customHeight="1" s="24"/>
+    <row r="635" ht="15.75" customHeight="1" s="24"/>
+    <row r="636" ht="15.75" customHeight="1" s="24"/>
+    <row r="637" ht="15.75" customHeight="1" s="24"/>
+    <row r="638" ht="15.75" customHeight="1" s="24"/>
+    <row r="639" ht="15.75" customHeight="1" s="24"/>
+    <row r="640" ht="15.75" customHeight="1" s="24"/>
+    <row r="641" ht="15.75" customHeight="1" s="24"/>
+    <row r="642" ht="15.75" customHeight="1" s="24"/>
+    <row r="643" ht="15.75" customHeight="1" s="24"/>
+    <row r="644" ht="15.75" customHeight="1" s="24"/>
+    <row r="645" ht="15.75" customHeight="1" s="24"/>
+    <row r="646" ht="15.75" customHeight="1" s="24"/>
+    <row r="647" ht="15.75" customHeight="1" s="24"/>
+    <row r="648" ht="15.75" customHeight="1" s="24"/>
+    <row r="649" ht="15.75" customHeight="1" s="24"/>
+    <row r="650" ht="15.75" customHeight="1" s="24"/>
+    <row r="651" ht="15.75" customHeight="1" s="24"/>
+    <row r="652" ht="15.75" customHeight="1" s="24"/>
+    <row r="653" ht="15.75" customHeight="1" s="24"/>
+    <row r="654" ht="15.75" customHeight="1" s="24"/>
+    <row r="655" ht="15.75" customHeight="1" s="24"/>
+    <row r="656" ht="15.75" customHeight="1" s="24"/>
+    <row r="657" ht="15.75" customHeight="1" s="24"/>
+    <row r="658" ht="15.75" customHeight="1" s="24"/>
+    <row r="659" ht="15.75" customHeight="1" s="24"/>
+    <row r="660" ht="15.75" customHeight="1" s="24"/>
+    <row r="661" ht="15.75" customHeight="1" s="24"/>
+    <row r="662" ht="15.75" customHeight="1" s="24"/>
+    <row r="663" ht="15.75" customHeight="1" s="24"/>
+    <row r="664" ht="15.75" customHeight="1" s="24"/>
+    <row r="665" ht="15.75" customHeight="1" s="24"/>
+    <row r="666" ht="15.75" customHeight="1" s="24"/>
+    <row r="667" ht="15.75" customHeight="1" s="24"/>
+    <row r="668" ht="15.75" customHeight="1" s="24"/>
+    <row r="669" ht="15.75" customHeight="1" s="24"/>
+    <row r="670" ht="15.75" customHeight="1" s="24"/>
+    <row r="671" ht="15.75" customHeight="1" s="24"/>
+    <row r="672" ht="15.75" customHeight="1" s="24"/>
+    <row r="673" ht="15.75" customHeight="1" s="24"/>
+    <row r="674" ht="15.75" customHeight="1" s="24"/>
+    <row r="675" ht="15.75" customHeight="1" s="24"/>
+    <row r="676" ht="15.75" customHeight="1" s="24"/>
+    <row r="677" ht="15.75" customHeight="1" s="24"/>
+    <row r="678" ht="15.75" customHeight="1" s="24"/>
+    <row r="679" ht="15.75" customHeight="1" s="24"/>
+    <row r="680" ht="15.75" customHeight="1" s="24"/>
+    <row r="681" ht="15.75" customHeight="1" s="24"/>
+    <row r="682" ht="15.75" customHeight="1" s="24"/>
+    <row r="683" ht="15.75" customHeight="1" s="24"/>
+    <row r="684" ht="15.75" customHeight="1" s="24"/>
+    <row r="685" ht="15.75" customHeight="1" s="24"/>
+    <row r="686" ht="15.75" customHeight="1" s="24"/>
+    <row r="687" ht="15.75" customHeight="1" s="24"/>
+    <row r="688" ht="15.75" customHeight="1" s="24"/>
+    <row r="689" ht="15.75" customHeight="1" s="24"/>
+    <row r="690" ht="15.75" customHeight="1" s="24"/>
+    <row r="691" ht="15.75" customHeight="1" s="24"/>
+    <row r="692" ht="15.75" customHeight="1" s="24"/>
+    <row r="693" ht="15.75" customHeight="1" s="24"/>
+    <row r="694" ht="15.75" customHeight="1" s="24"/>
+    <row r="695" ht="15.75" customHeight="1" s="24"/>
+    <row r="696" ht="15.75" customHeight="1" s="24"/>
+    <row r="697" ht="15.75" customHeight="1" s="24"/>
+    <row r="698" ht="15.75" customHeight="1" s="24"/>
+    <row r="699" ht="15.75" customHeight="1" s="24"/>
+    <row r="700" ht="15.75" customHeight="1" s="24"/>
+    <row r="701" ht="15.75" customHeight="1" s="24"/>
+    <row r="702" ht="15.75" customHeight="1" s="24"/>
+    <row r="703" ht="15.75" customHeight="1" s="24"/>
+    <row r="704" ht="15.75" customHeight="1" s="24"/>
+    <row r="705" ht="15.75" customHeight="1" s="24"/>
+    <row r="706" ht="15.75" customHeight="1" s="24"/>
+    <row r="707" ht="15.75" customHeight="1" s="24"/>
+    <row r="708" ht="15.75" customHeight="1" s="24"/>
+    <row r="709" ht="15.75" customHeight="1" s="24"/>
+    <row r="710" ht="15.75" customHeight="1" s="24"/>
+    <row r="711" ht="15.75" customHeight="1" s="24"/>
+    <row r="712" ht="15.75" customHeight="1" s="24"/>
+    <row r="713" ht="15.75" customHeight="1" s="24"/>
+    <row r="714" ht="15.75" customHeight="1" s="24"/>
+    <row r="715" ht="15.75" customHeight="1" s="24"/>
+    <row r="716" ht="15.75" customHeight="1" s="24"/>
+    <row r="717" ht="15.75" customHeight="1" s="24"/>
+    <row r="718" ht="15.75" customHeight="1" s="24"/>
+    <row r="719" ht="15.75" customHeight="1" s="24"/>
+    <row r="720" ht="15.75" customHeight="1" s="24"/>
+    <row r="721" ht="15.75" customHeight="1" s="24"/>
+    <row r="722" ht="15.75" customHeight="1" s="24"/>
+    <row r="723" ht="15.75" customHeight="1" s="24"/>
+    <row r="724" ht="15.75" customHeight="1" s="24"/>
+    <row r="725" ht="15.75" customHeight="1" s="24"/>
+    <row r="726" ht="15.75" customHeight="1" s="24"/>
+    <row r="727" ht="15.75" customHeight="1" s="24"/>
+    <row r="728" ht="15.75" customHeight="1" s="24"/>
+    <row r="729" ht="15.75" customHeight="1" s="24"/>
+    <row r="730" ht="15.75" customHeight="1" s="24"/>
+    <row r="731" ht="15.75" customHeight="1" s="24"/>
+    <row r="732" ht="15.75" customHeight="1" s="24"/>
+    <row r="733" ht="15.75" customHeight="1" s="24"/>
+    <row r="734" ht="15.75" customHeight="1" s="24"/>
+    <row r="735" ht="15.75" customHeight="1" s="24"/>
+    <row r="736" ht="15.75" customHeight="1" s="24"/>
+    <row r="737" ht="15.75" customHeight="1" s="24"/>
+    <row r="738" ht="15.75" customHeight="1" s="24"/>
+    <row r="739" ht="15.75" customHeight="1" s="24"/>
+    <row r="740" ht="15.75" customHeight="1" s="24"/>
+    <row r="741" ht="15.75" customHeight="1" s="24"/>
+    <row r="742" ht="15.75" customHeight="1" s="24"/>
+    <row r="743" ht="15.75" customHeight="1" s="24"/>
+    <row r="744" ht="15.75" customHeight="1" s="24"/>
+    <row r="745" ht="15.75" customHeight="1" s="24"/>
+    <row r="746" ht="15.75" customHeight="1" s="24"/>
+    <row r="747" ht="15.75" customHeight="1" s="24"/>
+    <row r="748" ht="15.75" customHeight="1" s="24"/>
+    <row r="749" ht="15.75" customHeight="1" s="24"/>
+    <row r="750" ht="15.75" customHeight="1" s="24"/>
+    <row r="751" ht="15.75" customHeight="1" s="24"/>
+    <row r="752" ht="15.75" customHeight="1" s="24"/>
+    <row r="753" ht="15.75" customHeight="1" s="24"/>
+    <row r="754" ht="15.75" customHeight="1" s="24"/>
+    <row r="755" ht="15.75" customHeight="1" s="24"/>
+    <row r="756" ht="15.75" customHeight="1" s="24"/>
+    <row r="757" ht="15.75" customHeight="1" s="24"/>
+    <row r="758" ht="15.75" customHeight="1" s="24"/>
+    <row r="759" ht="15.75" customHeight="1" s="24"/>
+    <row r="760" ht="15.75" customHeight="1" s="24"/>
+    <row r="761" ht="15.75" customHeight="1" s="24"/>
+    <row r="762" ht="15.75" customHeight="1" s="24"/>
+    <row r="763" ht="15.75" customHeight="1" s="24"/>
+    <row r="764" ht="15.75" customHeight="1" s="24"/>
+    <row r="765" ht="15.75" customHeight="1" s="24"/>
+    <row r="766" ht="15.75" customHeight="1" s="24"/>
+    <row r="767" ht="15.75" customHeight="1" s="24"/>
+    <row r="768" ht="15.75" customHeight="1" s="24"/>
+    <row r="769" ht="15.75" customHeight="1" s="24"/>
+    <row r="770" ht="15.75" customHeight="1" s="24"/>
+    <row r="771" ht="15.75" customHeight="1" s="24"/>
+    <row r="772" ht="15.75" customHeight="1" s="24"/>
+    <row r="773" ht="15.75" customHeight="1" s="24"/>
+    <row r="774" ht="15.75" customHeight="1" s="24"/>
+    <row r="775" ht="15.75" customHeight="1" s="24"/>
+    <row r="776" ht="15.75" customHeight="1" s="24"/>
+    <row r="777" ht="15.75" customHeight="1" s="24"/>
+    <row r="778" ht="15.75" customHeight="1" s="24"/>
+    <row r="779" ht="15.75" customHeight="1" s="24"/>
+    <row r="780" ht="15.75" customHeight="1" s="24"/>
+    <row r="781" ht="15.75" customHeight="1" s="24"/>
+    <row r="782" ht="15.75" customHeight="1" s="24"/>
+    <row r="783" ht="15.75" customHeight="1" s="24"/>
+    <row r="784" ht="15.75" customHeight="1" s="24"/>
+    <row r="785" ht="15.75" customHeight="1" s="24"/>
+    <row r="786" ht="15.75" customHeight="1" s="24"/>
+    <row r="787" ht="15.75" customHeight="1" s="24"/>
+    <row r="788" ht="15.75" customHeight="1" s="24"/>
+    <row r="789" ht="15.75" customHeight="1" s="24"/>
+    <row r="790" ht="15.75" customHeight="1" s="24"/>
+    <row r="791" ht="15.75" customHeight="1" s="24"/>
+    <row r="792" ht="15.75" customHeight="1" s="24"/>
+    <row r="793" ht="15.75" customHeight="1" s="24"/>
+    <row r="794" ht="15.75" customHeight="1" s="24"/>
+    <row r="795" ht="15.75" customHeight="1" s="24"/>
+    <row r="796" ht="15.75" customHeight="1" s="24"/>
+    <row r="797" ht="15.75" customHeight="1" s="24"/>
+    <row r="798" ht="15.75" customHeight="1" s="24"/>
+    <row r="799" ht="15.75" customHeight="1" s="24"/>
+    <row r="800" ht="15.75" customHeight="1" s="24"/>
+    <row r="801" ht="15.75" customHeight="1" s="24"/>
+    <row r="802" ht="15.75" customHeight="1" s="24"/>
+    <row r="803" ht="15.75" customHeight="1" s="24"/>
+    <row r="804" ht="15.75" customHeight="1" s="24"/>
+    <row r="805" ht="15.75" customHeight="1" s="24"/>
+    <row r="806" ht="15.75" customHeight="1" s="24"/>
+    <row r="807" ht="15.75" customHeight="1" s="24"/>
+    <row r="808" ht="15.75" customHeight="1" s="24"/>
+    <row r="809" ht="15.75" customHeight="1" s="24"/>
+    <row r="810" ht="15.75" customHeight="1" s="24"/>
+    <row r="811" ht="15.75" customHeight="1" s="24"/>
+    <row r="812" ht="15.75" customHeight="1" s="24"/>
+    <row r="813" ht="15.75" customHeight="1" s="24"/>
+    <row r="814" ht="15.75" customHeight="1" s="24"/>
+    <row r="815" ht="15.75" customHeight="1" s="24"/>
+    <row r="816" ht="15.75" customHeight="1" s="24"/>
+    <row r="817" ht="15.75" customHeight="1" s="24"/>
+    <row r="818" ht="15.75" customHeight="1" s="24"/>
+    <row r="819" ht="15.75" customHeight="1" s="24"/>
+    <row r="820" ht="15.75" customHeight="1" s="24"/>
+    <row r="821" ht="15.75" customHeight="1" s="24"/>
+    <row r="822" ht="15.75" customHeight="1" s="24"/>
+    <row r="823" ht="15.75" customHeight="1" s="24"/>
+    <row r="824" ht="15.75" customHeight="1" s="24"/>
+    <row r="825" ht="15.75" customHeight="1" s="24"/>
+    <row r="826" ht="15.75" customHeight="1" s="24"/>
+    <row r="827" ht="15.75" customHeight="1" s="24"/>
+    <row r="828" ht="15.75" customHeight="1" s="24"/>
+    <row r="829" ht="15.75" customHeight="1" s="24"/>
+    <row r="830" ht="15.75" customHeight="1" s="24"/>
+    <row r="831" ht="15.75" customHeight="1" s="24"/>
+    <row r="832" ht="15.75" customHeight="1" s="24"/>
+    <row r="833" ht="15.75" customHeight="1" s="24"/>
+    <row r="834" ht="15.75" customHeight="1" s="24"/>
+    <row r="835" ht="15.75" customHeight="1" s="24"/>
+    <row r="836" ht="15.75" customHeight="1" s="24"/>
+    <row r="837" ht="15.75" customHeight="1" s="24"/>
+    <row r="838" ht="15.75" customHeight="1" s="24"/>
+    <row r="839" ht="15.75" customHeight="1" s="24"/>
+    <row r="840" ht="15.75" customHeight="1" s="24"/>
+    <row r="841" ht="15.75" customHeight="1" s="24"/>
+    <row r="842" ht="15.75" customHeight="1" s="24"/>
+    <row r="843" ht="15.75" customHeight="1" s="24"/>
+    <row r="844" ht="15.75" customHeight="1" s="24"/>
+    <row r="845" ht="15.75" customHeight="1" s="24"/>
+    <row r="846" ht="15.75" customHeight="1" s="24"/>
+    <row r="847" ht="15.75" customHeight="1" s="24"/>
+    <row r="848" ht="15.75" customHeight="1" s="24"/>
+    <row r="849" ht="15.75" customHeight="1" s="24"/>
+    <row r="850" ht="15.75" customHeight="1" s="24"/>
+    <row r="851" ht="15.75" customHeight="1" s="24"/>
+    <row r="852" ht="15.75" customHeight="1" s="24"/>
+    <row r="853" ht="15.75" customHeight="1" s="24"/>
+    <row r="854" ht="15.75" customHeight="1" s="24"/>
+    <row r="855" ht="15.75" customHeight="1" s="24"/>
+    <row r="856" ht="15.75" customHeight="1" s="24"/>
+    <row r="857" ht="15.75" customHeight="1" s="24"/>
+    <row r="858" ht="15.75" customHeight="1" s="24"/>
+    <row r="859" ht="15.75" customHeight="1" s="24"/>
+    <row r="860" ht="15.75" customHeight="1" s="24"/>
+    <row r="861" ht="15.75" customHeight="1" s="24"/>
+    <row r="862" ht="15.75" customHeight="1" s="24"/>
+    <row r="863" ht="15.75" customHeight="1" s="24"/>
+    <row r="864" ht="15.75" customHeight="1" s="24"/>
+    <row r="865" ht="15.75" customHeight="1" s="24"/>
+    <row r="866" ht="15.75" customHeight="1" s="24"/>
+    <row r="867" ht="15.75" customHeight="1" s="24"/>
+    <row r="868" ht="15.75" customHeight="1" s="24"/>
+    <row r="869" ht="15.75" customHeight="1" s="24"/>
+    <row r="870" ht="15.75" customHeight="1" s="24"/>
+    <row r="871" ht="15.75" customHeight="1" s="24"/>
+    <row r="872" ht="15.75" customHeight="1" s="24"/>
+    <row r="873" ht="15.75" customHeight="1" s="24"/>
+    <row r="874" ht="15.75" customHeight="1" s="24"/>
+    <row r="875" ht="15.75" customHeight="1" s="24"/>
+    <row r="876" ht="15.75" customHeight="1" s="24"/>
+    <row r="877" ht="15.75" customHeight="1" s="24"/>
+    <row r="878" ht="15.75" customHeight="1" s="24"/>
+    <row r="879" ht="15.75" customHeight="1" s="24"/>
+    <row r="880" ht="15.75" customHeight="1" s="24"/>
+    <row r="881" ht="15.75" customHeight="1" s="24"/>
+    <row r="882" ht="15.75" customHeight="1" s="24"/>
+    <row r="883" ht="15.75" customHeight="1" s="24"/>
+    <row r="884" ht="15.75" customHeight="1" s="24"/>
+    <row r="885" ht="15.75" customHeight="1" s="24"/>
+    <row r="886" ht="15.75" customHeight="1" s="24"/>
+    <row r="887" ht="15.75" customHeight="1" s="24"/>
+    <row r="888" ht="15.75" customHeight="1" s="24"/>
+    <row r="889" ht="15.75" customHeight="1" s="24"/>
+    <row r="890" ht="15.75" customHeight="1" s="24"/>
+    <row r="891" ht="15.75" customHeight="1" s="24"/>
+    <row r="892" ht="15.75" customHeight="1" s="24"/>
+    <row r="893" ht="15.75" customHeight="1" s="24"/>
+    <row r="894" ht="15.75" customHeight="1" s="24"/>
+    <row r="895" ht="15.75" customHeight="1" s="24"/>
+    <row r="896" ht="15.75" customHeight="1" s="24"/>
+    <row r="897" ht="15.75" customHeight="1" s="24"/>
+    <row r="898" ht="15.75" customHeight="1" s="24"/>
+    <row r="899" ht="15.75" customHeight="1" s="24"/>
+    <row r="900" ht="15.75" customHeight="1" s="24"/>
+    <row r="901" ht="15.75" customHeight="1" s="24"/>
+    <row r="902" ht="15.75" customHeight="1" s="24"/>
+    <row r="903" ht="15.75" customHeight="1" s="24"/>
+    <row r="904" ht="15.75" customHeight="1" s="24"/>
+    <row r="905" ht="15.75" customHeight="1" s="24"/>
+    <row r="906" ht="15.75" customHeight="1" s="24"/>
+    <row r="907" ht="15.75" customHeight="1" s="24"/>
+    <row r="908" ht="15.75" customHeight="1" s="24"/>
+    <row r="909" ht="15.75" customHeight="1" s="24"/>
+    <row r="910" ht="15.75" customHeight="1" s="24"/>
+    <row r="911" ht="15.75" customHeight="1" s="24"/>
+    <row r="912" ht="15.75" customHeight="1" s="24"/>
+    <row r="913" ht="15.75" customHeight="1" s="24"/>
+    <row r="914" ht="15.75" customHeight="1" s="24"/>
+    <row r="915" ht="15.75" customHeight="1" s="24"/>
+    <row r="916" ht="15.75" customHeight="1" s="24"/>
+    <row r="917" ht="15.75" customHeight="1" s="24"/>
+    <row r="918" ht="15.75" customHeight="1" s="24"/>
+    <row r="919" ht="15.75" customHeight="1" s="24"/>
+    <row r="920" ht="15.75" customHeight="1" s="24"/>
+    <row r="921" ht="15.75" customHeight="1" s="24"/>
+    <row r="922" ht="15.75" customHeight="1" s="24"/>
+    <row r="923" ht="15.75" customHeight="1" s="24"/>
+    <row r="924" ht="15.75" customHeight="1" s="24"/>
+    <row r="925" ht="15.75" customHeight="1" s="24"/>
+    <row r="926" ht="15.75" customHeight="1" s="24"/>
+    <row r="927" ht="15.75" customHeight="1" s="24"/>
+    <row r="928" ht="15.75" customHeight="1" s="24"/>
+    <row r="929" ht="15.75" customHeight="1" s="24"/>
+    <row r="930" ht="15.75" customHeight="1" s="24"/>
+    <row r="931" ht="15.75" customHeight="1" s="24"/>
+    <row r="932" ht="15.75" customHeight="1" s="24"/>
+    <row r="933" ht="15.75" customHeight="1" s="24"/>
+    <row r="934" ht="15.75" customHeight="1" s="24"/>
+    <row r="935" ht="15.75" customHeight="1" s="24"/>
+    <row r="936" ht="15.75" customHeight="1" s="24"/>
+    <row r="937" ht="15.75" customHeight="1" s="24"/>
+    <row r="938" ht="15.75" customHeight="1" s="24"/>
+    <row r="939" ht="15.75" customHeight="1" s="24"/>
+    <row r="940" ht="15.75" customHeight="1" s="24"/>
+    <row r="941" ht="15.75" customHeight="1" s="24"/>
+    <row r="942" ht="15.75" customHeight="1" s="24"/>
+    <row r="943" ht="15.75" customHeight="1" s="24"/>
+    <row r="944" ht="15.75" customHeight="1" s="24"/>
+    <row r="945" ht="15.75" customHeight="1" s="24"/>
+    <row r="946" ht="15.75" customHeight="1" s="24"/>
+    <row r="947" ht="15.75" customHeight="1" s="24"/>
+    <row r="948" ht="15.75" customHeight="1" s="24"/>
+    <row r="949" ht="15.75" customHeight="1" s="24"/>
+    <row r="950" ht="15.75" customHeight="1" s="24"/>
+    <row r="951" ht="15.75" customHeight="1" s="24"/>
+    <row r="952" ht="15.75" customHeight="1" s="24"/>
+    <row r="953" ht="15.75" customHeight="1" s="24"/>
+    <row r="954" ht="15.75" customHeight="1" s="24"/>
+    <row r="955" ht="15.75" customHeight="1" s="24"/>
+    <row r="956" ht="15.75" customHeight="1" s="24"/>
+    <row r="957" ht="15.75" customHeight="1" s="24"/>
+    <row r="958" ht="15.75" customHeight="1" s="24"/>
+    <row r="959" ht="15.75" customHeight="1" s="24"/>
+    <row r="960" ht="15.75" customHeight="1" s="24"/>
+    <row r="961" ht="15.75" customHeight="1" s="24"/>
+    <row r="962" ht="15.75" customHeight="1" s="24"/>
+    <row r="963" ht="15.75" customHeight="1" s="24"/>
+    <row r="964" ht="15.75" customHeight="1" s="24"/>
+    <row r="965" ht="15.75" customHeight="1" s="24"/>
+    <row r="966" ht="15.75" customHeight="1" s="24"/>
+    <row r="967" ht="15.75" customHeight="1" s="24"/>
+    <row r="968" ht="15.75" customHeight="1" s="24"/>
+    <row r="969" ht="15.75" customHeight="1" s="24"/>
+    <row r="970" ht="15.75" customHeight="1" s="24"/>
+    <row r="971" ht="15.75" customHeight="1" s="24"/>
+    <row r="972" ht="15.75" customHeight="1" s="24"/>
+    <row r="973" ht="15.75" customHeight="1" s="24"/>
+    <row r="974" ht="15.75" customHeight="1" s="24"/>
+    <row r="975" ht="15.75" customHeight="1" s="24"/>
+    <row r="976" ht="15.75" customHeight="1" s="24"/>
+    <row r="977" ht="15.75" customHeight="1" s="24"/>
+    <row r="978" ht="15.75" customHeight="1" s="24"/>
+    <row r="979" ht="15.75" customHeight="1" s="24"/>
+    <row r="980" ht="15.75" customHeight="1" s="24"/>
+    <row r="981" ht="15.75" customHeight="1" s="24"/>
+    <row r="982" ht="15.75" customHeight="1" s="24"/>
+    <row r="983" ht="15.75" customHeight="1" s="24"/>
+    <row r="984" ht="15.75" customHeight="1" s="24"/>
+    <row r="985" ht="15.75" customHeight="1" s="24"/>
+    <row r="986" ht="15.75" customHeight="1" s="24"/>
+    <row r="987" ht="15.75" customHeight="1" s="24"/>
+    <row r="988" ht="15.75" customHeight="1" s="24"/>
+    <row r="989" ht="15.75" customHeight="1" s="24"/>
+    <row r="990" ht="15.75" customHeight="1" s="24"/>
+    <row r="991" ht="15.75" customHeight="1" s="24"/>
+    <row r="992" ht="15.75" customHeight="1" s="24"/>
+    <row r="993" ht="15.75" customHeight="1" s="24"/>
+    <row r="994" ht="15.75" customHeight="1" s="24"/>
+    <row r="995" ht="15.75" customHeight="1" s="24"/>
+    <row r="996" ht="15.75" customHeight="1" s="24"/>
+    <row r="997" ht="15.75" customHeight="1" s="24"/>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
fix(deploy): bật Silero VAD cho speech, giữ Whisper large-v3
</commit_message>
<xml_diff>
--- a/docs/evidence/tc2-3-ai-usage/AI Prompt Log - W07 - 2026-10-26_2026-11-01.xlsx
+++ b/docs/evidence/tc2-3-ai-usage/AI Prompt Log - W07 - 2026-10-26_2026-11-01.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet name="Thắng" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Nguyên" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Sang" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Tổng hợp" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thắng" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nguyên" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sang" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tổng hợp" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
@@ -1011,29 +1011,95 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="36" customHeight="1" s="24">
-      <c r="A17" s="32" t="n"/>
-      <c r="B17" s="18" t="n"/>
-      <c r="C17" s="18" t="n"/>
-      <c r="D17" s="33" t="n"/>
-      <c r="E17" s="33" t="n"/>
-      <c r="F17" s="33" t="n"/>
-    </row>
-    <row r="18" ht="36" customHeight="1" s="24">
-      <c r="A18" s="25" t="n"/>
-      <c r="B18" s="26" t="n"/>
-      <c r="C18" s="26" t="n"/>
-      <c r="D18" s="27" t="n"/>
-      <c r="E18" s="27" t="n"/>
-      <c r="F18" s="27" t="n"/>
-    </row>
-    <row r="19" ht="36" customHeight="1" s="24">
-      <c r="A19" s="25" t="n"/>
-      <c r="B19" s="26" t="n"/>
-      <c r="C19" s="26" t="n"/>
-      <c r="D19" s="27" t="n"/>
-      <c r="E19" s="27" t="n"/>
-      <c r="F19" s="27" t="n"/>
+    <row r="17" ht="125" customHeight="1" s="24">
+      <c r="A17" s="39" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B17" s="40" t="inlineStr">
+        <is>
+          <t>Thắng</t>
+        </is>
+      </c>
+      <c r="C17" s="40" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="D17" s="41" t="inlineStr">
+        <is>
+          <t>Build image, tao PR va merge theo yeu cau</t>
+        </is>
+      </c>
+      <c r="E17" s="41" t="inlineStr">
+        <is>
+          <t>hãy build image mới và tạo PR chuẩn rồi merge vào main rồi đợi có người review</t>
+        </is>
+      </c>
+      <c r="F17" s="41" t="inlineStr">
+        <is>
+          <t>thang/deploy-silero-vad-2026-10-30.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="125" customHeight="1" s="24">
+      <c r="A18" s="39" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B18" s="40" t="inlineStr">
+        <is>
+          <t>Thắng</t>
+        </is>
+      </c>
+      <c r="C18" s="40" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="D18" s="41" t="inlineStr">
+        <is>
+          <t>Giai thich Whisper large-v3 va mo hinh cham</t>
+        </is>
+      </c>
+      <c r="E18" s="41" t="inlineStr">
+        <is>
+          <t>Tại sao tôi lại không dùng model này được faster-whisper-large-v3</t>
+        </is>
+      </c>
+      <c r="F18" s="41" t="inlineStr">
+        <is>
+          <t>thang/deploy-silero-vad-2026-10-30.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="125" customHeight="1" s="24">
+      <c r="A19" s="39" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B19" s="40" t="inlineStr">
+        <is>
+          <t>Thắng</t>
+        </is>
+      </c>
+      <c r="C19" s="40" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="D19" s="41" t="inlineStr">
+        <is>
+          <t>Chot pham vi chi bat Silero, giu large-v3</t>
+        </is>
+      </c>
+      <c r="E19" s="41" t="inlineStr">
+        <is>
+          <t>để lại model faster-whisper-large-v3 giữ nguyên và chỉ thêm VAD=1 thôi</t>
+        </is>
+      </c>
+      <c r="F19" s="41" t="inlineStr">
+        <is>
+          <t>thang/deploy-silero-vad-2026-10-30.md</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="36" customHeight="1" s="24">
       <c r="A20" s="25" t="n"/>
@@ -19084,7 +19150,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:F14"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.625" defaultRowHeight="14.25"/>
   <cols>
     <col width="24" customWidth="1" style="24" min="1" max="1"/>

</xml_diff>

<commit_message>
docs(W7): cập nhật báo cáo tuần 7 và AI Prompt Log tuần 7 (sheet Sang) ngày 30/10
Báo cáo: mục 1.3 các việc 29–30/10 (#80–#91: khôi phục main, D061–D065, deploy
EC2, sửa lỗi teammate không chạy được, rà phân quyền admin), kết quả kiểm thử,
vướng mắc mới (cổng thanh toán thử đang bật trên production, rủi ro dữ liệu cá
nhân sau D064, PR chờ merge) và kế hoạch tuần 8.
AI log W07 sheet Sang thêm 11 dòng (hàng 16–26), mỗi dòng có PR làm minh chứng;
README cập nhật số liệu W07 (14 Thắng, 3 Nguyên, 21 Sang, 38 tổng).
</commit_message>
<xml_diff>
--- a/docs/evidence/tc2-3-ai-usage/AI Prompt Log - W07 - 2026-10-26_2026-11-01.xlsx
+++ b/docs/evidence/tc2-3-ai-usage/AI Prompt Log - W07 - 2026-10-26_2026-11-01.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thắng" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nguyên" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sang" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tổng hợp" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Thắng" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Nguyên" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Sang" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Tổng hợp" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
@@ -13326,92 +13326,334 @@
       </c>
     </row>
     <row r="16" ht="36" customHeight="1" s="24">
-      <c r="A16" s="20" t="n"/>
-      <c r="B16" s="18" t="n"/>
-      <c r="C16" s="18" t="n"/>
-      <c r="D16" s="33" t="n"/>
-      <c r="E16" s="33" t="n"/>
-      <c r="F16" s="33" t="n"/>
+      <c r="A16" s="36" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B16" s="37" t="inlineStr">
+        <is>
+          <t>Sang</t>
+        </is>
+      </c>
+      <c r="C16" s="37" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="D16" s="38" t="inlineStr">
+        <is>
+          <t>Khôi phục main sau commit đồng bộ đưa nhầm bản cũ (ff683cc)</t>
+        </is>
+      </c>
+      <c r="E16" s="38" t="inlineStr">
+        <is>
+          <t>Commit đẩy thẳng lên main đưa lại bản cũ của toàn bộ mã nguồn: mất D058–D060, đưa lại artifact suy ra từ S&amp;I vào repo công khai và làm đỏ CI. Đưa cây mã về đúng bản #79, giữ commit lỗi trong lịch sử, kiểm CI trước khi merge.</t>
+        </is>
+      </c>
+      <c r="F16" s="38" t="inlineStr">
+        <is>
+          <t>https://github.com/ThanhSangLouis/ai-assessor-cefr/pull/80 (squash f4a6659)</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="36" customHeight="1" s="24">
-      <c r="A17" s="20" t="n"/>
-      <c r="B17" s="18" t="n"/>
-      <c r="C17" s="18" t="n"/>
-      <c r="D17" s="33" t="n"/>
-      <c r="E17" s="33" t="n"/>
-      <c r="F17" s="33" t="n"/>
+      <c r="A17" s="36" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B17" s="37" t="inlineStr">
+        <is>
+          <t>Sang</t>
+        </is>
+      </c>
+      <c r="C17" s="37" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="D17" s="38" t="inlineStr">
+        <is>
+          <t>D061: đo Mạch lạc bằng từ nối; sửa demo.sh để teammate chạy được</t>
+        </is>
+      </c>
+      <c r="E17" s="38" t="inlineStr">
+        <is>
+          <t>Nghiên cứu phản hồi của nhóm về hai tiêu chí Mạch lạc và Độ chính xác, chọn cách đo bằng chỉ số đọc được: liệt kê các kiểu từ nối trong bài làm bằng chứng cho Mạch lạc. Teammate báo không chạy được dự án: sửa demo.sh dùng MongoDB trong Docker và artifact giả lập khi thiếu model thật.</t>
+        </is>
+      </c>
+      <c r="F17" s="38" t="inlineStr">
+        <is>
+          <t>https://github.com/ThanhSangLouis/ai-assessor-cefr/pull/81 (squash cbfd87f)</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="36" customHeight="1" s="24">
-      <c r="A18" s="20" t="n"/>
-      <c r="B18" s="18" t="n"/>
-      <c r="C18" s="18" t="n"/>
-      <c r="D18" s="33" t="n"/>
-      <c r="E18" s="33" t="n"/>
-      <c r="F18" s="33" t="n"/>
+      <c r="A18" s="36" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B18" s="37" t="inlineStr">
+        <is>
+          <t>Sang</t>
+        </is>
+      </c>
+      <c r="C18" s="37" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="D18" s="38" t="inlineStr">
+        <is>
+          <t>Viết hướng dẫn chạy dự án cho AI agent của teammate</t>
+        </is>
+      </c>
+      <c r="E18" s="38" t="inlineStr">
+        <is>
+          <t>Ghi đầy đủ các cách chạy dự án (demo.sh, Whisper thật, Docker Compose, kiểm thử như CI, lỗi hay gặp) để AI agent của teammate đọc trước khi chạy; CLAUDE.md trỏ tới AGENTS.md; sửa các lệnh sai trong README.</t>
+        </is>
+      </c>
+      <c r="F18" s="38" t="inlineStr">
+        <is>
+          <t>https://github.com/ThanhSangLouis/ai-assessor-cefr/pull/83 (squash a5e19c5); docs/plan/CHAY_DU_AN_CHO_AI.md</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="36" customHeight="1" s="24">
-      <c r="A19" s="20" t="n"/>
-      <c r="B19" s="18" t="n"/>
-      <c r="C19" s="18" t="n"/>
-      <c r="D19" s="33" t="n"/>
-      <c r="E19" s="33" t="n"/>
-      <c r="F19" s="33" t="n"/>
+      <c r="A19" s="36" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B19" s="37" t="inlineStr">
+        <is>
+          <t>Sang</t>
+        </is>
+      </c>
+      <c r="C19" s="37" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="D19" s="38" t="inlineStr">
+        <is>
+          <t>D062: chỉ chấm năm tiêu chí, bỏ khía cạnh Tương tác</t>
+        </is>
+      </c>
+      <c r="E19" s="38" t="inlineStr">
+        <is>
+          <t>Nhóm chốt chỉ đánh giá năm tiêu chí; bỏ dòng Tương tác khỏi báo cáo, trang /bands và chú thích, cập nhật test và E2E.</t>
+        </is>
+      </c>
+      <c r="F19" s="38" t="inlineStr">
+        <is>
+          <t>https://github.com/ThanhSangLouis/ai-assessor-cefr/pull/84 (squash 24f6845)</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="36" customHeight="1" s="24">
-      <c r="A20" s="20" t="n"/>
-      <c r="B20" s="18" t="n"/>
-      <c r="C20" s="18" t="n"/>
-      <c r="D20" s="33" t="n"/>
-      <c r="E20" s="33" t="n"/>
-      <c r="F20" s="33" t="n"/>
+      <c r="A20" s="36" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B20" s="37" t="inlineStr">
+        <is>
+          <t>Sang</t>
+        </is>
+      </c>
+      <c r="C20" s="37" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="D20" s="38" t="inlineStr">
+        <is>
+          <t>Phối hợp phiên khác hoàn tất tự động deploy lên EC2</t>
+        </is>
+      </c>
+      <c r="E20" s="38" t="inlineStr">
+        <is>
+          <t>Trao đổi với phiên đang làm AWS runner để hoàn tất workflow deploy lên EC2 sau CI xanh, thêm bước CI kiểm thư mục cache Whisper và bản đồ triển khai cho AI agent.</t>
+        </is>
+      </c>
+      <c r="F20" s="38" t="inlineStr">
+        <is>
+          <t>https://github.com/ThanhSangLouis/ai-assessor-cefr/pull/82; https://github.com/ThanhSangLouis/ai-assessor-cefr/pull/86 (squash 99c4a8d)</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="36" customHeight="1" s="24">
-      <c r="A21" s="20" t="n"/>
-      <c r="B21" s="18" t="n"/>
-      <c r="C21" s="18" t="n"/>
-      <c r="D21" s="33" t="n"/>
-      <c r="E21" s="33" t="n"/>
-      <c r="F21" s="33" t="n"/>
+      <c r="A21" s="36" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B21" s="37" t="inlineStr">
+        <is>
+          <t>Sang</t>
+        </is>
+      </c>
+      <c r="C21" s="37" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="D21" s="38" t="inlineStr">
+        <is>
+          <t>D063: sinh viên đăng ký bằng Google; seed tài khoản khi deploy</t>
+        </is>
+      </c>
+      <c r="E21" s="38" t="inlineStr">
+        <is>
+          <t>Thêm đăng ký bằng Google cho sinh viên (bút danh ngẫu nhiên, chỉ lưu băm định danh Google), lệnh seed bộ tài khoản mẫu chạy sau mỗi lần deploy, hướng dẫn tạo OAuth client trên GCP và kiểm tra .env trên máy chủ; kiểm tra web sau deploy.</t>
+        </is>
+      </c>
+      <c r="F21" s="38" t="inlineStr">
+        <is>
+          <t>https://github.com/ThanhSangLouis/ai-assessor-cefr/pull/85 (squash 096b061)</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="36" customHeight="1" s="24">
-      <c r="A22" s="20" t="n"/>
-      <c r="B22" s="18" t="n"/>
-      <c r="C22" s="18" t="n"/>
-      <c r="D22" s="33" t="n"/>
-      <c r="E22" s="33" t="n"/>
-      <c r="F22" s="33" t="n"/>
+      <c r="A22" s="36" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B22" s="37" t="inlineStr">
+        <is>
+          <t>Sang</t>
+        </is>
+      </c>
+      <c r="C22" s="37" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="D22" s="38" t="inlineStr">
+        <is>
+          <t>D064: bỏ bước đồng ý điều khoản; logo Google; cập nhật sơ đồ lớp; kiểm chấm điểm toàn bộ</t>
+        </is>
+      </c>
+      <c r="E22" s="38" t="inlineStr">
+        <is>
+          <t>Hệ thống đã phục vụ người dùng thật nên bỏ hẳn bước đồng ý điều khoản (migration 8), thêm logo Google trên nút đăng nhập, cập nhật sơ đồ lớp và ERD; chạy thử chấm điểm với Whisper và model thật trên các dạng bài, chạy kiểm thử ba tầng với ba vai trò.</t>
+        </is>
+      </c>
+      <c r="F22" s="38" t="inlineStr">
+        <is>
+          <t>https://github.com/ThanhSangLouis/ai-assessor-cefr/pull/87 (squash 46ee31c)</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="36" customHeight="1" s="24">
-      <c r="A23" s="20" t="n"/>
-      <c r="B23" s="18" t="n"/>
-      <c r="C23" s="18" t="n"/>
-      <c r="D23" s="33" t="n"/>
-      <c r="E23" s="33" t="n"/>
-      <c r="F23" s="33" t="n"/>
+      <c r="A23" s="36" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B23" s="37" t="inlineStr">
+        <is>
+          <t>Sang</t>
+        </is>
+      </c>
+      <c r="C23" s="37" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="D23" s="38" t="inlineStr">
+        <is>
+          <t>Tái hiện lỗi teammate không chạy được trên bản clone mới và sửa</t>
+        </is>
+      </c>
+      <c r="E23" s="38" t="inlineStr">
+        <is>
+          <t>Kéo code mới nhất, clone sạch và cài như máy teammate: bật Whisper khi chưa cài nhóm asr làm mọi bài FAILED mà log không nói lý do; Mac Intel cài nhầm backend; nút Google không hiện khi thiếu khoá. Sửa demo.sh báo rõ, ghi lý do vào log, sửa điều kiện cài, thêm mục bật Google ở local.</t>
+        </is>
+      </c>
+      <c r="F23" s="38" t="inlineStr">
+        <is>
+          <t>https://github.com/ThanhSangLouis/ai-assessor-cefr/pull/89</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="36" customHeight="1" s="24">
-      <c r="A24" s="20" t="n"/>
-      <c r="B24" s="18" t="n"/>
-      <c r="C24" s="18" t="n"/>
-      <c r="D24" s="33" t="n"/>
-      <c r="E24" s="33" t="n"/>
-      <c r="F24" s="33" t="n"/>
+      <c r="A24" s="36" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B24" s="37" t="inlineStr">
+        <is>
+          <t>Sang</t>
+        </is>
+      </c>
+      <c r="C24" s="37" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="D24" s="38" t="inlineStr">
+        <is>
+          <t>Rà toàn bộ xác thực và phân quyền của vai trò quản trị</t>
+        </is>
+      </c>
+      <c r="E24" s="38" t="inlineStr">
+        <is>
+          <t>Kiểm tra vai trò admin đã phủ hết các trường hợp xác thực và phân quyền: liệt kê 184 route API cùng lớp chặn, viết test gọi thử mọi route bằng khách, sinh viên, giảng viên, admin mật khẩu tạm và admin; chặn trang /admin cho người không phải admin.</t>
+        </is>
+      </c>
+      <c r="F24" s="38" t="inlineStr">
+        <is>
+          <t>https://github.com/ThanhSangLouis/ai-assessor-cefr/pull/90; tests/test_admin_access.py</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="36" customHeight="1" s="24">
-      <c r="A25" s="20" t="n"/>
-      <c r="B25" s="18" t="n"/>
-      <c r="C25" s="18" t="n"/>
-      <c r="D25" s="33" t="n"/>
-      <c r="E25" s="33" t="n"/>
-      <c r="F25" s="33" t="n"/>
+      <c r="A25" s="36" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B25" s="37" t="inlineStr">
+        <is>
+          <t>Sang</t>
+        </is>
+      </c>
+      <c r="C25" s="37" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="D25" s="38" t="inlineStr">
+        <is>
+          <t>D065: tự đăng ký bằng mật khẩu và quên mật khẩu bằng mã khôi phục</t>
+        </is>
+      </c>
+      <c r="E25" s="38" t="inlineStr">
+        <is>
+          <t>Làm tính năng đăng ký và quên mật khẩu khi hệ thống không lưu email: bút danh ngẫu nhiên, mã khôi phục dùng một lần lưu dạng băm, khoá khi đoán sai, giới hạn tốc độ; thẻ mã khôi phục ở trang Tài khoản; test tích hợp và E2E.</t>
+        </is>
+      </c>
+      <c r="F25" s="38" t="inlineStr">
+        <is>
+          <t>https://github.com/ThanhSangLouis/ai-assessor-cefr/pull/91; docs/test/TEST_PLAN_D065.md</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="36" customHeight="1" s="24">
-      <c r="A26" s="20" t="n"/>
-      <c r="B26" s="18" t="n"/>
-      <c r="C26" s="18" t="n"/>
-      <c r="D26" s="33" t="n"/>
-      <c r="E26" s="33" t="n"/>
-      <c r="F26" s="33" t="n"/>
+      <c r="A26" s="36" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B26" s="37" t="inlineStr">
+        <is>
+          <t>Sang</t>
+        </is>
+      </c>
+      <c r="C26" s="37" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="D26" s="38" t="inlineStr">
+        <is>
+          <t>Cập nhật báo cáo tuần 7 và AI Prompt Log tuần 7</t>
+        </is>
+      </c>
+      <c r="E26" s="38" t="inlineStr">
+        <is>
+          <t>Cập nhật báo cáo tiến độ tuần 7 và nhật ký sử dụng AI cho các việc ngày 29–30/10, đối chiếu từng dòng với PR thật.</t>
+        </is>
+      </c>
+      <c r="F26" s="38" t="inlineStr">
+        <is>
+          <t>docs/reports/week-07/bao-cao-tuan-07-sang.md; docs/evidence/tc2-3-ai-usage/README.md</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="36" customHeight="1" s="24">
       <c r="A27" s="20" t="n"/>
@@ -19150,7 +19392,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A2:F14"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.625" defaultRowHeight="14.25"/>
   <cols>
     <col width="24" customWidth="1" style="24" min="1" max="1"/>

</xml_diff>

<commit_message>
docs(W7): cập nhật báo cáo tuần 7 và AI Prompt Log ngày 30/10 (#92)
* docs(W7): cập nhật báo cáo tuần 7 và AI Prompt Log tuần 7 (sheet Sang) ngày 30/10

Báo cáo: mục 1.3 các việc 29–30/10 (#80–#91: khôi phục main, D061–D065, deploy
EC2, sửa lỗi teammate không chạy được, rà phân quyền admin), kết quả kiểm thử,
vướng mắc mới (cổng thanh toán thử đang bật trên production, rủi ro dữ liệu cá
nhân sau D064, PR chờ merge) và kế hoạch tuần 8.
AI log W07 sheet Sang thêm 11 dòng (hàng 16–26), mỗi dòng có PR làm minh chứng;
README cập nhật số liệu W07 (14 Thắng, 3 Nguyên, 21 Sang, 38 tổng).

* docs(W7): #89–#91 đã merge, bỏ vướng mắc chờ merge
</commit_message>
<xml_diff>
--- a/docs/evidence/tc2-3-ai-usage/AI Prompt Log - W07 - 2026-10-26_2026-11-01.xlsx
+++ b/docs/evidence/tc2-3-ai-usage/AI Prompt Log - W07 - 2026-10-26_2026-11-01.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thắng" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nguyên" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sang" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tổng hợp" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Thắng" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Nguyên" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Sang" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Tổng hợp" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
@@ -13326,92 +13326,334 @@
       </c>
     </row>
     <row r="16" ht="36" customHeight="1" s="24">
-      <c r="A16" s="20" t="n"/>
-      <c r="B16" s="18" t="n"/>
-      <c r="C16" s="18" t="n"/>
-      <c r="D16" s="33" t="n"/>
-      <c r="E16" s="33" t="n"/>
-      <c r="F16" s="33" t="n"/>
+      <c r="A16" s="36" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B16" s="37" t="inlineStr">
+        <is>
+          <t>Sang</t>
+        </is>
+      </c>
+      <c r="C16" s="37" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="D16" s="38" t="inlineStr">
+        <is>
+          <t>Khôi phục main sau commit đồng bộ đưa nhầm bản cũ (ff683cc)</t>
+        </is>
+      </c>
+      <c r="E16" s="38" t="inlineStr">
+        <is>
+          <t>Commit đẩy thẳng lên main đưa lại bản cũ của toàn bộ mã nguồn: mất D058–D060, đưa lại artifact suy ra từ S&amp;I vào repo công khai và làm đỏ CI. Đưa cây mã về đúng bản #79, giữ commit lỗi trong lịch sử, kiểm CI trước khi merge.</t>
+        </is>
+      </c>
+      <c r="F16" s="38" t="inlineStr">
+        <is>
+          <t>https://github.com/ThanhSangLouis/ai-assessor-cefr/pull/80 (squash f4a6659)</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="36" customHeight="1" s="24">
-      <c r="A17" s="20" t="n"/>
-      <c r="B17" s="18" t="n"/>
-      <c r="C17" s="18" t="n"/>
-      <c r="D17" s="33" t="n"/>
-      <c r="E17" s="33" t="n"/>
-      <c r="F17" s="33" t="n"/>
+      <c r="A17" s="36" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B17" s="37" t="inlineStr">
+        <is>
+          <t>Sang</t>
+        </is>
+      </c>
+      <c r="C17" s="37" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="D17" s="38" t="inlineStr">
+        <is>
+          <t>D061: đo Mạch lạc bằng từ nối; sửa demo.sh để teammate chạy được</t>
+        </is>
+      </c>
+      <c r="E17" s="38" t="inlineStr">
+        <is>
+          <t>Nghiên cứu phản hồi của nhóm về hai tiêu chí Mạch lạc và Độ chính xác, chọn cách đo bằng chỉ số đọc được: liệt kê các kiểu từ nối trong bài làm bằng chứng cho Mạch lạc. Teammate báo không chạy được dự án: sửa demo.sh dùng MongoDB trong Docker và artifact giả lập khi thiếu model thật.</t>
+        </is>
+      </c>
+      <c r="F17" s="38" t="inlineStr">
+        <is>
+          <t>https://github.com/ThanhSangLouis/ai-assessor-cefr/pull/81 (squash cbfd87f)</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="36" customHeight="1" s="24">
-      <c r="A18" s="20" t="n"/>
-      <c r="B18" s="18" t="n"/>
-      <c r="C18" s="18" t="n"/>
-      <c r="D18" s="33" t="n"/>
-      <c r="E18" s="33" t="n"/>
-      <c r="F18" s="33" t="n"/>
+      <c r="A18" s="36" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B18" s="37" t="inlineStr">
+        <is>
+          <t>Sang</t>
+        </is>
+      </c>
+      <c r="C18" s="37" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="D18" s="38" t="inlineStr">
+        <is>
+          <t>Viết hướng dẫn chạy dự án cho AI agent của teammate</t>
+        </is>
+      </c>
+      <c r="E18" s="38" t="inlineStr">
+        <is>
+          <t>Ghi đầy đủ các cách chạy dự án (demo.sh, Whisper thật, Docker Compose, kiểm thử như CI, lỗi hay gặp) để AI agent của teammate đọc trước khi chạy; CLAUDE.md trỏ tới AGENTS.md; sửa các lệnh sai trong README.</t>
+        </is>
+      </c>
+      <c r="F18" s="38" t="inlineStr">
+        <is>
+          <t>https://github.com/ThanhSangLouis/ai-assessor-cefr/pull/83 (squash a5e19c5); docs/plan/CHAY_DU_AN_CHO_AI.md</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="36" customHeight="1" s="24">
-      <c r="A19" s="20" t="n"/>
-      <c r="B19" s="18" t="n"/>
-      <c r="C19" s="18" t="n"/>
-      <c r="D19" s="33" t="n"/>
-      <c r="E19" s="33" t="n"/>
-      <c r="F19" s="33" t="n"/>
+      <c r="A19" s="36" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B19" s="37" t="inlineStr">
+        <is>
+          <t>Sang</t>
+        </is>
+      </c>
+      <c r="C19" s="37" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="D19" s="38" t="inlineStr">
+        <is>
+          <t>D062: chỉ chấm năm tiêu chí, bỏ khía cạnh Tương tác</t>
+        </is>
+      </c>
+      <c r="E19" s="38" t="inlineStr">
+        <is>
+          <t>Nhóm chốt chỉ đánh giá năm tiêu chí; bỏ dòng Tương tác khỏi báo cáo, trang /bands và chú thích, cập nhật test và E2E.</t>
+        </is>
+      </c>
+      <c r="F19" s="38" t="inlineStr">
+        <is>
+          <t>https://github.com/ThanhSangLouis/ai-assessor-cefr/pull/84 (squash 24f6845)</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="36" customHeight="1" s="24">
-      <c r="A20" s="20" t="n"/>
-      <c r="B20" s="18" t="n"/>
-      <c r="C20" s="18" t="n"/>
-      <c r="D20" s="33" t="n"/>
-      <c r="E20" s="33" t="n"/>
-      <c r="F20" s="33" t="n"/>
+      <c r="A20" s="36" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B20" s="37" t="inlineStr">
+        <is>
+          <t>Sang</t>
+        </is>
+      </c>
+      <c r="C20" s="37" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="D20" s="38" t="inlineStr">
+        <is>
+          <t>Phối hợp phiên khác hoàn tất tự động deploy lên EC2</t>
+        </is>
+      </c>
+      <c r="E20" s="38" t="inlineStr">
+        <is>
+          <t>Trao đổi với phiên đang làm AWS runner để hoàn tất workflow deploy lên EC2 sau CI xanh, thêm bước CI kiểm thư mục cache Whisper và bản đồ triển khai cho AI agent.</t>
+        </is>
+      </c>
+      <c r="F20" s="38" t="inlineStr">
+        <is>
+          <t>https://github.com/ThanhSangLouis/ai-assessor-cefr/pull/82; https://github.com/ThanhSangLouis/ai-assessor-cefr/pull/86 (squash 99c4a8d)</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="36" customHeight="1" s="24">
-      <c r="A21" s="20" t="n"/>
-      <c r="B21" s="18" t="n"/>
-      <c r="C21" s="18" t="n"/>
-      <c r="D21" s="33" t="n"/>
-      <c r="E21" s="33" t="n"/>
-      <c r="F21" s="33" t="n"/>
+      <c r="A21" s="36" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B21" s="37" t="inlineStr">
+        <is>
+          <t>Sang</t>
+        </is>
+      </c>
+      <c r="C21" s="37" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="D21" s="38" t="inlineStr">
+        <is>
+          <t>D063: sinh viên đăng ký bằng Google; seed tài khoản khi deploy</t>
+        </is>
+      </c>
+      <c r="E21" s="38" t="inlineStr">
+        <is>
+          <t>Thêm đăng ký bằng Google cho sinh viên (bút danh ngẫu nhiên, chỉ lưu băm định danh Google), lệnh seed bộ tài khoản mẫu chạy sau mỗi lần deploy, hướng dẫn tạo OAuth client trên GCP và kiểm tra .env trên máy chủ; kiểm tra web sau deploy.</t>
+        </is>
+      </c>
+      <c r="F21" s="38" t="inlineStr">
+        <is>
+          <t>https://github.com/ThanhSangLouis/ai-assessor-cefr/pull/85 (squash 096b061)</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="36" customHeight="1" s="24">
-      <c r="A22" s="20" t="n"/>
-      <c r="B22" s="18" t="n"/>
-      <c r="C22" s="18" t="n"/>
-      <c r="D22" s="33" t="n"/>
-      <c r="E22" s="33" t="n"/>
-      <c r="F22" s="33" t="n"/>
+      <c r="A22" s="36" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B22" s="37" t="inlineStr">
+        <is>
+          <t>Sang</t>
+        </is>
+      </c>
+      <c r="C22" s="37" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="D22" s="38" t="inlineStr">
+        <is>
+          <t>D064: bỏ bước đồng ý điều khoản; logo Google; cập nhật sơ đồ lớp; kiểm chấm điểm toàn bộ</t>
+        </is>
+      </c>
+      <c r="E22" s="38" t="inlineStr">
+        <is>
+          <t>Hệ thống đã phục vụ người dùng thật nên bỏ hẳn bước đồng ý điều khoản (migration 8), thêm logo Google trên nút đăng nhập, cập nhật sơ đồ lớp và ERD; chạy thử chấm điểm với Whisper và model thật trên các dạng bài, chạy kiểm thử ba tầng với ba vai trò.</t>
+        </is>
+      </c>
+      <c r="F22" s="38" t="inlineStr">
+        <is>
+          <t>https://github.com/ThanhSangLouis/ai-assessor-cefr/pull/87 (squash 46ee31c)</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="36" customHeight="1" s="24">
-      <c r="A23" s="20" t="n"/>
-      <c r="B23" s="18" t="n"/>
-      <c r="C23" s="18" t="n"/>
-      <c r="D23" s="33" t="n"/>
-      <c r="E23" s="33" t="n"/>
-      <c r="F23" s="33" t="n"/>
+      <c r="A23" s="36" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B23" s="37" t="inlineStr">
+        <is>
+          <t>Sang</t>
+        </is>
+      </c>
+      <c r="C23" s="37" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="D23" s="38" t="inlineStr">
+        <is>
+          <t>Tái hiện lỗi teammate không chạy được trên bản clone mới và sửa</t>
+        </is>
+      </c>
+      <c r="E23" s="38" t="inlineStr">
+        <is>
+          <t>Kéo code mới nhất, clone sạch và cài như máy teammate: bật Whisper khi chưa cài nhóm asr làm mọi bài FAILED mà log không nói lý do; Mac Intel cài nhầm backend; nút Google không hiện khi thiếu khoá. Sửa demo.sh báo rõ, ghi lý do vào log, sửa điều kiện cài, thêm mục bật Google ở local.</t>
+        </is>
+      </c>
+      <c r="F23" s="38" t="inlineStr">
+        <is>
+          <t>https://github.com/ThanhSangLouis/ai-assessor-cefr/pull/89</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="36" customHeight="1" s="24">
-      <c r="A24" s="20" t="n"/>
-      <c r="B24" s="18" t="n"/>
-      <c r="C24" s="18" t="n"/>
-      <c r="D24" s="33" t="n"/>
-      <c r="E24" s="33" t="n"/>
-      <c r="F24" s="33" t="n"/>
+      <c r="A24" s="36" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B24" s="37" t="inlineStr">
+        <is>
+          <t>Sang</t>
+        </is>
+      </c>
+      <c r="C24" s="37" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="D24" s="38" t="inlineStr">
+        <is>
+          <t>Rà toàn bộ xác thực và phân quyền của vai trò quản trị</t>
+        </is>
+      </c>
+      <c r="E24" s="38" t="inlineStr">
+        <is>
+          <t>Kiểm tra vai trò admin đã phủ hết các trường hợp xác thực và phân quyền: liệt kê 184 route API cùng lớp chặn, viết test gọi thử mọi route bằng khách, sinh viên, giảng viên, admin mật khẩu tạm và admin; chặn trang /admin cho người không phải admin.</t>
+        </is>
+      </c>
+      <c r="F24" s="38" t="inlineStr">
+        <is>
+          <t>https://github.com/ThanhSangLouis/ai-assessor-cefr/pull/90; tests/test_admin_access.py</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="36" customHeight="1" s="24">
-      <c r="A25" s="20" t="n"/>
-      <c r="B25" s="18" t="n"/>
-      <c r="C25" s="18" t="n"/>
-      <c r="D25" s="33" t="n"/>
-      <c r="E25" s="33" t="n"/>
-      <c r="F25" s="33" t="n"/>
+      <c r="A25" s="36" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B25" s="37" t="inlineStr">
+        <is>
+          <t>Sang</t>
+        </is>
+      </c>
+      <c r="C25" s="37" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="D25" s="38" t="inlineStr">
+        <is>
+          <t>D065: tự đăng ký bằng mật khẩu và quên mật khẩu bằng mã khôi phục</t>
+        </is>
+      </c>
+      <c r="E25" s="38" t="inlineStr">
+        <is>
+          <t>Làm tính năng đăng ký và quên mật khẩu khi hệ thống không lưu email: bút danh ngẫu nhiên, mã khôi phục dùng một lần lưu dạng băm, khoá khi đoán sai, giới hạn tốc độ; thẻ mã khôi phục ở trang Tài khoản; test tích hợp và E2E.</t>
+        </is>
+      </c>
+      <c r="F25" s="38" t="inlineStr">
+        <is>
+          <t>https://github.com/ThanhSangLouis/ai-assessor-cefr/pull/91; docs/test/TEST_PLAN_D065.md</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="36" customHeight="1" s="24">
-      <c r="A26" s="20" t="n"/>
-      <c r="B26" s="18" t="n"/>
-      <c r="C26" s="18" t="n"/>
-      <c r="D26" s="33" t="n"/>
-      <c r="E26" s="33" t="n"/>
-      <c r="F26" s="33" t="n"/>
+      <c r="A26" s="36" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B26" s="37" t="inlineStr">
+        <is>
+          <t>Sang</t>
+        </is>
+      </c>
+      <c r="C26" s="37" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="D26" s="38" t="inlineStr">
+        <is>
+          <t>Cập nhật báo cáo tuần 7 và AI Prompt Log tuần 7</t>
+        </is>
+      </c>
+      <c r="E26" s="38" t="inlineStr">
+        <is>
+          <t>Cập nhật báo cáo tiến độ tuần 7 và nhật ký sử dụng AI cho các việc ngày 29–30/10, đối chiếu từng dòng với PR thật.</t>
+        </is>
+      </c>
+      <c r="F26" s="38" t="inlineStr">
+        <is>
+          <t>docs/reports/week-07/bao-cao-tuan-07-sang.md; docs/evidence/tc2-3-ai-usage/README.md</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="36" customHeight="1" s="24">
       <c r="A27" s="20" t="n"/>
@@ -19150,7 +19392,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A2:F14"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.625" defaultRowHeight="14.25"/>
   <cols>
     <col width="24" customWidth="1" style="24" min="1" max="1"/>

</xml_diff>